<commit_message>
2. Criação da pasta 'imagens'
Realizei a criação da pasta 'imagens', onde estarão localizados alguns arquivos relacionados a imagem. Assim como, também, iniciei o processo de apresentação do projeto.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Área de Trabalho\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C70DF8B-0900-4309-9EE4-C77318665FF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C942B785-7779-4A6A-B730-733D9CADF967}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Apresentação" sheetId="3" r:id="rId1"/>
@@ -499,6 +499,272 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>168366</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>154997</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="8835496" cy="405432"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="CaixaDeTexto 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F16D9131-B0A3-F0E7-827F-539C48FC9E0C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1380639" y="345497"/>
+          <a:ext cx="8835496" cy="405432"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="2000" b="1"/>
+            <a:t>Análise Financeira das Transferências do Tottenham Hotspur (2019/20 - 2025/26)</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>60614</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>129886</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1255344" cy="327141"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="CaixaDeTexto 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BC7727EF-C1D5-58F7-6A00-6791417BC2E5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="60614" y="701386"/>
+          <a:ext cx="1255344" cy="327141"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1500" b="1"/>
+            <a:t>1. Introdução</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>60612</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>43296</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="11074979" cy="1407437"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4" name="CaixaDeTexto 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5D370021-CD04-67C3-5959-C83BAFFB0CE5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="60612" y="1186296"/>
+          <a:ext cx="11074979" cy="1407437"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200"/>
+            <a:t>	O </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1"/>
+            <a:t>Tottenham Hotspur </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0"/>
+            <a:t>é um clube</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+            <a:t> profissional de futebol fundado em 1882, localizado em Londres, Inglaterra. Reconhecido historicamente por sua tradição no futebol inglês, o clube participa da </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0"/>
+            <a:t>Premier League</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+            <a:t>, uma das ligas esportivas mais valiosas e competitivas do mundo.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+            <a:t>	Nas últimas temporadas, o Tottenham passou por importantes mudanças esportivas e financeiras, incluindo elevados investimentos no mercado de transferências, reformulação do elenco e negociações de grande impacto financeiro, como a venda de atletas estratégicos e a contratação de jogadores jovens com potencial de valorização.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+            <a:t>	Nesse contexto, o mercado de transferências tornou-se um dos principais pilares da gestão esportiva moderna, exigindo análises cada vez mais detalhadas sobre investimentos, vendas de jogadores e sustentabilidade financeira.</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>424296</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>352946</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>171000</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Imagem 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2537A6D7-BCAE-5EA4-9F35-2551E0933569}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1636569" y="2857500"/>
+          <a:ext cx="1747059" cy="3600000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -793,6 +1059,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
3. Seção 'Introdução' da Apresentação
Conclusão da seção Introdução da aba de Apresentação, onde é feita uma apresentação inicial sobre o Tottenham Hotspur.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C942B785-7779-4A6A-B730-733D9CADF967}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2DA8343-EC0C-4E09-AE41-50942E58E281}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -717,15 +717,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>424296</xdr:colOff>
+      <xdr:colOff>424297</xdr:colOff>
       <xdr:row>15</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>352946</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>171000</xdr:rowOff>
+      <xdr:colOff>595151</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>99869</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -754,8 +754,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1636569" y="2857500"/>
-          <a:ext cx="1747059" cy="3600000"/>
+          <a:off x="1627455" y="2757237"/>
+          <a:ext cx="1975591" cy="3960000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -764,6 +764,239 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>602250</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>113835</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>471604</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>177363</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Imagem 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{26EF4C72-DA2F-9572-BF40-30CA6DE32DEF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4888500" y="2733210"/>
+          <a:ext cx="5380247" cy="3992591"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:effectLst>
+          <a:softEdge rad="25400"/>
+        </a:effectLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>297655</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>51027</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2289858" cy="264560"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="8" name="CaixaDeTexto 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BB783D0A-3520-A8FE-81DB-C9BEB8E65D78}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1522298" y="6973661"/>
+          <a:ext cx="2289858" cy="264560"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1100" i="1"/>
+            <a:t>Escudo atual do Tottenham Hotspur</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>603817</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>25513</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3739485" cy="264560"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="9" name="CaixaDeTexto 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{67C620EE-9B7E-6468-8F23-6D3ADB66F364}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5502388" y="6948147"/>
+          <a:ext cx="3739485" cy="264560"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1100" i="1"/>
+            <a:t>Tottenham Hotspur Stadium,</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1100" i="1" baseline="0"/>
+            <a:t> atual estádio da equipe londrina</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1100" i="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>108659</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>83622</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1948482" cy="327141"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="10" name="CaixaDeTexto 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3B639A6B-6503-407B-8B08-590395381102}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="108659" y="7513122"/>
+          <a:ext cx="1948482" cy="327141"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1500" b="1"/>
+            <a:t>2. Objetivo do Projeto</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 

</xml_diff>

<commit_message>
4. Seção 'Objetivo do Projeto'
Conclusão da seção 'Objetivo do Projeto'.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2DA8343-EC0C-4E09-AE41-50942E58E281}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31824488-2A05-4894-B121-E0A40F184D5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -866,6 +866,7 @@
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
+          <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="pt-BR" sz="1100" i="1"/>
             <a:t>Escudo atual do Tottenham Hotspur</a:t>
@@ -924,6 +925,7 @@
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
+          <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="pt-BR" sz="1100" i="1"/>
             <a:t>Tottenham Hotspur Stadium,</a:t>
@@ -991,6 +993,84 @@
           <a:r>
             <a:rPr lang="pt-BR" sz="1500" b="1"/>
             <a:t>2. Objetivo do Projeto</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>224646</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>143774</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="11074979" cy="655949"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="11" name="CaixaDeTexto 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0F6DB5F7-4374-4779-B699-DD037B1E2E2E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="224646" y="8113672"/>
+          <a:ext cx="11074979" cy="655949"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200"/>
+            <a:t>	Este projeto tem</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" baseline="0"/>
+            <a:t> como principal objetivo </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0"/>
+            <a:t>analisar o comportamento financeiro</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+            <a:t> do Tottenham Hotspur no mercado de transferências entre as temporadas de 2019/20 e 2025/26, utilizando técnicas de limpeza, tratamento, exploração e visualização de dados.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+            <a:t>	A análise busca identificar padrões de investimento, tendências de mercado e possíveis estratégias adotadas pelo clube ao longo dos anos.</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>

</xml_diff>

<commit_message>
5. Seção 'Problemas de Negócio'
Conclusão da seção 'Problemas de Negócio'.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31824488-2A05-4894-B121-E0A40F184D5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9F62CA8-5474-4849-A541-D8F7C58CEDE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -506,7 +506,7 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>168366</xdr:colOff>
+      <xdr:colOff>168367</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>154997</xdr:rowOff>
     </xdr:from>
@@ -524,7 +524,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1380639" y="345497"/>
+          <a:off x="1393010" y="342095"/>
           <a:ext cx="8835496" cy="405432"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -583,7 +583,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="60614" y="701386"/>
+          <a:off x="60614" y="714375"/>
           <a:ext cx="1255344" cy="327141"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -628,7 +628,7 @@
       <xdr:row>6</xdr:row>
       <xdr:rowOff>43296</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="11074979" cy="1407437"/>
+    <xdr:ext cx="12331413" cy="1219565"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="4" name="CaixaDeTexto 3">
@@ -643,7 +643,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="60612" y="1186296"/>
-          <a:ext cx="11074979" cy="1407437"/>
+          <a:ext cx="12331413" cy="1219565"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1006,7 +1006,7 @@
       <xdr:row>41</xdr:row>
       <xdr:rowOff>143774</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="11074979" cy="655949"/>
+    <xdr:ext cx="12148329" cy="655949"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="11" name="CaixaDeTexto 10">
@@ -1020,8 +1020,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="224646" y="8113672"/>
-          <a:ext cx="11074979" cy="655949"/>
+          <a:off x="224646" y="7954274"/>
+          <a:ext cx="12148329" cy="655949"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1072,6 +1072,219 @@
             <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
             <a:t>	A análise busca identificar padrões de investimento, tendências de mercado e possíveis estratégias adotadas pelo clube ao longo dos anos.</a:t>
           </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>102895</xdr:colOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>169347</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2169569" cy="327141"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="12" name="CaixaDeTexto 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AB74C15D-C02A-4A02-84DD-B99CDAECFF78}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="102895" y="8741847"/>
+          <a:ext cx="2169569" cy="327141"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1500" b="1"/>
+            <a:t>3. Problemas do</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1500" b="1" baseline="0"/>
+            <a:t> Negócio</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1500" b="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>215121</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>181874</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="12148329" cy="1783180"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="13" name="CaixaDeTexto 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{79AD57C6-179F-4617-A9FA-C1D323C83959}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="215121" y="8975490"/>
+          <a:ext cx="12148329" cy="1783180"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200"/>
+            <a:t>	Durante a análise, serão investigadas algumas questões estratégicas relacionadas à</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" baseline="0"/>
+            <a:t> gestão financeira e esportiva do clube:</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200"/>
+            <a:t>• </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1"/>
+            <a:t>O Tottenham apresentou lucro ou prejuízo no mercado de transferências</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0"/>
+            <a:t> ao longo das temporadas?</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200"/>
+            <a:t>• </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1"/>
+            <a:t>Quais</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0"/>
+            <a:t> posições receberam maior volume de investimento?</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200"/>
+            <a:t>• </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1"/>
+            <a:t>O</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0"/>
+            <a:t> clube priorizou jogadores jovens ou atletas mais experientes?</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1"/>
+            <a:t>• Existe um perfil de contratação predominante em</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0"/>
+            <a:t> relação à nacionalidade dos atletas?</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1"/>
+            <a:t>• As vendas de jogadores compensaram financeiramente os investimentos realizados?</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1"/>
+            <a:t>• O perfil</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0"/>
+            <a:t> das contratações mudou ao longo das temporadas analisadas?</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1"/>
+            <a:t>• Quais negociações representaram maior impacto financeiro para o clube?</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1200" b="1" baseline="0"/>
         </a:p>
       </xdr:txBody>
     </xdr:sp>

</xml_diff>

<commit_message>
6. Seções 'Objetivos Analíticos' e 'Fonte dos Dados'
Conclusão das seções relacionadas a objetivos analíticos e fontes dos dados usados no projeto.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9F62CA8-5474-4849-A541-D8F7C58CEDE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCB77DF6-04F8-4ECF-8157-B2767E4C2F91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1252,8 +1252,12 @@
         <a:p>
           <a:pPr algn="l"/>
           <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0"/>
+            <a:t>•</a:t>
+          </a:r>
+          <a:r>
             <a:rPr lang="pt-BR" sz="1200" b="1"/>
-            <a:t>• Existe um perfil de contratação predominante em</a:t>
+            <a:t> Existe um perfil de contratação predominante em</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0"/>
@@ -1263,15 +1267,23 @@
         <a:p>
           <a:pPr algn="l"/>
           <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0"/>
+            <a:t>•</a:t>
+          </a:r>
+          <a:r>
             <a:rPr lang="pt-BR" sz="1200" b="1"/>
-            <a:t>• As vendas de jogadores compensaram financeiramente os investimentos realizados?</a:t>
+            <a:t> As vendas de jogadores compensaram financeiramente os investimentos realizados?</a:t>
           </a:r>
         </a:p>
         <a:p>
           <a:pPr algn="l"/>
           <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0"/>
+            <a:t>•</a:t>
+          </a:r>
+          <a:r>
             <a:rPr lang="pt-BR" sz="1200" b="1"/>
-            <a:t>• O perfil</a:t>
+            <a:t> O perfil</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0"/>
@@ -1281,10 +1293,521 @@
         <a:p>
           <a:pPr algn="l"/>
           <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0"/>
+            <a:t>•</a:t>
+          </a:r>
+          <a:r>
             <a:rPr lang="pt-BR" sz="1200" b="1"/>
-            <a:t>• Quais negociações representaram maior impacto financeiro para o clube?</a:t>
+            <a:t> Quais negociações representaram maior impacto financeiro para o clube?</a:t>
           </a:r>
           <a:endParaRPr lang="pt-BR" sz="1200" b="1" baseline="0"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>155690</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>131247</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1968744" cy="327141"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="14" name="CaixaDeTexto 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C8C0B1B2-3A34-4D73-9A18-CB06CE852679}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="155690" y="11180247"/>
+          <a:ext cx="1968744" cy="327141"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1500" b="1"/>
+            <a:t>4. Objetivos</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1500" b="1" baseline="0"/>
+            <a:t> Analíticos</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1500" b="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>157971</xdr:colOff>
+      <xdr:row>61</xdr:row>
+      <xdr:rowOff>31515</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="12148329" cy="1783180"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="15" name="CaixaDeTexto 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C138AC39-12F5-4772-B45A-AF48518A71D9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="157971" y="11652015"/>
+          <a:ext cx="12148329" cy="1783180"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200"/>
+            <a:t>	Para responder às questões propostas,</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" baseline="0"/>
+            <a:t> o projeto realizará:</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0"/>
+            <a:t>• Limpeza e padronização dos dados;</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0"/>
+            <a:t>• Tratamento de inconsistências e valores ausentes;</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0"/>
+            <a:t>• Conversão e normalização de valores financeiros;</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0"/>
+            <a:t>• Criação de indicadores financeiros;</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0"/>
+            <a:t>• Análise exploratória das transferências;</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0"/>
+            <a:t>• Construção</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+            <a:t> de visualizações e dashboards interativos;</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0"/>
+            <a:t>• Geração de insights financeiros e estratégicos</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>191230</xdr:colOff>
+      <xdr:row>71</xdr:row>
+      <xdr:rowOff>183202</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1782219" cy="327141"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="16" name="CaixaDeTexto 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3ACB6205-4CFC-421C-9819-82281BA4ECD7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="191230" y="13503770"/>
+          <a:ext cx="1782219" cy="327141"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1500" b="1"/>
+            <a:t>5. Fontes dos Dados</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>148252</xdr:colOff>
+      <xdr:row>74</xdr:row>
+      <xdr:rowOff>134541</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="12148329" cy="280205"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="17" name="CaixaDeTexto 16">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{77602AAC-4522-4B59-8F8C-9398EBE18384}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="148252" y="14519235"/>
+          <a:ext cx="12148329" cy="280205"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200"/>
+            <a:t>	Os dados utilizados neste projeto foram</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" baseline="0"/>
+            <a:t> obtidos por meio de plataformas públicas especializadas em futebol e mercado esportivo:</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>184669</xdr:colOff>
+      <xdr:row>76</xdr:row>
+      <xdr:rowOff>165230</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1229760" cy="280205"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="18" name="CaixaDeTexto 17">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4430E003-D00A-AF1C-8F35-41DEE617166C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="184669" y="14938699"/>
+          <a:ext cx="1229760" cy="280205"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>• </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" u="sng">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Transfermarkt;</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1200" u="sng">
+            <a:effectLst/>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>181559</xdr:colOff>
+      <xdr:row>78</xdr:row>
+      <xdr:rowOff>16327</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="905376" cy="280205"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="19" name="CaixaDeTexto 18">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A390E617-8C79-4F82-B598-BC446ECCA7EA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="181559" y="15178572"/>
+          <a:ext cx="905376" cy="280205"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>• </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" u="sng">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Sofascore</a:t>
+          </a:r>
         </a:p>
       </xdr:txBody>
     </xdr:sp>
@@ -1585,7 +2108,8 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
7. Aba 'Anotações' e 'Dados Tratados'
Criação da aba 'Anotações', que será utilizada para reunir justificativas relacionadas à tomadas de decisão que ocorreram durante a realização do projeto.

Além disso, também, dei início ao processo de tratamento de dados com formatações leves em colunas.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,20 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCB77DF6-04F8-4ECF-8157-B2767E4C2F91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C72A87F5-FE88-4217-8574-B8D653CECE69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Apresentação" sheetId="3" r:id="rId1"/>
     <sheet name="Dados Brutos" sheetId="1" r:id="rId2"/>
+    <sheet name="Dados Tratados" sheetId="4" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Dados Tratados'!$A$2:$I$2</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="150">
   <si>
     <t>temporada</t>
   </si>
@@ -441,13 +445,43 @@
   </si>
   <si>
     <t>Nottingham Forest</t>
+  </si>
+  <si>
+    <t>tipo_movimentação</t>
+  </si>
+  <si>
+    <t>valor_transferência</t>
+  </si>
+  <si>
+    <t>tipo_negociação</t>
+  </si>
+  <si>
+    <t>Qualitativa Ordinal</t>
+  </si>
+  <si>
+    <t>Qualitativa Nominal</t>
+  </si>
+  <si>
+    <t>Quantitativa Contínua</t>
+  </si>
+  <si>
+    <t>Quantitativa Discreta</t>
+  </si>
+  <si>
+    <t>Tanguy Ndombélé</t>
+  </si>
+  <si>
+    <t>Ivan Perišić</t>
+  </si>
+  <si>
+    <t>Pierre-Emile Høbjerg</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -459,6 +493,12 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -481,9 +521,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1808,6 +1857,605 @@
             </a:rPr>
             <a:t>Sofascore</a:t>
           </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>163195</xdr:colOff>
+      <xdr:row>80</xdr:row>
+      <xdr:rowOff>149331</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2363147" cy="327141"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="CaixaDeTexto 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CB7CF3C1-5A5B-47AD-B411-E2EA1B874DCC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="163195" y="15700351"/>
+          <a:ext cx="2363147" cy="327141"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1500" b="1"/>
+            <a:t>6. Apresentação do Projeto</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>97194</xdr:colOff>
+      <xdr:row>83</xdr:row>
+      <xdr:rowOff>77755</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="12148329" cy="2534668"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="20" name="CaixaDeTexto 19">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{79617BDE-CDDA-4EE1-868A-B05F9C3521DB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="97194" y="15889255"/>
+          <a:ext cx="12148329" cy="2534668"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200"/>
+            <a:t>	Este projeto contará</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" baseline="0"/>
+            <a:t> com o total de 6 abas, cada uma representando uma etapa diferente. São elas:</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>• </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Apresentação: </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>aba que</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> introduz o projeto, citando as motivações por trás da criação do mesmo e quais objetivos pretendem ser alcançados através de sua realização.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="pt-BR" sz="1200" b="0" baseline="0">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1100" b="1">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>• </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Dados</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> Brutos: </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>aba que contém os dados que serão utilizados no projeto em estado bruto, sem qualquer tipo de tratamento ou formatação.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="pt-BR" sz="1200" b="0" baseline="0">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="l" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1100" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>•</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Dados Tratados: </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>aba contendo os dados limpos e tratados, tendo passado por processos cruciais como verificação de dados ausenes e remoção de duplicatas.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="l" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:endParaRPr lang="pt-BR" sz="1200" b="0" baseline="0">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="l" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>•</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Análises: </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>aba contendo as análises que serão feitas baseando-se nas perguntas de negócio que buscam serem respondidas e nos dados tratados.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="l" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:endParaRPr lang="pt-BR" sz="1200" b="0" baseline="0">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="l" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>•</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Dashboard: </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>aba contendo o dashboard que será construído através da utilização de métricas importantes obtidas durante o processo das análises.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="l" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:endParaRPr lang="pt-BR" sz="1200" b="0" baseline="0">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="l" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>•</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Anotações: </a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1200">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+            <a:effectLst/>
+          </a:endParaRPr>
         </a:p>
       </xdr:txBody>
     </xdr:sp>
@@ -2837,4 +3485,740 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{121A8764-E71B-430A-8F79-2AFBC43701E9}">
+  <sheetPr>
+    <tabColor theme="6" tint="0.39997558519241921"/>
+  </sheetPr>
+  <dimension ref="A1:I25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="6" width="19" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>147</v>
+      </c>
+      <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3">
+        <v>22</v>
+      </c>
+      <c r="I3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" t="s">
+        <v>30</v>
+      </c>
+      <c r="F5" t="s">
+        <v>31</v>
+      </c>
+      <c r="G5" t="s">
+        <v>32</v>
+      </c>
+      <c r="H5">
+        <v>27</v>
+      </c>
+      <c r="I5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" t="s">
+        <v>36</v>
+      </c>
+      <c r="E6" t="s">
+        <v>37</v>
+      </c>
+      <c r="F6" t="s">
+        <v>38</v>
+      </c>
+      <c r="G6" t="s">
+        <v>39</v>
+      </c>
+      <c r="H6">
+        <v>25</v>
+      </c>
+      <c r="I6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" t="s">
+        <v>42</v>
+      </c>
+      <c r="D7" t="s">
+        <v>43</v>
+      </c>
+      <c r="E7" t="s">
+        <v>44</v>
+      </c>
+      <c r="F7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G7" t="s">
+        <v>46</v>
+      </c>
+      <c r="H7" t="s">
+        <v>47</v>
+      </c>
+      <c r="I7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8" t="s">
+        <v>50</v>
+      </c>
+      <c r="E8" t="s">
+        <v>51</v>
+      </c>
+      <c r="F8" t="s">
+        <v>52</v>
+      </c>
+      <c r="G8" t="s">
+        <v>53</v>
+      </c>
+      <c r="H8">
+        <v>33</v>
+      </c>
+      <c r="I8" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" t="s">
+        <v>131</v>
+      </c>
+      <c r="D9" t="s">
+        <v>133</v>
+      </c>
+      <c r="E9" t="s">
+        <v>132</v>
+      </c>
+      <c r="F9" t="s">
+        <v>134</v>
+      </c>
+      <c r="G9" t="s">
+        <v>135</v>
+      </c>
+      <c r="H9">
+        <v>28</v>
+      </c>
+      <c r="I9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" t="s">
+        <v>56</v>
+      </c>
+      <c r="D10" t="s">
+        <v>57</v>
+      </c>
+      <c r="E10" t="s">
+        <v>58</v>
+      </c>
+      <c r="F10" t="s">
+        <v>59</v>
+      </c>
+      <c r="G10" t="s">
+        <v>60</v>
+      </c>
+      <c r="H10">
+        <v>23</v>
+      </c>
+      <c r="I10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>55</v>
+      </c>
+      <c r="B11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" t="s">
+        <v>62</v>
+      </c>
+      <c r="D11" t="s">
+        <v>63</v>
+      </c>
+      <c r="E11" t="s">
+        <v>64</v>
+      </c>
+      <c r="F11" t="s">
+        <v>65</v>
+      </c>
+      <c r="G11" t="s">
+        <v>66</v>
+      </c>
+      <c r="H11">
+        <v>21</v>
+      </c>
+      <c r="I11" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>55</v>
+      </c>
+      <c r="B12" t="s">
+        <v>68</v>
+      </c>
+      <c r="C12" t="s">
+        <v>69</v>
+      </c>
+      <c r="D12" t="s">
+        <v>70</v>
+      </c>
+      <c r="E12" t="s">
+        <v>71</v>
+      </c>
+      <c r="F12" t="s">
+        <v>72</v>
+      </c>
+      <c r="G12" t="s">
+        <v>73</v>
+      </c>
+      <c r="H12">
+        <v>32</v>
+      </c>
+      <c r="I12" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B13" t="s">
+        <v>126</v>
+      </c>
+      <c r="C13" t="s">
+        <v>127</v>
+      </c>
+      <c r="D13" t="s">
+        <v>128</v>
+      </c>
+      <c r="E13" t="s">
+        <v>129</v>
+      </c>
+      <c r="F13" t="s">
+        <v>65</v>
+      </c>
+      <c r="G13" t="s">
+        <v>130</v>
+      </c>
+      <c r="H13">
+        <v>24</v>
+      </c>
+      <c r="I13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>75</v>
+      </c>
+      <c r="B14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" t="s">
+        <v>76</v>
+      </c>
+      <c r="D14" t="s">
+        <v>77</v>
+      </c>
+      <c r="E14" t="s">
+        <v>78</v>
+      </c>
+      <c r="F14" t="s">
+        <v>79</v>
+      </c>
+      <c r="G14" t="s">
+        <v>80</v>
+      </c>
+      <c r="H14">
+        <v>25</v>
+      </c>
+      <c r="I14" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>75</v>
+      </c>
+      <c r="B15" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" t="s">
+        <v>82</v>
+      </c>
+      <c r="D15" t="s">
+        <v>83</v>
+      </c>
+      <c r="E15" t="s">
+        <v>84</v>
+      </c>
+      <c r="F15" t="s">
+        <v>85</v>
+      </c>
+      <c r="G15" t="s">
+        <v>86</v>
+      </c>
+      <c r="H15" t="s">
+        <v>87</v>
+      </c>
+      <c r="I15" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>75</v>
+      </c>
+      <c r="B16" t="s">
+        <v>27</v>
+      </c>
+      <c r="C16" t="s">
+        <v>88</v>
+      </c>
+      <c r="D16" t="s">
+        <v>89</v>
+      </c>
+      <c r="E16" t="s">
+        <v>90</v>
+      </c>
+      <c r="F16" t="s">
+        <v>91</v>
+      </c>
+      <c r="G16" t="s">
+        <v>92</v>
+      </c>
+      <c r="H16">
+        <v>24</v>
+      </c>
+      <c r="I16" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>75</v>
+      </c>
+      <c r="C17" t="s">
+        <v>148</v>
+      </c>
+      <c r="E17" t="s">
+        <v>124</v>
+      </c>
+      <c r="F17" t="s">
+        <v>125</v>
+      </c>
+      <c r="H17">
+        <v>33</v>
+      </c>
+      <c r="I17" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>93</v>
+      </c>
+      <c r="B18" t="s">
+        <v>94</v>
+      </c>
+      <c r="C18" t="s">
+        <v>95</v>
+      </c>
+      <c r="D18" t="s">
+        <v>96</v>
+      </c>
+      <c r="E18" t="s">
+        <v>97</v>
+      </c>
+      <c r="F18" t="s">
+        <v>98</v>
+      </c>
+      <c r="G18" t="s">
+        <v>99</v>
+      </c>
+      <c r="H18">
+        <v>26</v>
+      </c>
+      <c r="I18" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>93</v>
+      </c>
+      <c r="B19" t="s">
+        <v>18</v>
+      </c>
+      <c r="C19" t="s">
+        <v>100</v>
+      </c>
+      <c r="D19" t="s">
+        <v>101</v>
+      </c>
+      <c r="E19" t="s">
+        <v>90</v>
+      </c>
+      <c r="F19" t="s">
+        <v>102</v>
+      </c>
+      <c r="G19" t="s">
+        <v>103</v>
+      </c>
+      <c r="H19">
+        <v>22</v>
+      </c>
+      <c r="I19" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>93</v>
+      </c>
+      <c r="B20" t="s">
+        <v>48</v>
+      </c>
+      <c r="C20" t="s">
+        <v>104</v>
+      </c>
+      <c r="D20" t="s">
+        <v>105</v>
+      </c>
+      <c r="E20" t="s">
+        <v>106</v>
+      </c>
+      <c r="F20" t="s">
+        <v>107</v>
+      </c>
+      <c r="G20" t="s">
+        <v>108</v>
+      </c>
+      <c r="H20">
+        <v>30</v>
+      </c>
+      <c r="I20" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>93</v>
+      </c>
+      <c r="B21" t="s">
+        <v>48</v>
+      </c>
+      <c r="C21" t="s">
+        <v>104</v>
+      </c>
+      <c r="D21" t="s">
+        <v>105</v>
+      </c>
+      <c r="E21" t="s">
+        <v>106</v>
+      </c>
+      <c r="F21" t="s">
+        <v>107</v>
+      </c>
+      <c r="G21" t="s">
+        <v>108</v>
+      </c>
+      <c r="H21">
+        <v>30</v>
+      </c>
+      <c r="I21" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>93</v>
+      </c>
+      <c r="B22" t="s">
+        <v>18</v>
+      </c>
+      <c r="C22" t="s">
+        <v>136</v>
+      </c>
+      <c r="D22" t="s">
+        <v>137</v>
+      </c>
+      <c r="E22" t="s">
+        <v>138</v>
+      </c>
+      <c r="F22" t="s">
+        <v>139</v>
+      </c>
+      <c r="H22">
+        <v>22</v>
+      </c>
+      <c r="I22" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>109</v>
+      </c>
+      <c r="B23" t="s">
+        <v>10</v>
+      </c>
+      <c r="C23" t="s">
+        <v>110</v>
+      </c>
+      <c r="D23" t="s">
+        <v>111</v>
+      </c>
+      <c r="E23" t="s">
+        <v>97</v>
+      </c>
+      <c r="F23" t="s">
+        <v>112</v>
+      </c>
+      <c r="G23" t="s">
+        <v>113</v>
+      </c>
+      <c r="H23">
+        <v>26</v>
+      </c>
+      <c r="I23" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>109</v>
+      </c>
+      <c r="B24" t="s">
+        <v>18</v>
+      </c>
+      <c r="C24" t="s">
+        <v>114</v>
+      </c>
+      <c r="D24" t="s">
+        <v>115</v>
+      </c>
+      <c r="E24" t="s">
+        <v>116</v>
+      </c>
+      <c r="F24" t="s">
+        <v>117</v>
+      </c>
+      <c r="G24" t="s">
+        <v>118</v>
+      </c>
+      <c r="H24" t="s">
+        <v>119</v>
+      </c>
+      <c r="I24" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>109</v>
+      </c>
+      <c r="B25" t="s">
+        <v>48</v>
+      </c>
+      <c r="C25" t="s">
+        <v>149</v>
+      </c>
+      <c r="D25" t="s">
+        <v>36</v>
+      </c>
+      <c r="E25" t="s">
+        <v>30</v>
+      </c>
+      <c r="F25" t="s">
+        <v>121</v>
+      </c>
+      <c r="G25" t="s">
+        <v>122</v>
+      </c>
+      <c r="H25">
+        <v>29</v>
+      </c>
+      <c r="I25" t="s">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:I2" xr:uid="{121A8764-E71B-430A-8F79-2AFBC43701E9}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:I25">
+    <sortCondition ref="A3:A25"/>
+  </sortState>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
17. Início das Análises
Início das Análises com as Análises Descritivas Gerais da planilha.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC968F1C-28B1-4E58-B5FF-4CEA5EBF5BA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA813A67-4545-49C7-95BE-C83D264CC3F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Apresentação" sheetId="3" r:id="rId1"/>
@@ -2222,7 +2222,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>aba contendo os dados limpos e tratados, tendo passado por processos cruciais como verificação de dados ausenes e remoção de duplicatas.</a:t>
+            <a:t>aba contendo os dados limpos e tratados, tendo passado por processos cruciais como verificação de dados ausentes e remoção de duplicatas.</a:t>
           </a:r>
         </a:p>
         <a:p>

</xml_diff>

<commit_message>
18. Começo da 1ª Análise
Começo da análise relacionada a lucro ou prejuízo.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -1,27 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA813A67-4545-49C7-95BE-C83D264CC3F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3442A26-E762-4488-A5D6-C47507F7A150}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Apresentação" sheetId="3" r:id="rId1"/>
     <sheet name="Dados Brutos" sheetId="1" r:id="rId2"/>
     <sheet name="Dados Tratados" sheetId="4" r:id="rId3"/>
-    <sheet name="Anotações" sheetId="5" r:id="rId4"/>
+    <sheet name="Análises" sheetId="6" r:id="rId4"/>
+    <sheet name="Anotações" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Dados Tratados'!$A$2:$I$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Dados Tratados'!$A$2:$I$24</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <pivotCaches>
+    <pivotCache cacheId="4" r:id="rId6"/>
+  </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -39,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="169">
   <si>
     <t>temporada</t>
   </si>
@@ -513,6 +517,39 @@
   </si>
   <si>
     <t>Empréstimo</t>
+  </si>
+  <si>
+    <t>Total de Transferências</t>
+  </si>
+  <si>
+    <t>Total de Entradas</t>
+  </si>
+  <si>
+    <t>Total de Saídas</t>
+  </si>
+  <si>
+    <t>Total de Jogadores</t>
+  </si>
+  <si>
+    <t>Total de Nacionalidades</t>
+  </si>
+  <si>
+    <t>Idade Média dos Jogadores</t>
+  </si>
+  <si>
+    <t>Total Geral</t>
+  </si>
+  <si>
+    <t>Temporadas</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Somas de Entradas e Saídas</t>
+  </si>
+  <si>
+    <t>Saldo por Temporada</t>
   </si>
 </sst>
 </file>
@@ -522,7 +559,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$£-809]#,##0.00"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -540,6 +577,14 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -562,7 +607,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -580,11 +625,145 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="41">
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1368,8 +1547,13 @@
           </a:r>
           <a:r>
             <a:rPr lang="pt-BR" sz="1200" b="1"/>
-            <a:t> As vendas de jogadores compensaram financeiramente os investimentos realizados?</a:t>
-          </a:r>
+            <a:t> Qual</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0"/>
+            <a:t> posições geraram maior retorno financeiro ao clube?</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1200" b="1"/>
         </a:p>
         <a:p>
           <a:pPr algn="l"/>
@@ -2527,6 +2711,261 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>848303</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>104775</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3234027" cy="405432"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="CaixaDeTexto 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{54F3D7A2-1728-47AF-B8F2-DC9F84FC265D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4925003" y="104775"/>
+          <a:ext cx="3234027" cy="405432"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="2000" b="1"/>
+            <a:t>Análise</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="2000" b="1" baseline="0"/>
+            <a:t> Descritiva dos Dados</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="2000" b="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>457200</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="4712251" cy="405432"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="CaixaDeTexto 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DC6DD0BC-1ECF-4085-86BC-5BBAFA85FFBE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1952625" y="1285875"/>
+          <a:ext cx="4712251" cy="405432"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="2000" b="1"/>
+            <a:t>1. Resultado</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="2000" b="1" baseline="0"/>
+            <a:t> Financeiro das Transferências</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>123168</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="9271128" cy="311496"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4" name="CaixaDeTexto 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DE15D2E5-0951-4C14-906B-6F98227F45DE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="1647168"/>
+          <a:ext cx="9271128" cy="311496"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0"/>
+            <a:t>Pergunta de Negócio: </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="1"/>
+            <a:t>O Tottenham apresentou lucro ou prejuízo no mercado de transferências ao longo das temporadas?</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>118502</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>139043</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="818815" cy="311496"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="6" name="CaixaDeTexto 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2B8224E1-89DA-44EA-BE9A-82CB0A9D9572}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="118502" y="2024199"/>
+          <a:ext cx="818815" cy="311496"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0"/>
+            <a:t>Análise: </a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>399871</xdr:colOff>
       <xdr:row>0</xdr:row>
@@ -3266,6 +3705,422 @@
     <xdr:clientData/>
   </xdr:oneCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Kaike Mendes" refreshedDate="46181.843427199077" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="22" xr:uid="{11AE0983-117D-40C8-AD52-16F3B61A0005}">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="A2:I24" sheet="Dados Tratados"/>
+  </cacheSource>
+  <cacheFields count="9">
+    <cacheField name="temporada" numFmtId="0">
+      <sharedItems count="6">
+        <s v="2019/20"/>
+        <s v="2020/21"/>
+        <s v="2021/22"/>
+        <s v="2022/23"/>
+        <s v="2023/24"/>
+        <s v="2024/25"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="tipo_movimentação" numFmtId="0">
+      <sharedItems count="2">
+        <s v="Entrada"/>
+        <s v="Saída"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="nome_jogador" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="posição" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="nacionalidade" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="clube" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="valor_transferência" numFmtId="164">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="95000000"/>
+    </cacheField>
+    <cacheField name="idade" numFmtId="1">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="18" maxValue="33"/>
+    </cacheField>
+    <cacheField name="tipo_negociação" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="22">
+  <r>
+    <x v="0"/>
+    <x v="0"/>
+    <s v="Tanguy Ndombélé"/>
+    <s v="Meio-campista"/>
+    <s v="França"/>
+    <s v="Lyon"/>
+    <n v="62000000"/>
+    <n v="22"/>
+    <s v="Compra"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="0"/>
+    <s v="Steven Bergwijn"/>
+    <s v="Atacante"/>
+    <s v="Holanda"/>
+    <s v="PSV Eindhoven"/>
+    <n v="30000000"/>
+    <n v="22"/>
+    <s v="Compra"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="1"/>
+    <s v="Christian Eriksen"/>
+    <s v="Meio-campista"/>
+    <s v="Dinamarca"/>
+    <s v="Inter Milan"/>
+    <n v="27000000"/>
+    <n v="27"/>
+    <s v="Venda"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="0"/>
+    <s v="Pierre-Emile Højbjerg"/>
+    <s v="Meio-campista"/>
+    <s v="Dinamarca"/>
+    <s v="Southampton"/>
+    <n v="16600000"/>
+    <n v="25"/>
+    <s v="Compra"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="0"/>
+    <s v="Sergio Reguilón"/>
+    <s v="Defensor"/>
+    <s v="Espanha"/>
+    <s v="Real Madrid"/>
+    <n v="30000000"/>
+    <n v="23"/>
+    <s v="Compra"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="1"/>
+    <s v="Jan Vertonghen"/>
+    <s v="Defensor"/>
+    <s v="Bélgica"/>
+    <s v="Benfica"/>
+    <n v="0"/>
+    <n v="33"/>
+    <s v="Livre"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="0"/>
+    <s v="Matt Doherty"/>
+    <s v="Defensor"/>
+    <s v="Irlanda"/>
+    <s v="Wolves"/>
+    <n v="16800000"/>
+    <n v="28"/>
+    <s v="Compra"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="0"/>
+    <s v="Cristian Romero"/>
+    <s v="Defensor"/>
+    <s v="Argentina"/>
+    <s v="Atalanta"/>
+    <n v="52000000"/>
+    <n v="23"/>
+    <s v="Compra"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="0"/>
+    <s v="Dejan Kulusevski"/>
+    <s v="Atacante"/>
+    <s v="Suécia"/>
+    <s v="Juventus"/>
+    <n v="0"/>
+    <n v="21"/>
+    <s v="Empréstimo"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="1"/>
+    <s v="Toby Alderweireld"/>
+    <s v="Defensor"/>
+    <s v="Bélgica"/>
+    <s v="Al Duhail"/>
+    <n v="13000000"/>
+    <n v="32"/>
+    <s v="Venda"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="0"/>
+    <s v="Rodrigo Bentancur"/>
+    <s v="Meio-campista"/>
+    <s v="Uruguai"/>
+    <s v="Juventus"/>
+    <n v="19000000"/>
+    <n v="24"/>
+    <s v="Compra"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <x v="0"/>
+    <s v="Richarlison"/>
+    <s v="Atacante"/>
+    <s v="Brasil"/>
+    <s v="Everton"/>
+    <n v="58000000"/>
+    <n v="25"/>
+    <s v="Compra"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <x v="0"/>
+    <s v="Yves Bissouma"/>
+    <s v="Meio-campista"/>
+    <s v="Mali"/>
+    <s v="Brighton"/>
+    <n v="29000000"/>
+    <n v="25"/>
+    <s v="Compra"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <x v="1"/>
+    <s v="Steven Bergwijn"/>
+    <s v="Atacante"/>
+    <s v="Holanda"/>
+    <s v="Ajax"/>
+    <n v="31300000"/>
+    <n v="24"/>
+    <s v="Venda"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <x v="0"/>
+    <s v="Ivan Perišić"/>
+    <s v="Atacante"/>
+    <s v="Croácia"/>
+    <s v="Inter Milan"/>
+    <n v="0"/>
+    <n v="33"/>
+    <s v="Livre"/>
+  </r>
+  <r>
+    <x v="4"/>
+    <x v="0"/>
+    <s v="James Maddison"/>
+    <s v="Meio-campista"/>
+    <s v="Inglaterra"/>
+    <s v="Leicester City"/>
+    <n v="46300000"/>
+    <n v="26"/>
+    <s v="Compra"/>
+  </r>
+  <r>
+    <x v="4"/>
+    <x v="0"/>
+    <s v="Micky van de Ven"/>
+    <s v="Defensor"/>
+    <s v="Holanda"/>
+    <s v="Wolfsburg"/>
+    <n v="40000000"/>
+    <n v="22"/>
+    <s v="Compra"/>
+  </r>
+  <r>
+    <x v="4"/>
+    <x v="1"/>
+    <s v="Harry Kane"/>
+    <s v="Atacante"/>
+    <s v="Inglaterra"/>
+    <s v="Bayern München"/>
+    <n v="95000000"/>
+    <n v="30"/>
+    <s v="Venda"/>
+  </r>
+  <r>
+    <x v="4"/>
+    <x v="0"/>
+    <s v="Brennan Johnson"/>
+    <s v="Atacante"/>
+    <s v="País De Gales"/>
+    <s v="Nottingham Forest"/>
+    <n v="47500000"/>
+    <n v="22"/>
+    <s v="Compra"/>
+  </r>
+  <r>
+    <x v="5"/>
+    <x v="0"/>
+    <s v="Dominic Solanke"/>
+    <s v="Atacante"/>
+    <s v="Inglaterra"/>
+    <s v="Bournemouth"/>
+    <n v="65000000"/>
+    <n v="26"/>
+    <s v="Compra"/>
+  </r>
+  <r>
+    <x v="5"/>
+    <x v="0"/>
+    <s v="Archie Gray"/>
+    <s v="Meio-campista"/>
+    <s v="Inglaterra"/>
+    <s v="Leeds United"/>
+    <n v="41000000"/>
+    <n v="18"/>
+    <s v="Compra"/>
+  </r>
+  <r>
+    <x v="5"/>
+    <x v="1"/>
+    <s v="Pierre-Emile Højbjerg"/>
+    <s v="Meio-campista"/>
+    <s v="Dinamarca"/>
+    <s v="Olympique Marseille"/>
+    <n v="13500000"/>
+    <n v="29"/>
+    <s v="Venda"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Temporadas" colHeaderCaption="">
+  <location ref="A14:D22" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="9">
+    <pivotField axis="axisRow" showAll="0">
+      <items count="7">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="7">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="1"/>
+  </colFields>
+  <colItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Somas de Entradas e Saídas" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
+  </dataFields>
+  <formats count="6">
+    <format dxfId="16">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="14">
+      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="12">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="10">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="1" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="8">
+      <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="6">
+      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4427,7 +5282,7 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>48</v>
@@ -5006,7 +5861,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:I2" xr:uid="{121A8764-E71B-430A-8F79-2AFBC43701E9}"/>
+  <autoFilter ref="A2:I24" xr:uid="{121A8764-E71B-430A-8F79-2AFBC43701E9}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:I25">
     <sortCondition ref="A3:A25"/>
   </sortState>
@@ -5015,6 +5870,244 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90EE7059-D724-41CB-823A-E2EAAB06413B}">
+  <sheetPr>
+    <tabColor theme="6" tint="-0.249977111117893"/>
+  </sheetPr>
+  <dimension ref="A4:H22"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="26.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.5703125" customWidth="1"/>
+    <col min="3" max="3" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="25.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="C4" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="C5" s="2">
+        <f>COUNTA('Dados Tratados'!A3:A24)</f>
+        <v>22</v>
+      </c>
+      <c r="D5" s="2">
+        <f>COUNTIF('Dados Tratados'!B:B, "Entrada")</f>
+        <v>16</v>
+      </c>
+      <c r="E5" s="2">
+        <f>COUNTIF('Dados Tratados'!B:B, "Saída")</f>
+        <v>6</v>
+      </c>
+      <c r="F5" s="2">
+        <f>COUNTA(_xlfn.UNIQUE('Dados Tratados'!C3:C24, ,))</f>
+        <v>20</v>
+      </c>
+      <c r="G5" s="2">
+        <f>COUNTA(_xlfn.UNIQUE('Dados Tratados'!E3:E24, ,))</f>
+        <v>14</v>
+      </c>
+      <c r="H5" s="5">
+        <f>AVERAGE('Dados Tratados'!H3:H24)</f>
+        <v>25.454545454545453</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G15" s="6">
+        <f>C16-B16</f>
+        <v>-65000000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B16" s="6">
+        <v>92000000</v>
+      </c>
+      <c r="C16" s="6">
+        <v>27000000</v>
+      </c>
+      <c r="D16" s="6">
+        <v>119000000</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G16" s="6">
+        <f t="shared" ref="G16:G20" si="0">C17-B17</f>
+        <v>-63400000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B17" s="6">
+        <v>63400000</v>
+      </c>
+      <c r="C17" s="6">
+        <v>0</v>
+      </c>
+      <c r="D17" s="6">
+        <v>63400000</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G17" s="6">
+        <f t="shared" si="0"/>
+        <v>-58000000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B18" s="6">
+        <v>71000000</v>
+      </c>
+      <c r="C18" s="6">
+        <v>13000000</v>
+      </c>
+      <c r="D18" s="6">
+        <v>84000000</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="G18" s="6">
+        <f t="shared" si="0"/>
+        <v>-55700000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B19" s="6">
+        <v>87000000</v>
+      </c>
+      <c r="C19" s="6">
+        <v>31300000</v>
+      </c>
+      <c r="D19" s="6">
+        <v>118300000</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="G19" s="6">
+        <f t="shared" si="0"/>
+        <v>-38800000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B20" s="6">
+        <v>133800000</v>
+      </c>
+      <c r="C20" s="6">
+        <v>95000000</v>
+      </c>
+      <c r="D20" s="6">
+        <v>228800000</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="G20" s="6">
+        <f t="shared" si="0"/>
+        <v>-92500000</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B21" s="6">
+        <v>106000000</v>
+      </c>
+      <c r="C21" s="6">
+        <v>13500000</v>
+      </c>
+      <c r="D21" s="6">
+        <v>119500000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="B22" s="6">
+        <v>553200000</v>
+      </c>
+      <c r="C22" s="6">
+        <v>179800000</v>
+      </c>
+      <c r="D22" s="6">
+        <v>733000000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF0E5432-3B5D-4EC2-9644-5CAA892A13A9}">
   <sheetPr>
     <tabColor theme="1"/>

</xml_diff>

<commit_message>
19. Andamento da 1ª Análise
Andamento da 1ª análise com introdução de gráficos e começo da conclusão/insights.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr/>
+  <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3442A26-E762-4488-A5D6-C47507F7A150}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A26CE95-8C5C-4573-B9D7-25B650683D58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="4" r:id="rId6"/>
+    <pivotCache cacheId="0" r:id="rId6"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="169">
   <si>
     <t>temporada</t>
   </si>
@@ -587,12 +587,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -607,7 +613,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -635,116 +641,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="41">
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
+  <dxfs count="6">
     <dxf>
       <alignment horizontal="center"/>
     </dxf>
@@ -774,6 +679,2180 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="pt-BR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:pivotSource>
+    <c:name>[tottenham_transferencias.xlsx]Análises!Tabela dinâmica1</c:name>
+    <c:fmtId val="0"/>
+  </c:pivotSource>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="pt-BR"/>
+              <a:t>Valores Provenientes</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="pt-BR" baseline="0"/>
+              <a:t> de</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="pt-BR"/>
+              <a:t> Entradas</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="pt-BR" baseline="0"/>
+              <a:t> e Saídas</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="pt-BR"/>
+              <a:t> por Temporada (</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="pt-BR" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0"/>
+              <a:t>£</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="pt-BR"/>
+              <a:t>)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="pt-BR"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:pivotFmts>
+      <c:pivotFmt>
+        <c:idx val="0"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:numFmt formatCode="[$£-809]#,##0" sourceLinked="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="pt-BR"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="1"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:numFmt formatCode="[$£-809]#,##0" sourceLinked="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="pt-BR"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+    </c:pivotFmts>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Análises!$B$14:$B$15</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Entrada</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:numFmt formatCode="[$£-809]#,##0" sourceLinked="0"/>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="pt-BR"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Análises!$A$16:$A$22</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>2019/20</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2020/21</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2021/22</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2022/23</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2023/24</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2024/25</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Análises!$B$16:$B$22</c:f>
+              <c:numCache>
+                <c:formatCode>[$£-809]#,##0.00</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>92000000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>63400000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>71000000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>87000000</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>133800000</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>106000000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-5D17-42E1-897A-3727A62A8404}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Análises!$C$14:$C$15</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Saída</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:numFmt formatCode="[$£-809]#,##0" sourceLinked="0"/>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="pt-BR"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Análises!$A$16:$A$22</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>2019/20</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2020/21</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2021/22</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2022/23</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2023/24</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2024/25</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Análises!$C$16:$C$22</c:f>
+              <c:numCache>
+                <c:formatCode>[$£-809]#,##0.00</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>27000000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>13000000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>31300000</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>95000000</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>13500000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-5D17-42E1-897A-3727A62A8404}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="1745656976"/>
+        <c:axId val="1745657936"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1745656976"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="pt-BR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1745657936"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1745657936"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="[$£-809]#,##0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="pt-BR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1745656976"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="pt-BR"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="pt-BR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.78740157499999996" l="0.511811024" r="0.511811024" t="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+    <c:pageSetup/>
+  </c:printSettings>
+  <c:extLst>
+    <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
+      <c14:pivotOptions>
+        <c14:dropZoneFilter val="1"/>
+        <c14:dropZoneCategories val="1"/>
+        <c14:dropZoneData val="1"/>
+        <c14:dropZoneSeries val="1"/>
+        <c14:dropZonesVisible val="1"/>
+      </c14:pivotOptions>
+    </c:ext>
+    <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{E28EC0CA-F0BB-4C9C-879D-F8772B89E7AC}">
+      <c16:pivotOptions16>
+        <c16:showExpandCollapseFieldButtons val="1"/>
+      </c16:pivotOptions16>
+    </c:ext>
+  </c:extLst>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="pt-BR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="pt-BR"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Análises!$G$15</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Saldo por Temporada</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="pt-BR"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Análises!$F$16:$F$22</c:f>
+              <c:strCache>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>2019/20</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2020/21</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2021/22</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2022/23</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2023/24</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2024/25</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Total Geral</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Análises!$G$16:$G$22</c:f>
+              <c:numCache>
+                <c:formatCode>[$£-809]#,##0.00</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>-65000000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-63400000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-58000000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-55700000</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-38800000</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-92500000</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-373400000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-EF0E-4C2E-A93D-61AB7162C937}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="1861808064"/>
+        <c:axId val="1861817184"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1861808064"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="high"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="pt-BR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1861817184"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1861817184"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="[$£-809]#,##0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="pt-BR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1861808064"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="pt-BR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.78740157499999996" l="0.511811024" r="0.511811024" t="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2954,6 +5033,351 @@
             <a:t>Análise: </a:t>
           </a:r>
           <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>635046</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>183890</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>1335200</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>8504</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Gráfico 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{66F10C5D-81A9-1C04-2DE6-3DCBEE703DE0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>644922</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>7542</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>1379141</xdr:colOff>
+      <xdr:row>70</xdr:row>
+      <xdr:rowOff>168672</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="7" name="Gráfico 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{07FDB2B2-AA8A-09CD-E88C-108D88C17356}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>113183</xdr:colOff>
+      <xdr:row>71</xdr:row>
+      <xdr:rowOff>138636</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1781963" cy="311496"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="8" name="CaixaDeTexto 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4198BE4D-298A-4180-AF5F-0EC58BFA5784}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="113183" y="13940167"/>
+          <a:ext cx="1781963" cy="311496"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0"/>
+            <a:t>Conclusão</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t> e Insights</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0"/>
+            <a:t>: </a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>74161</xdr:colOff>
+      <xdr:row>73</xdr:row>
+      <xdr:rowOff>128278</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="10458504" cy="2064796"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="9" name="CaixaDeTexto 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6E667475-6A3D-452C-91E0-F7E4682A1787}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="74161" y="13824073"/>
+          <a:ext cx="10458504" cy="2064796"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0"/>
+            <a:t>A</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t> análise financeira baseada nas movimentações do Tottenham Hotspur entre as temporadas 2019/20 e 2024/25 demonstrou que</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>o clube manteve uma forte postura no que diz respeito à aquisição de atletas, chegando a investir cerca de </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400"/>
+            <a:t>£553.2m</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" baseline="0"/>
+            <a:t> durante todo o período.</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" baseline="0"/>
+            <a:t>Em contrapartida, também conseguimos perceber que o clube gerou menos da metade deste valor com a saída de seus ativos, reunindo um</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" baseline="0"/>
+            <a:t>total de </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400"/>
+            <a:t>£179.8m.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="0"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0"/>
+            <a:t>Outro</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t> ponto chamativo foi o déficit acumulado pelo clube, chegando aos </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>£373.4m em 2024/25</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>. O ápice do fenômeno ocorreu</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t> justamente no último período analisado, onde o valor esteve na marca de </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>£92.5m. Curiosamente, este número surgiu após uma</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>constante</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> decrescente de cinco temporadas consecutivas, o que pode indicar um possível desejo de reforçar o plantel de jogadores com</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>contratações pontuais e de extrema necessidade naquele momento.</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="0"/>
         </a:p>
       </xdr:txBody>
     </xdr:sp>
@@ -4007,7 +6431,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Temporadas" colHeaderCaption="">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Temporadas" colHeaderCaption="">
   <location ref="A14:D22" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField axis="axisRow" showAll="0">
@@ -4080,37 +6504,63 @@
     <dataField name="Somas de Entradas e Saídas" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="16">
+    <format dxfId="5">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="14">
+    <format dxfId="4">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="12">
+    <format dxfId="3">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="10">
+    <format dxfId="2">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="8">
+    <format dxfId="1">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="6">
+    <format dxfId="0">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
+  <chartFormats count="2">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
@@ -5877,10 +8327,10 @@
   <dimension ref="A4:H22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.5703125" customWidth="1"/>
+    <col min="1" max="1" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17.7109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="22.5703125" bestFit="1" customWidth="1"/>
@@ -5940,12 +8390,6 @@
       <c r="B14" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="F14" s="7" t="s">
-        <v>165</v>
-      </c>
-      <c r="G14" s="7" t="s">
-        <v>168</v>
-      </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
@@ -5960,12 +8404,11 @@
       <c r="D15" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="F15" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G15" s="6">
-        <f>C16-B16</f>
-        <v>-65000000</v>
+      <c r="F15" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="G15" s="11" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
@@ -5982,11 +8425,11 @@
         <v>119000000</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="G16" s="6">
-        <f t="shared" ref="G16:G20" si="0">C17-B17</f>
-        <v>-63400000</v>
+        <f>C16-B16</f>
+        <v>-65000000</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -6003,11 +8446,11 @@
         <v>63400000</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>55</v>
+        <v>34</v>
       </c>
       <c r="G17" s="6">
-        <f t="shared" si="0"/>
-        <v>-58000000</v>
+        <f>C17-B17</f>
+        <v>-63400000</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -6024,11 +8467,11 @@
         <v>84000000</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="G18" s="6">
-        <f t="shared" si="0"/>
-        <v>-55700000</v>
+        <f>C18-B18</f>
+        <v>-58000000</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -6045,11 +8488,11 @@
         <v>118300000</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>93</v>
+        <v>75</v>
       </c>
       <c r="G19" s="6">
-        <f t="shared" si="0"/>
-        <v>-38800000</v>
+        <f>C19-B19</f>
+        <v>-55700000</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -6066,11 +8509,11 @@
         <v>228800000</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="G20" s="6">
-        <f t="shared" si="0"/>
-        <v>-92500000</v>
+        <f>C20-B20</f>
+        <v>-38800000</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -6086,6 +8529,13 @@
       <c r="D21" s="6">
         <v>119500000</v>
       </c>
+      <c r="F21" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="G21" s="6">
+        <f>C21-B21</f>
+        <v>-92500000</v>
+      </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
@@ -6099,6 +8549,13 @@
       </c>
       <c r="D22" s="6">
         <v>733000000</v>
+      </c>
+      <c r="F22" s="12" t="s">
+        <v>164</v>
+      </c>
+      <c r="G22" s="6">
+        <f>C22-B22</f>
+        <v>-373400000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
20. 1ª Análise Concluída
Primeira análise concluída.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A26CE95-8C5C-4573-B9D7-25B650683D58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2218803-D210-4827-A5EE-41C2CB0E900C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5181,11 +5181,11 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>74161</xdr:colOff>
+      <xdr:colOff>28575</xdr:colOff>
       <xdr:row>73</xdr:row>
-      <xdr:rowOff>128278</xdr:rowOff>
+      <xdr:rowOff>113860</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="10458504" cy="2064796"/>
+    <xdr:ext cx="10458504" cy="2722284"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="9" name="CaixaDeTexto 8">
@@ -5199,8 +5199,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="74161" y="13824073"/>
-          <a:ext cx="10458504" cy="2064796"/>
+          <a:off x="28575" y="14020360"/>
+          <a:ext cx="10458504" cy="2722284"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5340,7 +5340,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>constante</a:t>
+            <a:t>decrescente constante</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="pt-BR" sz="1400" baseline="0">
@@ -5352,7 +5352,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t> decrescente de cinco temporadas consecutivas, o que pode indicar um possível desejo de reforçar o plantel de jogadores com</a:t>
+            <a:t> de cinco temporadas consecutivas, o que pode indicar um possível desejo de reforçar o plantel de jogadores com</a:t>
           </a:r>
           <a:br>
             <a:rPr lang="pt-BR" sz="1400" baseline="0">
@@ -5376,6 +5376,56 @@
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
             <a:t>contratações pontuais e de extrema necessidade naquele momento.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Em resumo, o Tottenham Hotspur sofreu prejuízo no mercado de transferências ao longo das temporadas analisadas pois, em cada uma,</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>investiu mais que arrecadou.</a:t>
           </a:r>
           <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="0"/>
         </a:p>

</xml_diff>

<commit_message>
21. Anotação 1ª Análise
Anotação sobre o que foi feito na primeira análise.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2218803-D210-4827-A5EE-41C2CB0E900C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBE32923-4F9E-40C0-BC79-50088556ABAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Apresentação" sheetId="3" r:id="rId1"/>
@@ -644,7 +644,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5433,6 +5433,133 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>262649</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>127309</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="4358565" cy="405432"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="10" name="CaixaDeTexto 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ADD2323A-2ACC-4756-82FC-396F30129351}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="15215102" y="1259526"/>
+          <a:ext cx="4358565" cy="405432"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="2000" b="1" baseline="0"/>
+            <a:t>2. Volume de Investimento por Posição</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>7518</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>110048</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="6052491" cy="311496"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="11" name="CaixaDeTexto 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{69AB0A73-C9BA-48BB-9A2A-B059995BA2FB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="14342643" y="1634048"/>
+          <a:ext cx="6052491" cy="311496"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0"/>
+            <a:t>Pergunta de Negócio: </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="1"/>
+            <a:t>Quais posições receberam</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="1" baseline="0"/>
+            <a:t> maior volume de investimento?</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -5634,6 +5761,711 @@
             <a:rPr lang="pt-BR" sz="1200" baseline="0"/>
             <a:t> planilha, foi identificada uma duplicação de cabeçalho, onde os nomes das colunas acabaram sendo introduzidos nos campos de valores da planilha. A decisão tomada nesta ocasião foi excluir a linha, visto que a mesma não possuía dados relevantes.</a:t>
           </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200"/>
+            <a:t> </a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200"/>
+            <a:t>• Na coluna </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1"/>
+            <a:t>'temporada'</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0"/>
+            <a:t>, </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+            <a:t>todos os dados que não seguiam o padrão (YYYY/YY) foram formatados para que fossem apresentados desta maneira. Foi utilizada a ferramenta Localizar e Selecionar para substituir ocorrências onde o sinal de traço - estava presente ao invés do sinal de barra /.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>• </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Na</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> coluna </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>'tipo_movimentação'</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>, existem apenas dois valores: Entrada ou Saída. Contudo, haviam ocorrências de valores semelhantes escritos de formas diferentes, como ENTRADA e saida, por exemplo. Em vista disso, foi criada uma nova coluna com o mesmo nome porém com a formatação de todos os valores com a fórmula </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>=PRI.MAIÚSCULA()</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> para padronizar com a primeira letra maiúscula. Além disso, houveram a presença de dados ausentes. Como a base de dados não é tão grande, a decisão tomada foi pesquisar e incluir os dados faltantes na planilha.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="pt-BR" sz="1200" b="0" baseline="0">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>• </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>A coluna </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>'nome_jogador' </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>apresentou inconsistências como</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> falta de acentos e traços em nomes de determinados jogadores e elas foram resolvidas à mão. Analisando a variável, também conseguimos identificar a presença de um valor duplicado no caso do jogador Harry Kane e tratamos de excluí-lo com o auxílio da ferramenta Remover Duplicatas. Novamente, utilizamos a fórmula </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>=PRI.MAIÚSCULA() </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>para formatar corretamente o texto.</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1200" b="0"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="pt-BR" sz="1200"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>• </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Na</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> coluna </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>'posição'</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>, foi identificada a presença de diversas posições distribuídas inconsistentemente. Em busca de padronizar os valores desta coluna, os mesmos foram modificados para que seguissem uma de três categorias: Defensor, Meio-campista ou Atacante. Desta forma, eles estarão em melhor estado quando as análises forem realizadas.</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1200"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="pt-BR" sz="1200"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200"/>
+            <a:t>• Semelhantemente</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" baseline="0"/>
+            <a:t> às outras colunas, </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0"/>
+            <a:t>'nacionalidade'</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+            <a:t> também apresentou registros inconsistentes quanto a formatação de letras maiúsculas, minúsculas e espaços desnecessários. Ambos os problemas foram resolvidos através da combinação das fórmulas </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0"/>
+            <a:t>=ARRUMAR() </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+            <a:t>e </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0"/>
+            <a:t>=PRI.MAIÚSCULA()</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+            <a:t>.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="pt-BR" sz="1200"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1100" b="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>• </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Em</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>'clube'</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>, apenas pequenas correções relacionadas aos nomes dos clubes foram realizadas.</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1200"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="pt-BR" sz="1200"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1100" b="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>• </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Na</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> coluna </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>'valor_transferencia'</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>, foi possível identificar diversas inconsistências. Primeiramente, os dados estavam disponibilizados em formatos monetários diferentes (por exemplo, 35M e 45.000.000 na mesma coluna), o que nos levou a modificar cada um dos registros manualmente. Esta decisão foi tomada considerando, principalmente, o tamanho da base de dados. Caso a mesma fosse maior, seria necessária outra abordagem. Em seguida, formatamos os valores como Número e para Moeda. Alguns jogadores estão com instâncias onde o 0 está presente, o que indica que sua entrada/saída não custou dinheiro ao clube.</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1200"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="pt-BR" sz="1200"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0"/>
+            <a:t>•</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1"/>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0"/>
+            <a:t>Em</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+            <a:t> relação à coluna </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0"/>
+            <a:t>'idade'</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+            <a:t>, foi necessário formatá-la inteiramente como Número para que seus valores assumissem o tipo correto.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0"/>
+            <a:t>•</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1"/>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0"/>
+            <a:t>Na</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+            <a:t> coluna </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0"/>
+            <a:t>'tipo_negociacao'</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+            <a:t>, foram utilizadas as fórmulas </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0"/>
+            <a:t>=ARRUMAR()</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+            <a:t> e </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0"/>
+            <a:t>=PRI.MAIÚSCULA() </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+            <a:t>para formatarmos os valores.</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1200" b="0"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>182274</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1089722" cy="327141"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="CaixaDeTexto 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6C786A4C-B0FC-4E5F-AD02-BC4A3FA750C2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="182274" y="7448550"/>
+          <a:ext cx="1089722" cy="327141"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1500" b="1"/>
+            <a:t>2. Análises:</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>190500</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="12148329" cy="6479979"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="6" name="CaixaDeTexto 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B3276CCD-3451-4463-A90F-1B3080FC64A9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="190500" y="7867650"/>
+          <a:ext cx="12148329" cy="6479979"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200"/>
+            <a:t>• </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1"/>
+            <a:t>1ª</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0"/>
+            <a:t> análise: </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+            <a:t>No processo da primeira análise, criei uma tabela dinâmica baseando-se em três colunas essenciais: </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0"/>
+            <a:t>temporada</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+            <a:t>, </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0"/>
+            <a:t>tipo_movimentação </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+            <a:t>e </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0"/>
+            <a:t>valor_transferência</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+            <a:t>. Utilizei tipo_movimentação como coluna para disponibilizar as duas categorias presentes nela: "Entrada" ou "Saída". Desta forma, cada uma seria apresentada como uma coluna diferente na visualização da tabela dinâmica. Por fim, incluí valor_transferência no campo de valores para mostrar cada cifra no formato de soma.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
+            <a:t>Após isso, criei uma tabela adjacente que demonstra de forma explícita os saldos ao final de cada temporada. Baseando-se nas duas tabelas, criei gráficos dinâmicos que representam visualmente estes valores.</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1200" baseline="0"/>
         </a:p>
         <a:p>
           <a:pPr algn="l"/>
@@ -8478,7 +9310,7 @@
         <v>9</v>
       </c>
       <c r="G16" s="6">
-        <f>C16-B16</f>
+        <f t="shared" ref="G16:G22" si="0">C16-B16</f>
         <v>-65000000</v>
       </c>
     </row>
@@ -8499,7 +9331,7 @@
         <v>34</v>
       </c>
       <c r="G17" s="6">
-        <f>C17-B17</f>
+        <f t="shared" si="0"/>
         <v>-63400000</v>
       </c>
     </row>
@@ -8520,7 +9352,7 @@
         <v>55</v>
       </c>
       <c r="G18" s="6">
-        <f>C18-B18</f>
+        <f t="shared" si="0"/>
         <v>-58000000</v>
       </c>
     </row>
@@ -8541,7 +9373,7 @@
         <v>75</v>
       </c>
       <c r="G19" s="6">
-        <f>C19-B19</f>
+        <f t="shared" si="0"/>
         <v>-55700000</v>
       </c>
     </row>
@@ -8562,7 +9394,7 @@
         <v>93</v>
       </c>
       <c r="G20" s="6">
-        <f>C20-B20</f>
+        <f t="shared" si="0"/>
         <v>-38800000</v>
       </c>
     </row>
@@ -8583,7 +9415,7 @@
         <v>109</v>
       </c>
       <c r="G21" s="6">
-        <f>C21-B21</f>
+        <f t="shared" si="0"/>
         <v>-92500000</v>
       </c>
     </row>
@@ -8604,7 +9436,7 @@
         <v>164</v>
       </c>
       <c r="G22" s="6">
-        <f>C22-B22</f>
+        <f t="shared" si="0"/>
         <v>-373400000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
23. Anotações sobre a Segunda Análise
Anotações e justificativas sobre a segunda análise.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD420858-ACB3-4AC1-BCF5-2FD571E1725C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08D515FF-8892-4E15-9813-41109F1A6D23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="2" r:id="rId6"/>
+    <pivotCache cacheId="0" r:id="rId6"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -570,7 +570,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="[$£-809]#,##0.00"/>
-    <numFmt numFmtId="167" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -626,7 +626,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -658,43 +658,17 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="52">
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
+  <dxfs count="15">
     <dxf>
       <alignment horizontal="general"/>
     </dxf>
@@ -718,93 +692,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general"/>
     </dxf>
     <dxf>
       <alignment horizontal="center"/>
@@ -2446,7 +2333,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="pt-BR"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -2483,6 +2370,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-CAE7-401C-9C6F-FAC5569D804B}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
@@ -2498,6 +2390,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-CAE7-401C-9C6F-FAC5569D804B}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="2"/>
@@ -2513,6 +2410,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-CAE7-401C-9C6F-FAC5569D804B}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dLbls>
             <c:spPr>
@@ -8560,7 +8462,7 @@
       <xdr:row>41</xdr:row>
       <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="12148329" cy="6479979"/>
+    <xdr:ext cx="12148329" cy="7231467"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="6" name="CaixaDeTexto 5">
@@ -8575,7 +8477,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="190500" y="7867650"/>
-          <a:ext cx="12148329" cy="6479979"/>
+          <a:ext cx="12148329" cy="7231467"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -8651,10 +8553,153 @@
         <a:p>
           <a:pPr algn="l"/>
           <a:r>
-            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
-            <a:t>Após isso, criei uma tabela adjacente que demonstra de forma explícita os saldos ao final de cada temporada. Baseando-se nas duas tabelas, criei gráficos dinâmicos que representam visualmente estes valores.</a:t>
-          </a:r>
-          <a:endParaRPr lang="pt-BR" sz="1200" baseline="0"/>
+            <a:rPr lang="pt-BR" sz="1200">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>• </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>2ª</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> análise: </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Na segunda análise, utilizei a variável </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>posição</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> juntamente à coluna </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>tipo_movimentação</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> filtrada pelo valor "Entrada" para especificar que eu desejava obter apenas os dados de quem chegou ao clube. Em seguida, no campo de Valores, introduzi as cifras somadas destes jogadores através da inserção de </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>valor_transferência</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> na tabela dinâmica. Semelhante à análise anterior, também criei uma tabela adjacente porém contendo todas as posições dos jogadores e o quanto seus percentuais representavam em relação ao total. Para tanto, selecionei individualmente cada valor pela posição e dividi pelo resultado da soma entre todos.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="pt-BR" sz="1200" b="0" baseline="0">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Optei pelos gráficos de barras agrupadas e pizza pois contávamos com poucas categorias, o que se encaixava bem com a proposta de cada tipo de gráfico.</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
         </a:p>
         <a:p>
           <a:pPr algn="l"/>
@@ -9506,7 +9551,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
   <location ref="O14:P19" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField showAll="0"/>
@@ -9573,39 +9618,39 @@
     <dataField name="Soma do Valor das Transferências" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="0">
+    <format dxfId="8">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="1">
+    <format dxfId="7">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="2">
+    <format dxfId="6">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="3">
+    <format dxfId="5">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
     <format dxfId="4">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="5">
+    <format dxfId="3">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="6">
+    <format dxfId="2">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="7">
+    <format dxfId="1">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="8">
+    <format dxfId="0">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -9633,7 +9678,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Temporadas" colHeaderCaption="">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Temporadas" colHeaderCaption="">
   <location ref="A14:D22" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField axis="axisRow" showAll="0">
@@ -9706,34 +9751,34 @@
     <dataField name="Somas de Entradas e Saídas" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="51">
+    <format dxfId="14">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="50">
+    <format dxfId="13">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="49">
+    <format dxfId="12">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="48">
+    <format dxfId="11">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="47">
+    <format dxfId="10">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="46">
+    <format dxfId="9">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -11665,7 +11710,7 @@
       <c r="R16" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="S16" s="15">
+      <c r="S16" s="13">
         <f>P16/$P$19</f>
         <v>0.3866594360086768</v>
       </c>
@@ -11699,7 +11744,7 @@
       <c r="R17" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="S17" s="15">
+      <c r="S17" s="13">
         <f>P17/$P$19</f>
         <v>0.36243673174258856</v>
       </c>
@@ -11733,7 +11778,7 @@
       <c r="R18" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="S18" s="15">
+      <c r="S18" s="13">
         <f>P18/$P$19</f>
         <v>0.25090383224873464</v>
       </c>
@@ -11758,16 +11803,16 @@
         <f t="shared" si="0"/>
         <v>-55700000</v>
       </c>
-      <c r="O19" s="13" t="s">
+      <c r="O19" t="s">
         <v>164</v>
       </c>
       <c r="P19" s="6">
         <v>553200000</v>
       </c>
-      <c r="R19" s="14" t="s">
+      <c r="R19" s="12" t="s">
         <v>164</v>
       </c>
-      <c r="S19" s="16">
+      <c r="S19" s="14">
         <f>P19/$P$19</f>
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
24. Insights (2ª Análise)
Insights da segunda análise.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08D515FF-8892-4E15-9813-41109F1A6D23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A34317A1-8EC2-4DA9-9BB6-38844348299A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7651,6 +7651,282 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>581025</xdr:colOff>
+      <xdr:row>62</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1781963" cy="311496"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="15" name="CaixaDeTexto 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6B9B4CC9-E9A1-43A9-999E-E228B5EABAC3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="13077825" y="11938000"/>
+          <a:ext cx="1781963" cy="311496"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0"/>
+            <a:t>Conclusão</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t> e Insights</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0"/>
+            <a:t>: </a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>568050</xdr:colOff>
+      <xdr:row>64</xdr:row>
+      <xdr:rowOff>129560</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="10272749" cy="2064796"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="16" name="CaixaDeTexto 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{385B74E8-2973-4604-90FA-73736C5B9397}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="13067366" y="12206541"/>
+          <a:ext cx="10272749" cy="2064796"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>A análise dos investimentos por posições realizados pelo Tottenham Hotspur demonstrou que os meio-campistas receberam o maior</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>volume de recursos financeiros durante o período analisado, concentrando cerca de </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>38,7% </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>do total. Logo em seguida, temos os atacantes,</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>reunindo </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>36,2%</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t> e, por fim, os defensores, para os quais foram direcionados </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>25,1%</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>. Apesar dos meio-campistas liderarem o ranking,</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>a diferença em relação aos atacantes é de apenas </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>2,5%</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>, indicando uma distribuição relativamente equilibrada dos recursos destinados</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>a estes setores do campo.</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="0"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Em conjunto, meio-campistas e atacantes representaram aproximadamente </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>75%</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> dos investimentos realizados pelo clube, sugerindo uma</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>estratégia voltada à consolidação dos setores de criação e conclusão das jogadas, que concentraram parcela superior dos recursos</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>destinados às contratações.</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 

</xml_diff>

<commit_message>
25. Começo da 3ª Análise
Começo da terceira análise.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A34317A1-8EC2-4DA9-9BB6-38844348299A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF4C21BF-C0AE-46F5-B1A8-EDF52E14F9ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,11 +20,11 @@
     <sheet name="Anotações" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Dados Tratados'!$A$2:$I$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Dados Tratados'!$A$2:$J$24</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId6"/>
+    <pivotCache cacheId="3" r:id="rId6"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="179">
   <si>
     <t>temporada</t>
   </si>
@@ -562,6 +562,24 @@
   </si>
   <si>
     <t>Porcentagem (%) do Total</t>
+  </si>
+  <si>
+    <t>16-20</t>
+  </si>
+  <si>
+    <t>21-25</t>
+  </si>
+  <si>
+    <t>26-30</t>
+  </si>
+  <si>
+    <t>31-35</t>
+  </si>
+  <si>
+    <t>Faixa Etária</t>
+  </si>
+  <si>
+    <t>faixa_etária</t>
   </si>
 </sst>
 </file>
@@ -626,7 +644,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -664,11 +682,78 @@
     <xf numFmtId="165" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="15">
+  <dxfs count="36">
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
     <dxf>
       <alignment horizontal="general"/>
     </dxf>
@@ -7927,6 +8012,188 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>593286</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>188176</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="4305794" cy="405432"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="17" name="CaixaDeTexto 16">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BB23360E-3363-4B90-8200-4B643BDF7E29}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="26891811" y="1331176"/>
+          <a:ext cx="4305794" cy="405432"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="2000" b="1" baseline="0"/>
+            <a:t>3. Priorização por Jovens ou Veteranos</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>179646</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="7407734" cy="311496"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="18" name="CaixaDeTexto 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B6AEFFB1-CB89-40A3-ACF7-6E74306948B6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="25278021" y="1657350"/>
+          <a:ext cx="7407734" cy="311496"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0"/>
+            <a:t>Pergunta de Negócio: </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="1"/>
+            <a:t>O clube priorizou a contratação de jogadores jovens ou mais experientes?</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="818815" cy="311496"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="20" name="CaixaDeTexto 19">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BBC96D07-6941-4884-8AFF-35016342CB85}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="25774650" y="2038350"/>
+          <a:ext cx="818815" cy="311496"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0"/>
+            <a:t>Análise: </a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -9526,7 +9793,7 @@
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Kaike Mendes" refreshedDate="46181.843427199077" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="22" xr:uid="{11AE0983-117D-40C8-AD52-16F3B61A0005}">
   <cacheSource type="worksheet">
-    <worksheetSource ref="A2:I24" sheet="Dados Tratados"/>
+    <worksheetSource ref="A2:J24" sheet="Dados Tratados"/>
   </cacheSource>
   <cacheFields count="9">
     <cacheField name="temporada" numFmtId="0">
@@ -9565,7 +9832,35 @@
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="95000000"/>
     </cacheField>
     <cacheField name="idade" numFmtId="1">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="18" maxValue="33"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="18" maxValue="33" count="13">
+        <n v="22"/>
+        <n v="27"/>
+        <n v="25"/>
+        <n v="23"/>
+        <n v="33"/>
+        <n v="28"/>
+        <n v="21"/>
+        <n v="32"/>
+        <n v="24"/>
+        <n v="26"/>
+        <n v="30"/>
+        <n v="18"/>
+        <n v="29"/>
+      </sharedItems>
+      <fieldGroup base="7">
+        <rangePr autoStart="0" autoEnd="0" startNum="1" endNum="33" groupInterval="5"/>
+        <groupItems count="9">
+          <s v="&lt;1"/>
+          <s v="1-5"/>
+          <s v="6-10"/>
+          <s v="11-15"/>
+          <s v="16-20"/>
+          <s v="21-25"/>
+          <s v="26-30"/>
+          <s v="31-35"/>
+          <s v="&gt;36"/>
+        </groupItems>
+      </fieldGroup>
     </cacheField>
     <cacheField name="tipo_negociação" numFmtId="0">
       <sharedItems/>
@@ -9589,7 +9884,7 @@
     <s v="França"/>
     <s v="Lyon"/>
     <n v="62000000"/>
-    <n v="22"/>
+    <x v="0"/>
     <s v="Compra"/>
   </r>
   <r>
@@ -9600,7 +9895,7 @@
     <s v="Holanda"/>
     <s v="PSV Eindhoven"/>
     <n v="30000000"/>
-    <n v="22"/>
+    <x v="0"/>
     <s v="Compra"/>
   </r>
   <r>
@@ -9611,7 +9906,7 @@
     <s v="Dinamarca"/>
     <s v="Inter Milan"/>
     <n v="27000000"/>
-    <n v="27"/>
+    <x v="1"/>
     <s v="Venda"/>
   </r>
   <r>
@@ -9622,7 +9917,7 @@
     <s v="Dinamarca"/>
     <s v="Southampton"/>
     <n v="16600000"/>
-    <n v="25"/>
+    <x v="2"/>
     <s v="Compra"/>
   </r>
   <r>
@@ -9633,7 +9928,7 @@
     <s v="Espanha"/>
     <s v="Real Madrid"/>
     <n v="30000000"/>
-    <n v="23"/>
+    <x v="3"/>
     <s v="Compra"/>
   </r>
   <r>
@@ -9644,7 +9939,7 @@
     <s v="Bélgica"/>
     <s v="Benfica"/>
     <n v="0"/>
-    <n v="33"/>
+    <x v="4"/>
     <s v="Livre"/>
   </r>
   <r>
@@ -9655,7 +9950,7 @@
     <s v="Irlanda"/>
     <s v="Wolves"/>
     <n v="16800000"/>
-    <n v="28"/>
+    <x v="5"/>
     <s v="Compra"/>
   </r>
   <r>
@@ -9666,7 +9961,7 @@
     <s v="Argentina"/>
     <s v="Atalanta"/>
     <n v="52000000"/>
-    <n v="23"/>
+    <x v="3"/>
     <s v="Compra"/>
   </r>
   <r>
@@ -9677,7 +9972,7 @@
     <s v="Suécia"/>
     <s v="Juventus"/>
     <n v="0"/>
-    <n v="21"/>
+    <x v="6"/>
     <s v="Empréstimo"/>
   </r>
   <r>
@@ -9688,7 +9983,7 @@
     <s v="Bélgica"/>
     <s v="Al Duhail"/>
     <n v="13000000"/>
-    <n v="32"/>
+    <x v="7"/>
     <s v="Venda"/>
   </r>
   <r>
@@ -9699,7 +9994,7 @@
     <s v="Uruguai"/>
     <s v="Juventus"/>
     <n v="19000000"/>
-    <n v="24"/>
+    <x v="8"/>
     <s v="Compra"/>
   </r>
   <r>
@@ -9710,7 +10005,7 @@
     <s v="Brasil"/>
     <s v="Everton"/>
     <n v="58000000"/>
-    <n v="25"/>
+    <x v="2"/>
     <s v="Compra"/>
   </r>
   <r>
@@ -9721,7 +10016,7 @@
     <s v="Mali"/>
     <s v="Brighton"/>
     <n v="29000000"/>
-    <n v="25"/>
+    <x v="2"/>
     <s v="Compra"/>
   </r>
   <r>
@@ -9732,7 +10027,7 @@
     <s v="Holanda"/>
     <s v="Ajax"/>
     <n v="31300000"/>
-    <n v="24"/>
+    <x v="8"/>
     <s v="Venda"/>
   </r>
   <r>
@@ -9743,7 +10038,7 @@
     <s v="Croácia"/>
     <s v="Inter Milan"/>
     <n v="0"/>
-    <n v="33"/>
+    <x v="4"/>
     <s v="Livre"/>
   </r>
   <r>
@@ -9754,7 +10049,7 @@
     <s v="Inglaterra"/>
     <s v="Leicester City"/>
     <n v="46300000"/>
-    <n v="26"/>
+    <x v="9"/>
     <s v="Compra"/>
   </r>
   <r>
@@ -9765,7 +10060,7 @@
     <s v="Holanda"/>
     <s v="Wolfsburg"/>
     <n v="40000000"/>
-    <n v="22"/>
+    <x v="0"/>
     <s v="Compra"/>
   </r>
   <r>
@@ -9776,7 +10071,7 @@
     <s v="Inglaterra"/>
     <s v="Bayern München"/>
     <n v="95000000"/>
-    <n v="30"/>
+    <x v="10"/>
     <s v="Venda"/>
   </r>
   <r>
@@ -9787,7 +10082,7 @@
     <s v="País De Gales"/>
     <s v="Nottingham Forest"/>
     <n v="47500000"/>
-    <n v="22"/>
+    <x v="0"/>
     <s v="Compra"/>
   </r>
   <r>
@@ -9798,7 +10093,7 @@
     <s v="Inglaterra"/>
     <s v="Bournemouth"/>
     <n v="65000000"/>
-    <n v="26"/>
+    <x v="9"/>
     <s v="Compra"/>
   </r>
   <r>
@@ -9809,7 +10104,7 @@
     <s v="Inglaterra"/>
     <s v="Leeds United"/>
     <n v="41000000"/>
-    <n v="18"/>
+    <x v="11"/>
     <s v="Compra"/>
   </r>
   <r>
@@ -9820,14 +10115,96 @@
     <s v="Dinamarca"/>
     <s v="Olympique Marseille"/>
     <n v="13500000"/>
-    <n v="29"/>
+    <x v="12"/>
     <s v="Venda"/>
   </r>
 </pivotCacheRecords>
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{996EC5F2-74EB-477F-A9D9-AF44A2544855}" name="Tabela dinâmica3" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Faixa Etária">
+  <location ref="Y14:Y19" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="9">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item h="1" x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField axis="axisRow" numFmtId="1" showAll="0">
+      <items count="10">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="7"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <formats count="1">
+    <format dxfId="5">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="7" count="4">
+            <x v="4"/>
+            <x v="5"/>
+            <x v="6"/>
+            <x v="7"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
   <location ref="O14:P19" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField showAll="0"/>
@@ -9862,7 +10239,20 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField dataField="1" numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0">
+      <items count="10">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField showAll="0"/>
   </pivotFields>
   <rowFields count="1">
@@ -9894,39 +10284,39 @@
     <dataField name="Soma do Valor das Transferências" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="8">
+    <format dxfId="29">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="7">
+    <format dxfId="28">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="6">
+    <format dxfId="27">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="5">
+    <format dxfId="26">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="4">
+    <format dxfId="25">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="3">
+    <format dxfId="24">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="2">
+    <format dxfId="23">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="1">
+    <format dxfId="22">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="0">
+    <format dxfId="21">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -9953,8 +10343,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Temporadas" colHeaderCaption="">
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Temporadas" colHeaderCaption="">
   <location ref="A14:D22" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField axis="axisRow" showAll="0">
@@ -9980,7 +10370,20 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField dataField="1" numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0">
+      <items count="10">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField showAll="0"/>
   </pivotFields>
   <rowFields count="1">
@@ -10027,34 +10430,34 @@
     <dataField name="Somas de Entradas e Saídas" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="14">
+    <format dxfId="35">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="13">
+    <format dxfId="34">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="12">
+    <format dxfId="33">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="11">
+    <format dxfId="32">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="10">
+    <format dxfId="31">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="9">
+    <format dxfId="30">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -11124,7 +11527,7 @@
   <sheetPr>
     <tabColor theme="6" tint="0.39997558519241921"/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
@@ -11133,11 +11536,13 @@
     <col min="5" max="5" width="20.42578125" customWidth="1"/>
     <col min="6" max="6" width="19.85546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="23" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.85546875" customWidth="1"/>
+    <col min="10" max="10" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>143</v>
       </c>
@@ -11163,10 +11568,13 @@
         <v>146</v>
       </c>
       <c r="I1" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="J1" s="2" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -11191,11 +11599,14 @@
       <c r="H2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="I2" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="J2" s="4" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>9</v>
       </c>
@@ -11220,11 +11631,15 @@
       <c r="H3" s="5">
         <v>22</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="5" t="str">
+        <f>IF(H3&lt;=20,"Muito Jovem",IF(AND(H3&gt;=21,H3&lt;=25),"Jovem",IF(AND(H3&gt;=26,H3&lt;=30),"Experiente",IF(H3&gt;31,"Veterano"))))</f>
+        <v>Jovem</v>
+      </c>
+      <c r="J3" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
@@ -11249,11 +11664,15 @@
       <c r="H4" s="5">
         <v>22</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="I4" s="5" t="str">
+        <f t="shared" ref="I4:I24" si="0">IF(H4&lt;=20,"Muito Jovem",IF(AND(H4&gt;=21,H4&lt;=25),"Jovem",IF(AND(H4&gt;=26,H4&lt;=30),"Experiente",IF(H4&gt;31,"Veterano"))))</f>
+        <v>Jovem</v>
+      </c>
+      <c r="J4" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>9</v>
       </c>
@@ -11278,11 +11697,15 @@
       <c r="H5" s="5">
         <v>27</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="I5" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Experiente</v>
+      </c>
+      <c r="J5" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>34</v>
       </c>
@@ -11307,11 +11730,15 @@
       <c r="H6" s="5">
         <v>25</v>
       </c>
-      <c r="I6" s="2" t="s">
+      <c r="I6" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Jovem</v>
+      </c>
+      <c r="J6" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>34</v>
       </c>
@@ -11336,11 +11763,15 @@
       <c r="H7" s="5">
         <v>23</v>
       </c>
-      <c r="I7" s="2" t="s">
+      <c r="I7" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Jovem</v>
+      </c>
+      <c r="J7" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>34</v>
       </c>
@@ -11365,11 +11796,15 @@
       <c r="H8" s="5">
         <v>33</v>
       </c>
-      <c r="I8" s="2" t="s">
+      <c r="I8" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Veterano</v>
+      </c>
+      <c r="J8" s="2" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>34</v>
       </c>
@@ -11394,11 +11829,15 @@
       <c r="H9" s="5">
         <v>28</v>
       </c>
-      <c r="I9" s="2" t="s">
+      <c r="I9" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Experiente</v>
+      </c>
+      <c r="J9" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>55</v>
       </c>
@@ -11423,11 +11862,15 @@
       <c r="H10" s="5">
         <v>23</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="I10" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Jovem</v>
+      </c>
+      <c r="J10" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>55</v>
       </c>
@@ -11452,11 +11895,15 @@
       <c r="H11" s="5">
         <v>21</v>
       </c>
-      <c r="I11" s="2" t="s">
+      <c r="I11" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Jovem</v>
+      </c>
+      <c r="J11" s="2" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>55</v>
       </c>
@@ -11481,11 +11928,15 @@
       <c r="H12" s="5">
         <v>32</v>
       </c>
-      <c r="I12" s="2" t="s">
+      <c r="I12" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Veterano</v>
+      </c>
+      <c r="J12" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>55</v>
       </c>
@@ -11510,11 +11961,15 @@
       <c r="H13" s="5">
         <v>24</v>
       </c>
-      <c r="I13" s="2" t="s">
+      <c r="I13" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Jovem</v>
+      </c>
+      <c r="J13" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>75</v>
       </c>
@@ -11539,11 +11994,15 @@
       <c r="H14" s="5">
         <v>25</v>
       </c>
-      <c r="I14" s="2" t="s">
+      <c r="I14" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Jovem</v>
+      </c>
+      <c r="J14" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>75</v>
       </c>
@@ -11568,11 +12027,15 @@
       <c r="H15" s="5">
         <v>25</v>
       </c>
-      <c r="I15" s="2" t="s">
+      <c r="I15" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Jovem</v>
+      </c>
+      <c r="J15" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>75</v>
       </c>
@@ -11597,11 +12060,15 @@
       <c r="H16" s="5">
         <v>24</v>
       </c>
-      <c r="I16" s="2" t="s">
+      <c r="I16" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Jovem</v>
+      </c>
+      <c r="J16" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>75</v>
       </c>
@@ -11626,11 +12093,15 @@
       <c r="H17" s="5">
         <v>33</v>
       </c>
-      <c r="I17" s="2" t="s">
+      <c r="I17" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Veterano</v>
+      </c>
+      <c r="J17" s="2" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>93</v>
       </c>
@@ -11655,11 +12126,15 @@
       <c r="H18" s="5">
         <v>26</v>
       </c>
-      <c r="I18" s="2" t="s">
+      <c r="I18" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Experiente</v>
+      </c>
+      <c r="J18" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>93</v>
       </c>
@@ -11684,11 +12159,15 @@
       <c r="H19" s="5">
         <v>22</v>
       </c>
-      <c r="I19" s="2" t="s">
+      <c r="I19" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Jovem</v>
+      </c>
+      <c r="J19" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>93</v>
       </c>
@@ -11713,11 +12192,15 @@
       <c r="H20" s="5">
         <v>30</v>
       </c>
-      <c r="I20" s="2" t="s">
+      <c r="I20" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Experiente</v>
+      </c>
+      <c r="J20" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>93</v>
       </c>
@@ -11742,11 +12225,15 @@
       <c r="H21" s="5">
         <v>22</v>
       </c>
-      <c r="I21" s="2" t="s">
+      <c r="I21" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Jovem</v>
+      </c>
+      <c r="J21" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>109</v>
       </c>
@@ -11771,11 +12258,15 @@
       <c r="H22" s="5">
         <v>26</v>
       </c>
-      <c r="I22" s="2" t="s">
+      <c r="I22" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Experiente</v>
+      </c>
+      <c r="J22" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>109</v>
       </c>
@@ -11800,11 +12291,15 @@
       <c r="H23" s="5">
         <v>18</v>
       </c>
-      <c r="I23" s="2" t="s">
+      <c r="I23" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Muito Jovem</v>
+      </c>
+      <c r="J23" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>109</v>
       </c>
@@ -11829,13 +12324,17 @@
       <c r="H24" s="5">
         <v>29</v>
       </c>
-      <c r="I24" s="2" t="s">
+      <c r="I24" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>Experiente</v>
+      </c>
+      <c r="J24" s="2" t="s">
         <v>33</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:I24" xr:uid="{121A8764-E71B-430A-8F79-2AFBC43701E9}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:I25">
+  <autoFilter ref="A2:J24" xr:uid="{121A8764-E71B-430A-8F79-2AFBC43701E9}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:J25">
     <sortCondition ref="A3:A25"/>
   </sortState>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -11847,13 +12346,11 @@
   <sheetPr>
     <tabColor theme="6" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A4:S22"/>
+  <dimension ref="A4:Y22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="14.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.140625" customWidth="1"/>
     <col min="6" max="6" width="17.7109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="22.5703125" bestFit="1" customWidth="1"/>
@@ -11863,9 +12360,12 @@
     <col min="17" max="17" width="14.85546875" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="19" max="20" width="24.140625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="27" max="28" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="C4" s="7" t="s">
         <v>158</v>
       </c>
@@ -11885,7 +12385,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="C5" s="2">
         <f>COUNTA('Dados Tratados'!A3:A24)</f>
         <v>22</v>
@@ -11911,7 +12411,7 @@
         <v>25.454545454545453</v>
       </c>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
         <v>167</v>
       </c>
@@ -11924,8 +12424,11 @@
       <c r="P14" s="10" t="s">
         <v>171</v>
       </c>
+      <c r="Y14" s="8" t="s">
+        <v>177</v>
+      </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
         <v>165</v>
       </c>
@@ -11956,8 +12459,11 @@
       <c r="S15" s="11" t="s">
         <v>172</v>
       </c>
+      <c r="Y15" s="5" t="s">
+        <v>173</v>
+      </c>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>9</v>
       </c>
@@ -11990,8 +12496,11 @@
         <f>P16/$P$19</f>
         <v>0.3866594360086768</v>
       </c>
+      <c r="Y16" s="5" t="s">
+        <v>174</v>
+      </c>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>34</v>
       </c>
@@ -12024,8 +12533,11 @@
         <f>P17/$P$19</f>
         <v>0.36243673174258856</v>
       </c>
+      <c r="Y17" s="5" t="s">
+        <v>175</v>
+      </c>
     </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>55</v>
       </c>
@@ -12058,8 +12570,11 @@
         <f>P18/$P$19</f>
         <v>0.25090383224873464</v>
       </c>
+      <c r="Y18" s="5" t="s">
+        <v>176</v>
+      </c>
     </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>75</v>
       </c>
@@ -12079,7 +12594,7 @@
         <f t="shared" si="0"/>
         <v>-55700000</v>
       </c>
-      <c r="O19" t="s">
+      <c r="O19" s="16" t="s">
         <v>164</v>
       </c>
       <c r="P19" s="6">
@@ -12092,8 +12607,11 @@
         <f>P19/$P$19</f>
         <v>1</v>
       </c>
+      <c r="Y19" s="15" t="s">
+        <v>164</v>
+      </c>
     </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>93</v>
       </c>
@@ -12114,7 +12632,7 @@
         <v>-38800000</v>
       </c>
     </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>109</v>
       </c>
@@ -12135,7 +12653,7 @@
         <v>-92500000</v>
       </c>
     </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
         <v>164</v>
       </c>
@@ -12158,8 +12676,8 @@
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId3"/>
-  <drawing r:id="rId4"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId4"/>
+  <drawing r:id="rId5"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
27. Continuação da 3ª Análise
Continuação da terceira análise (tabela dinâmica).
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF4C21BF-C0AE-46F5-B1A8-EDF52E14F9ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ECC86BE-BE9A-411D-B77D-CD562B5D6DDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="3" r:id="rId6"/>
+    <pivotCache cacheId="19" r:id="rId6"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="181">
   <si>
     <t>temporada</t>
   </si>
@@ -564,22 +564,28 @@
     <t>Porcentagem (%) do Total</t>
   </si>
   <si>
-    <t>16-20</t>
-  </si>
-  <si>
-    <t>21-25</t>
-  </si>
-  <si>
-    <t>26-30</t>
-  </si>
-  <si>
-    <t>31-35</t>
-  </si>
-  <si>
     <t>Faixa Etária</t>
   </si>
   <si>
     <t>faixa_etária</t>
+  </si>
+  <si>
+    <t>Contagem de Jogadores</t>
+  </si>
+  <si>
+    <t>Jovem (21-25 anos)</t>
+  </si>
+  <si>
+    <t>Experiente (26-30 anos)</t>
+  </si>
+  <si>
+    <t>Veterano (31+ anos)</t>
+  </si>
+  <si>
+    <t>Muito Jovem (16-20 anos)</t>
+  </si>
+  <si>
+    <t>Porcentagem (% do Total)</t>
   </si>
 </sst>
 </file>
@@ -590,7 +596,7 @@
     <numFmt numFmtId="164" formatCode="[$£-809]#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -611,6 +617,13 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -641,10 +654,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -682,15 +696,145 @@
     <xf numFmtId="165" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="9" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Porcentagem" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="36">
+  <dxfs count="108">
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
     <dxf>
       <alignment horizontal="center"/>
     </dxf>
@@ -753,6 +897,99 @@
     </dxf>
     <dxf>
       <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
     </dxf>
     <dxf>
       <alignment horizontal="general"/>
@@ -8015,11 +8252,11 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>25</xdr:col>
-      <xdr:colOff>593286</xdr:colOff>
+      <xdr:colOff>256688</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>188176</xdr:rowOff>
+      <xdr:rowOff>169126</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="4305794" cy="405432"/>
+    <xdr:ext cx="3588355" cy="405432"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="17" name="CaixaDeTexto 16">
@@ -8033,8 +8270,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="26891811" y="1331176"/>
-          <a:ext cx="4305794" cy="405432"/>
+          <a:off x="26955263" y="1312126"/>
+          <a:ext cx="3588355" cy="405432"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -8064,7 +8301,7 @@
           <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="pt-BR" sz="2000" b="1" baseline="0"/>
-            <a:t>3. Priorização por Jovens ou Veteranos</a:t>
+            <a:t>3. Perfil Etário das Contratações</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -8073,10 +8310,10 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>24</xdr:col>
-      <xdr:colOff>179646</xdr:colOff>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>560646</xdr:colOff>
       <xdr:row>8</xdr:row>
-      <xdr:rowOff>133350</xdr:rowOff>
+      <xdr:rowOff>114300</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="7407734" cy="311496"/>
     <xdr:sp macro="" textlink="">
@@ -8092,7 +8329,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="25278021" y="1657350"/>
+          <a:off x="25049421" y="1638300"/>
           <a:ext cx="7407734" cy="311496"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -9791,11 +10028,11 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Kaike Mendes" refreshedDate="46181.843427199077" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="22" xr:uid="{11AE0983-117D-40C8-AD52-16F3B61A0005}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Kaike Mendes" refreshedDate="46195.801321412036" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="22" xr:uid="{11AE0983-117D-40C8-AD52-16F3B61A0005}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A2:J24" sheet="Dados Tratados"/>
   </cacheSource>
-  <cacheFields count="9">
+  <cacheFields count="10">
     <cacheField name="temporada" numFmtId="0">
       <sharedItems count="6">
         <s v="2019/20"/>
@@ -9862,6 +10099,18 @@
         </groupItems>
       </fieldGroup>
     </cacheField>
+    <cacheField name="faixa_etária" numFmtId="1">
+      <sharedItems count="8">
+        <s v="Jovem (21-25 anos)"/>
+        <s v="Experiente (26-30 anos)"/>
+        <s v="Veterano (31+ anos)"/>
+        <s v="Muito Jovem (16-20 anos)"/>
+        <s v="Jovem" u="1"/>
+        <s v="Experiente" u="1"/>
+        <s v="Veterano" u="1"/>
+        <s v="Muito Jovem" u="1"/>
+      </sharedItems>
+    </cacheField>
     <cacheField name="tipo_negociação" numFmtId="0">
       <sharedItems/>
     </cacheField>
@@ -9885,6 +10134,7 @@
     <s v="Lyon"/>
     <n v="62000000"/>
     <x v="0"/>
+    <x v="0"/>
     <s v="Compra"/>
   </r>
   <r>
@@ -9895,6 +10145,7 @@
     <s v="Holanda"/>
     <s v="PSV Eindhoven"/>
     <n v="30000000"/>
+    <x v="0"/>
     <x v="0"/>
     <s v="Compra"/>
   </r>
@@ -9907,6 +10158,7 @@
     <s v="Inter Milan"/>
     <n v="27000000"/>
     <x v="1"/>
+    <x v="1"/>
     <s v="Venda"/>
   </r>
   <r>
@@ -9918,6 +10170,7 @@
     <s v="Southampton"/>
     <n v="16600000"/>
     <x v="2"/>
+    <x v="0"/>
     <s v="Compra"/>
   </r>
   <r>
@@ -9929,6 +10182,7 @@
     <s v="Real Madrid"/>
     <n v="30000000"/>
     <x v="3"/>
+    <x v="0"/>
     <s v="Compra"/>
   </r>
   <r>
@@ -9940,6 +10194,7 @@
     <s v="Benfica"/>
     <n v="0"/>
     <x v="4"/>
+    <x v="2"/>
     <s v="Livre"/>
   </r>
   <r>
@@ -9951,6 +10206,7 @@
     <s v="Wolves"/>
     <n v="16800000"/>
     <x v="5"/>
+    <x v="1"/>
     <s v="Compra"/>
   </r>
   <r>
@@ -9962,6 +10218,7 @@
     <s v="Atalanta"/>
     <n v="52000000"/>
     <x v="3"/>
+    <x v="0"/>
     <s v="Compra"/>
   </r>
   <r>
@@ -9973,6 +10230,7 @@
     <s v="Juventus"/>
     <n v="0"/>
     <x v="6"/>
+    <x v="0"/>
     <s v="Empréstimo"/>
   </r>
   <r>
@@ -9984,6 +10242,7 @@
     <s v="Al Duhail"/>
     <n v="13000000"/>
     <x v="7"/>
+    <x v="2"/>
     <s v="Venda"/>
   </r>
   <r>
@@ -9995,6 +10254,7 @@
     <s v="Juventus"/>
     <n v="19000000"/>
     <x v="8"/>
+    <x v="0"/>
     <s v="Compra"/>
   </r>
   <r>
@@ -10006,6 +10266,7 @@
     <s v="Everton"/>
     <n v="58000000"/>
     <x v="2"/>
+    <x v="0"/>
     <s v="Compra"/>
   </r>
   <r>
@@ -10017,6 +10278,7 @@
     <s v="Brighton"/>
     <n v="29000000"/>
     <x v="2"/>
+    <x v="0"/>
     <s v="Compra"/>
   </r>
   <r>
@@ -10028,6 +10290,7 @@
     <s v="Ajax"/>
     <n v="31300000"/>
     <x v="8"/>
+    <x v="0"/>
     <s v="Venda"/>
   </r>
   <r>
@@ -10039,6 +10302,7 @@
     <s v="Inter Milan"/>
     <n v="0"/>
     <x v="4"/>
+    <x v="2"/>
     <s v="Livre"/>
   </r>
   <r>
@@ -10050,6 +10314,7 @@
     <s v="Leicester City"/>
     <n v="46300000"/>
     <x v="9"/>
+    <x v="1"/>
     <s v="Compra"/>
   </r>
   <r>
@@ -10060,6 +10325,7 @@
     <s v="Holanda"/>
     <s v="Wolfsburg"/>
     <n v="40000000"/>
+    <x v="0"/>
     <x v="0"/>
     <s v="Compra"/>
   </r>
@@ -10072,6 +10338,7 @@
     <s v="Bayern München"/>
     <n v="95000000"/>
     <x v="10"/>
+    <x v="1"/>
     <s v="Venda"/>
   </r>
   <r>
@@ -10082,6 +10349,7 @@
     <s v="País De Gales"/>
     <s v="Nottingham Forest"/>
     <n v="47500000"/>
+    <x v="0"/>
     <x v="0"/>
     <s v="Compra"/>
   </r>
@@ -10094,6 +10362,7 @@
     <s v="Bournemouth"/>
     <n v="65000000"/>
     <x v="9"/>
+    <x v="1"/>
     <s v="Compra"/>
   </r>
   <r>
@@ -10105,6 +10374,7 @@
     <s v="Leeds United"/>
     <n v="41000000"/>
     <x v="11"/>
+    <x v="3"/>
     <s v="Compra"/>
   </r>
   <r>
@@ -10116,20 +10386,21 @@
     <s v="Olympique Marseille"/>
     <n v="13500000"/>
     <x v="12"/>
+    <x v="1"/>
     <s v="Venda"/>
   </r>
 </pivotCacheRecords>
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{996EC5F2-74EB-477F-A9D9-AF44A2544855}" name="Tabela dinâmica3" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Faixa Etária">
-  <location ref="Y14:Y19" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="9">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{996EC5F2-74EB-477F-A9D9-AF44A2544855}" name="Tabela dinâmica3" cacheId="19" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Faixa Etária" colHeaderCaption="Tipo de Movimentação">
+  <location ref="Y14:Z20" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="10">
     <pivotField showAll="0"/>
-    <pivotField showAll="0">
+    <pivotField axis="axisCol" showAll="0">
       <items count="3">
+        <item h="1" x="1"/>
         <item x="0"/>
-        <item h="1" x="1"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -10138,24 +10409,24 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField numFmtId="164" showAll="0"/>
-    <pivotField axis="axisRow" numFmtId="1" showAll="0">
-      <items count="10">
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField axis="axisRow" dataField="1" showAll="0">
+      <items count="9">
+        <item m="1" x="5"/>
+        <item m="1" x="4"/>
+        <item m="1" x="7"/>
+        <item m="1" x="6"/>
+        <item x="3"/>
         <item x="0"/>
         <item x="1"/>
         <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
         <item t="default"/>
       </items>
     </pivotField>
     <pivotField showAll="0"/>
   </pivotFields>
   <rowFields count="1">
-    <field x="7"/>
+    <field x="8"/>
   </rowFields>
   <rowItems count="5">
     <i>
@@ -10174,21 +10445,56 @@
       <x/>
     </i>
   </rowItems>
+  <colFields count="1">
+    <field x="1"/>
+  </colFields>
   <colItems count="1">
-    <i/>
+    <i>
+      <x v="1"/>
+    </i>
   </colItems>
-  <formats count="1">
-    <format dxfId="5">
+  <dataFields count="1">
+    <dataField name="Contagem de Jogadores" fld="8" subtotal="count" baseField="8" baseItem="0"/>
+  </dataFields>
+  <formats count="9">
+    <format dxfId="9">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="8" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="10">
+      <pivotArea field="8" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="11">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
-          <reference field="7" count="4">
-            <x v="4"/>
-            <x v="5"/>
-            <x v="6"/>
-            <x v="7"/>
-          </reference>
+          <reference field="8" count="0"/>
         </references>
       </pivotArea>
+    </format>
+    <format dxfId="12">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+    <format dxfId="13">
+      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="14">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="15">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="1" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="16">
+      <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
+    </format>
+    <format dxfId="0">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
@@ -10204,9 +10510,9 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="19" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
   <location ref="O14:P19" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="9">
+  <pivotFields count="10">
     <pivotField showAll="0"/>
     <pivotField axis="axisCol" showAll="0">
       <items count="3">
@@ -10239,20 +10545,8 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField dataField="1" numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0">
-      <items count="10">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField showAll="0"/>
     <pivotField showAll="0"/>
   </pivotFields>
   <rowFields count="1">
@@ -10284,39 +10578,39 @@
     <dataField name="Soma do Valor das Transferências" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="29">
+    <format dxfId="101">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="28">
+    <format dxfId="100">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="27">
+    <format dxfId="99">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="26">
+    <format dxfId="98">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="25">
+    <format dxfId="97">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="24">
+    <format dxfId="96">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="23">
+    <format dxfId="95">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="22">
+    <format dxfId="94">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="21">
+    <format dxfId="93">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -10344,9 +10638,9 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Temporadas" colHeaderCaption="">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="19" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Temporadas" colHeaderCaption="">
   <location ref="A14:D22" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="9">
+  <pivotFields count="10">
     <pivotField axis="axisRow" showAll="0">
       <items count="7">
         <item x="0"/>
@@ -10370,20 +10664,8 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField dataField="1" numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0">
-      <items count="10">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField showAll="0"/>
     <pivotField showAll="0"/>
   </pivotFields>
   <rowFields count="1">
@@ -10430,34 +10712,34 @@
     <dataField name="Somas de Entradas e Saídas" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="35">
+    <format dxfId="107">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="34">
+    <format dxfId="106">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="33">
+    <format dxfId="105">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="32">
+    <format dxfId="104">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="31">
+    <format dxfId="103">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="30">
+    <format dxfId="102">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -11537,7 +11819,7 @@
     <col min="6" max="6" width="19.85546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="23" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.85546875" customWidth="1"/>
+    <col min="9" max="9" width="22.28515625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="19.85546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="20.140625" bestFit="1" customWidth="1"/>
   </cols>
@@ -11600,7 +11882,7 @@
         <v>7</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="J2" s="4" t="s">
         <v>142</v>
@@ -11632,8 +11914,8 @@
         <v>22</v>
       </c>
       <c r="I3" s="5" t="str">
-        <f>IF(H3&lt;=20,"Muito Jovem",IF(AND(H3&gt;=21,H3&lt;=25),"Jovem",IF(AND(H3&gt;=26,H3&lt;=30),"Experiente",IF(H3&gt;31,"Veterano"))))</f>
-        <v>Jovem</v>
+        <f t="shared" ref="I3:I24" si="0">IF(H3&lt;=20,"Muito Jovem (16-20 anos)",IF(AND(H3&gt;=21,H3&lt;=25),"Jovem (21-25 anos)",IF(AND(H3&gt;=26,H3&lt;=30),"Experiente (26-30 anos)",IF(H3&gt;31,"Veterano (31+ anos)"))))</f>
+        <v>Jovem (21-25 anos)</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>16</v>
@@ -11665,8 +11947,8 @@
         <v>22</v>
       </c>
       <c r="I4" s="5" t="str">
-        <f t="shared" ref="I4:I24" si="0">IF(H4&lt;=20,"Muito Jovem",IF(AND(H4&gt;=21,H4&lt;=25),"Jovem",IF(AND(H4&gt;=26,H4&lt;=30),"Experiente",IF(H4&gt;31,"Veterano"))))</f>
-        <v>Jovem</v>
+        <f t="shared" si="0"/>
+        <v>Jovem (21-25 anos)</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>16</v>
@@ -11699,7 +11981,7 @@
       </c>
       <c r="I5" s="5" t="str">
         <f t="shared" si="0"/>
-        <v>Experiente</v>
+        <v>Experiente (26-30 anos)</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>33</v>
@@ -11732,7 +12014,7 @@
       </c>
       <c r="I6" s="5" t="str">
         <f t="shared" si="0"/>
-        <v>Jovem</v>
+        <v>Jovem (21-25 anos)</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>16</v>
@@ -11765,7 +12047,7 @@
       </c>
       <c r="I7" s="5" t="str">
         <f t="shared" si="0"/>
-        <v>Jovem</v>
+        <v>Jovem (21-25 anos)</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>16</v>
@@ -11798,7 +12080,7 @@
       </c>
       <c r="I8" s="5" t="str">
         <f t="shared" si="0"/>
-        <v>Veterano</v>
+        <v>Veterano (31+ anos)</v>
       </c>
       <c r="J8" s="2" t="s">
         <v>53</v>
@@ -11830,8 +12112,8 @@
         <v>28</v>
       </c>
       <c r="I9" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>Experiente</v>
+        <f>IF(H9&lt;=20,"Muito Jovem (16-20 anos)",IF(AND(H9&gt;=21,H9&lt;=25),"Jovem (21-25 anos)",IF(AND(H9&gt;=26,H9&lt;=30),"Experiente (26-30 anos)",IF(H9&gt;31,"Veterano (31+ anos)"))))</f>
+        <v>Experiente (26-30 anos)</v>
       </c>
       <c r="J9" s="2" t="s">
         <v>16</v>
@@ -11864,7 +12146,7 @@
       </c>
       <c r="I10" s="5" t="str">
         <f t="shared" si="0"/>
-        <v>Jovem</v>
+        <v>Jovem (21-25 anos)</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>16</v>
@@ -11897,7 +12179,7 @@
       </c>
       <c r="I11" s="5" t="str">
         <f t="shared" si="0"/>
-        <v>Jovem</v>
+        <v>Jovem (21-25 anos)</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>157</v>
@@ -11930,7 +12212,7 @@
       </c>
       <c r="I12" s="5" t="str">
         <f t="shared" si="0"/>
-        <v>Veterano</v>
+        <v>Veterano (31+ anos)</v>
       </c>
       <c r="J12" s="2" t="s">
         <v>33</v>
@@ -11963,7 +12245,7 @@
       </c>
       <c r="I13" s="5" t="str">
         <f t="shared" si="0"/>
-        <v>Jovem</v>
+        <v>Jovem (21-25 anos)</v>
       </c>
       <c r="J13" s="2" t="s">
         <v>16</v>
@@ -11996,7 +12278,7 @@
       </c>
       <c r="I14" s="5" t="str">
         <f t="shared" si="0"/>
-        <v>Jovem</v>
+        <v>Jovem (21-25 anos)</v>
       </c>
       <c r="J14" s="2" t="s">
         <v>16</v>
@@ -12029,7 +12311,7 @@
       </c>
       <c r="I15" s="5" t="str">
         <f t="shared" si="0"/>
-        <v>Jovem</v>
+        <v>Jovem (21-25 anos)</v>
       </c>
       <c r="J15" s="2" t="s">
         <v>16</v>
@@ -12062,7 +12344,7 @@
       </c>
       <c r="I16" s="5" t="str">
         <f t="shared" si="0"/>
-        <v>Jovem</v>
+        <v>Jovem (21-25 anos)</v>
       </c>
       <c r="J16" s="2" t="s">
         <v>33</v>
@@ -12095,7 +12377,7 @@
       </c>
       <c r="I17" s="5" t="str">
         <f t="shared" si="0"/>
-        <v>Veterano</v>
+        <v>Veterano (31+ anos)</v>
       </c>
       <c r="J17" s="2" t="s">
         <v>53</v>
@@ -12128,7 +12410,7 @@
       </c>
       <c r="I18" s="5" t="str">
         <f t="shared" si="0"/>
-        <v>Experiente</v>
+        <v>Experiente (26-30 anos)</v>
       </c>
       <c r="J18" s="2" t="s">
         <v>16</v>
@@ -12161,7 +12443,7 @@
       </c>
       <c r="I19" s="5" t="str">
         <f t="shared" si="0"/>
-        <v>Jovem</v>
+        <v>Jovem (21-25 anos)</v>
       </c>
       <c r="J19" s="2" t="s">
         <v>16</v>
@@ -12194,7 +12476,7 @@
       </c>
       <c r="I20" s="5" t="str">
         <f t="shared" si="0"/>
-        <v>Experiente</v>
+        <v>Experiente (26-30 anos)</v>
       </c>
       <c r="J20" s="2" t="s">
         <v>33</v>
@@ -12227,7 +12509,7 @@
       </c>
       <c r="I21" s="5" t="str">
         <f t="shared" si="0"/>
-        <v>Jovem</v>
+        <v>Jovem (21-25 anos)</v>
       </c>
       <c r="J21" s="2" t="s">
         <v>16</v>
@@ -12260,7 +12542,7 @@
       </c>
       <c r="I22" s="5" t="str">
         <f t="shared" si="0"/>
-        <v>Experiente</v>
+        <v>Experiente (26-30 anos)</v>
       </c>
       <c r="J22" s="2" t="s">
         <v>16</v>
@@ -12293,7 +12575,7 @@
       </c>
       <c r="I23" s="5" t="str">
         <f t="shared" si="0"/>
-        <v>Muito Jovem</v>
+        <v>Muito Jovem (16-20 anos)</v>
       </c>
       <c r="J23" s="2" t="s">
         <v>16</v>
@@ -12326,7 +12608,7 @@
       </c>
       <c r="I24" s="5" t="str">
         <f t="shared" si="0"/>
-        <v>Experiente</v>
+        <v>Experiente (26-30 anos)</v>
       </c>
       <c r="J24" s="2" t="s">
         <v>33</v>
@@ -12346,7 +12628,7 @@
   <sheetPr>
     <tabColor theme="6" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A4:Y22"/>
+  <dimension ref="A4:AC22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.5703125" bestFit="1" customWidth="1"/>
@@ -12360,12 +12642,14 @@
     <col min="17" max="17" width="14.85546875" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="19" max="20" width="24.140625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="27" max="28" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="24" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="26.28515625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="24" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="24.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:29" x14ac:dyDescent="0.25">
       <c r="C4" s="7" t="s">
         <v>158</v>
       </c>
@@ -12385,7 +12669,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:29" x14ac:dyDescent="0.25">
       <c r="C5" s="2">
         <f>COUNTA('Dados Tratados'!A3:A24)</f>
         <v>22</v>
@@ -12411,7 +12695,7 @@
         <v>25.454545454545453</v>
       </c>
     </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
         <v>167</v>
       </c>
@@ -12424,11 +12708,14 @@
       <c r="P14" s="10" t="s">
         <v>171</v>
       </c>
-      <c r="Y14" s="8" t="s">
-        <v>177</v>
+      <c r="Y14" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="Z14" s="10" t="s">
+        <v>171</v>
       </c>
     </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
         <v>165</v>
       </c>
@@ -12459,11 +12746,20 @@
       <c r="S15" s="11" t="s">
         <v>172</v>
       </c>
-      <c r="Y15" s="5" t="s">
+      <c r="Y15" s="10" t="s">
         <v>173</v>
       </c>
+      <c r="Z15" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="AB15" s="11" t="s">
+        <v>173</v>
+      </c>
+      <c r="AC15" s="11" t="s">
+        <v>180</v>
+      </c>
     </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>9</v>
       </c>
@@ -12496,11 +12792,21 @@
         <f>P16/$P$19</f>
         <v>0.3866594360086768</v>
       </c>
-      <c r="Y16" s="5" t="s">
-        <v>174</v>
+      <c r="Y16" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="Z16" s="16">
+        <v>1</v>
+      </c>
+      <c r="AB16" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="AC16" s="18">
+        <f>Z16/$Z$20</f>
+        <v>6.25E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>34</v>
       </c>
@@ -12533,11 +12839,21 @@
         <f>P17/$P$19</f>
         <v>0.36243673174258856</v>
       </c>
-      <c r="Y17" s="5" t="s">
-        <v>175</v>
+      <c r="Y17" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="Z17" s="16">
+        <v>11</v>
+      </c>
+      <c r="AB17" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="AC17" s="18">
+        <f t="shared" ref="AC17:AC20" si="1">Z17/$Z$20</f>
+        <v>0.6875</v>
       </c>
     </row>
-    <row r="18" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>55</v>
       </c>
@@ -12570,11 +12886,21 @@
         <f>P18/$P$19</f>
         <v>0.25090383224873464</v>
       </c>
-      <c r="Y18" s="5" t="s">
-        <v>176</v>
+      <c r="Y18" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="Z18" s="16">
+        <v>3</v>
+      </c>
+      <c r="AB18" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="AC18" s="18">
+        <f t="shared" si="1"/>
+        <v>0.1875</v>
       </c>
     </row>
-    <row r="19" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>75</v>
       </c>
@@ -12594,7 +12920,7 @@
         <f t="shared" si="0"/>
         <v>-55700000</v>
       </c>
-      <c r="O19" s="16" t="s">
+      <c r="O19" s="15" t="s">
         <v>164</v>
       </c>
       <c r="P19" s="6">
@@ -12607,11 +12933,21 @@
         <f>P19/$P$19</f>
         <v>1</v>
       </c>
-      <c r="Y19" s="15" t="s">
-        <v>164</v>
+      <c r="Y19" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="Z19" s="16">
+        <v>1</v>
+      </c>
+      <c r="AB19" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="AC19" s="18">
+        <f t="shared" si="1"/>
+        <v>6.25E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>93</v>
       </c>
@@ -12631,8 +12967,21 @@
         <f t="shared" si="0"/>
         <v>-38800000</v>
       </c>
+      <c r="Y20" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="Z20" s="16">
+        <v>16</v>
+      </c>
+      <c r="AB20" s="12" t="s">
+        <v>164</v>
+      </c>
+      <c r="AC20" s="17">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
     </row>
-    <row r="21" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>109</v>
       </c>
@@ -12653,7 +13002,7 @@
         <v>-92500000</v>
       </c>
     </row>
-    <row r="22" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
         <v>164</v>
       </c>

</xml_diff>

<commit_message>
28. Ajuste dos Gráficos
Ajuste dos gráficos da terceira análise.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ECC86BE-BE9A-411D-B77D-CD562B5D6DDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C12CAC09-8E9C-459D-A256-AA3F1846CC9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="19" r:id="rId6"/>
+    <pivotCache cacheId="0" r:id="rId6"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -658,7 +658,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -696,14 +696,13 @@
     <xf numFmtId="165" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="9" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -711,7 +710,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentagem" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="108">
+  <dxfs count="42">
     <dxf>
       <alignment horizontal="center"/>
     </dxf>
@@ -774,204 +773,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general"/>
     </dxf>
     <dxf>
       <alignment horizontal="center"/>
@@ -2231,7 +2032,7 @@
         <c:idx val="0"/>
         <c:spPr>
           <a:solidFill>
-            <a:schemeClr val="accent1"/>
+            <a:schemeClr val="accent3"/>
           </a:solidFill>
           <a:ln>
             <a:noFill/>
@@ -2307,7 +2108,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent1"/>
+              <a:schemeClr val="accent3"/>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -2946,6 +2747,806 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="pt-BR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:pivotSource>
+    <c:name>[tottenham_transferencias.xlsx]Análises!Tabela dinâmica3</c:name>
+    <c:fmtId val="2"/>
+  </c:pivotSource>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Quantidade de Contratações por Faixa</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> Etária</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="pt-BR"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:pivotFmts>
+      <c:pivotFmt>
+        <c:idx val="0"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="pt-BR"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+    </c:pivotFmts>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Análises!$Z$14:$Z$15</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Entrada</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="pt-BR"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Análises!$Y$16:$Y$20</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Muito Jovem (16-20 anos)</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Veterano (31+ anos)</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Experiente (26-30 anos)</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Jovem (21-25 anos)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Análises!$Z$16:$Z$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>11</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-33A2-407E-819F-CD69739D33E5}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="130"/>
+        <c:axId val="1871569328"/>
+        <c:axId val="1871575088"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1871569328"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="pt-BR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1871575088"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1871575088"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="pt-BR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1871569328"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="pt-BR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.78740157499999996" l="0.511811024" r="0.511811024" t="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+    <c:pageSetup/>
+  </c:printSettings>
+  <c:extLst>
+    <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
+      <c14:pivotOptions>
+        <c14:dropZoneFilter val="1"/>
+        <c14:dropZoneCategories val="1"/>
+        <c14:dropZoneData val="1"/>
+      </c14:pivotOptions>
+    </c:ext>
+    <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{E28EC0CA-F0BB-4C9C-879D-F8772B89E7AC}">
+      <c16:pivotOptions16>
+        <c16:showExpandCollapseFieldButtons val="1"/>
+      </c16:pivotOptions16>
+    </c:ext>
+  </c:extLst>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="pt-BR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Distribuição das Contratações por</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> Faixa Etária (%) </a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.19742450851606"/>
+          <c:y val="3.8593154911404401E-2"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="pt-BR"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:pieChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Análises!$AC$15</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Porcentagem (% do Total)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="3"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="pt-BR"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="1"/>
+            <c:leaderLines>
+              <c:spPr>
+                <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="35000"/>
+                      <a:lumOff val="65000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:round/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+            </c:leaderLines>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Análises!$AB$16:$AB$19</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Muito Jovem (16-20 anos)</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Jovem (21-25 anos)</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Experiente (26-30 anos)</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Veterano (31+ anos)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Análises!$AC$16:$AC$19</c:f>
+              <c:numCache>
+                <c:formatCode>0%</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>6.25E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>6.25E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.1875</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.6875</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-9201-49E7-805C-B05D6A165FC1}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+      </c:pieChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="pt-BR"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="pt-BR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.78740157499999996" l="0.511811024" r="0.511811024" t="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -3106,6 +3707,86 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors6.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
   <cs:axisTitle>
@@ -4618,6 +5299,1030 @@
 </file>
 
 <file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="25400">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="216">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style6.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -8431,6 +10136,78 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>609157</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>5538</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>1600200</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="19" name="Gráfico 18">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{38D6C836-3A56-17E2-128E-560DC3676132}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>655617</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>13853</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>989610</xdr:colOff>
+      <xdr:row>59</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="22" name="Gráfico 21">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B8A48BDB-A6DB-9E0A-3760-D2730846DE3E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -10393,7 +12170,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{996EC5F2-74EB-477F-A9D9-AF44A2544855}" name="Tabela dinâmica3" cacheId="19" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Faixa Etária" colHeaderCaption="Tipo de Movimentação">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{996EC5F2-74EB-477F-A9D9-AF44A2544855}" name="Tabela dinâmica3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Faixa Etária" colHeaderCaption="Tipo de Movimentação">
   <location ref="Y14:Z20" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField showAll="0"/>
@@ -10410,7 +12187,7 @@
     <pivotField showAll="0"/>
     <pivotField numFmtId="164" showAll="0"/>
     <pivotField numFmtId="1" showAll="0"/>
-    <pivotField axis="axisRow" dataField="1" showAll="0">
+    <pivotField axis="axisRow" dataField="1" showAll="0" sortType="ascending">
       <items count="9">
         <item m="1" x="5"/>
         <item m="1" x="4"/>
@@ -10422,6 +12199,18 @@
         <item x="2"/>
         <item t="default"/>
       </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="2">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+            <reference field="1" count="1" selected="0">
+              <x v="1"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
     </pivotField>
     <pivotField showAll="0"/>
   </pivotFields>
@@ -10433,13 +12222,13 @@
       <x v="4"/>
     </i>
     <i>
-      <x v="5"/>
+      <x v="7"/>
     </i>
     <i>
       <x v="6"/>
     </i>
     <i>
-      <x v="7"/>
+      <x v="5"/>
     </i>
     <i t="grand">
       <x/>
@@ -10457,46 +12246,57 @@
     <dataField name="Contagem de Jogadores" fld="8" subtotal="count" baseField="8" baseItem="0"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="9">
+    <format dxfId="26">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="10">
+    <format dxfId="25">
       <pivotArea field="8" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="11">
+    <format dxfId="24">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="12">
+    <format dxfId="23">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="13">
+    <format dxfId="22">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="14">
+    <format dxfId="21">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="15">
+    <format dxfId="20">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="16">
+    <format dxfId="19">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="0">
+    <format dxfId="18">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
+  <chartFormats count="1">
+    <chartFormat chart="2" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
@@ -10510,7 +12310,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="19" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
   <location ref="O14:P19" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField showAll="0"/>
@@ -10578,39 +12378,39 @@
     <dataField name="Soma do Valor das Transferências" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="101">
+    <format dxfId="35">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="100">
+    <format dxfId="34">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="99">
+    <format dxfId="33">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="98">
+    <format dxfId="32">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="97">
+    <format dxfId="31">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="96">
+    <format dxfId="30">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="95">
+    <format dxfId="29">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="94">
+    <format dxfId="28">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="93">
+    <format dxfId="27">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -10638,7 +12438,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="19" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Temporadas" colHeaderCaption="">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Temporadas" colHeaderCaption="">
   <location ref="A14:D22" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField axis="axisRow" showAll="0">
@@ -10712,34 +12512,34 @@
     <dataField name="Somas de Entradas e Saídas" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="107">
+    <format dxfId="41">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="106">
+    <format dxfId="40">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="105">
+    <format dxfId="39">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="104">
+    <format dxfId="38">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="103">
+    <format dxfId="37">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="102">
+    <format dxfId="36">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -12795,13 +14595,13 @@
       <c r="Y16" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="Z16" s="16">
+      <c r="Z16" s="17">
         <v>1</v>
       </c>
       <c r="AB16" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="AC16" s="18">
+      <c r="AC16" s="16">
         <f>Z16/$Z$20</f>
         <v>6.25E-2</v>
       </c>
@@ -12840,17 +14640,17 @@
         <v>0.36243673174258856</v>
       </c>
       <c r="Y17" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="Z17" s="16">
-        <v>11</v>
+        <v>178</v>
+      </c>
+      <c r="Z17" s="17">
+        <v>1</v>
       </c>
       <c r="AB17" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="AC17" s="18">
+      <c r="AC17" s="16">
         <f t="shared" ref="AC17:AC20" si="1">Z17/$Z$20</f>
-        <v>0.6875</v>
+        <v>6.25E-2</v>
       </c>
     </row>
     <row r="18" spans="1:29" x14ac:dyDescent="0.25">
@@ -12889,13 +14689,13 @@
       <c r="Y18" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="Z18" s="16">
+      <c r="Z18" s="17">
         <v>3</v>
       </c>
       <c r="AB18" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="AC18" s="18">
+      <c r="AC18" s="16">
         <f t="shared" si="1"/>
         <v>0.1875</v>
       </c>
@@ -12920,7 +14720,7 @@
         <f t="shared" si="0"/>
         <v>-55700000</v>
       </c>
-      <c r="O19" s="15" t="s">
+      <c r="O19" t="s">
         <v>164</v>
       </c>
       <c r="P19" s="6">
@@ -12934,17 +14734,17 @@
         <v>1</v>
       </c>
       <c r="Y19" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="Z19" s="16">
-        <v>1</v>
+        <v>176</v>
+      </c>
+      <c r="Z19" s="17">
+        <v>11</v>
       </c>
       <c r="AB19" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="AC19" s="18">
+      <c r="AC19" s="16">
         <f t="shared" si="1"/>
-        <v>6.25E-2</v>
+        <v>0.6875</v>
       </c>
     </row>
     <row r="20" spans="1:29" x14ac:dyDescent="0.25">
@@ -12970,13 +14770,13 @@
       <c r="Y20" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="Z20" s="16">
+      <c r="Z20" s="17">
         <v>16</v>
       </c>
       <c r="AB20" s="12" t="s">
         <v>164</v>
       </c>
-      <c r="AC20" s="17">
+      <c r="AC20" s="15">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
29. Construção da Conclusão
Construção da conclusão da análise.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C12CAC09-8E9C-459D-A256-AA3F1846CC9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD3EA7E2-65AB-4C1B-850C-F974E6543587}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId6"/>
+    <pivotCache cacheId="16" r:id="rId6"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -658,7 +658,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -705,66 +705,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentagem" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="42">
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
+  <dxfs count="24">
     <dxf>
       <alignment horizontal="center"/>
     </dxf>
@@ -3415,13 +3362,13 @@
                   <c:v>Muito Jovem (16-20 anos)</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Jovem (21-25 anos)</c:v>
+                  <c:v>Veterano (31+ anos)</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>Experiente (26-30 anos)</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Veterano (31+ anos)</c:v>
+                  <c:v>Jovem (21-25 anos)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -10208,6 +10155,304 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>542925</xdr:colOff>
+      <xdr:row>59</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1781963" cy="311496"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="23" name="CaixaDeTexto 22">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AA244325-9335-4DA8-9815-568B8D059AC2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="25031700" y="11363325"/>
+          <a:ext cx="1781963" cy="311496"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0"/>
+            <a:t>Conclusão</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t> e Insights</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0"/>
+            <a:t>: </a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>165224</xdr:colOff>
+      <xdr:row>61</xdr:row>
+      <xdr:rowOff>116366</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="10997818" cy="2503121"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="24" name="CaixaDeTexto 23">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5D63FC72-E26D-4E62-BEC9-52F80CCEB75A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="23429587" y="11627239"/>
+          <a:ext cx="10997818" cy="2503121"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>Evidenciou-se, após análise, que o perfil etário mais buscado pelo Tottenham Hotspur em suas contratações concentra-se em atletas</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>jovens</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t> na faixa de 21 a 25 anos, representando cerca de </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>69</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>% das entradas durante o período analisado. Somando-o com a porcentagem</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>apresentada pela categoria </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>muito jovem</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>, chega-se à conclusão de que </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>75%</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t> de todas as movimentações admissionais priorizaram jogadores</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>até 25 anos de idade, portanto, </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>jovens</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>.</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>Em contrapartida, os atletas </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>experientes</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t> e </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>veteranos</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t> representaram, juntos, </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>25%</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t> do total, sendo </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>19%</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t> e </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>6%</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>, respectivamente. Nota-se,</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>durante as temporadas analisadas, que o clube se distanciou de contratações "extremas", como as de jogadores muito jovens e veteranos, visto que</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>ambas representam apenas </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>12</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>% da totalidade quando somadas. Pelo ponto de vista adotado, as categorias intermediárias reúnem-se em </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>88%</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>,</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>concentrando a maioria das contratações em atletas de </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>21</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t> até </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>30</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t> anos.</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>Resumidamente, o Tottenham Hotspur priorizou jogadores jovens em relação aos experientes</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="0"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -11805,7 +12050,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Kaike Mendes" refreshedDate="46195.801321412036" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="22" xr:uid="{11AE0983-117D-40C8-AD52-16F3B61A0005}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Kaike Mendes" refreshedDate="46196.442077430554" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="22" xr:uid="{11AE0983-117D-40C8-AD52-16F3B61A0005}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A2:J24" sheet="Dados Tratados"/>
   </cacheSource>
@@ -12170,7 +12415,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{996EC5F2-74EB-477F-A9D9-AF44A2544855}" name="Tabela dinâmica3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Faixa Etária" colHeaderCaption="Tipo de Movimentação">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{996EC5F2-74EB-477F-A9D9-AF44A2544855}" name="Tabela dinâmica3" cacheId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Faixa Etária" colHeaderCaption="Tipo de Movimentação">
   <location ref="Y14:Z20" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField showAll="0"/>
@@ -12246,43 +12491,43 @@
     <dataField name="Contagem de Jogadores" fld="8" subtotal="count" baseField="8" baseItem="0"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="26">
+    <format dxfId="8">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="25">
+    <format dxfId="7">
       <pivotArea field="8" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="24">
+    <format dxfId="6">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="23">
+    <format dxfId="5">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="22">
+    <format dxfId="4">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="21">
+    <format dxfId="3">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="20">
+    <format dxfId="2">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="19">
+    <format dxfId="1">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="18">
+    <format dxfId="0">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -12310,7 +12555,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
   <location ref="O14:P19" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField showAll="0"/>
@@ -12378,39 +12623,39 @@
     <dataField name="Soma do Valor das Transferências" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="35">
+    <format dxfId="17">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="34">
+    <format dxfId="16">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="33">
+    <format dxfId="15">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="32">
+    <format dxfId="14">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="31">
+    <format dxfId="13">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="30">
+    <format dxfId="12">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="29">
+    <format dxfId="11">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="28">
+    <format dxfId="10">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="27">
+    <format dxfId="9">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -12438,7 +12683,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Temporadas" colHeaderCaption="">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Temporadas" colHeaderCaption="">
   <location ref="A14:D22" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField axis="axisRow" showAll="0">
@@ -12512,34 +12757,34 @@
     <dataField name="Somas de Entradas e Saídas" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="41">
+    <format dxfId="23">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="40">
+    <format dxfId="22">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="39">
+    <format dxfId="21">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="38">
+    <format dxfId="20">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="37">
+    <format dxfId="19">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="36">
+    <format dxfId="18">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -14646,7 +14891,7 @@
         <v>1</v>
       </c>
       <c r="AB17" s="2" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="AC17" s="16">
         <f t="shared" ref="AC17:AC20" si="1">Z17/$Z$20</f>
@@ -14720,7 +14965,7 @@
         <f t="shared" si="0"/>
         <v>-55700000</v>
       </c>
-      <c r="O19" t="s">
+      <c r="O19" s="18" t="s">
         <v>164</v>
       </c>
       <c r="P19" s="6">
@@ -14740,7 +14985,7 @@
         <v>11</v>
       </c>
       <c r="AB19" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="AC19" s="16">
         <f t="shared" si="1"/>

</xml_diff>

<commit_message>
29. Conclusão da Análise
Término da terceira análise.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD3EA7E2-65AB-4C1B-850C-F974E6543587}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6898C039-C506-42E4-BF22-B0CD2A6F9019}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -10225,12 +10225,12 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>165224</xdr:colOff>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>517167</xdr:colOff>
       <xdr:row>61</xdr:row>
-      <xdr:rowOff>116366</xdr:rowOff>
+      <xdr:rowOff>130610</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="10997818" cy="2503121"/>
+    <xdr:ext cx="11036163" cy="2722284"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="24" name="CaixaDeTexto 23">
@@ -10244,8 +10244,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="23429587" y="11627239"/>
-          <a:ext cx="10997818" cy="2503121"/>
+          <a:off x="24392568" y="11641483"/>
+          <a:ext cx="11036163" cy="2722284"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -10445,7 +10445,30 @@
           </a:br>
           <a:r>
             <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
-            <a:t>Resumidamente, o Tottenham Hotspur priorizou jogadores jovens em relação aos experientes</a:t>
+            <a:t>Resumidamente, o Tottenham Hotspur priorizou jogadores jovens em relação aos experientes, especificamente atletas entre a faixa de </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>21</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t> a </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>25</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t> anos,</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>sugerindo uma possível estratégia voltada ao equilíbro entre desempenho esportivo e desenvolvimento de ativos.</a:t>
           </a:r>
           <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="0"/>
         </a:p>

</xml_diff>

<commit_message>
31. Começo da análise
Começando a quarta análise.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28E5FC33-1D24-41D4-BB81-A60A8499C099}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A1DD0CA-4E8E-4407-8BD3-C4D161982EB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Apresentação" sheetId="3" r:id="rId1"/>
@@ -25,6 +25,7 @@
   <calcPr calcId="191029"/>
   <pivotCaches>
     <pivotCache cacheId="0" r:id="rId6"/>
+    <pivotCache cacheId="5" r:id="rId7"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="183">
   <si>
     <t>temporada</t>
   </si>
@@ -586,6 +587,12 @@
   </si>
   <si>
     <t>Porcentagem (% do Total)</t>
+  </si>
+  <si>
+    <t>Contagem de nacionalidade</t>
+  </si>
+  <si>
+    <t>Nacionalidades</t>
   </si>
 </sst>
 </file>
@@ -658,7 +665,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -702,12 +709,129 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentagem" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="24">
+  <dxfs count="62">
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
     <dxf>
       <alignment horizontal="center"/>
     </dxf>
@@ -10492,6 +10616,193 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>37</xdr:col>
+      <xdr:colOff>176839</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>167784</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3858750" cy="405432"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="21" name="CaixaDeTexto 20">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{73338A40-233F-40C6-AA68-0038EF48CC69}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="38627287" y="1300001"/>
+          <a:ext cx="3858750" cy="405432"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="2000" b="1" baseline="0"/>
+            <a:t>4. Contratações por Nacionalidade</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>35</xdr:col>
+      <xdr:colOff>532230</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>133079</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="8122545" cy="311496"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="25" name="CaixaDeTexto 24">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8A9CB241-16C3-4FA3-AFA6-8681B1186EDB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="36574471" y="1642702"/>
+          <a:ext cx="8122545" cy="311496"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0"/>
+            <a:t>Pergunta de Negócio: </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="1"/>
+            <a:t>Existe um perfil de</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="1" baseline="0"/>
+            <a:t> contratação predominante em relação à nacionalidade dos atletas?</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>35</xdr:col>
+      <xdr:colOff>584080</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>143774</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="818815" cy="311496"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="26" name="CaixaDeTexto 25">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EF0BE010-78C9-4789-BBF0-912093708FC7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="36626321" y="2030802"/>
+          <a:ext cx="818815" cy="311496"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0"/>
+            <a:t>Análise: </a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -12254,6 +12565,66 @@
         <s v="Veterano" u="1"/>
         <s v="Muito Jovem" u="1"/>
       </sharedItems>
+    </cacheField>
+    <cacheField name="tipo_negociação" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Kaike Mendes" refreshedDate="46198.806584606478" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="22" xr:uid="{DDD0AD49-FD94-41C1-9F64-39D91F4A0370}">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="B2:J24" sheet="Dados Tratados"/>
+  </cacheSource>
+  <cacheFields count="9">
+    <cacheField name="tipo_movimentação" numFmtId="0">
+      <sharedItems count="2">
+        <s v="Entrada"/>
+        <s v="Saída"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="nome_jogador" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="posição" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="nacionalidade" numFmtId="0">
+      <sharedItems count="14">
+        <s v="França"/>
+        <s v="Holanda"/>
+        <s v="Dinamarca"/>
+        <s v="Espanha"/>
+        <s v="Bélgica"/>
+        <s v="Irlanda"/>
+        <s v="Argentina"/>
+        <s v="Suécia"/>
+        <s v="Uruguai"/>
+        <s v="Brasil"/>
+        <s v="Mali"/>
+        <s v="Croácia"/>
+        <s v="Inglaterra"/>
+        <s v="País De Gales"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="clube" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="valor_transferência" numFmtId="164">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="95000000"/>
+    </cacheField>
+    <cacheField name="idade" numFmtId="1">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="18" maxValue="33"/>
+    </cacheField>
+    <cacheField name="faixa_etária" numFmtId="1">
+      <sharedItems/>
     </cacheField>
     <cacheField name="tipo_negociação" numFmtId="0">
       <sharedItems/>
@@ -12536,7 +12907,394 @@
 </pivotCacheRecords>
 </file>
 
+<file path=xl/pivotCache/pivotCacheRecords2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="22">
+  <r>
+    <x v="0"/>
+    <s v="Tanguy Ndombélé"/>
+    <s v="Meio-campista"/>
+    <x v="0"/>
+    <s v="Lyon"/>
+    <n v="62000000"/>
+    <n v="22"/>
+    <s v="Jovem (21-25 anos)"/>
+    <s v="Compra"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <s v="Steven Bergwijn"/>
+    <s v="Atacante"/>
+    <x v="1"/>
+    <s v="PSV Eindhoven"/>
+    <n v="30000000"/>
+    <n v="22"/>
+    <s v="Jovem (21-25 anos)"/>
+    <s v="Compra"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <s v="Christian Eriksen"/>
+    <s v="Meio-campista"/>
+    <x v="2"/>
+    <s v="Inter Milan"/>
+    <n v="27000000"/>
+    <n v="27"/>
+    <s v="Experiente (26-30 anos)"/>
+    <s v="Venda"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <s v="Pierre-Emile Højbjerg"/>
+    <s v="Meio-campista"/>
+    <x v="2"/>
+    <s v="Southampton"/>
+    <n v="16600000"/>
+    <n v="25"/>
+    <s v="Jovem (21-25 anos)"/>
+    <s v="Compra"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <s v="Sergio Reguilón"/>
+    <s v="Defensor"/>
+    <x v="3"/>
+    <s v="Real Madrid"/>
+    <n v="30000000"/>
+    <n v="23"/>
+    <s v="Jovem (21-25 anos)"/>
+    <s v="Compra"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <s v="Jan Vertonghen"/>
+    <s v="Defensor"/>
+    <x v="4"/>
+    <s v="Benfica"/>
+    <n v="0"/>
+    <n v="33"/>
+    <s v="Veterano (31+ anos)"/>
+    <s v="Livre"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <s v="Matt Doherty"/>
+    <s v="Defensor"/>
+    <x v="5"/>
+    <s v="Wolves"/>
+    <n v="16800000"/>
+    <n v="28"/>
+    <s v="Experiente (26-30 anos)"/>
+    <s v="Compra"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <s v="Cristian Romero"/>
+    <s v="Defensor"/>
+    <x v="6"/>
+    <s v="Atalanta"/>
+    <n v="52000000"/>
+    <n v="23"/>
+    <s v="Jovem (21-25 anos)"/>
+    <s v="Compra"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <s v="Dejan Kulusevski"/>
+    <s v="Atacante"/>
+    <x v="7"/>
+    <s v="Juventus"/>
+    <n v="0"/>
+    <n v="21"/>
+    <s v="Jovem (21-25 anos)"/>
+    <s v="Empréstimo"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <s v="Toby Alderweireld"/>
+    <s v="Defensor"/>
+    <x v="4"/>
+    <s v="Al Duhail"/>
+    <n v="13000000"/>
+    <n v="32"/>
+    <s v="Veterano (31+ anos)"/>
+    <s v="Venda"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <s v="Rodrigo Bentancur"/>
+    <s v="Meio-campista"/>
+    <x v="8"/>
+    <s v="Juventus"/>
+    <n v="19000000"/>
+    <n v="24"/>
+    <s v="Jovem (21-25 anos)"/>
+    <s v="Compra"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <s v="Richarlison"/>
+    <s v="Atacante"/>
+    <x v="9"/>
+    <s v="Everton"/>
+    <n v="58000000"/>
+    <n v="25"/>
+    <s v="Jovem (21-25 anos)"/>
+    <s v="Compra"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <s v="Yves Bissouma"/>
+    <s v="Meio-campista"/>
+    <x v="10"/>
+    <s v="Brighton"/>
+    <n v="29000000"/>
+    <n v="25"/>
+    <s v="Jovem (21-25 anos)"/>
+    <s v="Compra"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <s v="Steven Bergwijn"/>
+    <s v="Atacante"/>
+    <x v="1"/>
+    <s v="Ajax"/>
+    <n v="31300000"/>
+    <n v="24"/>
+    <s v="Jovem (21-25 anos)"/>
+    <s v="Venda"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <s v="Ivan Perišić"/>
+    <s v="Atacante"/>
+    <x v="11"/>
+    <s v="Inter Milan"/>
+    <n v="0"/>
+    <n v="33"/>
+    <s v="Veterano (31+ anos)"/>
+    <s v="Livre"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <s v="James Maddison"/>
+    <s v="Meio-campista"/>
+    <x v="12"/>
+    <s v="Leicester City"/>
+    <n v="46300000"/>
+    <n v="26"/>
+    <s v="Experiente (26-30 anos)"/>
+    <s v="Compra"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <s v="Micky van de Ven"/>
+    <s v="Defensor"/>
+    <x v="1"/>
+    <s v="Wolfsburg"/>
+    <n v="40000000"/>
+    <n v="22"/>
+    <s v="Jovem (21-25 anos)"/>
+    <s v="Compra"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <s v="Harry Kane"/>
+    <s v="Atacante"/>
+    <x v="12"/>
+    <s v="Bayern München"/>
+    <n v="95000000"/>
+    <n v="30"/>
+    <s v="Experiente (26-30 anos)"/>
+    <s v="Venda"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <s v="Brennan Johnson"/>
+    <s v="Atacante"/>
+    <x v="13"/>
+    <s v="Nottingham Forest"/>
+    <n v="47500000"/>
+    <n v="22"/>
+    <s v="Jovem (21-25 anos)"/>
+    <s v="Compra"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <s v="Dominic Solanke"/>
+    <s v="Atacante"/>
+    <x v="12"/>
+    <s v="Bournemouth"/>
+    <n v="65000000"/>
+    <n v="26"/>
+    <s v="Experiente (26-30 anos)"/>
+    <s v="Compra"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <s v="Archie Gray"/>
+    <s v="Meio-campista"/>
+    <x v="12"/>
+    <s v="Leeds United"/>
+    <n v="41000000"/>
+    <n v="18"/>
+    <s v="Muito Jovem (16-20 anos)"/>
+    <s v="Compra"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <s v="Pierre-Emile Højbjerg"/>
+    <s v="Meio-campista"/>
+    <x v="2"/>
+    <s v="Olympique Marseille"/>
+    <n v="13500000"/>
+    <n v="29"/>
+    <s v="Experiente (26-30 anos)"/>
+    <s v="Venda"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{904CEA3A-CD0A-459C-A420-1FB249800D4C}" name="Tabela dinâmica4" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Nacionalidades" colHeaderCaption="Contagem de Jogadores">
+  <location ref="AK14:AL29" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="9">
+    <pivotField axis="axisCol" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item h="1" x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" dataField="1" showAll="0">
+      <items count="15">
+        <item x="6"/>
+        <item x="4"/>
+        <item x="9"/>
+        <item x="11"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="12"/>
+        <item x="5"/>
+        <item x="10"/>
+        <item x="13"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="3"/>
+  </rowFields>
+  <rowItems count="14">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="0"/>
+  </colFields>
+  <colItems count="1">
+    <i>
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Contagem de nacionalidade" fld="3" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="6">
+    <format dxfId="37">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="3" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="36">
+      <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="35">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="3" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="34">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+    <format dxfId="32">
+      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="6">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{996EC5F2-74EB-477F-A9D9-AF44A2544855}" name="Tabela dinâmica3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Faixa Etária" colHeaderCaption="Tipo de Movimentação">
   <location ref="Y14:Z20" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -12613,43 +13371,43 @@
     <dataField name="Contagem de Jogadores" fld="8" subtotal="count" baseField="8" baseItem="0"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="8">
+    <format dxfId="46">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="7">
+    <format dxfId="45">
       <pivotArea field="8" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="6">
+    <format dxfId="44">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="5">
+    <format dxfId="43">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="4">
+    <format dxfId="42">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="3">
+    <format dxfId="41">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="2">
+    <format dxfId="40">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="1">
+    <format dxfId="39">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="0">
+    <format dxfId="38">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -12676,7 +13434,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
   <location ref="O14:P19" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -12745,39 +13503,39 @@
     <dataField name="Soma do Valor das Transferências" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="17">
+    <format dxfId="55">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="16">
+    <format dxfId="54">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="15">
+    <format dxfId="53">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="14">
+    <format dxfId="52">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="13">
+    <format dxfId="51">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="12">
+    <format dxfId="50">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="11">
+    <format dxfId="49">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="10">
+    <format dxfId="48">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="9">
+    <format dxfId="47">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -12804,8 +13562,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Temporadas" colHeaderCaption="">
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6" rowHeaderCaption="Temporadas" colHeaderCaption="">
   <location ref="A14:D22" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField axis="axisRow" showAll="0">
@@ -12879,34 +13637,34 @@
     <dataField name="Somas de Entradas e Saídas" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="23">
+    <format dxfId="61">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="22">
+    <format dxfId="60">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="21">
+    <format dxfId="59">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="20">
+    <format dxfId="58">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="19">
+    <format dxfId="57">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="18">
+    <format dxfId="56">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -14795,7 +15553,7 @@
   <sheetPr>
     <tabColor theme="6" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A4:AC22"/>
+  <dimension ref="A4:AL29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.5703125" bestFit="1" customWidth="1"/>
@@ -14814,9 +15572,12 @@
     <col min="27" max="27" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="24" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="24.140625" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="27" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="39" max="40" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:38" x14ac:dyDescent="0.25">
       <c r="C4" s="7" t="s">
         <v>158</v>
       </c>
@@ -14836,7 +15597,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="5" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:38" x14ac:dyDescent="0.25">
       <c r="C5" s="2">
         <f>COUNTA('Dados Tratados'!A3:A24)</f>
         <v>22</v>
@@ -14862,7 +15623,7 @@
         <v>25.454545454545453</v>
       </c>
     </row>
-    <row r="14" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
         <v>167</v>
       </c>
@@ -14881,8 +15642,14 @@
       <c r="Z14" s="10" t="s">
         <v>171</v>
       </c>
+      <c r="AK14" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="AL14" s="8" t="s">
+        <v>175</v>
+      </c>
     </row>
-    <row r="15" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
         <v>165</v>
       </c>
@@ -14925,8 +15692,14 @@
       <c r="AC15" s="11" t="s">
         <v>180</v>
       </c>
+      <c r="AK15" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="AL15" s="2" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="16" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>9</v>
       </c>
@@ -14972,8 +15745,14 @@
         <f>Z16/$Z$20</f>
         <v>6.25E-2</v>
       </c>
+      <c r="AK16" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="AL16" s="17">
+        <v>1</v>
+      </c>
     </row>
-    <row r="17" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>34</v>
       </c>
@@ -15019,8 +15798,14 @@
         <f t="shared" ref="AC17:AC20" si="1">Z17/$Z$20</f>
         <v>6.25E-2</v>
       </c>
+      <c r="AK17" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="AL17" s="17">
+        <v>1</v>
+      </c>
     </row>
-    <row r="18" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>55</v>
       </c>
@@ -15066,8 +15851,14 @@
         <f t="shared" si="1"/>
         <v>0.1875</v>
       </c>
+      <c r="AK18" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="AL18" s="17">
+        <v>1</v>
+      </c>
     </row>
-    <row r="19" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>75</v>
       </c>
@@ -15113,8 +15904,14 @@
         <f t="shared" si="1"/>
         <v>0.6875</v>
       </c>
+      <c r="AK19" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="AL19" s="17">
+        <v>1</v>
+      </c>
     </row>
-    <row r="20" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>93</v>
       </c>
@@ -15147,8 +15944,14 @@
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
+      <c r="AK20" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="AL20" s="17">
+        <v>1</v>
+      </c>
     </row>
-    <row r="21" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>109</v>
       </c>
@@ -15168,8 +15971,14 @@
         <f t="shared" si="0"/>
         <v>-92500000</v>
       </c>
+      <c r="AK21" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="AL21" s="17">
+        <v>1</v>
+      </c>
     </row>
-    <row r="22" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
         <v>164</v>
       </c>
@@ -15189,11 +15998,73 @@
         <f t="shared" si="0"/>
         <v>-373400000</v>
       </c>
+      <c r="AK22" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="AL22" s="17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:38" x14ac:dyDescent="0.25">
+      <c r="AK23" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="AL23" s="17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:38" x14ac:dyDescent="0.25">
+      <c r="AK24" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="AL24" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:38" x14ac:dyDescent="0.25">
+      <c r="AK25" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="AL25" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:38" x14ac:dyDescent="0.25">
+      <c r="AK26" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="AL26" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:38" x14ac:dyDescent="0.25">
+      <c r="AK27" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="AL27" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:38" x14ac:dyDescent="0.25">
+      <c r="AK28" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="AL28" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:38" x14ac:dyDescent="0.25">
+      <c r="AK29" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="AL29" s="17">
+        <v>16</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId4"/>
-  <drawing r:id="rId5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId5"/>
+  <drawing r:id="rId6"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
32. Continuação da Análise
Pequenas modificações na quarta análise.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A1DD0CA-4E8E-4407-8BD3-C4D161982EB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1B29CE1-271A-42ED-B2B5-5B9C94F254CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
   <calcPr calcId="191029"/>
   <pivotCaches>
     <pivotCache cacheId="0" r:id="rId6"/>
-    <pivotCache cacheId="5" r:id="rId7"/>
+    <pivotCache cacheId="1" r:id="rId7"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -665,7 +665,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -709,93 +709,12 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentagem" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="62">
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
+  <dxfs count="30">
     <dxf>
       <alignment horizontal="center"/>
     </dxf>
@@ -861,24 +780,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="general"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
     </dxf>
     <dxf>
       <alignment horizontal="center"/>
@@ -7684,11 +7585,11 @@
           </a:r>
           <a:r>
             <a:rPr lang="pt-BR" sz="1200" b="1"/>
-            <a:t> Existe um perfil de contratação predominante em</a:t>
+            <a:t> Existe um padrão</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0"/>
-            <a:t> relação à nacionalidade dos atletas?</a:t>
+            <a:t> de nacionalidades nas contratações realizadas pelo Tottenham Hotspur?</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -10619,11 +10520,11 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>37</xdr:col>
-      <xdr:colOff>176839</xdr:colOff>
+      <xdr:colOff>341371</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>167784</xdr:rowOff>
+      <xdr:rowOff>176770</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="3858750" cy="405432"/>
+    <xdr:ext cx="3961021" cy="405432"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="21" name="CaixaDeTexto 20">
@@ -10637,8 +10538,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="38627287" y="1300001"/>
-          <a:ext cx="3858750" cy="405432"/>
+          <a:off x="38791819" y="1308987"/>
+          <a:ext cx="3961021" cy="405432"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -10668,7 +10569,7 @@
           <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="pt-BR" sz="2000" b="1" baseline="0"/>
-            <a:t>4. Contratações por Nacionalidade</a:t>
+            <a:t>4. Nacionalidades das Contratações</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -10678,11 +10579,11 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>35</xdr:col>
-      <xdr:colOff>532230</xdr:colOff>
+      <xdr:colOff>534477</xdr:colOff>
       <xdr:row>8</xdr:row>
-      <xdr:rowOff>133079</xdr:rowOff>
+      <xdr:rowOff>124093</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="8122545" cy="311496"/>
+    <xdr:ext cx="8405635" cy="311496"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="25" name="CaixaDeTexto 24">
@@ -10696,8 +10597,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="36574471" y="1642702"/>
-          <a:ext cx="8122545" cy="311496"/>
+          <a:off x="36576718" y="1633716"/>
+          <a:ext cx="8405635" cy="311496"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -10731,13 +10632,8 @@
           </a:r>
           <a:r>
             <a:rPr lang="pt-BR" sz="1400" b="0" i="1"/>
-            <a:t>Existe um perfil de</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="0" i="1" baseline="0"/>
-            <a:t> contratação predominante em relação à nacionalidade dos atletas?</a:t>
-          </a:r>
-          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="1"/>
+            <a:t>Existe um padrão de nacionalidades nas contratações realizadas pelo Tottenham Hotspur?</a:t>
+          </a:r>
         </a:p>
       </xdr:txBody>
     </xdr:sp>
@@ -13155,7 +13051,151 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{904CEA3A-CD0A-459C-A420-1FB249800D4C}" name="Tabela dinâmica4" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Nacionalidades" colHeaderCaption="Contagem de Jogadores">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6" rowHeaderCaption="Temporadas" colHeaderCaption="">
+  <location ref="A14:D22" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="10">
+    <pivotField axis="axisRow" showAll="0">
+      <items count="7">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="7">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="1"/>
+  </colFields>
+  <colItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Somas de Entradas e Saídas" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
+  </dataFields>
+  <formats count="6">
+    <format dxfId="5">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="4">
+      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="3">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="2">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="1" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="1">
+      <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="0">
+      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="2">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{904CEA3A-CD0A-459C-A420-1FB249800D4C}" name="Tabela dinâmica4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Nacionalidades" colHeaderCaption="Contagem de Jogadores">
   <location ref="AK14:AL29" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField axis="axisCol" showAll="0">
@@ -13251,27 +13291,27 @@
     <dataField name="Contagem de nacionalidade" fld="3" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="37">
+    <format dxfId="11">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="36">
+    <format dxfId="10">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="35">
+    <format dxfId="9">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="34">
+    <format dxfId="8">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="32">
+    <format dxfId="7">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
     <format dxfId="6">
@@ -13294,7 +13334,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{996EC5F2-74EB-477F-A9D9-AF44A2544855}" name="Tabela dinâmica3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Faixa Etária" colHeaderCaption="Tipo de Movimentação">
   <location ref="Y14:Z20" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -13371,43 +13411,43 @@
     <dataField name="Contagem de Jogadores" fld="8" subtotal="count" baseField="8" baseItem="0"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="46">
+    <format dxfId="20">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="45">
+    <format dxfId="19">
       <pivotArea field="8" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="44">
+    <format dxfId="18">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="43">
+    <format dxfId="17">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="42">
+    <format dxfId="16">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="41">
+    <format dxfId="15">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="40">
+    <format dxfId="14">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="39">
+    <format dxfId="13">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="38">
+    <format dxfId="12">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -13434,7 +13474,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
   <location ref="O14:P19" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -13503,39 +13543,39 @@
     <dataField name="Soma do Valor das Transferências" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="55">
+    <format dxfId="29">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="54">
+    <format dxfId="28">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="53">
+    <format dxfId="27">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="52">
+    <format dxfId="26">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="51">
+    <format dxfId="25">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="50">
+    <format dxfId="24">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="49">
+    <format dxfId="23">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="48">
+    <format dxfId="22">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="47">
+    <format dxfId="21">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -13545,150 +13585,6 @@
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
             <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6" rowHeaderCaption="Temporadas" colHeaderCaption="">
-  <location ref="A14:D22" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="10">
-    <pivotField axis="axisRow" showAll="0">
-      <items count="7">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisCol" showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="7">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="1"/>
-  </colFields>
-  <colItems count="3">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Somas de Entradas e Saídas" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
-  </dataFields>
-  <formats count="6">
-    <format dxfId="61">
-      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
-        <references count="1">
-          <reference field="0" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="60">
-      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
-    </format>
-    <format dxfId="59">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="0" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="58">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="1" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="57">
-      <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="56">
-      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="2">
-    <chartFormat chart="0" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="1" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="1"/>
           </reference>
         </references>
       </pivotArea>
@@ -15748,7 +15644,7 @@
       <c r="AK16" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="AL16" s="17">
+      <c r="AL16" s="2">
         <v>1</v>
       </c>
     </row>
@@ -15801,7 +15697,7 @@
       <c r="AK17" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="AL17" s="17">
+      <c r="AL17" s="2">
         <v>1</v>
       </c>
     </row>
@@ -15854,7 +15750,7 @@
       <c r="AK18" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="AL18" s="17">
+      <c r="AL18" s="2">
         <v>1</v>
       </c>
     </row>
@@ -15907,7 +15803,7 @@
       <c r="AK19" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="AL19" s="17">
+      <c r="AL19" s="2">
         <v>1</v>
       </c>
     </row>
@@ -15947,7 +15843,7 @@
       <c r="AK20" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="AL20" s="17">
+      <c r="AL20" s="2">
         <v>1</v>
       </c>
     </row>
@@ -15974,7 +15870,7 @@
       <c r="AK21" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="AL21" s="17">
+      <c r="AL21" s="2">
         <v>1</v>
       </c>
     </row>
@@ -16001,7 +15897,7 @@
       <c r="AK22" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="AL22" s="17">
+      <c r="AL22" s="2">
         <v>2</v>
       </c>
     </row>
@@ -16009,7 +15905,7 @@
       <c r="AK23" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="AL23" s="17">
+      <c r="AL23" s="2">
         <v>3</v>
       </c>
     </row>
@@ -16017,7 +15913,7 @@
       <c r="AK24" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="AL24" s="17">
+      <c r="AL24" s="2">
         <v>1</v>
       </c>
     </row>
@@ -16025,7 +15921,7 @@
       <c r="AK25" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="AL25" s="17">
+      <c r="AL25" s="2">
         <v>1</v>
       </c>
     </row>
@@ -16033,7 +15929,7 @@
       <c r="AK26" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="AL26" s="17">
+      <c r="AL26" s="2">
         <v>1</v>
       </c>
     </row>
@@ -16041,7 +15937,7 @@
       <c r="AK27" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="AL27" s="17">
+      <c r="AL27" s="2">
         <v>1</v>
       </c>
     </row>
@@ -16049,7 +15945,7 @@
       <c r="AK28" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="AL28" s="17">
+      <c r="AL28" s="2">
         <v>1</v>
       </c>
     </row>
@@ -16057,7 +15953,7 @@
       <c r="AK29" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="AL29" s="17">
+      <c r="AL29" s="2">
         <v>16</v>
       </c>
     </row>

</xml_diff>

<commit_message>
33. Continuação da Análise
Continuação da quarta análise.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1B29CE1-271A-42ED-B2B5-5B9C94F254CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60DB313B-E85E-492D-A72B-56390D68EFA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
   <calcPr calcId="191029"/>
   <pivotCaches>
     <pivotCache cacheId="0" r:id="rId6"/>
-    <pivotCache cacheId="1" r:id="rId7"/>
+    <pivotCache cacheId="2" r:id="rId7"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="185">
   <si>
     <t>temporada</t>
   </si>
@@ -589,10 +589,16 @@
     <t>Porcentagem (% do Total)</t>
   </si>
   <si>
-    <t>Contagem de nacionalidade</t>
-  </si>
-  <si>
     <t>Nacionalidades</t>
+  </si>
+  <si>
+    <t>Contagem de Nacionalidades</t>
+  </si>
+  <si>
+    <t>Origem das Contratações</t>
+  </si>
+  <si>
+    <t>Clubes</t>
   </si>
 </sst>
 </file>
@@ -665,7 +671,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -709,12 +715,157 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentagem" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="30">
+  <dxfs count="77">
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
     <dxf>
       <alignment horizontal="center"/>
     </dxf>
@@ -2148,13 +2299,13 @@
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>Meio-campista</c:v>
+                  <c:v>Defensor</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>Atacante</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Defensor</c:v>
+                  <c:v>Meio-campista</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2166,13 +2317,13 @@
                 <c:formatCode>[$£-809]#,##0.00</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>213900000</c:v>
+                  <c:v>138800000</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>200500000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>138800000</c:v>
+                  <c:v>213900000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2601,13 +2752,13 @@
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>0.3866594360086768</c:v>
+                  <c:v>0.25090383224873464</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0.36243673174258856</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.25090383224873464</c:v>
+                  <c:v>0.3866594360086768</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3535,6 +3686,500 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="pt-BR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:pivotSource>
+    <c:name>[tottenham_transferencias.xlsx]Análises!Tabela dinâmica4</c:name>
+    <c:fmtId val="1"/>
+  </c:pivotSource>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Quantidade de Contratações por Nacionalidade</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="pt-BR"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:pivotFmts>
+      <c:pivotFmt>
+        <c:idx val="0"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="pt-BR"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+    </c:pivotFmts>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Análises!$AL$14:$AL$15</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Entrada</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="pt-BR"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Análises!$AK$16:$AK$29</c:f>
+              <c:strCache>
+                <c:ptCount val="13"/>
+                <c:pt idx="0">
+                  <c:v>França</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Uruguai</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Argentina</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Croácia</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Irlanda</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Espanha</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Mali</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Dinamarca</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>País De Gales</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Brasil</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Suécia</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Holanda</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>Inglaterra</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Análises!$AL$16:$AL$29</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="13"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-1A9E-4121-B54A-AF5CB949493C}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="80"/>
+        <c:axId val="749467536"/>
+        <c:axId val="749468976"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="749467536"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="pt-BR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="749468976"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="749468976"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="3.5"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="pt-BR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="749467536"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+        <c:majorUnit val="1"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="pt-BR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.78740157499999996" l="0.511811024" r="0.511811024" t="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+    <c:pageSetup/>
+  </c:printSettings>
+  <c:extLst>
+    <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
+      <c14:pivotOptions>
+        <c14:dropZoneFilter val="1"/>
+        <c14:dropZoneCategories val="1"/>
+        <c14:dropZoneData val="1"/>
+      </c14:pivotOptions>
+    </c:ext>
+    <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{E28EC0CA-F0BB-4C9C-879D-F8772B89E7AC}">
+      <c16:pivotOptions16>
+        <c16:showExpandCollapseFieldButtons val="1"/>
+      </c16:pivotOptions16>
+    </c:ext>
+  </c:extLst>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -3775,6 +4420,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors7.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
   <cs:axisTitle>
@@ -6487,6 +7172,511 @@
       <cs:styleClr val="auto"/>
     </cs:lnRef>
     <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style7.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="216">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
@@ -10694,6 +11884,269 @@
             <a:t>Análise: </a:t>
           </a:r>
           <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>36</xdr:col>
+      <xdr:colOff>9721</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>189180</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>40</xdr:col>
+      <xdr:colOff>1827246</xdr:colOff>
+      <xdr:row>67</xdr:row>
+      <xdr:rowOff>170819</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="27" name="Gráfico 26">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BAFD9697-F798-3D87-C4A2-4DDD12DE16B9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>35</xdr:col>
+      <xdr:colOff>589473</xdr:colOff>
+      <xdr:row>68</xdr:row>
+      <xdr:rowOff>120222</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1781963" cy="311496"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="28" name="CaixaDeTexto 27">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{310F3297-2F08-48EB-9D6C-55DE52BDCEDB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="36622548" y="13074222"/>
+          <a:ext cx="1781963" cy="311496"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0"/>
+            <a:t>Conclusão</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t> e Insights</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0"/>
+            <a:t>: </a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>36</xdr:col>
+      <xdr:colOff>44470</xdr:colOff>
+      <xdr:row>70</xdr:row>
+      <xdr:rowOff>105249</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="11067773" cy="1845633"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="29" name="CaixaDeTexto 28">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8463A3B4-0C55-443D-9D86-0A55241C8A82}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="36697748" y="13314447"/>
+          <a:ext cx="11067773" cy="1845633"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>As contratações realizadas pelo Tottenham Hotspur durante o período contaram com a presença de atletas originários de diversos países do globo,</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>totalizando </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>13</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t> nacionalidades distintas divididas entre </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>16</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t> jogadores. A Inglaterra, com </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>3</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>, encontra-se no topo, seguida por Holanda com </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>2</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>e pelas consecutivas pátrias, como Brasil e Uruguai, que contabilizam apenas </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>1</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t> atleta cada.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>Embora os ingleses e holandeses liderem a lista, não há indícios suficientes para afirmar que o Tottenham Hotspur padronizou sua busca por talentos</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>ao concentrar-se em uma ou outra nacionalidade, visto que a diferença entre atletas é </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>mínima</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t> e a </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>diversidade</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t> de nações se faz presente. Cerca de </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>11</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>jogadores não são representados pelas bandeiras de Inglaterra ou Holanda.</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
         </a:p>
       </xdr:txBody>
     </xdr:sp>
@@ -12511,7 +13964,28 @@
       </sharedItems>
     </cacheField>
     <cacheField name="clube" numFmtId="0">
-      <sharedItems/>
+      <sharedItems count="20">
+        <s v="Lyon"/>
+        <s v="PSV Eindhoven"/>
+        <s v="Inter Milan"/>
+        <s v="Southampton"/>
+        <s v="Real Madrid"/>
+        <s v="Benfica"/>
+        <s v="Wolves"/>
+        <s v="Atalanta"/>
+        <s v="Juventus"/>
+        <s v="Al Duhail"/>
+        <s v="Everton"/>
+        <s v="Brighton"/>
+        <s v="Ajax"/>
+        <s v="Leicester City"/>
+        <s v="Wolfsburg"/>
+        <s v="Bayern München"/>
+        <s v="Nottingham Forest"/>
+        <s v="Bournemouth"/>
+        <s v="Leeds United"/>
+        <s v="Olympique Marseille"/>
+      </sharedItems>
     </cacheField>
     <cacheField name="valor_transferência" numFmtId="164">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="95000000"/>
@@ -12810,7 +14284,7 @@
     <s v="Tanguy Ndombélé"/>
     <s v="Meio-campista"/>
     <x v="0"/>
-    <s v="Lyon"/>
+    <x v="0"/>
     <n v="62000000"/>
     <n v="22"/>
     <s v="Jovem (21-25 anos)"/>
@@ -12821,7 +14295,7 @@
     <s v="Steven Bergwijn"/>
     <s v="Atacante"/>
     <x v="1"/>
-    <s v="PSV Eindhoven"/>
+    <x v="1"/>
     <n v="30000000"/>
     <n v="22"/>
     <s v="Jovem (21-25 anos)"/>
@@ -12832,7 +14306,7 @@
     <s v="Christian Eriksen"/>
     <s v="Meio-campista"/>
     <x v="2"/>
-    <s v="Inter Milan"/>
+    <x v="2"/>
     <n v="27000000"/>
     <n v="27"/>
     <s v="Experiente (26-30 anos)"/>
@@ -12843,7 +14317,7 @@
     <s v="Pierre-Emile Højbjerg"/>
     <s v="Meio-campista"/>
     <x v="2"/>
-    <s v="Southampton"/>
+    <x v="3"/>
     <n v="16600000"/>
     <n v="25"/>
     <s v="Jovem (21-25 anos)"/>
@@ -12854,7 +14328,7 @@
     <s v="Sergio Reguilón"/>
     <s v="Defensor"/>
     <x v="3"/>
-    <s v="Real Madrid"/>
+    <x v="4"/>
     <n v="30000000"/>
     <n v="23"/>
     <s v="Jovem (21-25 anos)"/>
@@ -12865,7 +14339,7 @@
     <s v="Jan Vertonghen"/>
     <s v="Defensor"/>
     <x v="4"/>
-    <s v="Benfica"/>
+    <x v="5"/>
     <n v="0"/>
     <n v="33"/>
     <s v="Veterano (31+ anos)"/>
@@ -12876,7 +14350,7 @@
     <s v="Matt Doherty"/>
     <s v="Defensor"/>
     <x v="5"/>
-    <s v="Wolves"/>
+    <x v="6"/>
     <n v="16800000"/>
     <n v="28"/>
     <s v="Experiente (26-30 anos)"/>
@@ -12887,7 +14361,7 @@
     <s v="Cristian Romero"/>
     <s v="Defensor"/>
     <x v="6"/>
-    <s v="Atalanta"/>
+    <x v="7"/>
     <n v="52000000"/>
     <n v="23"/>
     <s v="Jovem (21-25 anos)"/>
@@ -12898,7 +14372,7 @@
     <s v="Dejan Kulusevski"/>
     <s v="Atacante"/>
     <x v="7"/>
-    <s v="Juventus"/>
+    <x v="8"/>
     <n v="0"/>
     <n v="21"/>
     <s v="Jovem (21-25 anos)"/>
@@ -12909,7 +14383,7 @@
     <s v="Toby Alderweireld"/>
     <s v="Defensor"/>
     <x v="4"/>
-    <s v="Al Duhail"/>
+    <x v="9"/>
     <n v="13000000"/>
     <n v="32"/>
     <s v="Veterano (31+ anos)"/>
@@ -12920,7 +14394,7 @@
     <s v="Rodrigo Bentancur"/>
     <s v="Meio-campista"/>
     <x v="8"/>
-    <s v="Juventus"/>
+    <x v="8"/>
     <n v="19000000"/>
     <n v="24"/>
     <s v="Jovem (21-25 anos)"/>
@@ -12931,7 +14405,7 @@
     <s v="Richarlison"/>
     <s v="Atacante"/>
     <x v="9"/>
-    <s v="Everton"/>
+    <x v="10"/>
     <n v="58000000"/>
     <n v="25"/>
     <s v="Jovem (21-25 anos)"/>
@@ -12942,7 +14416,7 @@
     <s v="Yves Bissouma"/>
     <s v="Meio-campista"/>
     <x v="10"/>
-    <s v="Brighton"/>
+    <x v="11"/>
     <n v="29000000"/>
     <n v="25"/>
     <s v="Jovem (21-25 anos)"/>
@@ -12953,7 +14427,7 @@
     <s v="Steven Bergwijn"/>
     <s v="Atacante"/>
     <x v="1"/>
-    <s v="Ajax"/>
+    <x v="12"/>
     <n v="31300000"/>
     <n v="24"/>
     <s v="Jovem (21-25 anos)"/>
@@ -12964,7 +14438,7 @@
     <s v="Ivan Perišić"/>
     <s v="Atacante"/>
     <x v="11"/>
-    <s v="Inter Milan"/>
+    <x v="2"/>
     <n v="0"/>
     <n v="33"/>
     <s v="Veterano (31+ anos)"/>
@@ -12975,7 +14449,7 @@
     <s v="James Maddison"/>
     <s v="Meio-campista"/>
     <x v="12"/>
-    <s v="Leicester City"/>
+    <x v="13"/>
     <n v="46300000"/>
     <n v="26"/>
     <s v="Experiente (26-30 anos)"/>
@@ -12986,7 +14460,7 @@
     <s v="Micky van de Ven"/>
     <s v="Defensor"/>
     <x v="1"/>
-    <s v="Wolfsburg"/>
+    <x v="14"/>
     <n v="40000000"/>
     <n v="22"/>
     <s v="Jovem (21-25 anos)"/>
@@ -12997,7 +14471,7 @@
     <s v="Harry Kane"/>
     <s v="Atacante"/>
     <x v="12"/>
-    <s v="Bayern München"/>
+    <x v="15"/>
     <n v="95000000"/>
     <n v="30"/>
     <s v="Experiente (26-30 anos)"/>
@@ -13008,7 +14482,7 @@
     <s v="Brennan Johnson"/>
     <s v="Atacante"/>
     <x v="13"/>
-    <s v="Nottingham Forest"/>
+    <x v="16"/>
     <n v="47500000"/>
     <n v="22"/>
     <s v="Jovem (21-25 anos)"/>
@@ -13019,7 +14493,7 @@
     <s v="Dominic Solanke"/>
     <s v="Atacante"/>
     <x v="12"/>
-    <s v="Bournemouth"/>
+    <x v="17"/>
     <n v="65000000"/>
     <n v="26"/>
     <s v="Experiente (26-30 anos)"/>
@@ -13030,7 +14504,7 @@
     <s v="Archie Gray"/>
     <s v="Meio-campista"/>
     <x v="12"/>
-    <s v="Leeds United"/>
+    <x v="18"/>
     <n v="41000000"/>
     <n v="18"/>
     <s v="Muito Jovem (16-20 anos)"/>
@@ -13041,7 +14515,7 @@
     <s v="Pierre-Emile Højbjerg"/>
     <s v="Meio-campista"/>
     <x v="2"/>
-    <s v="Olympique Marseille"/>
+    <x v="19"/>
     <n v="13500000"/>
     <n v="29"/>
     <s v="Experiente (26-30 anos)"/>
@@ -13051,6 +14525,653 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FB686887-B509-4E7E-B605-6A13972A6E0B}" name="Tabela dinâmica5" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Origem das Contratações" colHeaderCaption="Contagem de Jogadores">
+  <location ref="AN14:AO47" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="9">
+    <pivotField axis="axisCol" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item h="1" x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" dataField="1" showAll="0">
+      <items count="15">
+        <item x="6"/>
+        <item x="4"/>
+        <item x="9"/>
+        <item x="11"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="12"/>
+        <item x="5"/>
+        <item x="10"/>
+        <item x="13"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="21">
+        <item x="12"/>
+        <item x="9"/>
+        <item x="7"/>
+        <item x="15"/>
+        <item x="5"/>
+        <item x="17"/>
+        <item x="11"/>
+        <item x="10"/>
+        <item x="2"/>
+        <item x="8"/>
+        <item x="18"/>
+        <item x="13"/>
+        <item x="0"/>
+        <item x="16"/>
+        <item x="19"/>
+        <item x="1"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item x="14"/>
+        <item x="6"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="2">
+    <field x="4"/>
+    <field x="3"/>
+  </rowFields>
+  <rowItems count="32">
+    <i>
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i r="1">
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i r="1">
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i r="1">
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i r="1">
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i r="1">
+      <x v="12"/>
+    </i>
+    <i r="1">
+      <x v="13"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i r="1">
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i r="1">
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i r="1">
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i r="1">
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="15"/>
+    </i>
+    <i r="1">
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="16"/>
+    </i>
+    <i r="1">
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="17"/>
+    </i>
+    <i r="1">
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="18"/>
+    </i>
+    <i r="1">
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="19"/>
+    </i>
+    <i r="1">
+      <x v="9"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="0"/>
+  </colFields>
+  <colItems count="1">
+    <i>
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Clubes" fld="3" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="46">
+    <format dxfId="45">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="44">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="43">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="42">
+      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
+    </format>
+    <format dxfId="41">
+      <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="40">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="4" count="15">
+            <x v="2"/>
+            <x v="5"/>
+            <x v="6"/>
+            <x v="7"/>
+            <x v="8"/>
+            <x v="9"/>
+            <x v="10"/>
+            <x v="11"/>
+            <x v="12"/>
+            <x v="13"/>
+            <x v="15"/>
+            <x v="16"/>
+            <x v="17"/>
+            <x v="18"/>
+            <x v="19"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="39">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="38">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="0"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="37">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="8"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="5"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="36">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="10"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="6"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="35">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="2"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="7"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="34">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="3"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="8"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="33">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="2">
+            <x v="12"/>
+            <x v="13"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="9"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="32">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="8"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="10"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="31">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="8"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="11"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="30">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="6"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="12"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="29">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="11"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="13"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="28">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="7"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="15"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="27">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="5"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="16"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="26">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="4"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="17"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="25">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="7"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="18"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="24">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="9"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="19"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="23">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="22">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="21">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="20">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="19">
+      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
+    </format>
+    <format dxfId="18">
+      <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="17">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="4" count="15">
+            <x v="2"/>
+            <x v="5"/>
+            <x v="6"/>
+            <x v="7"/>
+            <x v="8"/>
+            <x v="9"/>
+            <x v="10"/>
+            <x v="11"/>
+            <x v="12"/>
+            <x v="13"/>
+            <x v="15"/>
+            <x v="16"/>
+            <x v="17"/>
+            <x v="18"/>
+            <x v="19"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="16">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="15">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="0"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="14">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="8"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="5"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="13">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="10"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="6"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="12">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="2"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="7"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="11">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="3"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="8"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="10">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="2">
+            <x v="12"/>
+            <x v="13"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="9"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="9">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="8"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="10"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="8">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="8"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="11"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="7">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="6"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="12"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="6">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="11"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="13"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="5">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="7"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="15"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="4">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="5"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="16"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="3">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="4"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="17"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="2">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="7"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="18"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="1">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="9"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="19"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="0">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6" rowHeaderCaption="Temporadas" colHeaderCaption="">
   <location ref="A14:D22" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -13125,34 +15246,34 @@
     <dataField name="Somas de Entradas e Saídas" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="5">
+    <format dxfId="58">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="4">
+    <format dxfId="57">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="3">
+    <format dxfId="56">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="2">
+    <format dxfId="55">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="1">
+    <format dxfId="54">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="0">
+    <format dxfId="53">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -13194,8 +15315,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{904CEA3A-CD0A-459C-A420-1FB249800D4C}" name="Tabela dinâmica4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Nacionalidades" colHeaderCaption="Contagem de Jogadores">
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{904CEA3A-CD0A-459C-A420-1FB249800D4C}" name="Tabela dinâmica4" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Nacionalidades" colHeaderCaption="Contagem de Jogadores">
   <location ref="AK14:AL29" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField axis="axisCol" showAll="0">
@@ -13207,7 +15328,7 @@
     </pivotField>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField axis="axisRow" dataField="1" showAll="0">
+    <pivotField axis="axisRow" dataField="1" showAll="0" sortType="ascending">
       <items count="15">
         <item x="6"/>
         <item x="4"/>
@@ -13225,8 +15346,44 @@
         <item x="8"/>
         <item t="default"/>
       </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="2">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+            <reference field="0" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
     </pivotField>
-    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="21">
+        <item x="12"/>
+        <item x="9"/>
+        <item x="7"/>
+        <item x="15"/>
+        <item x="5"/>
+        <item x="17"/>
+        <item x="11"/>
+        <item x="10"/>
+        <item x="2"/>
+        <item x="8"/>
+        <item x="18"/>
+        <item x="13"/>
+        <item x="0"/>
+        <item x="16"/>
+        <item x="19"/>
+        <item x="1"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item x="14"/>
+        <item x="6"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField numFmtId="164" showAll="0"/>
     <pivotField numFmtId="1" showAll="0"/>
     <pivotField showAll="0"/>
@@ -13237,43 +15394,43 @@
   </rowFields>
   <rowItems count="14">
     <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i>
       <x/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="11"/>
     </i>
     <i>
       <x v="2"/>
     </i>
     <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
+      <x v="12"/>
     </i>
     <i>
       <x v="7"/>
     </i>
     <i>
       <x v="8"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="11"/>
-    </i>
-    <i>
-      <x v="12"/>
-    </i>
-    <i>
-      <x v="13"/>
     </i>
     <i t="grand">
       <x/>
@@ -13288,40 +15445,54 @@
     </i>
   </colItems>
   <dataFields count="1">
-    <dataField name="Contagem de nacionalidade" fld="3" subtotal="count" baseField="0" baseItem="0"/>
+    <dataField name="Contagem de Nacionalidades" fld="3" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
-  <formats count="6">
-    <format dxfId="11">
+  <formats count="7">
+    <format dxfId="46">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="10">
+    <format dxfId="47">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="9">
+    <format dxfId="48">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="8">
+    <format dxfId="49">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="7">
+    <format dxfId="50">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="6">
+    <format dxfId="51">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
+    <format dxfId="52">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
   </formats>
+  <chartFormats count="1">
+    <chartFormat chart="1" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
@@ -13334,7 +15505,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{996EC5F2-74EB-477F-A9D9-AF44A2544855}" name="Tabela dinâmica3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Faixa Etária" colHeaderCaption="Tipo de Movimentação">
   <location ref="Y14:Z20" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -13411,43 +15582,43 @@
     <dataField name="Contagem de Jogadores" fld="8" subtotal="count" baseField="8" baseItem="0"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="20">
+    <format dxfId="67">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="19">
+    <format dxfId="66">
       <pivotArea field="8" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="18">
+    <format dxfId="65">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="17">
+    <format dxfId="64">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="16">
+    <format dxfId="63">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="15">
+    <format dxfId="62">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="14">
+    <format dxfId="61">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="13">
+    <format dxfId="60">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="12">
+    <format dxfId="59">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -13474,7 +15645,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
   <location ref="O14:P19" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -13487,7 +15658,7 @@
       </items>
     </pivotField>
     <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0" sortType="descending">
+    <pivotField axis="axisRow" showAll="0" sortType="ascending">
       <items count="4">
         <item x="1"/>
         <item x="2"/>
@@ -13519,13 +15690,13 @@
   </rowFields>
   <rowItems count="4">
     <i>
-      <x v="2"/>
+      <x v="1"/>
     </i>
     <i>
       <x/>
     </i>
     <i>
-      <x v="1"/>
+      <x v="2"/>
     </i>
     <i t="grand">
       <x/>
@@ -13543,39 +15714,39 @@
     <dataField name="Soma do Valor das Transferências" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="29">
+    <format dxfId="76">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="28">
+    <format dxfId="75">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="27">
+    <format dxfId="74">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="26">
+    <format dxfId="73">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="25">
+    <format dxfId="72">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="24">
+    <format dxfId="71">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="23">
+    <format dxfId="70">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="22">
+    <format dxfId="69">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="21">
+    <format dxfId="68">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -15449,7 +17620,7 @@
   <sheetPr>
     <tabColor theme="6" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A4:AL29"/>
+  <dimension ref="A4:AO47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.5703125" bestFit="1" customWidth="1"/>
@@ -15468,12 +17639,14 @@
     <col min="27" max="27" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="24" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="24.140625" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="27" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="28.140625" bestFit="1" customWidth="1"/>
     <col min="38" max="38" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="39" max="40" width="11" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="11" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="28.7109375" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="27.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:41" x14ac:dyDescent="0.25">
       <c r="C4" s="7" t="s">
         <v>158</v>
       </c>
@@ -15493,7 +17666,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="5" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:41" x14ac:dyDescent="0.25">
       <c r="C5" s="2">
         <f>COUNTA('Dados Tratados'!A3:A24)</f>
         <v>22</v>
@@ -15519,7 +17692,7 @@
         <v>25.454545454545453</v>
       </c>
     </row>
-    <row r="14" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
         <v>167</v>
       </c>
@@ -15538,14 +17711,20 @@
       <c r="Z14" s="10" t="s">
         <v>171</v>
       </c>
-      <c r="AK14" s="8" t="s">
-        <v>181</v>
+      <c r="AK14" s="10" t="s">
+        <v>182</v>
       </c>
       <c r="AL14" s="8" t="s">
         <v>175</v>
       </c>
+      <c r="AN14" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="AO14" s="10" t="s">
+        <v>175</v>
+      </c>
     </row>
-    <row r="15" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
         <v>165</v>
       </c>
@@ -15589,13 +17768,19 @@
         <v>180</v>
       </c>
       <c r="AK15" s="10" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AL15" s="2" t="s">
         <v>18</v>
       </c>
+      <c r="AN15" s="10" t="s">
+        <v>183</v>
+      </c>
+      <c r="AO15" s="2" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="16" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>9</v>
       </c>
@@ -15616,17 +17801,17 @@
         <v>-65000000</v>
       </c>
       <c r="O16" s="2" t="s">
-        <v>156</v>
+        <v>70</v>
       </c>
       <c r="P16" s="6">
-        <v>213900000</v>
+        <v>138800000</v>
       </c>
       <c r="R16" s="2" t="s">
         <v>156</v>
       </c>
       <c r="S16" s="13">
         <f>P16/$P$19</f>
-        <v>0.3866594360086768</v>
+        <v>0.25090383224873464</v>
       </c>
       <c r="Y16" s="2" t="s">
         <v>179</v>
@@ -15642,13 +17827,19 @@
         <v>6.25E-2</v>
       </c>
       <c r="AK16" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="AL16" s="2">
+        <v>13</v>
+      </c>
+      <c r="AL16" s="17">
         <v>1</v>
       </c>
+      <c r="AN16" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="AO16" s="17">
+        <v>1</v>
+      </c>
     </row>
-    <row r="17" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>34</v>
       </c>
@@ -15695,13 +17886,19 @@
         <v>6.25E-2</v>
       </c>
       <c r="AK17" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="AL17" s="2">
+        <v>129</v>
+      </c>
+      <c r="AL17" s="17">
         <v>1</v>
       </c>
+      <c r="AN17" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="AO17" s="17">
+        <v>1</v>
+      </c>
     </row>
-    <row r="18" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>55</v>
       </c>
@@ -15722,17 +17919,17 @@
         <v>-58000000</v>
       </c>
       <c r="O18" s="2" t="s">
-        <v>70</v>
+        <v>156</v>
       </c>
       <c r="P18" s="6">
-        <v>138800000</v>
+        <v>213900000</v>
       </c>
       <c r="R18" s="2" t="s">
         <v>70</v>
       </c>
       <c r="S18" s="13">
         <f>P18/$P$19</f>
-        <v>0.25090383224873464</v>
+        <v>0.3866594360086768</v>
       </c>
       <c r="Y18" s="2" t="s">
         <v>177</v>
@@ -15748,13 +17945,19 @@
         <v>0.1875</v>
       </c>
       <c r="AK18" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="AL18" s="2">
+        <v>151</v>
+      </c>
+      <c r="AL18" s="17">
         <v>1</v>
       </c>
+      <c r="AN18" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="AO18" s="17">
+        <v>1</v>
+      </c>
     </row>
-    <row r="19" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>75</v>
       </c>
@@ -15774,7 +17977,7 @@
         <f t="shared" si="0"/>
         <v>-55700000</v>
       </c>
-      <c r="O19" t="s">
+      <c r="O19" s="18" t="s">
         <v>164</v>
       </c>
       <c r="P19" s="6">
@@ -15801,13 +18004,19 @@
         <v>0.6875</v>
       </c>
       <c r="AK19" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="AL19" s="2">
+        <v>124</v>
+      </c>
+      <c r="AL19" s="17">
         <v>1</v>
       </c>
+      <c r="AN19" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="AO19" s="17">
+        <v>1</v>
+      </c>
     </row>
-    <row r="20" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>93</v>
       </c>
@@ -15841,13 +18050,19 @@
         <v>1</v>
       </c>
       <c r="AK20" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="AL20" s="2">
+        <v>132</v>
+      </c>
+      <c r="AL20" s="17">
         <v>1</v>
       </c>
+      <c r="AN20" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="AO20" s="17">
+        <v>1</v>
+      </c>
     </row>
-    <row r="21" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>109</v>
       </c>
@@ -15868,13 +18083,19 @@
         <v>-92500000</v>
       </c>
       <c r="AK21" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="AL21" s="2">
+        <v>44</v>
+      </c>
+      <c r="AL21" s="17">
         <v>1</v>
       </c>
+      <c r="AN21" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="AO21" s="17">
+        <v>1</v>
+      </c>
     </row>
-    <row r="22" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
         <v>164</v>
       </c>
@@ -15895,72 +18116,264 @@
         <v>-373400000</v>
       </c>
       <c r="AK22" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="AL22" s="17">
+        <v>1</v>
+      </c>
+      <c r="AN22" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="AO22" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="AK23" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="AL23" s="17">
+        <v>1</v>
+      </c>
+      <c r="AN23" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="AO23" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="AK24" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="AL24" s="17">
+        <v>1</v>
+      </c>
+      <c r="AN24" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="AO24" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="AK25" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="AL25" s="17">
+        <v>1</v>
+      </c>
+      <c r="AN25" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="AO25" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="AK26" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="AL26" s="17">
+        <v>1</v>
+      </c>
+      <c r="AN26" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="AO26" s="17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="AK27" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="AL22" s="2">
+      <c r="AL27" s="17">
         <v>2</v>
       </c>
+      <c r="AN27" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="AO27" s="17">
+        <v>1</v>
+      </c>
     </row>
-    <row r="23" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="AK23" s="2" t="s">
+    <row r="28" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="AK28" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="AL23" s="2">
+      <c r="AL28" s="17">
         <v>3</v>
       </c>
+      <c r="AN28" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="AO28" s="17">
+        <v>1</v>
+      </c>
     </row>
-    <row r="24" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="AK24" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="AL24" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="AK25" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="AL25" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="AK26" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="AL26" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="AK27" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="AL27" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="AK28" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="AL28" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:41" x14ac:dyDescent="0.25">
       <c r="AK29" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="AL29" s="2">
+      <c r="AL29" s="17">
+        <v>16</v>
+      </c>
+      <c r="AN29" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="AO29" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="AN30" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="AO30" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="AN31" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="AO31" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="AN32" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="AO32" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="40:41" x14ac:dyDescent="0.25">
+      <c r="AN33" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="AO33" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="40:41" x14ac:dyDescent="0.25">
+      <c r="AN34" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="AO34" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="40:41" x14ac:dyDescent="0.25">
+      <c r="AN35" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="AO35" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="40:41" x14ac:dyDescent="0.25">
+      <c r="AN36" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="AO36" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="40:41" x14ac:dyDescent="0.25">
+      <c r="AN37" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="AO37" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="40:41" x14ac:dyDescent="0.25">
+      <c r="AN38" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="AO38" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="40:41" x14ac:dyDescent="0.25">
+      <c r="AN39" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="AO39" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="40:41" x14ac:dyDescent="0.25">
+      <c r="AN40" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="AO40" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="40:41" x14ac:dyDescent="0.25">
+      <c r="AN41" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="AO41" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="40:41" x14ac:dyDescent="0.25">
+      <c r="AN42" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="AO42" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="40:41" x14ac:dyDescent="0.25">
+      <c r="AN43" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="AO43" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="40:41" x14ac:dyDescent="0.25">
+      <c r="AN44" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="AO44" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="40:41" x14ac:dyDescent="0.25">
+      <c r="AN45" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="AO45" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="40:41" x14ac:dyDescent="0.25">
+      <c r="AN46" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="AO46" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="40:41" x14ac:dyDescent="0.25">
+      <c r="AN47" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="AO47" s="17">
         <v>16</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId5"/>
-  <drawing r:id="rId6"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId6"/>
+  <drawing r:id="rId7"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
34. Término da Conclusão
Término da quarta conclusão.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60DB313B-E85E-492D-A72B-56390D68EFA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{534F1DE2-6EF9-4A80-A694-4F56C5D30E65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
   <calcPr calcId="191029"/>
   <pivotCaches>
     <pivotCache cacheId="0" r:id="rId6"/>
-    <pivotCache cacheId="2" r:id="rId7"/>
+    <pivotCache cacheId="1" r:id="rId7"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -671,7 +671,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -715,16 +715,87 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentagem" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="77">
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
     <dxf>
       <alignment horizontal="center"/>
     </dxf>
@@ -862,81 +933,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
     </dxf>
     <dxf>
       <alignment horizontal="center"/>
@@ -11995,12 +11991,12 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>36</xdr:col>
-      <xdr:colOff>44470</xdr:colOff>
+      <xdr:col>35</xdr:col>
+      <xdr:colOff>259240</xdr:colOff>
       <xdr:row>70</xdr:row>
-      <xdr:rowOff>105249</xdr:rowOff>
+      <xdr:rowOff>125239</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="11067773" cy="1845633"/>
+    <xdr:ext cx="11907362" cy="2283959"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="29" name="CaixaDeTexto 28">
@@ -12014,8 +12010,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="36697748" y="13314447"/>
-          <a:ext cx="11067773" cy="1845633"/>
+          <a:off x="36301160" y="13222114"/>
+          <a:ext cx="11907362" cy="2283959"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -12088,19 +12084,19 @@
           <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
-            <a:t>e pelas consecutivas pátrias, como Brasil e Uruguai, que contabilizam apenas </a:t>
+            <a:t>enquanto as demais nacionalidades apresentam apenas </a:t>
           </a:r>
           <a:r>
             <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
-            <a:t>1</a:t>
+            <a:t>1 </a:t>
           </a:r>
           <a:r>
             <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
-            <a:t> atleta cada.</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="ctr"/>
+            <a:t>cada.</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
           <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
         </a:p>
         <a:p>
@@ -12130,23 +12126,44 @@
           </a:r>
           <a:r>
             <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
-            <a:t> de nações se faz presente. Cerca de </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
-            <a:t>11</a:t>
+            <a:t> de nações se faz presente. Além disso,</a:t>
           </a:r>
           <a:br>
             <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
           </a:br>
           <a:r>
             <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
-            <a:t>jogadores não são representados pelas bandeiras de Inglaterra ou Holanda.</a:t>
+            <a:t>cerca de </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>11 </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>ativos contratados não são representados pelas bandeiras de Inglaterra ou Holanda. Isso sugere uma possível estratégia adotada pelo departamento</a:t>
           </a:r>
           <a:br>
             <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
           </a:br>
-          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>de scouting do clube visando o mapeamento de atletas que estejam se desenvolvendo em outras ligas europeias, porém sem perder contato com as</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>novidades que surgem no mercado doméstico — uma vez que todos os jogadores ingleses foram contratados enquanto atuavam por equipes conterrâneas</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>como Leicester City, Bournemouth e Leeds United.</a:t>
+          </a:r>
         </a:p>
       </xdr:txBody>
     </xdr:sp>
@@ -14525,7 +14542,465 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FB686887-B509-4E7E-B605-6A13972A6E0B}" name="Tabela dinâmica5" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Origem das Contratações" colHeaderCaption="Contagem de Jogadores">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{904CEA3A-CD0A-459C-A420-1FB249800D4C}" name="Tabela dinâmica4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Nacionalidades" colHeaderCaption="Contagem de Jogadores">
+  <location ref="AK14:AL29" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="9">
+    <pivotField axis="axisCol" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item h="1" x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" dataField="1" showAll="0" sortType="ascending">
+      <items count="15">
+        <item x="6"/>
+        <item x="4"/>
+        <item x="9"/>
+        <item x="11"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="12"/>
+        <item x="5"/>
+        <item x="10"/>
+        <item x="13"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="2">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+            <reference field="0" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="21">
+        <item x="12"/>
+        <item x="9"/>
+        <item x="7"/>
+        <item x="15"/>
+        <item x="5"/>
+        <item x="17"/>
+        <item x="11"/>
+        <item x="10"/>
+        <item x="2"/>
+        <item x="8"/>
+        <item x="18"/>
+        <item x="13"/>
+        <item x="0"/>
+        <item x="16"/>
+        <item x="19"/>
+        <item x="1"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item x="14"/>
+        <item x="6"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="3"/>
+  </rowFields>
+  <rowItems count="14">
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="0"/>
+  </colFields>
+  <colItems count="1">
+    <i>
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Contagem de Nacionalidades" fld="3" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="7">
+    <format dxfId="6">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="3" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="5">
+      <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="4">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="3" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="3">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+    <format dxfId="2">
+      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="1">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="0">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="1">
+    <chartFormat chart="1" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{996EC5F2-74EB-477F-A9D9-AF44A2544855}" name="Tabela dinâmica3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Faixa Etária" colHeaderCaption="Tipo de Movimentação">
+  <location ref="Y14:Z20" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="10">
+    <pivotField showAll="0"/>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="3">
+        <item h="1" x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField axis="axisRow" dataField="1" showAll="0" sortType="ascending">
+      <items count="9">
+        <item m="1" x="5"/>
+        <item m="1" x="4"/>
+        <item m="1" x="7"/>
+        <item m="1" x="6"/>
+        <item x="3"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="2">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+            <reference field="1" count="1" selected="0">
+              <x v="1"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="8"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="1"/>
+  </colFields>
+  <colItems count="1">
+    <i>
+      <x v="1"/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Contagem de Jogadores" fld="8" subtotal="count" baseField="8" baseItem="0"/>
+  </dataFields>
+  <formats count="9">
+    <format dxfId="15">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="8" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="14">
+      <pivotArea field="8" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="13">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="8" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="12">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+    <format dxfId="11">
+      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="10">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="9">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="1" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="8">
+      <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
+    </format>
+    <format dxfId="7">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="1">
+    <chartFormat chart="2" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
+  <location ref="O14:P19" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="10">
+    <pivotField showAll="0"/>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="3">
+        <item h="1" x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0" sortType="ascending">
+      <items count="4">
+        <item x="1"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="2">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+            <reference field="1" count="1" selected="0">
+              <x v="1"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="3"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="1"/>
+  </colFields>
+  <colItems count="1">
+    <i>
+      <x v="1"/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Soma do Valor das Transferências" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
+  </dataFields>
+  <formats count="9">
+    <format dxfId="24">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="23">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="22">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="21">
+      <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
+    </format>
+    <format dxfId="20">
+      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="19">
+      <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="18">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="3" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="17">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="1" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="16">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="1">
+    <chartFormat chart="1" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FB686887-B509-4E7E-B605-6A13972A6E0B}" name="Tabela dinâmica5" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Origem das Contratações" colHeaderCaption="Contagem de Jogadores">
   <location ref="AN14:AO47" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField axis="axisCol" showAll="0">
@@ -14700,22 +15175,22 @@
     <dataField name="Clubes" fld="3" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="46">
-    <format dxfId="45">
+    <format dxfId="70">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="44">
+    <format dxfId="69">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="43">
+    <format dxfId="68">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="42">
+    <format dxfId="67">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="41">
+    <format dxfId="66">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="40">
+    <format dxfId="65">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="15">
@@ -14738,10 +15213,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="39">
+    <format dxfId="64">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="38">
+    <format dxfId="63">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14753,7 +15228,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="37">
+    <format dxfId="62">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14765,7 +15240,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="36">
+    <format dxfId="61">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14777,7 +15252,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="35">
+    <format dxfId="60">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14789,7 +15264,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="34">
+    <format dxfId="59">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14801,7 +15276,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="33">
+    <format dxfId="58">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="2">
@@ -14814,7 +15289,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="32">
+    <format dxfId="57">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14826,7 +15301,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="31">
+    <format dxfId="56">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14838,7 +15313,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="30">
+    <format dxfId="55">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14850,7 +15325,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="29">
+    <format dxfId="54">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14862,7 +15337,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="28">
+    <format dxfId="53">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14874,7 +15349,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="27">
+    <format dxfId="52">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14886,7 +15361,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="26">
+    <format dxfId="51">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14898,7 +15373,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="25">
+    <format dxfId="50">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14910,7 +15385,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="24">
+    <format dxfId="49">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14922,29 +15397,29 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="23">
+    <format dxfId="48">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="22">
+    <format dxfId="47">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="21">
+    <format dxfId="46">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="20">
+    <format dxfId="45">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="19">
+    <format dxfId="44">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="18">
+    <format dxfId="43">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="17">
+    <format dxfId="42">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="15">
@@ -14967,10 +15442,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="16">
+    <format dxfId="41">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="15">
+    <format dxfId="40">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14982,7 +15457,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="14">
+    <format dxfId="39">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14994,7 +15469,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="13">
+    <format dxfId="38">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -15006,7 +15481,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="12">
+    <format dxfId="37">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -15018,7 +15493,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="11">
+    <format dxfId="36">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -15030,7 +15505,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="10">
+    <format dxfId="35">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="2">
@@ -15043,7 +15518,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="9">
+    <format dxfId="34">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -15055,7 +15530,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="8">
+    <format dxfId="33">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -15067,7 +15542,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="7">
+    <format dxfId="32">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -15079,7 +15554,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="6">
+    <format dxfId="31">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -15091,7 +15566,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="5">
+    <format dxfId="30">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -15103,7 +15578,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="4">
+    <format dxfId="29">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -15115,7 +15590,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="3">
+    <format dxfId="28">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -15127,7 +15602,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="2">
+    <format dxfId="27">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -15139,7 +15614,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="1">
+    <format dxfId="26">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -15151,7 +15626,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="0">
+    <format dxfId="25">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
@@ -15171,7 +15646,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6" rowHeaderCaption="Temporadas" colHeaderCaption="">
   <location ref="A14:D22" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -15246,34 +15721,34 @@
     <dataField name="Somas de Entradas e Saídas" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="58">
+    <format dxfId="76">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="57">
+    <format dxfId="75">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="56">
+    <format dxfId="74">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="55">
+    <format dxfId="73">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="54">
+    <format dxfId="72">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="53">
+    <format dxfId="71">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -15298,464 +15773,6 @@
           </reference>
           <reference field="1" count="1" selected="0">
             <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{904CEA3A-CD0A-459C-A420-1FB249800D4C}" name="Tabela dinâmica4" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Nacionalidades" colHeaderCaption="Contagem de Jogadores">
-  <location ref="AK14:AL29" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="9">
-    <pivotField axis="axisCol" showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item h="1" x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" dataField="1" showAll="0" sortType="ascending">
-      <items count="15">
-        <item x="6"/>
-        <item x="4"/>
-        <item x="9"/>
-        <item x="11"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="12"/>
-        <item x="5"/>
-        <item x="10"/>
-        <item x="13"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item t="default"/>
-      </items>
-      <autoSortScope>
-        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
-          <references count="2">
-            <reference field="4294967294" count="1" selected="0">
-              <x v="0"/>
-            </reference>
-            <reference field="0" count="1" selected="0">
-              <x v="0"/>
-            </reference>
-          </references>
-        </pivotArea>
-      </autoSortScope>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="21">
-        <item x="12"/>
-        <item x="9"/>
-        <item x="7"/>
-        <item x="15"/>
-        <item x="5"/>
-        <item x="17"/>
-        <item x="11"/>
-        <item x="10"/>
-        <item x="2"/>
-        <item x="8"/>
-        <item x="18"/>
-        <item x="13"/>
-        <item x="0"/>
-        <item x="16"/>
-        <item x="19"/>
-        <item x="1"/>
-        <item x="4"/>
-        <item x="3"/>
-        <item x="14"/>
-        <item x="6"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="3"/>
-  </rowFields>
-  <rowItems count="14">
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="13"/>
-    </i>
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="11"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="12"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="0"/>
-  </colFields>
-  <colItems count="1">
-    <i>
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Contagem de Nacionalidades" fld="3" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="7">
-    <format dxfId="46">
-      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
-        <references count="1">
-          <reference field="3" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="47">
-      <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
-    </format>
-    <format dxfId="48">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="3" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="49">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
-    </format>
-    <format dxfId="50">
-      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="51">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="0" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="52">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="1">
-    <chartFormat chart="1" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{996EC5F2-74EB-477F-A9D9-AF44A2544855}" name="Tabela dinâmica3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Faixa Etária" colHeaderCaption="Tipo de Movimentação">
-  <location ref="Y14:Z20" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="10">
-    <pivotField showAll="0"/>
-    <pivotField axis="axisCol" showAll="0">
-      <items count="3">
-        <item h="1" x="1"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField axis="axisRow" dataField="1" showAll="0" sortType="ascending">
-      <items count="9">
-        <item m="1" x="5"/>
-        <item m="1" x="4"/>
-        <item m="1" x="7"/>
-        <item m="1" x="6"/>
-        <item x="3"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-      <autoSortScope>
-        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
-          <references count="2">
-            <reference field="4294967294" count="1" selected="0">
-              <x v="0"/>
-            </reference>
-            <reference field="1" count="1" selected="0">
-              <x v="1"/>
-            </reference>
-          </references>
-        </pivotArea>
-      </autoSortScope>
-    </pivotField>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="8"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="1"/>
-  </colFields>
-  <colItems count="1">
-    <i>
-      <x v="1"/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Contagem de Jogadores" fld="8" subtotal="count" baseField="8" baseItem="0"/>
-  </dataFields>
-  <formats count="9">
-    <format dxfId="67">
-      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
-        <references count="1">
-          <reference field="8" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="66">
-      <pivotArea field="8" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
-    </format>
-    <format dxfId="65">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="8" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="64">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
-    </format>
-    <format dxfId="63">
-      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="62">
-      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="61">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="1" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="60">
-      <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
-    </format>
-    <format dxfId="59">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="1">
-    <chartFormat chart="2" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
-  <location ref="O14:P19" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="10">
-    <pivotField showAll="0"/>
-    <pivotField axis="axisCol" showAll="0">
-      <items count="3">
-        <item h="1" x="1"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0" sortType="ascending">
-      <items count="4">
-        <item x="1"/>
-        <item x="2"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-      <autoSortScope>
-        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
-          <references count="2">
-            <reference field="4294967294" count="1" selected="0">
-              <x v="0"/>
-            </reference>
-            <reference field="1" count="1" selected="0">
-              <x v="1"/>
-            </reference>
-          </references>
-        </pivotArea>
-      </autoSortScope>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="3"/>
-  </rowFields>
-  <rowItems count="4">
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="1"/>
-  </colFields>
-  <colItems count="1">
-    <i>
-      <x v="1"/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Soma do Valor das Transferências" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
-  </dataFields>
-  <formats count="9">
-    <format dxfId="76">
-      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="75">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="74">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="73">
-      <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
-    </format>
-    <format dxfId="72">
-      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="71">
-      <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
-    </format>
-    <format dxfId="70">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="3" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="69">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="1" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="68">
-      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="1">
-    <chartFormat chart="1" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
           </reference>
         </references>
       </pivotArea>
@@ -17829,13 +17846,13 @@
       <c r="AK16" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="AL16" s="17">
+      <c r="AL16" s="2">
         <v>1</v>
       </c>
       <c r="AN16" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="AO16" s="17">
+      <c r="AO16" s="2">
         <v>1</v>
       </c>
     </row>
@@ -17888,13 +17905,13 @@
       <c r="AK17" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="AL17" s="17">
+      <c r="AL17" s="2">
         <v>1</v>
       </c>
       <c r="AN17" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="AO17" s="17">
+      <c r="AO17" s="2">
         <v>1</v>
       </c>
     </row>
@@ -17947,13 +17964,13 @@
       <c r="AK18" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="AL18" s="17">
+      <c r="AL18" s="2">
         <v>1</v>
       </c>
       <c r="AN18" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="AO18" s="17">
+      <c r="AO18" s="2">
         <v>1</v>
       </c>
     </row>
@@ -17977,7 +17994,7 @@
         <f t="shared" si="0"/>
         <v>-55700000</v>
       </c>
-      <c r="O19" s="18" t="s">
+      <c r="O19" t="s">
         <v>164</v>
       </c>
       <c r="P19" s="6">
@@ -18006,13 +18023,13 @@
       <c r="AK19" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="AL19" s="17">
+      <c r="AL19" s="2">
         <v>1</v>
       </c>
       <c r="AN19" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="AO19" s="17">
+      <c r="AO19" s="2">
         <v>1</v>
       </c>
     </row>
@@ -18052,13 +18069,13 @@
       <c r="AK20" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="AL20" s="17">
+      <c r="AL20" s="2">
         <v>1</v>
       </c>
       <c r="AN20" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="AO20" s="17">
+      <c r="AO20" s="2">
         <v>1</v>
       </c>
     </row>
@@ -18085,13 +18102,13 @@
       <c r="AK21" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="AL21" s="17">
+      <c r="AL21" s="2">
         <v>1</v>
       </c>
       <c r="AN21" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="AO21" s="17">
+      <c r="AO21" s="2">
         <v>1</v>
       </c>
     </row>
@@ -18118,13 +18135,13 @@
       <c r="AK22" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="AL22" s="17">
+      <c r="AL22" s="2">
         <v>1</v>
       </c>
       <c r="AN22" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="AO22" s="17">
+      <c r="AO22" s="2">
         <v>1</v>
       </c>
     </row>
@@ -18132,13 +18149,13 @@
       <c r="AK23" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="AL23" s="17">
+      <c r="AL23" s="2">
         <v>1</v>
       </c>
       <c r="AN23" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="AO23" s="17">
+      <c r="AO23" s="2">
         <v>1</v>
       </c>
     </row>
@@ -18146,13 +18163,13 @@
       <c r="AK24" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="AL24" s="17">
+      <c r="AL24" s="2">
         <v>1</v>
       </c>
       <c r="AN24" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="AO24" s="17">
+      <c r="AO24" s="2">
         <v>1</v>
       </c>
     </row>
@@ -18160,13 +18177,13 @@
       <c r="AK25" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="AL25" s="17">
+      <c r="AL25" s="2">
         <v>1</v>
       </c>
       <c r="AN25" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="AO25" s="17">
+      <c r="AO25" s="2">
         <v>1</v>
       </c>
     </row>
@@ -18174,13 +18191,13 @@
       <c r="AK26" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="AL26" s="17">
+      <c r="AL26" s="2">
         <v>1</v>
       </c>
       <c r="AN26" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="AO26" s="17">
+      <c r="AO26" s="2">
         <v>2</v>
       </c>
     </row>
@@ -18188,13 +18205,13 @@
       <c r="AK27" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="AL27" s="17">
+      <c r="AL27" s="2">
         <v>2</v>
       </c>
       <c r="AN27" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="AO27" s="17">
+      <c r="AO27" s="2">
         <v>1</v>
       </c>
     </row>
@@ -18202,13 +18219,13 @@
       <c r="AK28" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="AL28" s="17">
+      <c r="AL28" s="2">
         <v>3</v>
       </c>
       <c r="AN28" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="AO28" s="17">
+      <c r="AO28" s="2">
         <v>1</v>
       </c>
     </row>
@@ -18216,13 +18233,13 @@
       <c r="AK29" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="AL29" s="17">
+      <c r="AL29" s="2">
         <v>16</v>
       </c>
       <c r="AN29" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="AO29" s="17">
+      <c r="AO29" s="2">
         <v>1</v>
       </c>
     </row>
@@ -18230,7 +18247,7 @@
       <c r="AN30" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="AO30" s="17">
+      <c r="AO30" s="2">
         <v>1</v>
       </c>
     </row>
@@ -18238,7 +18255,7 @@
       <c r="AN31" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="AO31" s="17">
+      <c r="AO31" s="2">
         <v>1</v>
       </c>
     </row>
@@ -18246,7 +18263,7 @@
       <c r="AN32" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="AO32" s="17">
+      <c r="AO32" s="2">
         <v>1</v>
       </c>
     </row>
@@ -18254,7 +18271,7 @@
       <c r="AN33" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="AO33" s="17">
+      <c r="AO33" s="2">
         <v>1</v>
       </c>
     </row>
@@ -18262,7 +18279,7 @@
       <c r="AN34" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="AO34" s="17">
+      <c r="AO34" s="2">
         <v>1</v>
       </c>
     </row>
@@ -18270,7 +18287,7 @@
       <c r="AN35" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="AO35" s="17">
+      <c r="AO35" s="2">
         <v>1</v>
       </c>
     </row>
@@ -18278,7 +18295,7 @@
       <c r="AN36" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="AO36" s="17">
+      <c r="AO36" s="2">
         <v>1</v>
       </c>
     </row>
@@ -18286,7 +18303,7 @@
       <c r="AN37" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="AO37" s="17">
+      <c r="AO37" s="2">
         <v>1</v>
       </c>
     </row>
@@ -18294,7 +18311,7 @@
       <c r="AN38" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="AO38" s="17">
+      <c r="AO38" s="2">
         <v>1</v>
       </c>
     </row>
@@ -18302,7 +18319,7 @@
       <c r="AN39" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="AO39" s="17">
+      <c r="AO39" s="2">
         <v>1</v>
       </c>
     </row>
@@ -18310,7 +18327,7 @@
       <c r="AN40" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="AO40" s="17">
+      <c r="AO40" s="2">
         <v>1</v>
       </c>
     </row>
@@ -18318,7 +18335,7 @@
       <c r="AN41" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="AO41" s="17">
+      <c r="AO41" s="2">
         <v>1</v>
       </c>
     </row>
@@ -18326,7 +18343,7 @@
       <c r="AN42" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="AO42" s="17">
+      <c r="AO42" s="2">
         <v>1</v>
       </c>
     </row>
@@ -18334,7 +18351,7 @@
       <c r="AN43" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="AO43" s="17">
+      <c r="AO43" s="2">
         <v>1</v>
       </c>
     </row>
@@ -18342,7 +18359,7 @@
       <c r="AN44" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="AO44" s="17">
+      <c r="AO44" s="2">
         <v>1</v>
       </c>
     </row>
@@ -18350,7 +18367,7 @@
       <c r="AN45" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="AO45" s="17">
+      <c r="AO45" s="2">
         <v>1</v>
       </c>
     </row>
@@ -18358,7 +18375,7 @@
       <c r="AN46" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="AO46" s="17">
+      <c r="AO46" s="2">
         <v>1</v>
       </c>
     </row>
@@ -18366,7 +18383,7 @@
       <c r="AN47" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="AO47" s="17">
+      <c r="AO47" s="2">
         <v>16</v>
       </c>
     </row>

</xml_diff>

<commit_message>
36. Começo da Análise
Começo da quinta análise.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79BB8CF1-1D39-44FB-8DA8-FE292C7ACB79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C78B24D5-1790-47A4-AD4B-391A532F1D1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Apresentação" sheetId="3" r:id="rId1"/>
@@ -24,7 +24,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId6"/>
+    <pivotCache cacheId="4" r:id="rId6"/>
     <pivotCache cacheId="1" r:id="rId7"/>
   </pivotCaches>
   <extLst>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="185">
   <si>
     <t>temporada</t>
   </si>
@@ -671,7 +671,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -715,12 +715,2311 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentagem" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="77">
+  <dxfs count="843">
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="0.0%"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
     <dxf>
       <alignment horizontal="general"/>
     </dxf>
@@ -8662,7 +10961,7 @@
       <xdr:row>47</xdr:row>
       <xdr:rowOff>181874</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="12148329" cy="1783180"/>
+    <xdr:ext cx="12148329" cy="1595309"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="13" name="CaixaDeTexto 12">
@@ -8676,8 +10975,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="215121" y="8975490"/>
-          <a:ext cx="12148329" cy="1783180"/>
+          <a:off x="215121" y="9135374"/>
+          <a:ext cx="12148329" cy="1595309"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -8793,21 +11092,6 @@
             <a:t> posições geraram maior retorno financeiro ao clube?</a:t>
           </a:r>
           <a:endParaRPr lang="pt-BR" sz="1200" b="1"/>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1200" b="0"/>
-            <a:t>•</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1200" b="1"/>
-            <a:t> O perfil</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0"/>
-            <a:t> das contratações mudou ao longo das temporadas analisadas?</a:t>
-          </a:r>
         </a:p>
         <a:p>
           <a:pPr algn="l"/>
@@ -12169,6 +14453,193 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>52</xdr:col>
+      <xdr:colOff>1626495</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>144531</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2477025" cy="405432"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="30" name="CaixaDeTexto 29">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{10162775-C05E-4213-A566-3C891D20B9F1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="53061495" y="1276748"/>
+          <a:ext cx="2477025" cy="405432"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="2000" b="1" baseline="0"/>
+            <a:t>5. Retorno Financeiro</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>51</xdr:col>
+      <xdr:colOff>527048</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>125801</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="6129498" cy="311496"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="31" name="CaixaDeTexto 30">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{27A7B400-F5D7-451E-A9A4-6871BEE4414A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="51351010" y="1635424"/>
+          <a:ext cx="6129498" cy="311496"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0"/>
+            <a:t>Pergunta de Negócio: </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="1"/>
+            <a:t>Quais posições</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="1" baseline="0"/>
+            <a:t> geraram maior retorno financeiro ao clube?</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>51</xdr:col>
+      <xdr:colOff>557123</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>125802</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="818815" cy="311496"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="32" name="CaixaDeTexto 31">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7B90AB71-F8D7-44F2-B99C-C54B52711ED8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="51381085" y="2012830"/>
+          <a:ext cx="818815" cy="311496"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0"/>
+            <a:t>Análise: </a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -13584,7 +16055,28 @@
       </sharedItems>
     </cacheField>
     <cacheField name="nome_jogador" numFmtId="0">
-      <sharedItems/>
+      <sharedItems count="20">
+        <s v="Tanguy Ndombélé"/>
+        <s v="Steven Bergwijn"/>
+        <s v="Christian Eriksen"/>
+        <s v="Pierre-Emile Højbjerg"/>
+        <s v="Sergio Reguilón"/>
+        <s v="Jan Vertonghen"/>
+        <s v="Matt Doherty"/>
+        <s v="Cristian Romero"/>
+        <s v="Dejan Kulusevski"/>
+        <s v="Toby Alderweireld"/>
+        <s v="Rodrigo Bentancur"/>
+        <s v="Richarlison"/>
+        <s v="Yves Bissouma"/>
+        <s v="Ivan Perišić"/>
+        <s v="James Maddison"/>
+        <s v="Micky van de Ven"/>
+        <s v="Harry Kane"/>
+        <s v="Brennan Johnson"/>
+        <s v="Dominic Solanke"/>
+        <s v="Archie Gray"/>
+      </sharedItems>
     </cacheField>
     <cacheField name="posição" numFmtId="0">
       <sharedItems count="3">
@@ -13743,7 +16235,7 @@
   <r>
     <x v="0"/>
     <x v="0"/>
-    <s v="Tanguy Ndombélé"/>
+    <x v="0"/>
     <x v="0"/>
     <s v="França"/>
     <s v="Lyon"/>
@@ -13755,7 +16247,7 @@
   <r>
     <x v="0"/>
     <x v="0"/>
-    <s v="Steven Bergwijn"/>
+    <x v="1"/>
     <x v="1"/>
     <s v="Holanda"/>
     <s v="PSV Eindhoven"/>
@@ -13767,7 +16259,7 @@
   <r>
     <x v="0"/>
     <x v="1"/>
-    <s v="Christian Eriksen"/>
+    <x v="2"/>
     <x v="0"/>
     <s v="Dinamarca"/>
     <s v="Inter Milan"/>
@@ -13779,7 +16271,7 @@
   <r>
     <x v="1"/>
     <x v="0"/>
-    <s v="Pierre-Emile Højbjerg"/>
+    <x v="3"/>
     <x v="0"/>
     <s v="Dinamarca"/>
     <s v="Southampton"/>
@@ -13791,7 +16283,7 @@
   <r>
     <x v="1"/>
     <x v="0"/>
-    <s v="Sergio Reguilón"/>
+    <x v="4"/>
     <x v="2"/>
     <s v="Espanha"/>
     <s v="Real Madrid"/>
@@ -13803,7 +16295,7 @@
   <r>
     <x v="1"/>
     <x v="1"/>
-    <s v="Jan Vertonghen"/>
+    <x v="5"/>
     <x v="2"/>
     <s v="Bélgica"/>
     <s v="Benfica"/>
@@ -13815,7 +16307,7 @@
   <r>
     <x v="1"/>
     <x v="0"/>
-    <s v="Matt Doherty"/>
+    <x v="6"/>
     <x v="2"/>
     <s v="Irlanda"/>
     <s v="Wolves"/>
@@ -13827,7 +16319,7 @@
   <r>
     <x v="2"/>
     <x v="0"/>
-    <s v="Cristian Romero"/>
+    <x v="7"/>
     <x v="2"/>
     <s v="Argentina"/>
     <s v="Atalanta"/>
@@ -13839,7 +16331,7 @@
   <r>
     <x v="2"/>
     <x v="0"/>
-    <s v="Dejan Kulusevski"/>
+    <x v="8"/>
     <x v="1"/>
     <s v="Suécia"/>
     <s v="Juventus"/>
@@ -13851,7 +16343,7 @@
   <r>
     <x v="2"/>
     <x v="1"/>
-    <s v="Toby Alderweireld"/>
+    <x v="9"/>
     <x v="2"/>
     <s v="Bélgica"/>
     <s v="Al Duhail"/>
@@ -13863,7 +16355,7 @@
   <r>
     <x v="2"/>
     <x v="0"/>
-    <s v="Rodrigo Bentancur"/>
+    <x v="10"/>
     <x v="0"/>
     <s v="Uruguai"/>
     <s v="Juventus"/>
@@ -13875,7 +16367,7 @@
   <r>
     <x v="3"/>
     <x v="0"/>
-    <s v="Richarlison"/>
+    <x v="11"/>
     <x v="1"/>
     <s v="Brasil"/>
     <s v="Everton"/>
@@ -13887,7 +16379,7 @@
   <r>
     <x v="3"/>
     <x v="0"/>
-    <s v="Yves Bissouma"/>
+    <x v="12"/>
     <x v="0"/>
     <s v="Mali"/>
     <s v="Brighton"/>
@@ -13899,7 +16391,7 @@
   <r>
     <x v="3"/>
     <x v="1"/>
-    <s v="Steven Bergwijn"/>
+    <x v="1"/>
     <x v="1"/>
     <s v="Holanda"/>
     <s v="Ajax"/>
@@ -13911,7 +16403,7 @@
   <r>
     <x v="3"/>
     <x v="0"/>
-    <s v="Ivan Perišić"/>
+    <x v="13"/>
     <x v="1"/>
     <s v="Croácia"/>
     <s v="Inter Milan"/>
@@ -13923,7 +16415,7 @@
   <r>
     <x v="4"/>
     <x v="0"/>
-    <s v="James Maddison"/>
+    <x v="14"/>
     <x v="0"/>
     <s v="Inglaterra"/>
     <s v="Leicester City"/>
@@ -13935,7 +16427,7 @@
   <r>
     <x v="4"/>
     <x v="0"/>
-    <s v="Micky van de Ven"/>
+    <x v="15"/>
     <x v="2"/>
     <s v="Holanda"/>
     <s v="Wolfsburg"/>
@@ -13947,7 +16439,7 @@
   <r>
     <x v="4"/>
     <x v="1"/>
-    <s v="Harry Kane"/>
+    <x v="16"/>
     <x v="1"/>
     <s v="Inglaterra"/>
     <s v="Bayern München"/>
@@ -13959,7 +16451,7 @@
   <r>
     <x v="4"/>
     <x v="0"/>
-    <s v="Brennan Johnson"/>
+    <x v="17"/>
     <x v="1"/>
     <s v="País De Gales"/>
     <s v="Nottingham Forest"/>
@@ -13971,7 +16463,7 @@
   <r>
     <x v="5"/>
     <x v="0"/>
-    <s v="Dominic Solanke"/>
+    <x v="18"/>
     <x v="1"/>
     <s v="Inglaterra"/>
     <s v="Bournemouth"/>
@@ -13983,7 +16475,7 @@
   <r>
     <x v="5"/>
     <x v="0"/>
-    <s v="Archie Gray"/>
+    <x v="19"/>
     <x v="0"/>
     <s v="Inglaterra"/>
     <s v="Leeds United"/>
@@ -13995,7 +16487,7 @@
   <r>
     <x v="5"/>
     <x v="1"/>
-    <s v="Pierre-Emile Højbjerg"/>
+    <x v="3"/>
     <x v="0"/>
     <s v="Dinamarca"/>
     <s v="Olympique Marseille"/>
@@ -14255,7 +16747,217 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A313B9B0-7D32-4F4A-9400-E25F20E67AB4}" name="Tabela dinâmica7" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
+  <location ref="BA14:BB19" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="10">
+    <pivotField showAll="0"/>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="3">
+        <item h="1" x="0"/>
+        <item n="Saída" x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="21">
+        <item x="19"/>
+        <item x="17"/>
+        <item x="2"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="18"/>
+        <item x="16"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="15"/>
+        <item x="3"/>
+        <item x="11"/>
+        <item x="10"/>
+        <item x="4"/>
+        <item x="1"/>
+        <item x="0"/>
+        <item x="9"/>
+        <item x="12"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0" sortType="descending">
+      <items count="4">
+        <item x="1"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="2">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+            <reference field="1" count="1" selected="0">
+              <x v="1"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="3"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="1"/>
+  </colFields>
+  <colItems count="1">
+    <i>
+      <x v="1"/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Soma do Valor das Transferências" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
+  </dataFields>
+  <formats count="16">
+    <format dxfId="0">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="3" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="1">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="2">
+      <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
+    </format>
+    <format dxfId="3">
+      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="4">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="3" count="1">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="5">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="3" count="1">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="6">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="3" count="1">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="7">
+      <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="8">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="3" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="9">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="1" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="10">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="3" count="1">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="11">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="3" count="1">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="12">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="3" count="1">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="13">
+      <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="14">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="3" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="15">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="1" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
   <location ref="O14:P19" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField showAll="0"/>
@@ -14323,39 +17025,39 @@
     <dataField name="Soma do Valor das Transferências" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="8">
+    <format dxfId="774">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="7">
+    <format dxfId="773">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="6">
+    <format dxfId="772">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="5">
+    <format dxfId="771">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="4">
+    <format dxfId="770">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="3">
+    <format dxfId="769">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="2">
+    <format dxfId="768">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="1">
+    <format dxfId="767">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="0">
+    <format dxfId="766">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -14382,7 +17084,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FB686887-B509-4E7E-B605-6A13972A6E0B}" name="Tabela dinâmica5" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Origem das Contratações" colHeaderCaption="Contagem de Jogadores">
   <location ref="AN14:AO47" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
@@ -14558,22 +17260,22 @@
     <dataField name="Clubes" fld="3" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="46">
-    <format dxfId="54">
+    <format dxfId="820">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="53">
+    <format dxfId="819">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="52">
+    <format dxfId="818">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="51">
+    <format dxfId="817">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="50">
+    <format dxfId="816">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="49">
+    <format dxfId="815">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="15">
@@ -14596,10 +17298,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="48">
+    <format dxfId="814">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="47">
+    <format dxfId="813">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14611,7 +17313,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="46">
+    <format dxfId="812">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14623,7 +17325,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="45">
+    <format dxfId="811">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14635,7 +17337,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="44">
+    <format dxfId="810">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14647,7 +17349,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="43">
+    <format dxfId="809">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14659,7 +17361,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="42">
+    <format dxfId="808">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="2">
@@ -14672,7 +17374,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="41">
+    <format dxfId="807">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14684,7 +17386,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="40">
+    <format dxfId="806">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14696,7 +17398,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="39">
+    <format dxfId="805">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14708,7 +17410,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="38">
+    <format dxfId="804">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14720,7 +17422,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="37">
+    <format dxfId="803">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14732,7 +17434,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="36">
+    <format dxfId="802">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14744,7 +17446,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="35">
+    <format dxfId="801">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14756,7 +17458,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="34">
+    <format dxfId="800">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14768,7 +17470,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="33">
+    <format dxfId="799">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14780,29 +17482,29 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="32">
+    <format dxfId="798">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="31">
+    <format dxfId="797">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="30">
+    <format dxfId="796">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="29">
+    <format dxfId="795">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="28">
+    <format dxfId="794">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="27">
+    <format dxfId="793">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="26">
+    <format dxfId="792">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="15">
@@ -14825,10 +17527,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="25">
+    <format dxfId="791">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="24">
+    <format dxfId="790">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14840,7 +17542,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="23">
+    <format dxfId="789">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14852,7 +17554,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="22">
+    <format dxfId="788">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14864,7 +17566,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="21">
+    <format dxfId="787">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14876,7 +17578,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="20">
+    <format dxfId="786">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14888,7 +17590,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="19">
+    <format dxfId="785">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="2">
@@ -14901,7 +17603,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="18">
+    <format dxfId="784">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14913,7 +17615,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="17">
+    <format dxfId="783">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14925,7 +17627,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="16">
+    <format dxfId="782">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14937,7 +17639,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="15">
+    <format dxfId="781">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14949,7 +17651,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="14">
+    <format dxfId="780">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14961,7 +17663,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="13">
+    <format dxfId="779">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14973,7 +17675,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="12">
+    <format dxfId="778">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14985,7 +17687,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="11">
+    <format dxfId="777">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -14997,7 +17699,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="10">
+    <format dxfId="776">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -15009,7 +17711,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="9">
+    <format dxfId="775">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
@@ -15029,8 +17731,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6" rowHeaderCaption="Temporadas" colHeaderCaption="">
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6" rowHeaderCaption="Temporadas" colHeaderCaption="">
   <location ref="A14:D22" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField axis="axisRow" showAll="0">
@@ -15104,34 +17806,34 @@
     <dataField name="Somas de Entradas e Saídas" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="60">
+    <format dxfId="826">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="59">
+    <format dxfId="825">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="58">
+    <format dxfId="824">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="57">
+    <format dxfId="823">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="56">
+    <format dxfId="822">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="55">
+    <format dxfId="821">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -15173,7 +17875,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{904CEA3A-CD0A-459C-A420-1FB249800D4C}" name="Tabela dinâmica4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Nacionalidades" colHeaderCaption="Contagem de Jogadores">
   <location ref="AK14:AL29" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
@@ -15306,37 +18008,37 @@
     <dataField name="Contagem de Nacionalidades" fld="3" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="7">
-    <format dxfId="67">
+    <format dxfId="833">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="66">
+    <format dxfId="832">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="65">
+    <format dxfId="831">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="64">
+    <format dxfId="830">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="63">
+    <format dxfId="829">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="62">
+    <format dxfId="828">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="61">
+    <format dxfId="827">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -15363,8 +18065,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{996EC5F2-74EB-477F-A9D9-AF44A2544855}" name="Tabela dinâmica3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Faixa Etária" colHeaderCaption="Tipo de Movimentação">
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{996EC5F2-74EB-477F-A9D9-AF44A2544855}" name="Tabela dinâmica3" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Faixa Etária" colHeaderCaption="Tipo de Movimentação">
   <location ref="Y14:Z20" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField showAll="0"/>
@@ -15440,43 +18142,43 @@
     <dataField name="Contagem de Jogadores" fld="8" subtotal="count" baseField="8" baseItem="0"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="76">
+    <format dxfId="842">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="75">
+    <format dxfId="841">
       <pivotArea field="8" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="74">
+    <format dxfId="840">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="73">
+    <format dxfId="839">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="72">
+    <format dxfId="838">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="71">
+    <format dxfId="837">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="70">
+    <format dxfId="836">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="69">
+    <format dxfId="835">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="68">
+    <format dxfId="834">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -17350,7 +20052,7 @@
   <sheetPr>
     <tabColor theme="6" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A4:AO47"/>
+  <dimension ref="A4:BE47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.5703125" bestFit="1" customWidth="1"/>
@@ -17374,9 +20076,14 @@
     <col min="39" max="39" width="11" bestFit="1" customWidth="1"/>
     <col min="40" max="40" width="28.7109375" bestFit="1" customWidth="1"/>
     <col min="41" max="41" width="27.5703125" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="32.42578125" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="11" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="25.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:57" x14ac:dyDescent="0.25">
       <c r="C4" s="7" t="s">
         <v>158</v>
       </c>
@@ -17396,7 +20103,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="5" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:57" x14ac:dyDescent="0.25">
       <c r="C5" s="2">
         <f>COUNTA('Dados Tratados'!A3:A24)</f>
         <v>22</v>
@@ -17422,7 +20129,7 @@
         <v>25.454545454545453</v>
       </c>
     </row>
-    <row r="14" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
         <v>167</v>
       </c>
@@ -17453,8 +20160,14 @@
       <c r="AO14" s="10" t="s">
         <v>175</v>
       </c>
+      <c r="BA14" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="BB14" s="10" t="s">
+        <v>171</v>
+      </c>
     </row>
-    <row r="15" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
         <v>165</v>
       </c>
@@ -17509,8 +20222,20 @@
       <c r="AO15" s="2" t="s">
         <v>18</v>
       </c>
+      <c r="BA15" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="BB15" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="BD15" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="BE15" s="11" t="s">
+        <v>172</v>
+      </c>
     </row>
-    <row r="16" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>9</v>
       </c>
@@ -17568,8 +20293,21 @@
       <c r="AO16" s="2">
         <v>1</v>
       </c>
+      <c r="BA16" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="BB16" s="6">
+        <v>126300000</v>
+      </c>
+      <c r="BD16" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="BE16" s="13">
+        <f>BB16/$BB$19</f>
+        <v>0.70244716351501668</v>
+      </c>
     </row>
-    <row r="17" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>34</v>
       </c>
@@ -17627,8 +20365,21 @@
       <c r="AO17" s="2">
         <v>1</v>
       </c>
+      <c r="BA17" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="BB17" s="6">
+        <v>40500000</v>
+      </c>
+      <c r="BD17" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="BE17" s="13">
+        <f t="shared" ref="BE17:BE19" si="2">BB17/$BB$19</f>
+        <v>0.22525027808676307</v>
+      </c>
     </row>
-    <row r="18" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>55</v>
       </c>
@@ -17686,8 +20437,21 @@
       <c r="AO18" s="2">
         <v>1</v>
       </c>
+      <c r="BA18" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="BB18" s="6">
+        <v>13000000</v>
+      </c>
+      <c r="BD18" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="BE18" s="13">
+        <f t="shared" si="2"/>
+        <v>7.2302558398220251E-2</v>
+      </c>
     </row>
-    <row r="19" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>75</v>
       </c>
@@ -17745,8 +20509,21 @@
       <c r="AO19" s="2">
         <v>1</v>
       </c>
+      <c r="BA19" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="BB19" s="6">
+        <v>179800000</v>
+      </c>
+      <c r="BD19" s="17" t="s">
+        <v>164</v>
+      </c>
+      <c r="BE19" s="14">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
     </row>
-    <row r="20" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>93</v>
       </c>
@@ -17792,7 +20569,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>109</v>
       </c>
@@ -17825,7 +20602,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
         <v>164</v>
       </c>
@@ -17858,7 +20635,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:57" x14ac:dyDescent="0.25">
       <c r="AK23" s="2" t="s">
         <v>30</v>
       </c>
@@ -17872,7 +20649,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:57" x14ac:dyDescent="0.25">
       <c r="AK24" s="2" t="s">
         <v>152</v>
       </c>
@@ -17886,7 +20663,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:57" x14ac:dyDescent="0.25">
       <c r="AK25" s="2" t="s">
         <v>78</v>
       </c>
@@ -17900,7 +20677,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:57" x14ac:dyDescent="0.25">
       <c r="AK26" s="2" t="s">
         <v>64</v>
       </c>
@@ -17914,7 +20691,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="27" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:57" x14ac:dyDescent="0.25">
       <c r="AK27" s="2" t="s">
         <v>90</v>
       </c>
@@ -17928,7 +20705,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:57" x14ac:dyDescent="0.25">
       <c r="AK28" s="2" t="s">
         <v>97</v>
       </c>
@@ -17942,7 +20719,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:57" x14ac:dyDescent="0.25">
       <c r="AK29" s="9" t="s">
         <v>164</v>
       </c>
@@ -17956,7 +20733,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:57" x14ac:dyDescent="0.25">
       <c r="AN30" s="2" t="s">
         <v>97</v>
       </c>
@@ -17964,7 +20741,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:57" x14ac:dyDescent="0.25">
       <c r="AN31" s="2" t="s">
         <v>98</v>
       </c>
@@ -17972,7 +20749,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:57" x14ac:dyDescent="0.25">
       <c r="AN32" s="2" t="s">
         <v>97</v>
       </c>
@@ -18102,8 +20879,8 @@
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId6"/>
-  <drawing r:id="rId7"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId7"/>
+  <drawing r:id="rId8"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
39. Ajustando os Gráficos
Ajuste dos gráficos da quinta análise.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A47BD357-609C-45D8-A693-94F21DEA55EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6519BE88-1524-45B8-B1B9-A956EDD4AF9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="516" uniqueCount="187">
   <si>
     <t>temporada</t>
   </si>
@@ -750,60 +750,30 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentagem" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="273">
+  <dxfs count="95">
     <dxf>
-      <alignment horizontal="center" indent="0"/>
+      <alignment horizontal="center"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" indent="0"/>
+      <alignment horizontal="center"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" indent="0"/>
+      <alignment horizontal="center"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" indent="0"/>
+      <alignment horizontal="center"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
+      <alignment horizontal="center"/>
     </dxf>
     <dxf>
       <alignment horizontal="center"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="165" formatCode="0.0%"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" indent="0"/>
@@ -852,444 +822,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="0.0%"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="0.0%"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="0.0%"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="0.0%"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="0.0%"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="0.0%"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="0.0%"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="0.0%"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="0.0%"/>
     </dxf>
     <dxf>
       <alignment horizontal="center"/>
@@ -1478,73 +1010,7 @@
       <alignment horizontal="center"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="general"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
     </dxf>
     <dxf>
       <alignment horizontal="center"/>
@@ -4864,7 +4330,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="pt-BR"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -4901,6 +4367,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-F68C-485D-B549-889B4687A93E}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
@@ -4916,6 +4387,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-F68C-485D-B549-889B4687A93E}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="2"/>
@@ -4931,6 +4407,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-F68C-485D-B549-889B4687A93E}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dLbls>
             <c:spPr>
@@ -5136,126 +4617,63 @@
       <c:style val="2"/>
     </mc:Fallback>
   </mc:AlternateContent>
-  <c:pivotSource>
-    <c:name>[tottenham_transferencias.xlsx]Análises!Tabela dinâmica8</c:name>
-    <c:fmtId val="2"/>
-  </c:pivotSource>
   <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Retorno Financeiro por Jogador</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="pt-BR"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
     <c:autoTitleDeleted val="0"/>
-    <c:pivotFmts>
-      <c:pivotFmt>
-        <c:idx val="0"/>
-        <c:spPr>
-          <a:solidFill>
-            <a:schemeClr val="accent3"/>
-          </a:solidFill>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:marker>
-          <c:symbol val="none"/>
-        </c:marker>
-        <c:dLbl>
-          <c:idx val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="75000"/>
-                      <a:lumOff val="25000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="pt-BR"/>
-            </a:p>
-          </c:txPr>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
-          </c:extLst>
-        </c:dLbl>
-      </c:pivotFmt>
-      <c:pivotFmt>
-        <c:idx val="1"/>
-        <c:spPr>
-          <a:solidFill>
-            <a:schemeClr val="accent1"/>
-          </a:solidFill>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:marker>
-          <c:symbol val="none"/>
-        </c:marker>
-        <c:dLbl>
-          <c:idx val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="75000"/>
-                      <a:lumOff val="25000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="pt-BR"/>
-            </a:p>
-          </c:txPr>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
-          </c:extLst>
-        </c:dLbl>
-      </c:pivotFmt>
-    </c:pivotFmts>
     <c:plotArea>
       <c:layout/>
       <c:barChart>
@@ -5267,11 +4685,11 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Análises!$BB$14:$BB$16</c:f>
+              <c:f>Anotações!$G$103</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Saída - Soma do Valores</c:v>
+                  <c:v>Soma do Valores</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -5286,171 +4704,113 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="pt-BR"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
           <c:cat>
-            <c:multiLvlStrRef>
-              <c:f>Análises!$BA$17:$BA$26</c:f>
-              <c:multiLvlStrCache>
-                <c:ptCount val="6"/>
-                <c:lvl>
-                  <c:pt idx="0">
-                    <c:v>Harry Kane</c:v>
-                  </c:pt>
-                  <c:pt idx="1">
-                    <c:v>Steven Bergwijn</c:v>
-                  </c:pt>
-                  <c:pt idx="2">
-                    <c:v>Christian Eriksen</c:v>
-                  </c:pt>
-                  <c:pt idx="3">
-                    <c:v>Pierre-Emile Højbjerg</c:v>
-                  </c:pt>
-                  <c:pt idx="4">
-                    <c:v>Toby Alderweireld</c:v>
-                  </c:pt>
-                  <c:pt idx="5">
-                    <c:v>Jan Vertonghen</c:v>
-                  </c:pt>
-                </c:lvl>
-                <c:lvl>
-                  <c:pt idx="0">
-                    <c:v>Atacante</c:v>
-                  </c:pt>
-                  <c:pt idx="2">
-                    <c:v>Meio-campista</c:v>
-                  </c:pt>
-                  <c:pt idx="4">
-                    <c:v>Defensor</c:v>
-                  </c:pt>
-                </c:lvl>
-              </c:multiLvlStrCache>
-            </c:multiLvlStrRef>
+            <c:strRef>
+              <c:f>Anotações!$F$104:$F$108</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>Toby Alderweireld</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Pierre-Emile Højbjerg</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Christian Eriksen</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Steven Bergwijn</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Harry Kane</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Análises!$BB$17:$BB$26</c:f>
+              <c:f>Anotações!$G$104:$G$108</c:f>
               <c:numCache>
                 <c:formatCode>[$£-809]#,##0.00</c:formatCode>
-                <c:ptCount val="6"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>95000000</c:v>
+                  <c:v>13000000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>31300000</c:v>
+                  <c:v>13500000</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>27000000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>13500000</c:v>
+                  <c:v>31300000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>13000000</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>95000000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-B24A-4543-A891-BA87D420C4BF}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>Análises!$BC$14:$BC$16</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Saída - Porcentagem (%) do Total</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent2"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:cat>
-            <c:multiLvlStrRef>
-              <c:f>Análises!$BA$17:$BA$26</c:f>
-              <c:multiLvlStrCache>
-                <c:ptCount val="6"/>
-                <c:lvl>
-                  <c:pt idx="0">
-                    <c:v>Harry Kane</c:v>
-                  </c:pt>
-                  <c:pt idx="1">
-                    <c:v>Steven Bergwijn</c:v>
-                  </c:pt>
-                  <c:pt idx="2">
-                    <c:v>Christian Eriksen</c:v>
-                  </c:pt>
-                  <c:pt idx="3">
-                    <c:v>Pierre-Emile Højbjerg</c:v>
-                  </c:pt>
-                  <c:pt idx="4">
-                    <c:v>Toby Alderweireld</c:v>
-                  </c:pt>
-                  <c:pt idx="5">
-                    <c:v>Jan Vertonghen</c:v>
-                  </c:pt>
-                </c:lvl>
-                <c:lvl>
-                  <c:pt idx="0">
-                    <c:v>Atacante</c:v>
-                  </c:pt>
-                  <c:pt idx="2">
-                    <c:v>Meio-campista</c:v>
-                  </c:pt>
-                  <c:pt idx="4">
-                    <c:v>Defensor</c:v>
-                  </c:pt>
-                </c:lvl>
-              </c:multiLvlStrCache>
-            </c:multiLvlStrRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>Análises!$BC$17:$BC$26</c:f>
-              <c:numCache>
-                <c:formatCode>0.0%</c:formatCode>
-                <c:ptCount val="6"/>
-                <c:pt idx="0">
-                  <c:v>0.52836484983314791</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.17408231368186874</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.15016685205784205</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>7.5083426028921027E-2</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>7.2302558398220251E-2</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-B24A-4543-A891-BA87D420C4BF}"/>
+              <c16:uniqueId val="{00000000-D253-422C-9D21-3B6A446490F4}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5463,11 +4823,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="182"/>
-        <c:axId val="456556543"/>
-        <c:axId val="362412079"/>
+        <c:axId val="1430914512"/>
+        <c:axId val="1356498096"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="456556543"/>
+        <c:axId val="1430914512"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5510,27 +4870,55 @@
             <a:endParaRPr lang="pt-BR"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="362412079"/>
-        <c:crossesAt val="0"/>
+        <c:crossAx val="1356498096"/>
+        <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="362412079"/>
+        <c:axId val="1356498096"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
-        <c:delete val="1"/>
+        <c:delete val="0"/>
         <c:axPos val="b"/>
         <c:numFmt formatCode="[$£-809]#,##0.00" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="456556543"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="pt-BR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1430914512"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
+        <c:majorUnit val="13000000"/>
       </c:valAx>
       <c:spPr>
         <a:noFill/>
@@ -5581,20 +4969,6 @@
     <c:pageMargins b="0.78740157499999996" l="0.511811024" r="0.511811024" t="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
     <c:pageSetup/>
   </c:printSettings>
-  <c:extLst>
-    <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
-      <c14:pivotOptions>
-        <c14:dropZoneFilter val="1"/>
-        <c14:dropZoneCategories val="1"/>
-        <c14:dropZoneData val="1"/>
-      </c14:pivotOptions>
-    </c:ext>
-    <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{E28EC0CA-F0BB-4C9C-879D-F8772B89E7AC}">
-      <c16:pivotOptions16>
-        <c16:showExpandCollapseFieldButtons val="1"/>
-      </c16:pivotOptions16>
-    </c:ext>
-  </c:extLst>
 </c:chartSpace>
 </file>
 
@@ -14877,8 +14251,8 @@
     <xdr:to>
       <xdr:col>56</xdr:col>
       <xdr:colOff>942975</xdr:colOff>
-      <xdr:row>45</xdr:row>
-      <xdr:rowOff>161925</xdr:rowOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -14907,25 +14281,27 @@
     <xdr:from>
       <xdr:col>52</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>46</xdr:row>
-      <xdr:rowOff>176212</xdr:rowOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>9717</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>57</xdr:col>
-      <xdr:colOff>1666875</xdr:colOff>
-      <xdr:row>67</xdr:row>
-      <xdr:rowOff>178594</xdr:rowOff>
+      <xdr:col>58</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>68</xdr:row>
+      <xdr:rowOff>179716</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="35" name="Gráfico 34">
+        <xdr:cNvPr id="36" name="Gráfico 35">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7FCFC15E-DA44-F229-7A9E-BB32B7D047FB}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{24624CA1-503A-4D91-9CE4-3967074146C9}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="0"/>
@@ -16292,8 +15668,8 @@
       <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>96703</xdr:colOff>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>115753</xdr:colOff>
       <xdr:row>58</xdr:row>
       <xdr:rowOff>57203</xdr:rowOff>
     </xdr:to>
@@ -16328,6 +15704,65 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>74</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1089722" cy="327141"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="7" name="CaixaDeTexto 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{143FA442-043C-4235-B065-81436679E673}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1219200" y="14097000"/>
+          <a:ext cx="1089722" cy="327141"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1500" b="1"/>
+            <a:t>2. Análises:</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -17046,7 +16481,151 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4F5027D2-D537-4505-8DBC-54A417F72129}" name="Tabela dinâmica8" cacheId="0" dataPosition="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="8" rowHeaderCaption="Posições e Jogadores" colHeaderCaption="Tipo de Movimentação">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6" rowHeaderCaption="Temporadas" colHeaderCaption="">
+  <location ref="A14:D22" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="10">
+    <pivotField axis="axisRow" showAll="0">
+      <items count="7">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="7">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="1"/>
+  </colFields>
+  <colItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Somas de Entradas e Saídas" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
+  </dataFields>
+  <formats count="6">
+    <format dxfId="5">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="4">
+      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="3">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="2">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="1" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="1">
+      <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="0">
+      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="2">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4F5027D2-D537-4505-8DBC-54A417F72129}" name="Tabela dinâmica8" cacheId="0" dataPosition="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10" rowHeaderCaption="Posições e Jogadores" colHeaderCaption="Tipo de Movimentação">
   <location ref="BA14:BC26" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField showAll="0"/>
@@ -17175,7 +16754,7 @@
     <dataField name="Porcentagem (%) do Total" fld="6" showDataAs="percentOfTotal" baseField="0" baseItem="0" numFmtId="10"/>
   </dataFields>
   <formats count="18">
-    <format dxfId="0">
+    <format dxfId="23">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -17184,7 +16763,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="1">
+    <format dxfId="22">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -17197,7 +16776,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="2">
+    <format dxfId="21">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -17206,7 +16785,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="3">
+    <format dxfId="20">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -17219,7 +16798,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="4">
+    <format dxfId="19">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -17228,7 +16807,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="5">
+    <format dxfId="18">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -17241,26 +16820,26 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="6">
+    <format dxfId="17">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="7">
+    <format dxfId="16">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="8">
+    <format dxfId="15">
       <pivotArea field="-2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="1"/>
     </format>
-    <format dxfId="9">
+    <format dxfId="14">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="10">
+    <format dxfId="13">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="11">
+    <format dxfId="12">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -17273,7 +16852,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="12">
+    <format dxfId="11">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -17286,7 +16865,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="13">
+    <format dxfId="10">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -17299,14 +16878,14 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="14">
+    <format dxfId="9">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="15">
+    <format dxfId="8">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -17317,10 +16896,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="16">
+    <format dxfId="7">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="17">
+    <format dxfId="6">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
@@ -17699,7 +17278,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FB686887-B509-4E7E-B605-6A13972A6E0B}" name="Tabela dinâmica5" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Origem das Contratações" colHeaderCaption="Contagem de Jogadores">
   <location ref="AN14:AO47" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
@@ -17875,22 +17454,22 @@
     <dataField name="Clubes" fld="3" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="46">
-    <format dxfId="225">
+    <format dxfId="69">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="224">
+    <format dxfId="68">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="223">
+    <format dxfId="67">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="222">
+    <format dxfId="66">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="221">
+    <format dxfId="65">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="220">
+    <format dxfId="64">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="15">
@@ -17913,10 +17492,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="219">
+    <format dxfId="63">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="218">
+    <format dxfId="62">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -17928,7 +17507,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="217">
+    <format dxfId="61">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -17940,7 +17519,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="216">
+    <format dxfId="60">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -17952,7 +17531,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="215">
+    <format dxfId="59">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -17964,7 +17543,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="214">
+    <format dxfId="58">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -17976,7 +17555,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="213">
+    <format dxfId="57">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="2">
@@ -17989,7 +17568,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="212">
+    <format dxfId="56">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18001,7 +17580,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="211">
+    <format dxfId="55">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18013,7 +17592,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="210">
+    <format dxfId="54">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18025,7 +17604,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="209">
+    <format dxfId="53">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18037,7 +17616,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="208">
+    <format dxfId="52">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18049,7 +17628,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="207">
+    <format dxfId="51">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18061,7 +17640,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="206">
+    <format dxfId="50">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18073,7 +17652,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="205">
+    <format dxfId="49">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18085,7 +17664,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="204">
+    <format dxfId="48">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18097,29 +17676,29 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="203">
+    <format dxfId="47">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="202">
+    <format dxfId="46">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="201">
+    <format dxfId="45">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="200">
+    <format dxfId="44">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="199">
+    <format dxfId="43">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="198">
+    <format dxfId="42">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="197">
+    <format dxfId="41">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="15">
@@ -18142,10 +17721,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="196">
+    <format dxfId="40">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="195">
+    <format dxfId="39">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18157,7 +17736,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="194">
+    <format dxfId="38">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18169,7 +17748,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="193">
+    <format dxfId="37">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18181,7 +17760,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="192">
+    <format dxfId="36">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18193,7 +17772,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="191">
+    <format dxfId="35">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18205,7 +17784,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="190">
+    <format dxfId="34">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="2">
@@ -18218,7 +17797,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="189">
+    <format dxfId="33">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18230,7 +17809,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="188">
+    <format dxfId="32">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18242,7 +17821,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="187">
+    <format dxfId="31">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18254,7 +17833,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="186">
+    <format dxfId="30">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18266,7 +17845,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="185">
+    <format dxfId="29">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18278,7 +17857,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="184">
+    <format dxfId="28">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18290,7 +17869,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="183">
+    <format dxfId="27">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18302,7 +17881,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="182">
+    <format dxfId="26">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18314,7 +17893,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="181">
+    <format dxfId="25">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18326,7 +17905,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="180">
+    <format dxfId="24">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
@@ -18346,7 +17925,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{996EC5F2-74EB-477F-A9D9-AF44A2544855}" name="Tabela dinâmica3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Faixa Etária" colHeaderCaption="Tipo de Movimentação">
   <location ref="Y14:Z20" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -18423,43 +18002,43 @@
     <dataField name="Contagem de Jogadores" fld="8" subtotal="count" baseField="8" baseItem="0"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="234">
+    <format dxfId="78">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="233">
+    <format dxfId="77">
       <pivotArea field="8" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="232">
+    <format dxfId="76">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="231">
+    <format dxfId="75">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="230">
+    <format dxfId="74">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="229">
+    <format dxfId="73">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="228">
+    <format dxfId="72">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="227">
+    <format dxfId="71">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="226">
+    <format dxfId="70">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -18486,7 +18065,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{904CEA3A-CD0A-459C-A420-1FB249800D4C}" name="Tabela dinâmica4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Nacionalidades" colHeaderCaption="Contagem de Jogadores">
   <location ref="AK14:AL29" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
@@ -18619,37 +18198,37 @@
     <dataField name="Contagem de Nacionalidades" fld="3" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="7">
-    <format dxfId="241">
+    <format dxfId="85">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="240">
+    <format dxfId="84">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="239">
+    <format dxfId="83">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="238">
+    <format dxfId="82">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="237">
+    <format dxfId="81">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="236">
+    <format dxfId="80">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="235">
+    <format dxfId="79">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -18676,7 +18255,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
   <location ref="O14:P19" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -18745,39 +18324,39 @@
     <dataField name="Soma do Valor das Transferências" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="266">
+    <format dxfId="94">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="265">
+    <format dxfId="93">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="264">
+    <format dxfId="92">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="263">
+    <format dxfId="91">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="262">
+    <format dxfId="90">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="261">
+    <format dxfId="89">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="260">
+    <format dxfId="88">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="259">
+    <format dxfId="87">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="258">
+    <format dxfId="86">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -18787,150 +18366,6 @@
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
             <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6" rowHeaderCaption="Temporadas" colHeaderCaption="">
-  <location ref="A14:D22" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="10">
-    <pivotField axis="axisRow" showAll="0">
-      <items count="7">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisCol" showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="7">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="1"/>
-  </colFields>
-  <colItems count="3">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Somas de Entradas e Saídas" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
-  </dataFields>
-  <formats count="6">
-    <format dxfId="272">
-      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
-        <references count="1">
-          <reference field="0" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="271">
-      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
-    </format>
-    <format dxfId="270">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="0" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="269">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="1" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="268">
-      <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="267">
-      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="2">
-    <chartFormat chart="0" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="1" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="1"/>
           </reference>
         </references>
       </pivotArea>
@@ -20824,7 +20259,7 @@
     <col min="55" max="55" width="24.140625" bestFit="1" customWidth="1"/>
     <col min="56" max="56" width="12.7109375" customWidth="1"/>
     <col min="57" max="57" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="34.7109375" bestFit="1" customWidth="1"/>
     <col min="59" max="59" width="17.7109375" bestFit="1" customWidth="1"/>
     <col min="60" max="60" width="20.42578125" bestFit="1" customWidth="1"/>
     <col min="61" max="61" width="15.85546875" bestFit="1" customWidth="1"/>
@@ -20842,7 +20277,7 @@
     <col min="74" max="74" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:61" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:58" x14ac:dyDescent="0.25">
       <c r="C4" s="7" t="s">
         <v>158</v>
       </c>
@@ -20862,7 +20297,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="5" spans="1:61" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:58" x14ac:dyDescent="0.25">
       <c r="C5" s="2">
         <f>COUNTA('Dados Tratados'!A3:A24)</f>
         <v>22</v>
@@ -20888,7 +20323,7 @@
         <v>25.454545454545453</v>
       </c>
     </row>
-    <row r="14" spans="1:61" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:58" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
         <v>167</v>
       </c>
@@ -20931,7 +20366,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="15" spans="1:61" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:58" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
         <v>165</v>
       </c>
@@ -20998,7 +20433,7 @@
         <v>0.70199999999999996</v>
       </c>
     </row>
-    <row r="16" spans="1:61" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:58" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>9</v>
       </c>
@@ -21070,12 +20505,6 @@
       </c>
       <c r="BF16" s="13">
         <v>0.22500000000000001</v>
-      </c>
-      <c r="BH16" s="17" t="s">
-        <v>185</v>
-      </c>
-      <c r="BI16" s="17" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="17" spans="1:61" x14ac:dyDescent="0.25">
@@ -21151,12 +20580,6 @@
       <c r="BF17" s="13">
         <v>7.1999999999999995E-2</v>
       </c>
-      <c r="BH17" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="BI17" s="19">
-        <v>126300000</v>
-      </c>
     </row>
     <row r="18" spans="1:61" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
@@ -21231,12 +20654,6 @@
       <c r="BF18" s="14">
         <v>1</v>
       </c>
-      <c r="BH18" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="BI18" s="6">
-        <v>95000000</v>
-      </c>
     </row>
     <row r="19" spans="1:61" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
@@ -21305,12 +20722,6 @@
       <c r="BC19" s="13">
         <v>0.17408231368186874</v>
       </c>
-      <c r="BH19" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="BI19" s="6">
-        <v>31300000</v>
-      </c>
     </row>
     <row r="20" spans="1:61" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
@@ -21366,12 +20777,6 @@
       <c r="BC20" s="13">
         <v>0.22525027808676307</v>
       </c>
-      <c r="BH20" s="18" t="s">
-        <v>156</v>
-      </c>
-      <c r="BI20" s="19">
-        <v>40500000</v>
-      </c>
     </row>
     <row r="21" spans="1:61" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
@@ -21414,12 +20819,6 @@
       <c r="BC21" s="13">
         <v>0.15016685205784205</v>
       </c>
-      <c r="BH21" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="BI21" s="6">
-        <v>27000000</v>
-      </c>
     </row>
     <row r="22" spans="1:61" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
@@ -21462,12 +20861,6 @@
       <c r="BC22" s="13">
         <v>7.5083426028921027E-2</v>
       </c>
-      <c r="BH22" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="BI22" s="6">
-        <v>13500000</v>
-      </c>
     </row>
     <row r="23" spans="1:61" x14ac:dyDescent="0.25">
       <c r="AK23" s="2" t="s">
@@ -21491,12 +20884,6 @@
       <c r="BC23" s="13">
         <v>7.2302558398220251E-2</v>
       </c>
-      <c r="BH23" s="18" t="s">
-        <v>70</v>
-      </c>
-      <c r="BI23" s="19">
-        <v>13000000</v>
-      </c>
     </row>
     <row r="24" spans="1:61" x14ac:dyDescent="0.25">
       <c r="AK24" s="2" t="s">
@@ -21520,12 +20907,6 @@
       <c r="BC24" s="13">
         <v>7.2302558398220251E-2</v>
       </c>
-      <c r="BH24" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="BI24" s="6">
-        <v>13000000</v>
-      </c>
     </row>
     <row r="25" spans="1:61" x14ac:dyDescent="0.25">
       <c r="AK25" s="2" t="s">
@@ -21549,12 +20930,8 @@
       <c r="BC25" s="13">
         <v>0</v>
       </c>
-      <c r="BH25" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="BI25" s="6">
-        <v>0</v>
-      </c>
+      <c r="BH25" s="2"/>
+      <c r="BI25" s="6"/>
     </row>
     <row r="26" spans="1:61" x14ac:dyDescent="0.25">
       <c r="AK26" s="2" t="s">
@@ -21777,9 +21154,66 @@
   <sheetPr>
     <tabColor theme="1"/>
   </sheetPr>
-  <dimension ref="A1"/>
+  <dimension ref="F103:G110"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="6" max="6" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="103" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F103" s="17" t="s">
+        <v>185</v>
+      </c>
+      <c r="G103" s="17" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="104" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F104" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="G104" s="6">
+        <v>13000000</v>
+      </c>
+    </row>
+    <row r="105" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F105" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="G105" s="6">
+        <v>13500000</v>
+      </c>
+    </row>
+    <row r="106" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F106" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G106" s="6">
+        <v>27000000</v>
+      </c>
+    </row>
+    <row r="107" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F107" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="G107" s="6">
+        <v>31300000</v>
+      </c>
+    </row>
+    <row r="108" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F108" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="G108" s="6">
+        <v>95000000</v>
+      </c>
+    </row>
+    <row r="110" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F110" s="18"/>
+      <c r="G110" s="19"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
40. Começo do Insight
Começo do insight/conclusão da análise.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6519BE88-1524-45B8-B1B9-A956EDD4AF9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A1E6970-C7D2-464D-B0C7-A3CB1A2AC0D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="516" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="188">
   <si>
     <t>temporada</t>
   </si>
@@ -606,6 +606,9 @@
   <si>
     <t>Soma do Valores</t>
   </si>
+  <si>
+    <t>Saídas/Vendas de Jogadores em %</t>
+  </si>
 </sst>
 </file>
 
@@ -692,7 +695,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -745,12 +748,40 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentagem" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="95">
+    <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
     <dxf>
       <alignment horizontal="center"/>
     </dxf>
@@ -984,33 +1015,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general"/>
     </dxf>
     <dxf>
       <alignment horizontal="center"/>
@@ -14186,7 +14190,7 @@
       <xdr:col>51</xdr:col>
       <xdr:colOff>557123</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>125802</xdr:rowOff>
+      <xdr:rowOff>150018</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="818815" cy="311496"/>
     <xdr:sp macro="" textlink="">
@@ -14202,7 +14206,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="51381085" y="2012830"/>
+          <a:off x="51435153" y="2087306"/>
           <a:ext cx="818815" cy="311496"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -14315,6 +14319,384 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>51</xdr:col>
+      <xdr:colOff>581185</xdr:colOff>
+      <xdr:row>69</xdr:row>
+      <xdr:rowOff>113008</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1781963" cy="311496"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="33" name="CaixaDeTexto 32">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9B05069A-EEB4-42D4-9F08-80E24546E4AA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="51459215" y="13480296"/>
+          <a:ext cx="1781963" cy="311496"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0"/>
+            <a:t>Conclusão</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t> e Insights</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0"/>
+            <a:t>: </a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>51</xdr:col>
+      <xdr:colOff>517568</xdr:colOff>
+      <xdr:row>71</xdr:row>
+      <xdr:rowOff>144850</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="12167626" cy="2503121"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="35" name="CaixaDeTexto 34">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{794FF18C-FFBB-4D14-8AC1-6C1ABCA94038}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="53467043" y="13670350"/>
+          <a:ext cx="12167626" cy="2503121"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>Após o período analisado, identificou-se que o Tottenham Hotspur reuniu cerca de </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400"/>
+            <a:t>£179.8 milhões através das</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" baseline="0"/>
+            <a:t> vendas e saídas de jogadores. O valor contrasta</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" baseline="0"/>
+            <a:t>significativamente com a quantia de </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>£553.2 milhões gasta pelo clube em contratações ao longo do mesmo espaço de tempo, representando aproximadamente</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>24,5% </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>de</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> todas as movimentações financeiras. As despedidas consistiram em atacantes, meio-campistas e defensores </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1100" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>— </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>espelhando, respectivamente, </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>70,2%</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>, </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>22,5%</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>e </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>7,2% </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>do total.</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>Embora os ingleses e holandeses liderem a lista, não há indícios suficientes para afirmar que o Tottenham Hotspur padronizou sua busca por talentos</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>ao concentrar-se em uma ou outra nacionalidade, visto que a diferença entre atletas é </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>mínima</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t> e a </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>diversidade</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t> de nações se faz presente. Além disso,</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>cerca de </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>11 </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>ativos contratados não são representados pelas bandeiras de Inglaterra ou Holanda. Isso sugere uma possível estratégia adotada pelo departamento</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>de scouting do clube visando o mapeamento de atletas que estejam se desenvolvendo em outras ligas europeias, porém sem perder contato com as</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>novidades que surgem no mercado doméstico — uma vez que todos os jogadores ingleses foram contratados enquanto atuavam por equipes conterrâneas</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>como Leicester City, Bournemouth e Leeds United.</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -16481,6 +16863,134 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
+  <location ref="O14:P19" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="10">
+    <pivotField showAll="0"/>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="3">
+        <item h="1" x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0" sortType="ascending">
+      <items count="4">
+        <item x="1"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="2">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+            <reference field="1" count="1" selected="0">
+              <x v="1"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="3"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="1"/>
+  </colFields>
+  <colItems count="1">
+    <i>
+      <x v="1"/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Soma do Valor das Transferências" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
+  </dataFields>
+  <formats count="9">
+    <format dxfId="8">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="7">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="6">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="5">
+      <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
+    </format>
+    <format dxfId="4">
+      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="3">
+      <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="2">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="3" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="1">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="1" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="0">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="1">
+    <chartFormat chart="1" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6" rowHeaderCaption="Temporadas" colHeaderCaption="">
   <location ref="A14:D22" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -16555,34 +17065,34 @@
     <dataField name="Somas de Entradas e Saídas" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="5">
+    <format dxfId="14">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="4">
+    <format dxfId="13">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="3">
+    <format dxfId="12">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="2">
+    <format dxfId="11">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="1">
+    <format dxfId="10">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="0">
+    <format dxfId="9">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -16624,7 +17134,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4F5027D2-D537-4505-8DBC-54A417F72129}" name="Tabela dinâmica8" cacheId="0" dataPosition="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10" rowHeaderCaption="Posições e Jogadores" colHeaderCaption="Tipo de Movimentação">
   <location ref="BA14:BC26" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
   <pivotFields count="10">
@@ -16754,7 +17264,7 @@
     <dataField name="Porcentagem (%) do Total" fld="6" showDataAs="percentOfTotal" baseField="0" baseItem="0" numFmtId="10"/>
   </dataFields>
   <formats count="18">
-    <format dxfId="23">
+    <format dxfId="32">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -16763,7 +17273,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="22">
+    <format dxfId="31">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -16776,7 +17286,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="21">
+    <format dxfId="30">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -16785,7 +17295,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="20">
+    <format dxfId="29">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -16798,7 +17308,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="19">
+    <format dxfId="28">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -16807,7 +17317,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="18">
+    <format dxfId="27">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -16820,26 +17330,26 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="17">
+    <format dxfId="26">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="16">
+    <format dxfId="25">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="15">
+    <format dxfId="24">
       <pivotArea field="-2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="1"/>
     </format>
-    <format dxfId="14">
+    <format dxfId="23">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="13">
+    <format dxfId="22">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="12">
+    <format dxfId="21">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -16852,7 +17362,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="11">
+    <format dxfId="20">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -16865,7 +17375,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="10">
+    <format dxfId="19">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -16878,14 +17388,14 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="9">
+    <format dxfId="18">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="8">
+    <format dxfId="17">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -16896,10 +17406,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="7">
+    <format dxfId="16">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="6">
+    <format dxfId="15">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
@@ -17278,7 +17788,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FB686887-B509-4E7E-B605-6A13972A6E0B}" name="Tabela dinâmica5" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Origem das Contratações" colHeaderCaption="Contagem de Jogadores">
   <location ref="AN14:AO47" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
@@ -17454,22 +17964,22 @@
     <dataField name="Clubes" fld="3" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="46">
-    <format dxfId="69">
+    <format dxfId="78">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="68">
+    <format dxfId="77">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="67">
+    <format dxfId="76">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="66">
+    <format dxfId="75">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="65">
+    <format dxfId="74">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="64">
+    <format dxfId="73">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="15">
@@ -17492,10 +18002,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="63">
+    <format dxfId="72">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="62">
+    <format dxfId="71">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -17507,7 +18017,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="61">
+    <format dxfId="70">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -17519,7 +18029,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="60">
+    <format dxfId="69">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -17531,7 +18041,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="59">
+    <format dxfId="68">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -17543,7 +18053,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="58">
+    <format dxfId="67">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -17555,7 +18065,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="57">
+    <format dxfId="66">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="2">
@@ -17568,7 +18078,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="56">
+    <format dxfId="65">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -17580,7 +18090,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="55">
+    <format dxfId="64">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -17592,7 +18102,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="54">
+    <format dxfId="63">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -17604,7 +18114,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="53">
+    <format dxfId="62">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -17616,7 +18126,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="52">
+    <format dxfId="61">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -17628,7 +18138,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="51">
+    <format dxfId="60">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -17640,7 +18150,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="50">
+    <format dxfId="59">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -17652,7 +18162,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="49">
+    <format dxfId="58">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -17664,7 +18174,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="48">
+    <format dxfId="57">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -17676,29 +18186,29 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="47">
+    <format dxfId="56">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="46">
+    <format dxfId="55">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="45">
+    <format dxfId="54">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="44">
+    <format dxfId="53">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="43">
+    <format dxfId="52">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="42">
+    <format dxfId="51">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="41">
+    <format dxfId="50">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="15">
@@ -17721,10 +18231,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="40">
+    <format dxfId="49">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="39">
+    <format dxfId="48">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -17736,7 +18246,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="38">
+    <format dxfId="47">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -17748,7 +18258,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="37">
+    <format dxfId="46">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -17760,7 +18270,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="36">
+    <format dxfId="45">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -17772,7 +18282,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="35">
+    <format dxfId="44">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -17784,7 +18294,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="34">
+    <format dxfId="43">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="2">
@@ -17797,7 +18307,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="33">
+    <format dxfId="42">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -17809,7 +18319,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="32">
+    <format dxfId="41">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -17821,7 +18331,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="31">
+    <format dxfId="40">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -17833,7 +18343,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="30">
+    <format dxfId="39">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -17845,7 +18355,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="29">
+    <format dxfId="38">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -17857,7 +18367,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="28">
+    <format dxfId="37">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -17869,7 +18379,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="27">
+    <format dxfId="36">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -17881,7 +18391,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="26">
+    <format dxfId="35">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -17893,7 +18403,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="25">
+    <format dxfId="34">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -17905,7 +18415,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="24">
+    <format dxfId="33">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
@@ -17925,7 +18435,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{996EC5F2-74EB-477F-A9D9-AF44A2544855}" name="Tabela dinâmica3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Faixa Etária" colHeaderCaption="Tipo de Movimentação">
   <location ref="Y14:Z20" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -18002,43 +18512,43 @@
     <dataField name="Contagem de Jogadores" fld="8" subtotal="count" baseField="8" baseItem="0"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="78">
+    <format dxfId="87">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="77">
+    <format dxfId="86">
       <pivotArea field="8" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="76">
+    <format dxfId="85">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="75">
+    <format dxfId="84">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="74">
+    <format dxfId="83">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="73">
+    <format dxfId="82">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="72">
+    <format dxfId="81">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="71">
+    <format dxfId="80">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="70">
+    <format dxfId="79">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -18065,7 +18575,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{904CEA3A-CD0A-459C-A420-1FB249800D4C}" name="Tabela dinâmica4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Nacionalidades" colHeaderCaption="Contagem de Jogadores">
   <location ref="AK14:AL29" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
@@ -18198,166 +18708,38 @@
     <dataField name="Contagem de Nacionalidades" fld="3" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="7">
-    <format dxfId="85">
+    <format dxfId="94">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="84">
+    <format dxfId="93">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="83">
+    <format dxfId="92">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="82">
+    <format dxfId="91">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="81">
+    <format dxfId="90">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="80">
+    <format dxfId="89">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="79">
+    <format dxfId="88">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="1">
-    <chartFormat chart="1" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
-  <location ref="O14:P19" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="10">
-    <pivotField showAll="0"/>
-    <pivotField axis="axisCol" showAll="0">
-      <items count="3">
-        <item h="1" x="1"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0" sortType="ascending">
-      <items count="4">
-        <item x="1"/>
-        <item x="2"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-      <autoSortScope>
-        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
-          <references count="2">
-            <reference field="4294967294" count="1" selected="0">
-              <x v="0"/>
-            </reference>
-            <reference field="1" count="1" selected="0">
-              <x v="1"/>
-            </reference>
-          </references>
-        </pivotArea>
-      </autoSortScope>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="3"/>
-  </rowFields>
-  <rowItems count="4">
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="1"/>
-  </colFields>
-  <colItems count="1">
-    <i>
-      <x v="1"/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Soma do Valor das Transferências" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
-  </dataFields>
-  <formats count="9">
-    <format dxfId="94">
-      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="93">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="92">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="91">
-      <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
-    </format>
-    <format dxfId="90">
-      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="89">
-      <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
-    </format>
-    <format dxfId="88">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="3" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="87">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="1" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="86">
-      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
   <chartFormats count="1">
@@ -20234,11 +20616,14 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="4" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.140625" customWidth="1"/>
     <col min="6" max="6" width="17.7109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="22.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="25.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="32" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="31.140625" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="26.28515625" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="14.85546875" bestFit="1" customWidth="1"/>
@@ -20296,6 +20681,9 @@
       <c r="H4" s="7" t="s">
         <v>163</v>
       </c>
+      <c r="I4" s="7" t="s">
+        <v>187</v>
+      </c>
     </row>
     <row r="5" spans="1:58" x14ac:dyDescent="0.25">
       <c r="C5" s="2">
@@ -20321,6 +20709,10 @@
       <c r="H5" s="5">
         <f>AVERAGE('Dados Tratados'!H3:H24)</f>
         <v>25.454545454545453</v>
+      </c>
+      <c r="I5" s="20">
+        <f>(C22/D22)*100</f>
+        <v>24.529331514324692</v>
       </c>
     </row>
     <row r="14" spans="1:58" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
41. Andamento do Insight
Construindo o insight.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A1E6970-C7D2-464D-B0C7-A3CB1A2AC0D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37E56EBA-BA2B-48A6-8B4C-04F9D7360E57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -14390,11 +14390,11 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>51</xdr:col>
-      <xdr:colOff>517568</xdr:colOff>
-      <xdr:row>71</xdr:row>
-      <xdr:rowOff>144850</xdr:rowOff>
+      <xdr:colOff>340727</xdr:colOff>
+      <xdr:row>72</xdr:row>
+      <xdr:rowOff>173513</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="12167626" cy="2503121"/>
+    <xdr:ext cx="12521313" cy="2064796"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="35" name="CaixaDeTexto 34">
@@ -14408,8 +14408,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="53467043" y="13670350"/>
-          <a:ext cx="12167626" cy="2503121"/>
+          <a:off x="53290202" y="13889513"/>
+          <a:ext cx="12521313" cy="2064796"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -14631,67 +14631,270 @@
           <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
-            <a:t>Embora os ingleses e holandeses liderem a lista, não há indícios suficientes para afirmar que o Tottenham Hotspur padronizou sua busca por talentos</a:t>
+            <a:t>Entre as posições, os atacantes se destacam. Suas saídas renderam </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>£126.3 milhões </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>aos cofres do clube,</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> valor superior ao dobro da soma entre os meio-campistas e </a:t>
           </a:r>
           <a:br>
-            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:rPr lang="pt-BR" sz="1400" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
           </a:br>
           <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
-            <a:t>ao concentrar-se em uma ou outra nacionalidade, visto que a diferença entre atletas é </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
-            <a:t>mínima</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
-            <a:t> e a </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
-            <a:t>diversidade</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
-            <a:t> de nações se faz presente. Além disso,</a:t>
+            <a:rPr lang="pt-BR" sz="1400" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>defensores. Um peso ainda maior vai para Harry Kane </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1100" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>— </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>sozinho, o inglês gerou </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>£95 milhões</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>, quantia que se sobrepõe à</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> adição dos valores de todos os jogadores</a:t>
           </a:r>
           <a:br>
-            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
           </a:br>
           <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
-            <a:t>cerca de </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
-            <a:t>11 </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
-            <a:t>ativos contratados não são representados pelas bandeiras de Inglaterra ou Holanda. Isso sugere uma possível estratégia adotada pelo departamento</a:t>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>restantes</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>.</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> Semelhantemente, a venda de Steve Bergwijn, girando em torno de </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>£31.3 milhões</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>, também</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> trouxe impactos positivos. Embora o setor de criação das jogadas,</a:t>
           </a:r>
           <a:br>
-            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
           </a:br>
           <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
-            <a:t>de scouting do clube visando o mapeamento de atletas que estejam se desenvolvendo em outras ligas europeias, porém sem perder contato com as</a:t>
-          </a:r>
-          <a:br>
-            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
-          </a:br>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
-            <a:t>novidades que surgem no mercado doméstico — uma vez que todos os jogadores ingleses foram contratados enquanto atuavam por equipes conterrâneas</a:t>
-          </a:r>
-          <a:br>
-            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
-          </a:br>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
-            <a:t>como Leicester City, Bournemouth e Leeds United.</a:t>
-          </a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>formado por Christian Eriksen e Pierre-Emile Højbjerg, tenha reunido </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>£40.5 milhões</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> ao todo, o atacante</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> holandês cobre grande parte desse valor</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
         </a:p>
       </xdr:txBody>
     </xdr:sp>

</xml_diff>

<commit_message>
42. Conclusão do Insight
Término do insight da quinta análise.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37E56EBA-BA2B-48A6-8B4C-04F9D7360E57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55CE6822-705D-4792-8BC6-0D5A21DB2B0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Apresentação" sheetId="3" r:id="rId1"/>
@@ -756,6 +756,27 @@
   </cellStyles>
   <dxfs count="95">
     <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="general"/>
     </dxf>
     <dxf>
@@ -991,27 +1012,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
     </dxf>
     <dxf>
       <alignment horizontal="center"/>
@@ -14390,11 +14390,11 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>51</xdr:col>
-      <xdr:colOff>340727</xdr:colOff>
-      <xdr:row>72</xdr:row>
-      <xdr:rowOff>173513</xdr:rowOff>
+      <xdr:colOff>495942</xdr:colOff>
+      <xdr:row>71</xdr:row>
+      <xdr:rowOff>106664</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="12521313" cy="2064796"/>
+    <xdr:ext cx="12668083" cy="2941446"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="35" name="CaixaDeTexto 34">
@@ -14408,8 +14408,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="53290202" y="13889513"/>
-          <a:ext cx="12521313" cy="2064796"/>
+          <a:off x="53445417" y="13632164"/>
+          <a:ext cx="12668083" cy="2941446"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -14501,7 +14501,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>de</a:t>
+            <a:t>do</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
@@ -14513,7 +14513,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t> todas as movimentações financeiras. As despedidas consistiram em atacantes, meio-campistas e defensores </a:t>
+            <a:t> montante aplicado pelo clube no mercado. As despedidas consistiram em atacantes, meio-campistas e defensores </a:t>
           </a:r>
           <a:r>
             <a:rPr lang="pt-BR" sz="1100" b="0" i="0" baseline="0">
@@ -14773,7 +14773,31 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>restantes</a:t>
+            <a:t>restantes e que representa </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>52,8</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>% do retorno financeiro obtido ao longo de seis temporadas</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="pt-BR" sz="1400" b="0">
@@ -14785,7 +14809,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>.</a:t>
+            <a:t>. O</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
@@ -14797,43 +14821,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t> Semelhantemente, a venda de Steve Bergwijn, girando em torno de </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="1">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>£31.3 milhões</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>, também</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t> trouxe impactos positivos. Embora o setor de criação das jogadas,</a:t>
+            <a:t> impacto da categoria torna-se ainda mais visível quando Steve Bergwijn,</a:t>
           </a:r>
           <a:br>
             <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
@@ -14856,7 +14844,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>formado por Christian Eriksen e Pierre-Emile Højbjerg, tenha reunido </a:t>
+            <a:t>seu companheiro, entra na equação: a saída do holandês garantiu </a:t>
           </a:r>
           <a:r>
             <a:rPr lang="pt-BR" sz="1400" b="1">
@@ -14868,7 +14856,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>£40.5 milhões</a:t>
+            <a:t>£31.3 milhões</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="pt-BR" sz="1400" b="0">
@@ -14880,7 +14868,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t> ao todo, o atacante</a:t>
+            <a:t> para a equipe, superando</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
@@ -14892,7 +14880,111 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t> holandês cobre grande parte desse valor</a:t>
+            <a:t> individualmente o preço de ambos os atletas responsáveis pela</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>administração do meio-campo, sendo eles Christian Eriksen e Pierre-Emile Højbjerg.</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Em resumo, os </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>atacantes</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> geraram maior retorno financeiro ao Tottenham Hotspur. Baseando-se na base de dados atual, não é possível identificar a razão por trás da</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>valorização dos mesmos.</a:t>
           </a:r>
           <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
         </a:p>
@@ -17066,6 +17158,196 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{904CEA3A-CD0A-459C-A420-1FB249800D4C}" name="Tabela dinâmica4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Nacionalidades" colHeaderCaption="Contagem de Jogadores">
+  <location ref="AK14:AL29" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="9">
+    <pivotField axis="axisCol" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item h="1" x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" dataField="1" showAll="0" sortType="ascending">
+      <items count="15">
+        <item x="6"/>
+        <item x="4"/>
+        <item x="9"/>
+        <item x="11"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="12"/>
+        <item x="5"/>
+        <item x="10"/>
+        <item x="13"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="2">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+            <reference field="0" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="21">
+        <item x="12"/>
+        <item x="9"/>
+        <item x="7"/>
+        <item x="15"/>
+        <item x="5"/>
+        <item x="17"/>
+        <item x="11"/>
+        <item x="10"/>
+        <item x="2"/>
+        <item x="8"/>
+        <item x="18"/>
+        <item x="13"/>
+        <item x="0"/>
+        <item x="16"/>
+        <item x="19"/>
+        <item x="1"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item x="14"/>
+        <item x="6"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="3"/>
+  </rowFields>
+  <rowItems count="14">
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="0"/>
+  </colFields>
+  <colItems count="1">
+    <i>
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Contagem de Nacionalidades" fld="3" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="7">
+    <format dxfId="6">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="3" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="5">
+      <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="4">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="3" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="3">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+    <format dxfId="2">
+      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="1">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="0">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="1">
+    <chartFormat chart="1" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
   <location ref="O14:P19" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -17134,39 +17416,39 @@
     <dataField name="Soma do Valor das Transferências" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="8">
+    <format dxfId="15">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="7">
+    <format dxfId="14">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="6">
+    <format dxfId="13">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="5">
+    <format dxfId="12">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="4">
+    <format dxfId="11">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="3">
+    <format dxfId="10">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="2">
+    <format dxfId="9">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="1">
+    <format dxfId="8">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="0">
+    <format dxfId="7">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -17193,7 +17475,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6" rowHeaderCaption="Temporadas" colHeaderCaption="">
   <location ref="A14:D22" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -17268,34 +17550,34 @@
     <dataField name="Somas de Entradas e Saídas" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="14">
+    <format dxfId="21">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="13">
+    <format dxfId="20">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="12">
+    <format dxfId="19">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="11">
+    <format dxfId="18">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="10">
+    <format dxfId="17">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="9">
+    <format dxfId="16">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -17337,7 +17619,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4F5027D2-D537-4505-8DBC-54A417F72129}" name="Tabela dinâmica8" cacheId="0" dataPosition="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10" rowHeaderCaption="Posições e Jogadores" colHeaderCaption="Tipo de Movimentação">
   <location ref="BA14:BC26" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
   <pivotFields count="10">
@@ -17467,7 +17749,7 @@
     <dataField name="Porcentagem (%) do Total" fld="6" showDataAs="percentOfTotal" baseField="0" baseItem="0" numFmtId="10"/>
   </dataFields>
   <formats count="18">
-    <format dxfId="32">
+    <format dxfId="39">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -17476,7 +17758,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="31">
+    <format dxfId="38">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -17489,7 +17771,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="30">
+    <format dxfId="37">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -17498,7 +17780,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="29">
+    <format dxfId="36">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -17511,7 +17793,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="28">
+    <format dxfId="35">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -17520,7 +17802,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="27">
+    <format dxfId="34">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -17533,26 +17815,26 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="26">
+    <format dxfId="33">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="25">
+    <format dxfId="32">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="24">
+    <format dxfId="31">
       <pivotArea field="-2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="1"/>
     </format>
-    <format dxfId="23">
+    <format dxfId="30">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="22">
+    <format dxfId="29">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="21">
+    <format dxfId="28">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -17565,7 +17847,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="20">
+    <format dxfId="27">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -17578,7 +17860,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="19">
+    <format dxfId="26">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -17591,14 +17873,14 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="18">
+    <format dxfId="25">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="17">
+    <format dxfId="24">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -17609,10 +17891,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="16">
+    <format dxfId="23">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="15">
+    <format dxfId="22">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
@@ -17991,7 +18273,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FB686887-B509-4E7E-B605-6A13972A6E0B}" name="Tabela dinâmica5" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Origem das Contratações" colHeaderCaption="Contagem de Jogadores">
   <location ref="AN14:AO47" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
@@ -18167,22 +18449,22 @@
     <dataField name="Clubes" fld="3" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="46">
-    <format dxfId="78">
+    <format dxfId="85">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="77">
+    <format dxfId="84">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="76">
+    <format dxfId="83">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="75">
+    <format dxfId="82">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="74">
+    <format dxfId="81">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="73">
+    <format dxfId="80">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="15">
@@ -18205,10 +18487,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="72">
+    <format dxfId="79">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="71">
+    <format dxfId="78">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18220,7 +18502,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="70">
+    <format dxfId="77">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18232,7 +18514,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="69">
+    <format dxfId="76">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18244,7 +18526,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="68">
+    <format dxfId="75">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18256,7 +18538,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="67">
+    <format dxfId="74">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18268,7 +18550,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="66">
+    <format dxfId="73">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="2">
@@ -18281,7 +18563,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="65">
+    <format dxfId="72">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18293,7 +18575,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="64">
+    <format dxfId="71">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18305,7 +18587,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="63">
+    <format dxfId="70">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18317,7 +18599,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="62">
+    <format dxfId="69">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18329,7 +18611,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="61">
+    <format dxfId="68">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18341,7 +18623,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="60">
+    <format dxfId="67">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18353,7 +18635,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="59">
+    <format dxfId="66">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18365,7 +18647,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="58">
+    <format dxfId="65">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18377,7 +18659,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="57">
+    <format dxfId="64">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18389,29 +18671,29 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="56">
+    <format dxfId="63">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="55">
+    <format dxfId="62">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="54">
+    <format dxfId="61">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="53">
+    <format dxfId="60">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="52">
+    <format dxfId="59">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="51">
+    <format dxfId="58">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="50">
+    <format dxfId="57">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="15">
@@ -18434,10 +18716,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="49">
+    <format dxfId="56">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="48">
+    <format dxfId="55">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18449,7 +18731,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="47">
+    <format dxfId="54">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18461,7 +18743,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="46">
+    <format dxfId="53">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18473,7 +18755,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="45">
+    <format dxfId="52">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18485,7 +18767,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="44">
+    <format dxfId="51">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18497,7 +18779,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="43">
+    <format dxfId="50">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="2">
@@ -18510,7 +18792,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="42">
+    <format dxfId="49">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18522,7 +18804,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="41">
+    <format dxfId="48">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18534,7 +18816,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="40">
+    <format dxfId="47">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18546,7 +18828,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="39">
+    <format dxfId="46">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18558,7 +18840,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="38">
+    <format dxfId="45">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18570,7 +18852,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="37">
+    <format dxfId="44">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18582,7 +18864,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="36">
+    <format dxfId="43">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18594,7 +18876,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="35">
+    <format dxfId="42">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18606,7 +18888,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="34">
+    <format dxfId="41">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18618,7 +18900,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="33">
+    <format dxfId="40">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
@@ -18638,7 +18920,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{996EC5F2-74EB-477F-A9D9-AF44A2544855}" name="Tabela dinâmica3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Faixa Etária" colHeaderCaption="Tipo de Movimentação">
   <location ref="Y14:Z20" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -18715,216 +18997,20 @@
     <dataField name="Contagem de Jogadores" fld="8" subtotal="count" baseField="8" baseItem="0"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="87">
+    <format dxfId="94">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="86">
+    <format dxfId="93">
       <pivotArea field="8" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
-    </format>
-    <format dxfId="85">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="8" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="84">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
-    </format>
-    <format dxfId="83">
-      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="82">
-      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="81">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="1" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="80">
-      <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
-    </format>
-    <format dxfId="79">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="1">
-    <chartFormat chart="2" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{904CEA3A-CD0A-459C-A420-1FB249800D4C}" name="Tabela dinâmica4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Nacionalidades" colHeaderCaption="Contagem de Jogadores">
-  <location ref="AK14:AL29" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="9">
-    <pivotField axis="axisCol" showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item h="1" x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" dataField="1" showAll="0" sortType="ascending">
-      <items count="15">
-        <item x="6"/>
-        <item x="4"/>
-        <item x="9"/>
-        <item x="11"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="12"/>
-        <item x="5"/>
-        <item x="10"/>
-        <item x="13"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item t="default"/>
-      </items>
-      <autoSortScope>
-        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
-          <references count="2">
-            <reference field="4294967294" count="1" selected="0">
-              <x v="0"/>
-            </reference>
-            <reference field="0" count="1" selected="0">
-              <x v="0"/>
-            </reference>
-          </references>
-        </pivotArea>
-      </autoSortScope>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="21">
-        <item x="12"/>
-        <item x="9"/>
-        <item x="7"/>
-        <item x="15"/>
-        <item x="5"/>
-        <item x="17"/>
-        <item x="11"/>
-        <item x="10"/>
-        <item x="2"/>
-        <item x="8"/>
-        <item x="18"/>
-        <item x="13"/>
-        <item x="0"/>
-        <item x="16"/>
-        <item x="19"/>
-        <item x="1"/>
-        <item x="4"/>
-        <item x="3"/>
-        <item x="14"/>
-        <item x="6"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="3"/>
-  </rowFields>
-  <rowItems count="14">
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="13"/>
-    </i>
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="11"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="12"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="0"/>
-  </colFields>
-  <colItems count="1">
-    <i>
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Contagem de Nacionalidades" fld="3" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="7">
-    <format dxfId="94">
-      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
-        <references count="1">
-          <reference field="3" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="93">
-      <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
     <format dxfId="92">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
-          <reference field="3" count="0"/>
+          <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
@@ -18935,18 +19021,24 @@
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
     <format dxfId="89">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="88">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
-          <reference field="0" count="0"/>
+          <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="88">
+    <format dxfId="87">
+      <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
+    </format>
+    <format dxfId="86">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
   <chartFormats count="1">
-    <chartFormat chart="1" format="0" series="1">
+    <chartFormat chart="2" format="0" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">

</xml_diff>

<commit_message>
43. Anotações 5ª análise
Anotações sobre a quinta análise.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55CE6822-705D-4792-8BC6-0D5A21DB2B0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{321C7001-6480-4AED-B868-FA0F3B74247A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -777,6 +777,33 @@
       <alignment horizontal="center"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="general"/>
     </dxf>
     <dxf>
@@ -1012,33 +1039,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -15803,7 +15803,7 @@
       <xdr:row>41</xdr:row>
       <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="12148329" cy="6072945"/>
+    <xdr:ext cx="12148329" cy="7403693"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="6" name="CaixaDeTexto 5">
@@ -15818,7 +15818,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="190500" y="7867650"/>
-          <a:ext cx="12148329" cy="6072945"/>
+          <a:ext cx="12148329" cy="7403693"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -16315,6 +16315,225 @@
             </a:rPr>
             <a:t>• </a:t>
           </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>5ª</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> análise: </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>A quinta análise foi construída de uma forma semelhante à terceira e diferente da segunda que, em teoria, seria sua contraparte. A pergunta de negócio relacionada a ela consistia em: </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" i="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>"Quais posições geraram maior retorno financeiro ao clube?"</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>. Pensando nisso, realizei uma tabela dinâmica com a variável </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>posição</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> enquanto a filtrava pelo valor </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Saída</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> da coluna </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>tipo_movimentação</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>. Ao invés de apenas incluir essas duas variáveis, decidi adicionar a coluna </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>jogador</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> na tabela para que a análise se tornasse algo mais rico. Além de evidenciar quais posições, de fato, geraram maior retorno financeiro ao Tottenham Hotspur, também foram incluídos quais jogadores contribuiram para este processo.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="pt-BR" sz="1200" b="0" i="0" baseline="0">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Essa decisão foi algo que enriqueceu o conteúdo da análise, visto que, em decorrência dela, percebemos que mais da metade desse retorno financeiro concentrou-se em apenas um jogador — no caso, </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Harry Kane</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>.</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1200" b="1" baseline="0">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
           <a:endParaRPr lang="pt-BR" sz="1200"/>
         </a:p>
         <a:p>
@@ -16383,10 +16602,10 @@
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>74</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>276225</xdr:colOff>
+      <xdr:row>82</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1089722" cy="327141"/>
     <xdr:sp macro="" textlink="">
@@ -16402,7 +16621,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1219200" y="14097000"/>
+          <a:off x="276225" y="15697200"/>
           <a:ext cx="1089722" cy="327141"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -17158,6 +17377,146 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{996EC5F2-74EB-477F-A9D9-AF44A2544855}" name="Tabela dinâmica3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Faixa Etária" colHeaderCaption="Tipo de Movimentação">
+  <location ref="Y14:Z20" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="10">
+    <pivotField showAll="0"/>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="3">
+        <item h="1" x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField axis="axisRow" dataField="1" showAll="0" sortType="ascending">
+      <items count="9">
+        <item m="1" x="5"/>
+        <item m="1" x="4"/>
+        <item m="1" x="7"/>
+        <item m="1" x="6"/>
+        <item x="3"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="2">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+            <reference field="1" count="1" selected="0">
+              <x v="1"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="8"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="1"/>
+  </colFields>
+  <colItems count="1">
+    <i>
+      <x v="1"/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Contagem de Jogadores" fld="8" subtotal="count" baseField="8" baseItem="0"/>
+  </dataFields>
+  <formats count="9">
+    <format dxfId="8">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="8" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="7">
+      <pivotArea field="8" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="6">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="8" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="5">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+    <format dxfId="4">
+      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="3">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="2">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="1" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="1">
+      <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
+    </format>
+    <format dxfId="0">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="1">
+    <chartFormat chart="2" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{904CEA3A-CD0A-459C-A420-1FB249800D4C}" name="Tabela dinâmica4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Nacionalidades" colHeaderCaption="Contagem de Jogadores">
   <location ref="AK14:AL29" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
@@ -17290,37 +17649,37 @@
     <dataField name="Contagem de Nacionalidades" fld="3" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="7">
-    <format dxfId="6">
+    <format dxfId="15">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="5">
+    <format dxfId="14">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="4">
+    <format dxfId="13">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="3">
+    <format dxfId="12">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="2">
+    <format dxfId="11">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="1">
+    <format dxfId="10">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="0">
+    <format dxfId="9">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -17347,7 +17706,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
   <location ref="O14:P19" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -17416,39 +17775,39 @@
     <dataField name="Soma do Valor das Transferências" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="15">
+    <format dxfId="24">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="14">
+    <format dxfId="23">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="13">
+    <format dxfId="22">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="12">
+    <format dxfId="21">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="11">
+    <format dxfId="20">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="10">
+    <format dxfId="19">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="9">
+    <format dxfId="18">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="8">
+    <format dxfId="17">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="7">
+    <format dxfId="16">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -17475,7 +17834,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6" rowHeaderCaption="Temporadas" colHeaderCaption="">
   <location ref="A14:D22" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -17550,34 +17909,34 @@
     <dataField name="Somas de Entradas e Saídas" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="21">
+    <format dxfId="30">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="20">
+    <format dxfId="29">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="19">
+    <format dxfId="28">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="18">
+    <format dxfId="27">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="17">
+    <format dxfId="26">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="16">
+    <format dxfId="25">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -17619,7 +17978,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4F5027D2-D537-4505-8DBC-54A417F72129}" name="Tabela dinâmica8" cacheId="0" dataPosition="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10" rowHeaderCaption="Posições e Jogadores" colHeaderCaption="Tipo de Movimentação">
   <location ref="BA14:BC26" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
   <pivotFields count="10">
@@ -17749,7 +18108,7 @@
     <dataField name="Porcentagem (%) do Total" fld="6" showDataAs="percentOfTotal" baseField="0" baseItem="0" numFmtId="10"/>
   </dataFields>
   <formats count="18">
-    <format dxfId="39">
+    <format dxfId="48">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -17758,7 +18117,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="38">
+    <format dxfId="47">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -17771,7 +18130,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="37">
+    <format dxfId="46">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -17780,7 +18139,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="36">
+    <format dxfId="45">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -17793,7 +18152,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="35">
+    <format dxfId="44">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -17802,7 +18161,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="34">
+    <format dxfId="43">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -17815,26 +18174,26 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="33">
+    <format dxfId="42">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="32">
+    <format dxfId="41">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="31">
+    <format dxfId="40">
       <pivotArea field="-2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="1"/>
     </format>
-    <format dxfId="30">
+    <format dxfId="39">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="29">
+    <format dxfId="38">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="28">
+    <format dxfId="37">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -17847,7 +18206,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="27">
+    <format dxfId="36">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -17860,7 +18219,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="26">
+    <format dxfId="35">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -17873,14 +18232,14 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="25">
+    <format dxfId="34">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="24">
+    <format dxfId="33">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -17891,10 +18250,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="23">
+    <format dxfId="32">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="22">
+    <format dxfId="31">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
@@ -18273,7 +18632,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FB686887-B509-4E7E-B605-6A13972A6E0B}" name="Tabela dinâmica5" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Origem das Contratações" colHeaderCaption="Contagem de Jogadores">
   <location ref="AN14:AO47" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
@@ -18449,22 +18808,22 @@
     <dataField name="Clubes" fld="3" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="46">
-    <format dxfId="85">
+    <format dxfId="94">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="84">
+    <format dxfId="93">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="83">
+    <format dxfId="92">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="82">
+    <format dxfId="91">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="81">
+    <format dxfId="90">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="80">
+    <format dxfId="89">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="15">
@@ -18487,10 +18846,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="79">
+    <format dxfId="88">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="78">
+    <format dxfId="87">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18502,7 +18861,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="77">
+    <format dxfId="86">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18514,7 +18873,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="76">
+    <format dxfId="85">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18526,7 +18885,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="75">
+    <format dxfId="84">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18538,7 +18897,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="74">
+    <format dxfId="83">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18550,7 +18909,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="73">
+    <format dxfId="82">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="2">
@@ -18563,7 +18922,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="72">
+    <format dxfId="81">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18575,7 +18934,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="71">
+    <format dxfId="80">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18587,7 +18946,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="70">
+    <format dxfId="79">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18599,7 +18958,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="69">
+    <format dxfId="78">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18611,7 +18970,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="68">
+    <format dxfId="77">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18623,7 +18982,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="67">
+    <format dxfId="76">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18635,7 +18994,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="66">
+    <format dxfId="75">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18647,7 +19006,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="65">
+    <format dxfId="74">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18659,7 +19018,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="64">
+    <format dxfId="73">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18671,29 +19030,29 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="63">
+    <format dxfId="72">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="62">
+    <format dxfId="71">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="61">
+    <format dxfId="70">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="60">
+    <format dxfId="69">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="59">
+    <format dxfId="68">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="58">
+    <format dxfId="67">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="57">
+    <format dxfId="66">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="15">
@@ -18716,10 +19075,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="56">
+    <format dxfId="65">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="55">
+    <format dxfId="64">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18731,7 +19090,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="54">
+    <format dxfId="63">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18743,7 +19102,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="53">
+    <format dxfId="62">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18755,7 +19114,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="52">
+    <format dxfId="61">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18767,7 +19126,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="51">
+    <format dxfId="60">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18779,7 +19138,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="50">
+    <format dxfId="59">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="2">
@@ -18792,7 +19151,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="49">
+    <format dxfId="58">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18804,7 +19163,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="48">
+    <format dxfId="57">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18816,7 +19175,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="47">
+    <format dxfId="56">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18828,7 +19187,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="46">
+    <format dxfId="55">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18840,7 +19199,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="45">
+    <format dxfId="54">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18852,7 +19211,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="44">
+    <format dxfId="53">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18864,7 +19223,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="43">
+    <format dxfId="52">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18876,7 +19235,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="42">
+    <format dxfId="51">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18888,7 +19247,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="41">
+    <format dxfId="50">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18900,7 +19259,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="40">
+    <format dxfId="49">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
@@ -18908,146 +19267,6 @@
       </pivotArea>
     </format>
   </formats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{996EC5F2-74EB-477F-A9D9-AF44A2544855}" name="Tabela dinâmica3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Faixa Etária" colHeaderCaption="Tipo de Movimentação">
-  <location ref="Y14:Z20" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="10">
-    <pivotField showAll="0"/>
-    <pivotField axis="axisCol" showAll="0">
-      <items count="3">
-        <item h="1" x="1"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField axis="axisRow" dataField="1" showAll="0" sortType="ascending">
-      <items count="9">
-        <item m="1" x="5"/>
-        <item m="1" x="4"/>
-        <item m="1" x="7"/>
-        <item m="1" x="6"/>
-        <item x="3"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-      <autoSortScope>
-        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
-          <references count="2">
-            <reference field="4294967294" count="1" selected="0">
-              <x v="0"/>
-            </reference>
-            <reference field="1" count="1" selected="0">
-              <x v="1"/>
-            </reference>
-          </references>
-        </pivotArea>
-      </autoSortScope>
-    </pivotField>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="8"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="1"/>
-  </colFields>
-  <colItems count="1">
-    <i>
-      <x v="1"/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Contagem de Jogadores" fld="8" subtotal="count" baseField="8" baseItem="0"/>
-  </dataFields>
-  <formats count="9">
-    <format dxfId="94">
-      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
-        <references count="1">
-          <reference field="8" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="93">
-      <pivotArea field="8" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
-    </format>
-    <format dxfId="92">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="8" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="91">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
-    </format>
-    <format dxfId="90">
-      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="89">
-      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="88">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="1" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="87">
-      <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
-    </format>
-    <format dxfId="86">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="1">
-    <chartFormat chart="2" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">

</xml_diff>

<commit_message>
44. Começo da 6ª análise
Começando a sexta análise por reunir as evidências das outras análises.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{321C7001-6480-4AED-B868-FA0F3B74247A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61A5BBC2-47E8-416D-A77A-3C0EF743D7F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Apresentação" sheetId="3" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="523" uniqueCount="194">
   <si>
     <t>temporada</t>
   </si>
@@ -609,6 +609,24 @@
   <si>
     <t>Saídas/Vendas de Jogadores em %</t>
   </si>
+  <si>
+    <t>Investimento no Período</t>
+  </si>
+  <si>
+    <t>Retorno no Período</t>
+  </si>
+  <si>
+    <t>Saldo Total no Período</t>
+  </si>
+  <si>
+    <t>Inv. em Meio-campistas</t>
+  </si>
+  <si>
+    <t>Inv. em Atacantes</t>
+  </si>
+  <si>
+    <t>Inv. em Defensores</t>
+  </si>
 </sst>
 </file>
 
@@ -618,7 +636,7 @@
     <numFmt numFmtId="164" formatCode="[$£-809]#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -652,6 +670,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -673,7 +699,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -690,12 +716,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -749,12 +784,187 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentagem" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="95">
+  <dxfs count="104">
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="center"/>
     </dxf>
@@ -901,144 +1111,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -2383,13 +2455,13 @@
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>Defensor</c:v>
+                  <c:v>Meio-campista</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>Atacante</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Meio-campista</c:v>
+                  <c:v>Defensor</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2401,13 +2473,13 @@
                 <c:formatCode>[$£-809]#,##0.00</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>138800000</c:v>
+                  <c:v>213900000</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>200500000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>213900000</c:v>
+                  <c:v>138800000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2836,13 +2908,13 @@
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>0.25090383224873464</c:v>
+                  <c:v>0.3866594360086768</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0.36243673174258856</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.3866594360086768</c:v>
+                  <c:v>0.25090383224873464</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -10706,7 +10778,15 @@
           </a:r>
           <a:r>
             <a:rPr lang="pt-BR" sz="1200" b="1"/>
-            <a:t> Quais negociações representaram maior impacto financeiro para o clube?</a:t>
+            <a:t> O</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0"/>
+            <a:t> que todas as evidências nos dizem sobre a estratégia do Tottenham Hotspur no mercado de transferências</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1"/>
+            <a:t>?</a:t>
           </a:r>
           <a:endParaRPr lang="pt-BR" sz="1200" b="1" baseline="0"/>
         </a:p>
@@ -14987,6 +15067,377 @@
             <a:t>valorização dos mesmos.</a:t>
           </a:r>
           <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>64</xdr:col>
+      <xdr:colOff>690801</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>179894</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1527021" cy="405432"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="37" name="CaixaDeTexto 36">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A05B3AC1-D0C5-4D40-9153-DA77CE942B48}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="71167142" y="1322894"/>
+          <a:ext cx="1527021" cy="405432"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="2000" b="1" baseline="0"/>
+            <a:t>6. Conclusão</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>61</xdr:col>
+      <xdr:colOff>1302238</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>127911</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="8815876" cy="530658"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="38" name="CaixaDeTexto 37">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{679200D7-A3DE-4C25-99CE-17C6913BB572}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="67466352" y="1651911"/>
+          <a:ext cx="8815876" cy="530658"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0"/>
+            <a:t>Pergunta de Negócio: </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="1"/>
+            <a:t>Quais características</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="1" baseline="0"/>
+            <a:t> definiram a estratégia do Tottenham Hotspur no mercado de transferências</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="1" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="1" baseline="0"/>
+            <a:t>entre as temporadas 2019/20 até 2024/25?</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>61</xdr:col>
+      <xdr:colOff>1313446</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>125801</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1013483" cy="311496"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="39" name="CaixaDeTexto 38">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{55A26890-609E-40CD-8A3E-802A9AC8F926}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="67620026" y="2390235"/>
+          <a:ext cx="1013483" cy="311496"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0"/>
+            <a:t>Evidências:</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>61</xdr:col>
+      <xdr:colOff>1318427</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>152758</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="323615" cy="311496"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="40" name="CaixaDeTexto 39">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D99A57C2-1A06-425C-99E3-E928AC0EEC47}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="67625007" y="2794598"/>
+          <a:ext cx="323615" cy="311496"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0"/>
+            <a:t>1.</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>61</xdr:col>
+      <xdr:colOff>1305030</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>127598</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="323615" cy="311496"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="41" name="CaixaDeTexto 40">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8A89519C-77FC-4092-8894-B0F46E9A76A6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="67460485" y="3565257"/>
+          <a:ext cx="323615" cy="311496"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0"/>
+            <a:t>2.</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>61</xdr:col>
+      <xdr:colOff>1305030</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>127598</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="323615" cy="311496"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="42" name="CaixaDeTexto 41">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{453269F0-11F9-4971-A436-A9BEDAACC788}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="67469144" y="4335916"/>
+          <a:ext cx="323615" cy="311496"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0"/>
+            <a:t>3.</a:t>
+          </a:r>
         </a:p>
       </xdr:txBody>
     </xdr:sp>
@@ -17377,6 +17828,653 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FB686887-B509-4E7E-B605-6A13972A6E0B}" name="Tabela dinâmica5" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Origem das Contratações" colHeaderCaption="Contagem de Jogadores">
+  <location ref="AN14:AO47" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="9">
+    <pivotField axis="axisCol" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item h="1" x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" dataField="1" showAll="0">
+      <items count="15">
+        <item x="6"/>
+        <item x="4"/>
+        <item x="9"/>
+        <item x="11"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="12"/>
+        <item x="5"/>
+        <item x="10"/>
+        <item x="13"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="21">
+        <item x="12"/>
+        <item x="9"/>
+        <item x="7"/>
+        <item x="15"/>
+        <item x="5"/>
+        <item x="17"/>
+        <item x="11"/>
+        <item x="10"/>
+        <item x="2"/>
+        <item x="8"/>
+        <item x="18"/>
+        <item x="13"/>
+        <item x="0"/>
+        <item x="16"/>
+        <item x="19"/>
+        <item x="1"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item x="14"/>
+        <item x="6"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="2">
+    <field x="4"/>
+    <field x="3"/>
+  </rowFields>
+  <rowItems count="32">
+    <i>
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i r="1">
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i r="1">
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i r="1">
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i r="1">
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i r="1">
+      <x v="12"/>
+    </i>
+    <i r="1">
+      <x v="13"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i r="1">
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i r="1">
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i r="1">
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i r="1">
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="15"/>
+    </i>
+    <i r="1">
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="16"/>
+    </i>
+    <i r="1">
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="17"/>
+    </i>
+    <i r="1">
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="18"/>
+    </i>
+    <i r="1">
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="19"/>
+    </i>
+    <i r="1">
+      <x v="9"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="0"/>
+  </colFields>
+  <colItems count="1">
+    <i>
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Clubes" fld="3" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="46">
+    <format dxfId="54">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="53">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="52">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="51">
+      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
+    </format>
+    <format dxfId="50">
+      <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="49">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="4" count="15">
+            <x v="2"/>
+            <x v="5"/>
+            <x v="6"/>
+            <x v="7"/>
+            <x v="8"/>
+            <x v="9"/>
+            <x v="10"/>
+            <x v="11"/>
+            <x v="12"/>
+            <x v="13"/>
+            <x v="15"/>
+            <x v="16"/>
+            <x v="17"/>
+            <x v="18"/>
+            <x v="19"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="48">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="47">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="0"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="46">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="8"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="5"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="45">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="10"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="6"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="44">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="2"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="7"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="43">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="3"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="8"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="42">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="2">
+            <x v="12"/>
+            <x v="13"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="9"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="41">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="8"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="10"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="40">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="8"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="11"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="39">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="6"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="12"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="38">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="11"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="13"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="37">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="7"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="15"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="36">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="5"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="16"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="35">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="4"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="17"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="34">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="7"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="18"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="33">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="9"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="19"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="32">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="31">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="30">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="29">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="28">
+      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
+    </format>
+    <format dxfId="27">
+      <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="26">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="4" count="15">
+            <x v="2"/>
+            <x v="5"/>
+            <x v="6"/>
+            <x v="7"/>
+            <x v="8"/>
+            <x v="9"/>
+            <x v="10"/>
+            <x v="11"/>
+            <x v="12"/>
+            <x v="13"/>
+            <x v="15"/>
+            <x v="16"/>
+            <x v="17"/>
+            <x v="18"/>
+            <x v="19"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="25">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="24">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="0"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="23">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="8"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="5"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="22">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="10"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="6"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="21">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="2"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="7"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="20">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="3"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="8"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="19">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="2">
+            <x v="12"/>
+            <x v="13"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="9"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="18">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="8"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="10"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="17">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="8"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="11"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="16">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="6"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="12"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="15">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="11"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="13"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="14">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="7"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="15"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="13">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="5"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="16"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="12">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="4"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="17"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="11">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="7"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="18"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="10">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="9"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="19"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="9">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{996EC5F2-74EB-477F-A9D9-AF44A2544855}" name="Tabela dinâmica3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Faixa Etária" colHeaderCaption="Tipo de Movimentação">
   <location ref="Y14:Z20" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -17453,43 +18551,43 @@
     <dataField name="Contagem de Jogadores" fld="8" subtotal="count" baseField="8" baseItem="0"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="8">
+    <format dxfId="63">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="7">
+    <format dxfId="62">
       <pivotArea field="8" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="6">
+    <format dxfId="61">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="5">
+    <format dxfId="60">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="4">
+    <format dxfId="59">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="3">
+    <format dxfId="58">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="2">
+    <format dxfId="57">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="1">
+    <format dxfId="56">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="0">
+    <format dxfId="55">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -17516,7 +18614,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{904CEA3A-CD0A-459C-A420-1FB249800D4C}" name="Tabela dinâmica4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Nacionalidades" colHeaderCaption="Contagem de Jogadores">
   <location ref="AK14:AL29" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
@@ -17649,37 +18747,37 @@
     <dataField name="Contagem de Nacionalidades" fld="3" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="7">
-    <format dxfId="15">
+    <format dxfId="70">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="14">
+    <format dxfId="69">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="13">
+    <format dxfId="68">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="12">
+    <format dxfId="67">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="11">
+    <format dxfId="66">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="10">
+    <format dxfId="65">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="9">
+    <format dxfId="64">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -17706,7 +18804,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
   <location ref="O14:P19" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -17719,7 +18817,7 @@
       </items>
     </pivotField>
     <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0" sortType="ascending">
+    <pivotField axis="axisRow" showAll="0" sortType="descending">
       <items count="4">
         <item x="1"/>
         <item x="2"/>
@@ -17751,13 +18849,13 @@
   </rowFields>
   <rowItems count="4">
     <i>
-      <x v="1"/>
+      <x v="2"/>
     </i>
     <i>
       <x/>
     </i>
     <i>
-      <x v="2"/>
+      <x v="1"/>
     </i>
     <i t="grand">
       <x/>
@@ -17775,39 +18873,39 @@
     <dataField name="Soma do Valor das Transferências" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="24">
+    <format dxfId="79">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="23">
+    <format dxfId="78">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="22">
+    <format dxfId="77">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="21">
+    <format dxfId="76">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="20">
+    <format dxfId="75">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="19">
+    <format dxfId="74">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="18">
+    <format dxfId="73">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="17">
+    <format dxfId="72">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="16">
+    <format dxfId="71">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -17834,7 +18932,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6" rowHeaderCaption="Temporadas" colHeaderCaption="">
   <location ref="A14:D22" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -17909,34 +19007,34 @@
     <dataField name="Somas de Entradas e Saídas" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="30">
+    <format dxfId="85">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="29">
+    <format dxfId="84">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="28">
+    <format dxfId="83">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="27">
+    <format dxfId="82">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="26">
+    <format dxfId="81">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="25">
+    <format dxfId="80">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -17978,7 +19076,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4F5027D2-D537-4505-8DBC-54A417F72129}" name="Tabela dinâmica8" cacheId="0" dataPosition="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10" rowHeaderCaption="Posições e Jogadores" colHeaderCaption="Tipo de Movimentação">
   <location ref="BA14:BC26" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
   <pivotFields count="10">
@@ -18108,7 +19206,7 @@
     <dataField name="Porcentagem (%) do Total" fld="6" showDataAs="percentOfTotal" baseField="0" baseItem="0" numFmtId="10"/>
   </dataFields>
   <formats count="18">
-    <format dxfId="48">
+    <format dxfId="103">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -18117,7 +19215,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="47">
+    <format dxfId="102">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -18130,7 +19228,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="46">
+    <format dxfId="101">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -18139,7 +19237,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="45">
+    <format dxfId="100">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -18152,7 +19250,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="44">
+    <format dxfId="99">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -18161,7 +19259,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="43">
+    <format dxfId="98">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -18174,26 +19272,26 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="42">
+    <format dxfId="97">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="41">
+    <format dxfId="96">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="40">
+    <format dxfId="95">
       <pivotArea field="-2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="1"/>
     </format>
-    <format dxfId="39">
+    <format dxfId="94">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="38">
+    <format dxfId="93">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="37">
+    <format dxfId="92">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -18206,7 +19304,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="36">
+    <format dxfId="91">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -18219,7 +19317,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="35">
+    <format dxfId="90">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -18232,14 +19330,14 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="34">
+    <format dxfId="89">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="33">
+    <format dxfId="88">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -18250,10 +19348,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="32">
+    <format dxfId="87">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="31">
+    <format dxfId="86">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
@@ -18632,653 +19730,6 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FB686887-B509-4E7E-B605-6A13972A6E0B}" name="Tabela dinâmica5" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Origem das Contratações" colHeaderCaption="Contagem de Jogadores">
-  <location ref="AN14:AO47" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="9">
-    <pivotField axis="axisCol" showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item h="1" x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" dataField="1" showAll="0">
-      <items count="15">
-        <item x="6"/>
-        <item x="4"/>
-        <item x="9"/>
-        <item x="11"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="12"/>
-        <item x="5"/>
-        <item x="10"/>
-        <item x="13"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="21">
-        <item x="12"/>
-        <item x="9"/>
-        <item x="7"/>
-        <item x="15"/>
-        <item x="5"/>
-        <item x="17"/>
-        <item x="11"/>
-        <item x="10"/>
-        <item x="2"/>
-        <item x="8"/>
-        <item x="18"/>
-        <item x="13"/>
-        <item x="0"/>
-        <item x="16"/>
-        <item x="19"/>
-        <item x="1"/>
-        <item x="4"/>
-        <item x="3"/>
-        <item x="14"/>
-        <item x="6"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="2">
-    <field x="4"/>
-    <field x="3"/>
-  </rowFields>
-  <rowItems count="32">
-    <i>
-      <x v="2"/>
-    </i>
-    <i r="1">
-      <x/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i r="1">
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i r="1">
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i r="1">
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i r="1">
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i r="1">
-      <x v="12"/>
-    </i>
-    <i r="1">
-      <x v="13"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i r="1">
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="11"/>
-    </i>
-    <i r="1">
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="12"/>
-    </i>
-    <i r="1">
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="13"/>
-    </i>
-    <i r="1">
-      <x v="11"/>
-    </i>
-    <i>
-      <x v="15"/>
-    </i>
-    <i r="1">
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="16"/>
-    </i>
-    <i r="1">
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="17"/>
-    </i>
-    <i r="1">
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="18"/>
-    </i>
-    <i r="1">
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="19"/>
-    </i>
-    <i r="1">
-      <x v="9"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="0"/>
-  </colFields>
-  <colItems count="1">
-    <i>
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Clubes" fld="3" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="46">
-    <format dxfId="94">
-      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="93">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="92">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="91">
-      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
-    </format>
-    <format dxfId="90">
-      <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
-    </format>
-    <format dxfId="89">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="4" count="15">
-            <x v="2"/>
-            <x v="5"/>
-            <x v="6"/>
-            <x v="7"/>
-            <x v="8"/>
-            <x v="9"/>
-            <x v="10"/>
-            <x v="11"/>
-            <x v="12"/>
-            <x v="13"/>
-            <x v="15"/>
-            <x v="16"/>
-            <x v="17"/>
-            <x v="18"/>
-            <x v="19"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="88">
-      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="87">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="0"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="86">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="8"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="5"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="85">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="10"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="6"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="84">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="2"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="7"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="83">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="3"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="8"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="82">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="2">
-            <x v="12"/>
-            <x v="13"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="9"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="81">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="8"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="10"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="80">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="8"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="11"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="79">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="6"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="12"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="78">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="11"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="13"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="77">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="7"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="15"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="76">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="5"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="16"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="75">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="4"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="17"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="74">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="7"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="18"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="73">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="9"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="19"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="72">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="0" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="71">
-      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="70">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="69">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="68">
-      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
-    </format>
-    <format dxfId="67">
-      <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
-    </format>
-    <format dxfId="66">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="4" count="15">
-            <x v="2"/>
-            <x v="5"/>
-            <x v="6"/>
-            <x v="7"/>
-            <x v="8"/>
-            <x v="9"/>
-            <x v="10"/>
-            <x v="11"/>
-            <x v="12"/>
-            <x v="13"/>
-            <x v="15"/>
-            <x v="16"/>
-            <x v="17"/>
-            <x v="18"/>
-            <x v="19"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="65">
-      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="64">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="0"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="63">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="8"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="5"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="62">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="10"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="6"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="61">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="2"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="7"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="60">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="3"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="8"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="59">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="2">
-            <x v="12"/>
-            <x v="13"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="9"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="58">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="8"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="10"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="57">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="8"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="11"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="56">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="6"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="12"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="55">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="11"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="13"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="54">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="7"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="15"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="53">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="5"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="16"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="52">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="4"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="17"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="51">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="7"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="18"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="50">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="9"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="19"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="49">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="0" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-  </formats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -21126,7 +21577,7 @@
   <sheetPr>
     <tabColor theme="6" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A4:BI47"/>
+  <dimension ref="A4:BP47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.5703125" bestFit="1" customWidth="1"/>
@@ -21138,7 +21589,7 @@
     <col min="7" max="7" width="22.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="25.5703125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="32" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="31.28515625" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="26.28515625" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="14.85546875" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="14.28515625" bestFit="1" customWidth="1"/>
@@ -21164,11 +21615,11 @@
     <col min="61" max="61" width="15.85546875" bestFit="1" customWidth="1"/>
     <col min="62" max="62" width="20.42578125" bestFit="1" customWidth="1"/>
     <col min="63" max="63" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="65" max="65" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="12.7109375" customWidth="1"/>
     <col min="66" max="66" width="20.7109375" bestFit="1" customWidth="1"/>
     <col min="67" max="67" width="11" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="23.85546875" bestFit="1" customWidth="1"/>
     <col min="69" max="69" width="15.5703125" bestFit="1" customWidth="1"/>
     <col min="70" max="70" width="16" bestFit="1" customWidth="1"/>
     <col min="71" max="72" width="18" bestFit="1" customWidth="1"/>
@@ -21176,7 +21627,7 @@
     <col min="74" max="74" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:68" x14ac:dyDescent="0.25">
       <c r="C4" s="7" t="s">
         <v>158</v>
       </c>
@@ -21199,7 +21650,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="5" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:68" x14ac:dyDescent="0.25">
       <c r="C5" s="2">
         <f>COUNTA('Dados Tratados'!A3:A24)</f>
         <v>22</v>
@@ -21229,7 +21680,7 @@
         <v>24.529331514324692</v>
       </c>
     </row>
-    <row r="14" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
         <v>167</v>
       </c>
@@ -21272,7 +21723,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="15" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
         <v>165</v>
       </c>
@@ -21339,7 +21790,7 @@
         <v>0.70199999999999996</v>
       </c>
     </row>
-    <row r="16" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>9</v>
       </c>
@@ -21360,17 +21811,17 @@
         <v>-65000000</v>
       </c>
       <c r="O16" s="2" t="s">
-        <v>70</v>
+        <v>156</v>
       </c>
       <c r="P16" s="6">
-        <v>138800000</v>
+        <v>213900000</v>
       </c>
       <c r="R16" s="2" t="s">
         <v>156</v>
       </c>
       <c r="S16" s="13">
         <f>P16/$P$19</f>
-        <v>0.25090383224873464</v>
+        <v>0.3866594360086768</v>
       </c>
       <c r="Y16" s="2" t="s">
         <v>179</v>
@@ -21412,8 +21863,17 @@
       <c r="BF16" s="13">
         <v>0.22500000000000001</v>
       </c>
+      <c r="BL16" s="21" t="s">
+        <v>188</v>
+      </c>
+      <c r="BN16" s="21" t="s">
+        <v>189</v>
+      </c>
+      <c r="BP16" s="21" t="s">
+        <v>190</v>
+      </c>
     </row>
-    <row r="17" spans="1:61" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>34</v>
       </c>
@@ -21486,8 +21946,17 @@
       <c r="BF17" s="13">
         <v>7.1999999999999995E-2</v>
       </c>
+      <c r="BL17" s="22">
+        <v>553200000</v>
+      </c>
+      <c r="BN17" s="22">
+        <v>179800000</v>
+      </c>
+      <c r="BP17" s="6">
+        <v>-373400000</v>
+      </c>
     </row>
-    <row r="18" spans="1:61" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>55</v>
       </c>
@@ -21508,17 +21977,17 @@
         <v>-58000000</v>
       </c>
       <c r="O18" s="2" t="s">
-        <v>156</v>
+        <v>70</v>
       </c>
       <c r="P18" s="6">
-        <v>213900000</v>
+        <v>138800000</v>
       </c>
       <c r="R18" s="2" t="s">
         <v>70</v>
       </c>
       <c r="S18" s="13">
         <f>P18/$P$19</f>
-        <v>0.3866594360086768</v>
+        <v>0.25090383224873464</v>
       </c>
       <c r="Y18" s="2" t="s">
         <v>177</v>
@@ -21561,7 +22030,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:61" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>75</v>
       </c>
@@ -21581,7 +22050,7 @@
         <f t="shared" si="0"/>
         <v>-55700000</v>
       </c>
-      <c r="O19" t="s">
+      <c r="O19" s="23" t="s">
         <v>164</v>
       </c>
       <c r="P19" s="6">
@@ -21629,7 +22098,7 @@
         <v>0.17408231368186874</v>
       </c>
     </row>
-    <row r="20" spans="1:61" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>93</v>
       </c>
@@ -21683,8 +22152,17 @@
       <c r="BC20" s="13">
         <v>0.22525027808676307</v>
       </c>
+      <c r="BL20" s="21" t="s">
+        <v>191</v>
+      </c>
+      <c r="BN20" s="21" t="s">
+        <v>192</v>
+      </c>
+      <c r="BP20" s="21" t="s">
+        <v>193</v>
+      </c>
     </row>
-    <row r="21" spans="1:61" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>109</v>
       </c>
@@ -21725,8 +22203,17 @@
       <c r="BC21" s="13">
         <v>0.15016685205784205</v>
       </c>
+      <c r="BL21" s="13">
+        <v>0.3866594360086768</v>
+      </c>
+      <c r="BN21" s="24">
+        <v>0.36243673174258856</v>
+      </c>
+      <c r="BP21" s="24">
+        <v>0.25090383224873464</v>
+      </c>
     </row>
-    <row r="22" spans="1:61" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
         <v>164</v>
       </c>
@@ -21768,7 +22255,7 @@
         <v>7.5083426028921027E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:61" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:68" x14ac:dyDescent="0.25">
       <c r="AK23" s="2" t="s">
         <v>30</v>
       </c>
@@ -21791,7 +22278,7 @@
         <v>7.2302558398220251E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:61" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:68" x14ac:dyDescent="0.25">
       <c r="AK24" s="2" t="s">
         <v>152</v>
       </c>
@@ -21814,7 +22301,7 @@
         <v>7.2302558398220251E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:61" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:68" x14ac:dyDescent="0.25">
       <c r="AK25" s="2" t="s">
         <v>78</v>
       </c>
@@ -21839,7 +22326,7 @@
       <c r="BH25" s="2"/>
       <c r="BI25" s="6"/>
     </row>
-    <row r="26" spans="1:61" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:68" x14ac:dyDescent="0.25">
       <c r="AK26" s="2" t="s">
         <v>64</v>
       </c>
@@ -21862,7 +22349,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:61" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:68" x14ac:dyDescent="0.25">
       <c r="AK27" s="2" t="s">
         <v>90</v>
       </c>
@@ -21876,7 +22363,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:61" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:68" x14ac:dyDescent="0.25">
       <c r="AK28" s="2" t="s">
         <v>97</v>
       </c>
@@ -21890,7 +22377,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:61" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:68" x14ac:dyDescent="0.25">
       <c r="AK29" s="9" t="s">
         <v>164</v>
       </c>
@@ -21904,7 +22391,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:61" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:68" x14ac:dyDescent="0.25">
       <c r="AN30" s="2" t="s">
         <v>97</v>
       </c>
@@ -21912,7 +22399,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:61" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:68" x14ac:dyDescent="0.25">
       <c r="AN31" s="2" t="s">
         <v>98</v>
       </c>
@@ -21920,7 +22407,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:61" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:68" x14ac:dyDescent="0.25">
       <c r="AN32" s="2" t="s">
         <v>97</v>
       </c>

</xml_diff>

<commit_message>
45. Andamento da 6ª análise
Andamento da sexta análise.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61A5BBC2-47E8-416D-A77A-3C0EF743D7F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{738A07C3-70A6-4C8C-9AF5-B422EFC3A549}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="523" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="203">
   <si>
     <t>temporada</t>
   </si>
@@ -627,6 +627,33 @@
   <si>
     <t>Inv. em Defensores</t>
   </si>
+  <si>
+    <t>Jogadores Ingleses</t>
+  </si>
+  <si>
+    <t>Jogadores Holandeses</t>
+  </si>
+  <si>
+    <t>Cont. de Jovens</t>
+  </si>
+  <si>
+    <t>Cont. de Experientes</t>
+  </si>
+  <si>
+    <t>Cont. de Veteranos</t>
+  </si>
+  <si>
+    <t>Ret. de Meio-campistas</t>
+  </si>
+  <si>
+    <t>Ret. de Atacantes</t>
+  </si>
+  <si>
+    <t>Ret. de Defensores</t>
+  </si>
+  <si>
+    <t>Nacionalidades Diversas</t>
+  </si>
 </sst>
 </file>
 
@@ -636,7 +663,7 @@
     <numFmt numFmtId="164" formatCode="[$£-809]#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -671,6 +698,13 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="12"/>
       <color theme="1"/>
@@ -679,7 +713,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -696,6 +730,12 @@
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.79998168889431442"/>
         <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -730,7 +770,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -784,7 +824,8 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -794,39 +835,18 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentagem" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="104">
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general"/>
-    </dxf>
+  <dxfs count="95">
     <dxf>
       <alignment horizontal="center"/>
     </dxf>
@@ -15443,6 +15463,184 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>61</xdr:col>
+      <xdr:colOff>1327544</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>124134</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="323615" cy="311496"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="43" name="CaixaDeTexto 42">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AE75D060-754E-4F9C-8871-D7844C116DDC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="67491658" y="5103111"/>
+          <a:ext cx="323615" cy="311496"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0"/>
+            <a:t>4.</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>61</xdr:col>
+      <xdr:colOff>1315421</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>146649</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="323615" cy="311496"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="44" name="CaixaDeTexto 43">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9B0C7E65-58CB-46DB-8C54-63E085A68A71}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="67479535" y="5896285"/>
+          <a:ext cx="323615" cy="311496"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0"/>
+            <a:t>5.</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>61</xdr:col>
+      <xdr:colOff>1305995</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>146568</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="884216" cy="311496"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="45" name="CaixaDeTexto 44">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{268DAF49-0C02-48AB-B8BB-D0B8A7C661EF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="67726995" y="6676485"/>
+          <a:ext cx="884216" cy="311496"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0"/>
+            <a:t>Veredito:</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -18003,22 +18201,22 @@
     <dataField name="Clubes" fld="3" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="46">
-    <format dxfId="54">
+    <format dxfId="45">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="53">
+    <format dxfId="44">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="52">
+    <format dxfId="43">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="51">
+    <format dxfId="42">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="50">
+    <format dxfId="41">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="49">
+    <format dxfId="40">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="15">
@@ -18041,10 +18239,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="48">
+    <format dxfId="39">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="47">
+    <format dxfId="38">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18056,7 +18254,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="46">
+    <format dxfId="37">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18068,7 +18266,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="45">
+    <format dxfId="36">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18080,7 +18278,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="44">
+    <format dxfId="35">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18092,7 +18290,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="43">
+    <format dxfId="34">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18104,7 +18302,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="42">
+    <format dxfId="33">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="2">
@@ -18117,7 +18315,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="41">
+    <format dxfId="32">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18129,7 +18327,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="40">
+    <format dxfId="31">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18141,7 +18339,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="39">
+    <format dxfId="30">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18153,7 +18351,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="38">
+    <format dxfId="29">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18165,7 +18363,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="37">
+    <format dxfId="28">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18177,7 +18375,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="36">
+    <format dxfId="27">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18189,7 +18387,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="35">
+    <format dxfId="26">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18201,7 +18399,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="34">
+    <format dxfId="25">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18213,7 +18411,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="33">
+    <format dxfId="24">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18225,29 +18423,29 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="32">
+    <format dxfId="23">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="31">
+    <format dxfId="22">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="30">
+    <format dxfId="21">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="29">
+    <format dxfId="20">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="28">
+    <format dxfId="19">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="27">
+    <format dxfId="18">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="26">
+    <format dxfId="17">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="15">
@@ -18270,10 +18468,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="25">
+    <format dxfId="16">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="24">
+    <format dxfId="15">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18285,7 +18483,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="23">
+    <format dxfId="14">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18297,7 +18495,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="22">
+    <format dxfId="13">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18309,7 +18507,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="21">
+    <format dxfId="12">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18321,7 +18519,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="20">
+    <format dxfId="11">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18333,7 +18531,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="19">
+    <format dxfId="10">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="2">
@@ -18346,7 +18544,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="18">
+    <format dxfId="9">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18358,7 +18556,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="17">
+    <format dxfId="8">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18370,7 +18568,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="16">
+    <format dxfId="7">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18382,7 +18580,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="15">
+    <format dxfId="6">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18394,7 +18592,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="14">
+    <format dxfId="5">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18406,7 +18604,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="13">
+    <format dxfId="4">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18418,7 +18616,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="12">
+    <format dxfId="3">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18430,7 +18628,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="11">
+    <format dxfId="2">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18442,7 +18640,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="10">
+    <format dxfId="1">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -18454,7 +18652,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="9">
+    <format dxfId="0">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
@@ -18551,43 +18749,43 @@
     <dataField name="Contagem de Jogadores" fld="8" subtotal="count" baseField="8" baseItem="0"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="63">
+    <format dxfId="54">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="62">
+    <format dxfId="53">
       <pivotArea field="8" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="61">
+    <format dxfId="52">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="60">
+    <format dxfId="51">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="59">
+    <format dxfId="50">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="58">
+    <format dxfId="49">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="57">
+    <format dxfId="48">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="56">
+    <format dxfId="47">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="55">
+    <format dxfId="46">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -18747,37 +18945,37 @@
     <dataField name="Contagem de Nacionalidades" fld="3" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="7">
-    <format dxfId="70">
+    <format dxfId="61">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="69">
+    <format dxfId="60">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="68">
+    <format dxfId="59">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="67">
+    <format dxfId="58">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="66">
+    <format dxfId="57">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="65">
+    <format dxfId="56">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="64">
+    <format dxfId="55">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -18873,39 +19071,39 @@
     <dataField name="Soma do Valor das Transferências" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="79">
+    <format dxfId="70">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="78">
+    <format dxfId="69">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="77">
+    <format dxfId="68">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="76">
+    <format dxfId="67">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="75">
+    <format dxfId="66">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="74">
+    <format dxfId="65">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="73">
+    <format dxfId="64">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="72">
+    <format dxfId="63">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="71">
+    <format dxfId="62">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -19007,34 +19205,34 @@
     <dataField name="Somas de Entradas e Saídas" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="85">
+    <format dxfId="76">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="84">
+    <format dxfId="75">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="83">
+    <format dxfId="74">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="82">
+    <format dxfId="73">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="81">
+    <format dxfId="72">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="80">
+    <format dxfId="71">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -19206,7 +19404,7 @@
     <dataField name="Porcentagem (%) do Total" fld="6" showDataAs="percentOfTotal" baseField="0" baseItem="0" numFmtId="10"/>
   </dataFields>
   <formats count="18">
-    <format dxfId="103">
+    <format dxfId="94">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -19215,7 +19413,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="102">
+    <format dxfId="93">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -19228,7 +19426,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="101">
+    <format dxfId="92">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -19237,7 +19435,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="100">
+    <format dxfId="91">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -19250,7 +19448,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="99">
+    <format dxfId="90">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -19259,7 +19457,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="98">
+    <format dxfId="89">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -19272,26 +19470,26 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="97">
+    <format dxfId="88">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="96">
+    <format dxfId="87">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="95">
+    <format dxfId="86">
       <pivotArea field="-2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="1"/>
     </format>
-    <format dxfId="94">
+    <format dxfId="85">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="93">
+    <format dxfId="84">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="92">
+    <format dxfId="83">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -19304,7 +19502,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="91">
+    <format dxfId="82">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -19317,7 +19515,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="90">
+    <format dxfId="81">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -19330,14 +19528,14 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="89">
+    <format dxfId="80">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="88">
+    <format dxfId="79">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -19348,10 +19546,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="87">
+    <format dxfId="78">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="86">
+    <format dxfId="77">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
@@ -21577,7 +21775,7 @@
   <sheetPr>
     <tabColor theme="6" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A4:BP47"/>
+  <dimension ref="A4:BR47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.5703125" bestFit="1" customWidth="1"/>
@@ -21616,12 +21814,12 @@
     <col min="62" max="62" width="20.42578125" bestFit="1" customWidth="1"/>
     <col min="63" max="63" width="19.42578125" bestFit="1" customWidth="1"/>
     <col min="64" max="64" width="25.85546875" bestFit="1" customWidth="1"/>
-    <col min="65" max="65" width="12.7109375" customWidth="1"/>
-    <col min="66" max="66" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="11.28515625" customWidth="1"/>
+    <col min="66" max="66" width="24.140625" bestFit="1" customWidth="1"/>
     <col min="67" max="67" width="11" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="70" max="70" width="16" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="27.140625" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="11.85546875" customWidth="1"/>
+    <col min="70" max="70" width="22.5703125" bestFit="1" customWidth="1"/>
     <col min="71" max="72" width="18" bestFit="1" customWidth="1"/>
     <col min="73" max="73" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="74" max="74" width="11" bestFit="1" customWidth="1"/>
@@ -21863,17 +22061,17 @@
       <c r="BF16" s="13">
         <v>0.22500000000000001</v>
       </c>
-      <c r="BL16" s="21" t="s">
+      <c r="BL16" s="22" t="s">
         <v>188</v>
       </c>
-      <c r="BN16" s="21" t="s">
+      <c r="BN16" s="22" t="s">
         <v>189</v>
       </c>
-      <c r="BP16" s="21" t="s">
+      <c r="BP16" s="22" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="17" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>34</v>
       </c>
@@ -21946,17 +22144,17 @@
       <c r="BF17" s="13">
         <v>7.1999999999999995E-2</v>
       </c>
-      <c r="BL17" s="22">
+      <c r="BL17" s="23">
         <v>553200000</v>
       </c>
-      <c r="BN17" s="22">
+      <c r="BN17" s="23">
         <v>179800000</v>
       </c>
       <c r="BP17" s="6">
         <v>-373400000</v>
       </c>
     </row>
-    <row r="18" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>55</v>
       </c>
@@ -22030,7 +22228,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>75</v>
       </c>
@@ -22050,7 +22248,7 @@
         <f t="shared" si="0"/>
         <v>-55700000</v>
       </c>
-      <c r="O19" s="23" t="s">
+      <c r="O19" s="24" t="s">
         <v>164</v>
       </c>
       <c r="P19" s="6">
@@ -22098,7 +22296,7 @@
         <v>0.17408231368186874</v>
       </c>
     </row>
-    <row r="20" spans="1:68" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:70" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>93</v>
       </c>
@@ -22152,17 +22350,17 @@
       <c r="BC20" s="13">
         <v>0.22525027808676307</v>
       </c>
-      <c r="BL20" s="21" t="s">
+      <c r="BL20" s="22" t="s">
         <v>191</v>
       </c>
-      <c r="BN20" s="21" t="s">
+      <c r="BN20" s="22" t="s">
         <v>192</v>
       </c>
-      <c r="BP20" s="21" t="s">
+      <c r="BP20" s="22" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="21" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>109</v>
       </c>
@@ -22206,14 +22404,14 @@
       <c r="BL21" s="13">
         <v>0.3866594360086768</v>
       </c>
-      <c r="BN21" s="24">
+      <c r="BN21" s="25">
         <v>0.36243673174258856</v>
       </c>
-      <c r="BP21" s="24">
+      <c r="BP21" s="25">
         <v>0.25090383224873464</v>
       </c>
     </row>
-    <row r="22" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:70" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
         <v>164</v>
       </c>
@@ -22255,7 +22453,7 @@
         <v>7.5083426028921027E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:70" x14ac:dyDescent="0.25">
       <c r="AK23" s="2" t="s">
         <v>30</v>
       </c>
@@ -22278,7 +22476,7 @@
         <v>7.2302558398220251E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:70" ht="15.75" x14ac:dyDescent="0.25">
       <c r="AK24" s="2" t="s">
         <v>152</v>
       </c>
@@ -22300,8 +22498,18 @@
       <c r="BC24" s="13">
         <v>7.2302558398220251E-2</v>
       </c>
+      <c r="BL24" s="22" t="s">
+        <v>196</v>
+      </c>
+      <c r="BN24" s="22" t="s">
+        <v>197</v>
+      </c>
+      <c r="BP24" s="22" t="s">
+        <v>198</v>
+      </c>
+      <c r="BR24" s="26"/>
     </row>
-    <row r="25" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:70" x14ac:dyDescent="0.25">
       <c r="AK25" s="2" t="s">
         <v>78</v>
       </c>
@@ -22325,8 +22533,17 @@
       </c>
       <c r="BH25" s="2"/>
       <c r="BI25" s="6"/>
+      <c r="BL25" s="16">
+        <v>0.6875</v>
+      </c>
+      <c r="BN25" s="16">
+        <v>0.1875</v>
+      </c>
+      <c r="BP25" s="16">
+        <v>6.25E-2</v>
+      </c>
     </row>
-    <row r="26" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:70" x14ac:dyDescent="0.25">
       <c r="AK26" s="2" t="s">
         <v>64</v>
       </c>
@@ -22349,7 +22566,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:70" x14ac:dyDescent="0.25">
       <c r="AK27" s="2" t="s">
         <v>90</v>
       </c>
@@ -22363,7 +22580,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:70" ht="15.75" x14ac:dyDescent="0.25">
       <c r="AK28" s="2" t="s">
         <v>97</v>
       </c>
@@ -22376,8 +22593,19 @@
       <c r="AO28" s="2">
         <v>1</v>
       </c>
+      <c r="BL28" s="27" t="s">
+        <v>194</v>
+      </c>
+      <c r="BM28" s="21"/>
+      <c r="BN28" s="27" t="s">
+        <v>195</v>
+      </c>
+      <c r="BO28" s="21"/>
+      <c r="BP28" s="27" t="s">
+        <v>202</v>
+      </c>
     </row>
-    <row r="29" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:70" x14ac:dyDescent="0.25">
       <c r="AK29" s="9" t="s">
         <v>164</v>
       </c>
@@ -22390,8 +22618,19 @@
       <c r="AO29" s="2">
         <v>1</v>
       </c>
+      <c r="BL29" s="2">
+        <v>3</v>
+      </c>
+      <c r="BM29" s="2"/>
+      <c r="BN29" s="2">
+        <v>2</v>
+      </c>
+      <c r="BO29" s="2"/>
+      <c r="BP29" s="2">
+        <v>13</v>
+      </c>
     </row>
-    <row r="30" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:70" x14ac:dyDescent="0.25">
       <c r="AN30" s="2" t="s">
         <v>97</v>
       </c>
@@ -22399,7 +22638,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:70" x14ac:dyDescent="0.25">
       <c r="AN31" s="2" t="s">
         <v>98</v>
       </c>
@@ -22407,23 +22646,41 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:70" ht="15.75" x14ac:dyDescent="0.25">
       <c r="AN32" s="2" t="s">
         <v>97</v>
       </c>
       <c r="AO32" s="2">
         <v>1</v>
       </c>
+      <c r="BL32" s="27" t="s">
+        <v>200</v>
+      </c>
+      <c r="BN32" s="27" t="s">
+        <v>199</v>
+      </c>
+      <c r="BP32" s="27" t="s">
+        <v>201</v>
+      </c>
     </row>
-    <row r="33" spans="40:41" x14ac:dyDescent="0.25">
+    <row r="33" spans="40:68" x14ac:dyDescent="0.25">
       <c r="AN33" s="2" t="s">
         <v>14</v>
       </c>
       <c r="AO33" s="2">
         <v>1</v>
       </c>
+      <c r="BL33" s="13">
+        <v>0.70199999999999996</v>
+      </c>
+      <c r="BN33" s="13">
+        <v>0.22500000000000001</v>
+      </c>
+      <c r="BP33" s="13">
+        <v>7.1999999999999995E-2</v>
+      </c>
     </row>
-    <row r="34" spans="40:41" x14ac:dyDescent="0.25">
+    <row r="34" spans="40:68" x14ac:dyDescent="0.25">
       <c r="AN34" s="2" t="s">
         <v>13</v>
       </c>
@@ -22431,7 +22688,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="40:41" x14ac:dyDescent="0.25">
+    <row r="35" spans="40:68" x14ac:dyDescent="0.25">
       <c r="AN35" s="2" t="s">
         <v>139</v>
       </c>
@@ -22439,7 +22696,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="40:41" x14ac:dyDescent="0.25">
+    <row r="36" spans="40:68" x14ac:dyDescent="0.25">
       <c r="AN36" s="2" t="s">
         <v>152</v>
       </c>
@@ -22447,7 +22704,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="40:41" x14ac:dyDescent="0.25">
+    <row r="37" spans="40:68" x14ac:dyDescent="0.25">
       <c r="AN37" s="2" t="s">
         <v>22</v>
       </c>
@@ -22455,7 +22712,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="40:41" x14ac:dyDescent="0.25">
+    <row r="38" spans="40:68" x14ac:dyDescent="0.25">
       <c r="AN38" s="2" t="s">
         <v>90</v>
       </c>
@@ -22463,7 +22720,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="40:41" x14ac:dyDescent="0.25">
+    <row r="39" spans="40:68" x14ac:dyDescent="0.25">
       <c r="AN39" s="2" t="s">
         <v>45</v>
       </c>
@@ -22471,7 +22728,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="40:41" x14ac:dyDescent="0.25">
+    <row r="40" spans="40:68" x14ac:dyDescent="0.25">
       <c r="AN40" s="2" t="s">
         <v>44</v>
       </c>
@@ -22479,7 +22736,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="40:41" x14ac:dyDescent="0.25">
+    <row r="41" spans="40:68" x14ac:dyDescent="0.25">
       <c r="AN41" s="2" t="s">
         <v>38</v>
       </c>
@@ -22487,7 +22744,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="40:41" x14ac:dyDescent="0.25">
+    <row r="42" spans="40:68" x14ac:dyDescent="0.25">
       <c r="AN42" s="2" t="s">
         <v>30</v>
       </c>
@@ -22495,7 +22752,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="40:41" x14ac:dyDescent="0.25">
+    <row r="43" spans="40:68" x14ac:dyDescent="0.25">
       <c r="AN43" s="2" t="s">
         <v>102</v>
       </c>
@@ -22503,7 +22760,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="40:41" x14ac:dyDescent="0.25">
+    <row r="44" spans="40:68" x14ac:dyDescent="0.25">
       <c r="AN44" s="2" t="s">
         <v>90</v>
       </c>
@@ -22511,7 +22768,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="40:41" x14ac:dyDescent="0.25">
+    <row r="45" spans="40:68" x14ac:dyDescent="0.25">
       <c r="AN45" s="2" t="s">
         <v>134</v>
       </c>
@@ -22519,7 +22776,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="40:41" x14ac:dyDescent="0.25">
+    <row r="46" spans="40:68" x14ac:dyDescent="0.25">
       <c r="AN46" s="2" t="s">
         <v>132</v>
       </c>
@@ -22527,7 +22784,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="40:41" x14ac:dyDescent="0.25">
+    <row r="47" spans="40:68" x14ac:dyDescent="0.25">
       <c r="AN47" s="2" t="s">
         <v>164</v>
       </c>

</xml_diff>

<commit_message>
46. Começando a 6ª análise
Começando a sexta análise.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{738A07C3-70A6-4C8C-9AF5-B422EFC3A549}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E674E499-9D7C-44D5-B219-297EDF0556CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -770,7 +770,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -828,14 +828,13 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -847,6 +846,60 @@
     <cellStyle name="Porcentagem" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="95">
+    <dxf>
+      <numFmt numFmtId="165" formatCode="0.0%"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="center"/>
     </dxf>
@@ -1077,60 +1130,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="0.0%"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" indent="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -10798,11 +10797,11 @@
           </a:r>
           <a:r>
             <a:rPr lang="pt-BR" sz="1200" b="1"/>
-            <a:t> O</a:t>
+            <a:t> Quais características definiram a estratégia do Tottenham</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0"/>
-            <a:t> que todas as evidências nos dizem sobre a estratégia do Tottenham Hotspur no mercado de transferências</a:t>
+            <a:t> Hotspur no mercado de transferências entre as temporadas 2019/20 e 2024/25</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="pt-BR" sz="1200" b="1"/>
@@ -15636,6 +15635,471 @@
             <a:t>Veredito:</a:t>
           </a:r>
           <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>61</xdr:col>
+      <xdr:colOff>1218038</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>135466</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="12625956" cy="2941446"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="46" name="CaixaDeTexto 45">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{05105D5E-6C37-40B9-AE87-DE1276453FB9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="67492988" y="7041091"/>
+          <a:ext cx="12625956" cy="2941446"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="ctr">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>A análise financeira das movimentações no mercado de transferências de atletas realizadas pelo Tottenham Hotspur entre as temporadas 2019/20 e 2024/25 sugere que</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>o clube tenha adotado uma postura </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>incisiva</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t> no que diz respeito à contratações — uma vez que </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>£553.2 milhões </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>foram investidos em jogadores durante o período. Esse</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t> valor contrasta-se significativamente com os </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>£179.8 milhões </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>provenientes das saídas de atletas, onde 52,8% deste montante representava apenas um atleta: Harry Kane.</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>Entre as posições, os atacantes se destacam. Suas saídas renderam </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>£126.3 milhões </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>aos cofres do clube,</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> valor superior ao dobro da soma entre os meio-campistas e </a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>defensores. Um peso ainda maior vai para Harry Kane </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1100" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>— </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>sozinho, o inglês gerou </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>£95 milhões</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>, quantia que se sobrepõe à</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> adição dos valores de todos os jogadores</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>restantes e que representa </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>52,8</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>% do retorno financeiro obtido ao longo de seis temporadas</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>. O</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> impacto da categoria torna-se ainda mais visível quando Steve Bergwijn,</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>seu companheiro, entra na equação: a saída do holandês garantiu </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>£31.3 milhões</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> para a equipe, superando</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> individualmente o preço de ambos os atletas responsáveis pela</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>administração do meio-campo, sendo eles Christian Eriksen e Pierre-Emile Højbjerg.</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Em resumo, os </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>atacantes</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> geraram maior retorno financeiro ao Tottenham Hotspur. Baseando-se na base de dados atual, não é possível identificar a razão por trás da</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>valorização dos mesmos.</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
         </a:p>
       </xdr:txBody>
     </xdr:sp>
@@ -18026,1255 +18490,6 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FB686887-B509-4E7E-B605-6A13972A6E0B}" name="Tabela dinâmica5" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Origem das Contratações" colHeaderCaption="Contagem de Jogadores">
-  <location ref="AN14:AO47" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="9">
-    <pivotField axis="axisCol" showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item h="1" x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" dataField="1" showAll="0">
-      <items count="15">
-        <item x="6"/>
-        <item x="4"/>
-        <item x="9"/>
-        <item x="11"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="12"/>
-        <item x="5"/>
-        <item x="10"/>
-        <item x="13"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="21">
-        <item x="12"/>
-        <item x="9"/>
-        <item x="7"/>
-        <item x="15"/>
-        <item x="5"/>
-        <item x="17"/>
-        <item x="11"/>
-        <item x="10"/>
-        <item x="2"/>
-        <item x="8"/>
-        <item x="18"/>
-        <item x="13"/>
-        <item x="0"/>
-        <item x="16"/>
-        <item x="19"/>
-        <item x="1"/>
-        <item x="4"/>
-        <item x="3"/>
-        <item x="14"/>
-        <item x="6"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="2">
-    <field x="4"/>
-    <field x="3"/>
-  </rowFields>
-  <rowItems count="32">
-    <i>
-      <x v="2"/>
-    </i>
-    <i r="1">
-      <x/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i r="1">
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i r="1">
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i r="1">
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i r="1">
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i r="1">
-      <x v="12"/>
-    </i>
-    <i r="1">
-      <x v="13"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i r="1">
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="11"/>
-    </i>
-    <i r="1">
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="12"/>
-    </i>
-    <i r="1">
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="13"/>
-    </i>
-    <i r="1">
-      <x v="11"/>
-    </i>
-    <i>
-      <x v="15"/>
-    </i>
-    <i r="1">
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="16"/>
-    </i>
-    <i r="1">
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="17"/>
-    </i>
-    <i r="1">
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="18"/>
-    </i>
-    <i r="1">
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="19"/>
-    </i>
-    <i r="1">
-      <x v="9"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="0"/>
-  </colFields>
-  <colItems count="1">
-    <i>
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Clubes" fld="3" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="46">
-    <format dxfId="45">
-      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="44">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="43">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="42">
-      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
-    </format>
-    <format dxfId="41">
-      <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
-    </format>
-    <format dxfId="40">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="4" count="15">
-            <x v="2"/>
-            <x v="5"/>
-            <x v="6"/>
-            <x v="7"/>
-            <x v="8"/>
-            <x v="9"/>
-            <x v="10"/>
-            <x v="11"/>
-            <x v="12"/>
-            <x v="13"/>
-            <x v="15"/>
-            <x v="16"/>
-            <x v="17"/>
-            <x v="18"/>
-            <x v="19"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="39">
-      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="38">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="0"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="37">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="8"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="5"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="36">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="10"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="6"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="35">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="2"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="7"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="34">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="3"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="8"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="33">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="2">
-            <x v="12"/>
-            <x v="13"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="9"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="32">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="8"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="10"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="31">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="8"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="11"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="30">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="6"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="12"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="29">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="11"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="13"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="28">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="7"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="15"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="27">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="5"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="16"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="26">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="4"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="17"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="25">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="7"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="18"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="24">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="9"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="19"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="23">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="0" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="22">
-      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="21">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="20">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="19">
-      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
-    </format>
-    <format dxfId="18">
-      <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
-    </format>
-    <format dxfId="17">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="4" count="15">
-            <x v="2"/>
-            <x v="5"/>
-            <x v="6"/>
-            <x v="7"/>
-            <x v="8"/>
-            <x v="9"/>
-            <x v="10"/>
-            <x v="11"/>
-            <x v="12"/>
-            <x v="13"/>
-            <x v="15"/>
-            <x v="16"/>
-            <x v="17"/>
-            <x v="18"/>
-            <x v="19"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="16">
-      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="15">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="0"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="14">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="8"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="5"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="13">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="10"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="6"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="12">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="2"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="7"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="11">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="3"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="8"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="10">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="2">
-            <x v="12"/>
-            <x v="13"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="9"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="9">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="8"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="10"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="8">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="8"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="11"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="7">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="6"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="12"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="6">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="11"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="13"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="5">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="7"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="15"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="4">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="5"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="16"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="3">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="4"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="17"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="2">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="7"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="18"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="1">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="9"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="19"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="0">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="0" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-  </formats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{996EC5F2-74EB-477F-A9D9-AF44A2544855}" name="Tabela dinâmica3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Faixa Etária" colHeaderCaption="Tipo de Movimentação">
-  <location ref="Y14:Z20" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="10">
-    <pivotField showAll="0"/>
-    <pivotField axis="axisCol" showAll="0">
-      <items count="3">
-        <item h="1" x="1"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField axis="axisRow" dataField="1" showAll="0" sortType="ascending">
-      <items count="9">
-        <item m="1" x="5"/>
-        <item m="1" x="4"/>
-        <item m="1" x="7"/>
-        <item m="1" x="6"/>
-        <item x="3"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-      <autoSortScope>
-        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
-          <references count="2">
-            <reference field="4294967294" count="1" selected="0">
-              <x v="0"/>
-            </reference>
-            <reference field="1" count="1" selected="0">
-              <x v="1"/>
-            </reference>
-          </references>
-        </pivotArea>
-      </autoSortScope>
-    </pivotField>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="8"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="1"/>
-  </colFields>
-  <colItems count="1">
-    <i>
-      <x v="1"/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Contagem de Jogadores" fld="8" subtotal="count" baseField="8" baseItem="0"/>
-  </dataFields>
-  <formats count="9">
-    <format dxfId="54">
-      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
-        <references count="1">
-          <reference field="8" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="53">
-      <pivotArea field="8" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
-    </format>
-    <format dxfId="52">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="8" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="51">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
-    </format>
-    <format dxfId="50">
-      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="49">
-      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="48">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="1" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="47">
-      <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
-    </format>
-    <format dxfId="46">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="1">
-    <chartFormat chart="2" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{904CEA3A-CD0A-459C-A420-1FB249800D4C}" name="Tabela dinâmica4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Nacionalidades" colHeaderCaption="Contagem de Jogadores">
-  <location ref="AK14:AL29" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="9">
-    <pivotField axis="axisCol" showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item h="1" x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" dataField="1" showAll="0" sortType="ascending">
-      <items count="15">
-        <item x="6"/>
-        <item x="4"/>
-        <item x="9"/>
-        <item x="11"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="12"/>
-        <item x="5"/>
-        <item x="10"/>
-        <item x="13"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item t="default"/>
-      </items>
-      <autoSortScope>
-        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
-          <references count="2">
-            <reference field="4294967294" count="1" selected="0">
-              <x v="0"/>
-            </reference>
-            <reference field="0" count="1" selected="0">
-              <x v="0"/>
-            </reference>
-          </references>
-        </pivotArea>
-      </autoSortScope>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="21">
-        <item x="12"/>
-        <item x="9"/>
-        <item x="7"/>
-        <item x="15"/>
-        <item x="5"/>
-        <item x="17"/>
-        <item x="11"/>
-        <item x="10"/>
-        <item x="2"/>
-        <item x="8"/>
-        <item x="18"/>
-        <item x="13"/>
-        <item x="0"/>
-        <item x="16"/>
-        <item x="19"/>
-        <item x="1"/>
-        <item x="4"/>
-        <item x="3"/>
-        <item x="14"/>
-        <item x="6"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="3"/>
-  </rowFields>
-  <rowItems count="14">
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="13"/>
-    </i>
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="11"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="12"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="0"/>
-  </colFields>
-  <colItems count="1">
-    <i>
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Contagem de Nacionalidades" fld="3" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="7">
-    <format dxfId="61">
-      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
-        <references count="1">
-          <reference field="3" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="60">
-      <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
-    </format>
-    <format dxfId="59">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="3" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="58">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
-    </format>
-    <format dxfId="57">
-      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="56">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="0" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="55">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="1">
-    <chartFormat chart="1" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
-  <location ref="O14:P19" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="10">
-    <pivotField showAll="0"/>
-    <pivotField axis="axisCol" showAll="0">
-      <items count="3">
-        <item h="1" x="1"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0" sortType="descending">
-      <items count="4">
-        <item x="1"/>
-        <item x="2"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-      <autoSortScope>
-        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
-          <references count="2">
-            <reference field="4294967294" count="1" selected="0">
-              <x v="0"/>
-            </reference>
-            <reference field="1" count="1" selected="0">
-              <x v="1"/>
-            </reference>
-          </references>
-        </pivotArea>
-      </autoSortScope>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="3"/>
-  </rowFields>
-  <rowItems count="4">
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="1"/>
-  </colFields>
-  <colItems count="1">
-    <i>
-      <x v="1"/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Soma do Valor das Transferências" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
-  </dataFields>
-  <formats count="9">
-    <format dxfId="70">
-      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="69">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="68">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="67">
-      <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
-    </format>
-    <format dxfId="66">
-      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="65">
-      <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
-    </format>
-    <format dxfId="64">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="3" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="63">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="1" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="62">
-      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="1">
-    <chartFormat chart="1" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6" rowHeaderCaption="Temporadas" colHeaderCaption="">
-  <location ref="A14:D22" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="10">
-    <pivotField axis="axisRow" showAll="0">
-      <items count="7">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisCol" showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="7">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="1"/>
-  </colFields>
-  <colItems count="3">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Somas de Entradas e Saídas" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
-  </dataFields>
-  <formats count="6">
-    <format dxfId="76">
-      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
-        <references count="1">
-          <reference field="0" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="75">
-      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
-    </format>
-    <format dxfId="74">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="0" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="73">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="1" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="72">
-      <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="71">
-      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="2">
-    <chartFormat chart="0" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="1" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4F5027D2-D537-4505-8DBC-54A417F72129}" name="Tabela dinâmica8" cacheId="0" dataPosition="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10" rowHeaderCaption="Posições e Jogadores" colHeaderCaption="Tipo de Movimentação">
   <location ref="BA14:BC26" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
   <pivotFields count="10">
@@ -19404,7 +18619,7 @@
     <dataField name="Porcentagem (%) do Total" fld="6" showDataAs="percentOfTotal" baseField="0" baseItem="0" numFmtId="10"/>
   </dataFields>
   <formats count="18">
-    <format dxfId="94">
+    <format dxfId="17">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -19413,7 +18628,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="93">
+    <format dxfId="16">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -19426,7 +18641,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="92">
+    <format dxfId="15">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -19435,7 +18650,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="91">
+    <format dxfId="14">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -19448,7 +18663,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="90">
+    <format dxfId="13">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -19457,7 +18672,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="89">
+    <format dxfId="12">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -19470,26 +18685,26 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="88">
+    <format dxfId="11">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="87">
+    <format dxfId="10">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="86">
+    <format dxfId="9">
       <pivotArea field="-2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="1"/>
     </format>
-    <format dxfId="85">
+    <format dxfId="8">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="84">
+    <format dxfId="7">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="83">
+    <format dxfId="6">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -19502,7 +18717,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="82">
+    <format dxfId="5">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -19515,7 +18730,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="81">
+    <format dxfId="4">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -19528,14 +18743,14 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="80">
+    <format dxfId="3">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="79">
+    <format dxfId="2">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -19546,10 +18761,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="78">
+    <format dxfId="1">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="77">
+    <format dxfId="0">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
@@ -19928,6 +19143,1255 @@
 </pivotTableDefinition>
 </file>
 
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FB686887-B509-4E7E-B605-6A13972A6E0B}" name="Tabela dinâmica5" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Origem das Contratações" colHeaderCaption="Contagem de Jogadores">
+  <location ref="AN14:AO47" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="9">
+    <pivotField axis="axisCol" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item h="1" x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" dataField="1" showAll="0">
+      <items count="15">
+        <item x="6"/>
+        <item x="4"/>
+        <item x="9"/>
+        <item x="11"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="12"/>
+        <item x="5"/>
+        <item x="10"/>
+        <item x="13"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="21">
+        <item x="12"/>
+        <item x="9"/>
+        <item x="7"/>
+        <item x="15"/>
+        <item x="5"/>
+        <item x="17"/>
+        <item x="11"/>
+        <item x="10"/>
+        <item x="2"/>
+        <item x="8"/>
+        <item x="18"/>
+        <item x="13"/>
+        <item x="0"/>
+        <item x="16"/>
+        <item x="19"/>
+        <item x="1"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item x="14"/>
+        <item x="6"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="2">
+    <field x="4"/>
+    <field x="3"/>
+  </rowFields>
+  <rowItems count="32">
+    <i>
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i r="1">
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i r="1">
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i r="1">
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i r="1">
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i r="1">
+      <x v="12"/>
+    </i>
+    <i r="1">
+      <x v="13"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i r="1">
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i r="1">
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i r="1">
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i r="1">
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="15"/>
+    </i>
+    <i r="1">
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="16"/>
+    </i>
+    <i r="1">
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="17"/>
+    </i>
+    <i r="1">
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="18"/>
+    </i>
+    <i r="1">
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="19"/>
+    </i>
+    <i r="1">
+      <x v="9"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="0"/>
+  </colFields>
+  <colItems count="1">
+    <i>
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Clubes" fld="3" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="46">
+    <format dxfId="63">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="62">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="61">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="60">
+      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
+    </format>
+    <format dxfId="59">
+      <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="58">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="4" count="15">
+            <x v="2"/>
+            <x v="5"/>
+            <x v="6"/>
+            <x v="7"/>
+            <x v="8"/>
+            <x v="9"/>
+            <x v="10"/>
+            <x v="11"/>
+            <x v="12"/>
+            <x v="13"/>
+            <x v="15"/>
+            <x v="16"/>
+            <x v="17"/>
+            <x v="18"/>
+            <x v="19"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="57">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="56">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="0"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="55">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="8"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="5"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="54">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="10"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="6"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="53">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="2"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="7"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="52">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="3"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="8"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="51">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="2">
+            <x v="12"/>
+            <x v="13"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="9"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="50">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="8"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="10"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="49">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="8"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="11"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="48">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="6"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="12"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="47">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="11"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="13"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="46">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="7"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="15"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="45">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="5"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="16"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="44">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="4"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="17"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="43">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="7"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="18"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="42">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="9"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="19"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="41">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="40">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="39">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="38">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="37">
+      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
+    </format>
+    <format dxfId="36">
+      <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="35">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="4" count="15">
+            <x v="2"/>
+            <x v="5"/>
+            <x v="6"/>
+            <x v="7"/>
+            <x v="8"/>
+            <x v="9"/>
+            <x v="10"/>
+            <x v="11"/>
+            <x v="12"/>
+            <x v="13"/>
+            <x v="15"/>
+            <x v="16"/>
+            <x v="17"/>
+            <x v="18"/>
+            <x v="19"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="34">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="33">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="0"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="32">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="8"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="5"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="31">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="10"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="6"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="30">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="2"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="7"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="29">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="3"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="8"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="28">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="2">
+            <x v="12"/>
+            <x v="13"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="9"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="27">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="8"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="10"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="26">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="8"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="11"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="25">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="6"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="12"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="24">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="11"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="13"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="23">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="7"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="15"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="22">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="5"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="16"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="21">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="4"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="17"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="20">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="7"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="18"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="19">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="9"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="19"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="18">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{996EC5F2-74EB-477F-A9D9-AF44A2544855}" name="Tabela dinâmica3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Faixa Etária" colHeaderCaption="Tipo de Movimentação">
+  <location ref="Y14:Z20" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="10">
+    <pivotField showAll="0"/>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="3">
+        <item h="1" x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField axis="axisRow" dataField="1" showAll="0" sortType="ascending">
+      <items count="9">
+        <item m="1" x="5"/>
+        <item m="1" x="4"/>
+        <item m="1" x="7"/>
+        <item m="1" x="6"/>
+        <item x="3"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="2">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+            <reference field="1" count="1" selected="0">
+              <x v="1"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="8"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="1"/>
+  </colFields>
+  <colItems count="1">
+    <i>
+      <x v="1"/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Contagem de Jogadores" fld="8" subtotal="count" baseField="8" baseItem="0"/>
+  </dataFields>
+  <formats count="9">
+    <format dxfId="72">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="8" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="71">
+      <pivotArea field="8" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="70">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="8" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="69">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+    <format dxfId="68">
+      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="67">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="66">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="1" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="65">
+      <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
+    </format>
+    <format dxfId="64">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="1">
+    <chartFormat chart="2" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{904CEA3A-CD0A-459C-A420-1FB249800D4C}" name="Tabela dinâmica4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Nacionalidades" colHeaderCaption="Contagem de Jogadores">
+  <location ref="AK14:AL29" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="9">
+    <pivotField axis="axisCol" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item h="1" x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" dataField="1" showAll="0" sortType="ascending">
+      <items count="15">
+        <item x="6"/>
+        <item x="4"/>
+        <item x="9"/>
+        <item x="11"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="12"/>
+        <item x="5"/>
+        <item x="10"/>
+        <item x="13"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="2">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+            <reference field="0" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="21">
+        <item x="12"/>
+        <item x="9"/>
+        <item x="7"/>
+        <item x="15"/>
+        <item x="5"/>
+        <item x="17"/>
+        <item x="11"/>
+        <item x="10"/>
+        <item x="2"/>
+        <item x="8"/>
+        <item x="18"/>
+        <item x="13"/>
+        <item x="0"/>
+        <item x="16"/>
+        <item x="19"/>
+        <item x="1"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item x="14"/>
+        <item x="6"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="3"/>
+  </rowFields>
+  <rowItems count="14">
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="0"/>
+  </colFields>
+  <colItems count="1">
+    <i>
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Contagem de Nacionalidades" fld="3" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="7">
+    <format dxfId="79">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="3" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="78">
+      <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="77">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="3" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="76">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+    <format dxfId="75">
+      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="74">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="73">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="1">
+    <chartFormat chart="1" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
+  <location ref="O14:P19" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="10">
+    <pivotField showAll="0"/>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="3">
+        <item h="1" x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0" sortType="descending">
+      <items count="4">
+        <item x="1"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="2">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+            <reference field="1" count="1" selected="0">
+              <x v="1"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="3"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="1"/>
+  </colFields>
+  <colItems count="1">
+    <i>
+      <x v="1"/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Soma do Valor das Transferências" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
+  </dataFields>
+  <formats count="9">
+    <format dxfId="88">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="87">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="86">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="85">
+      <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
+    </format>
+    <format dxfId="84">
+      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="83">
+      <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="82">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="3" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="81">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="1" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="80">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="1">
+    <chartFormat chart="1" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6" rowHeaderCaption="Temporadas" colHeaderCaption="">
+  <location ref="A14:D22" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="10">
+    <pivotField axis="axisRow" showAll="0">
+      <items count="7">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="7">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="1"/>
+  </colFields>
+  <colItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Somas de Entradas e Saídas" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
+  </dataFields>
+  <formats count="6">
+    <format dxfId="94">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="93">
+      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="92">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="91">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="1" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="90">
+      <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="89">
+      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="2">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -22248,7 +22712,7 @@
         <f t="shared" si="0"/>
         <v>-55700000</v>
       </c>
-      <c r="O19" s="24" t="s">
+      <c r="O19" t="s">
         <v>164</v>
       </c>
       <c r="P19" s="6">
@@ -22404,10 +22868,10 @@
       <c r="BL21" s="13">
         <v>0.3866594360086768</v>
       </c>
-      <c r="BN21" s="25">
+      <c r="BN21" s="24">
         <v>0.36243673174258856</v>
       </c>
-      <c r="BP21" s="25">
+      <c r="BP21" s="24">
         <v>0.25090383224873464</v>
       </c>
     </row>
@@ -22507,7 +22971,7 @@
       <c r="BP24" s="22" t="s">
         <v>198</v>
       </c>
-      <c r="BR24" s="26"/>
+      <c r="BR24" s="25"/>
     </row>
     <row r="25" spans="1:70" x14ac:dyDescent="0.25">
       <c r="AK25" s="2" t="s">
@@ -22593,15 +23057,15 @@
       <c r="AO28" s="2">
         <v>1</v>
       </c>
-      <c r="BL28" s="27" t="s">
+      <c r="BL28" s="26" t="s">
         <v>194</v>
       </c>
       <c r="BM28" s="21"/>
-      <c r="BN28" s="27" t="s">
+      <c r="BN28" s="26" t="s">
         <v>195</v>
       </c>
       <c r="BO28" s="21"/>
-      <c r="BP28" s="27" t="s">
+      <c r="BP28" s="26" t="s">
         <v>202</v>
       </c>
     </row>
@@ -22653,13 +23117,13 @@
       <c r="AO32" s="2">
         <v>1</v>
       </c>
-      <c r="BL32" s="27" t="s">
+      <c r="BL32" s="26" t="s">
         <v>200</v>
       </c>
-      <c r="BN32" s="27" t="s">
+      <c r="BN32" s="26" t="s">
         <v>199</v>
       </c>
-      <c r="BP32" s="27" t="s">
+      <c r="BP32" s="26" t="s">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
47. Andamento da 6ª análise
Andamento da sexta análise.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E674E499-9D7C-44D5-B219-297EDF0556CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E6E42AA-B77E-4A94-95E7-BAF5C8A34A75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15735,6 +15735,18 @@
           <a:br>
             <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
           </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>Os fatos apresentados reforçam o indicativo de que a equipe assumiu uma identidade </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0"/>
+            <a:t>compradora</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>.</a:t>
+          </a:r>
           <a:br>
             <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
           </a:br>

</xml_diff>

<commit_message>
48. Andamento da 6ª análise
Andamento da sexta análise.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E6E42AA-B77E-4A94-95E7-BAF5C8A34A75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8076D85-2031-4329-97B0-2DDCB4189AF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -847,6 +847,24 @@
   </cellStyles>
   <dxfs count="95">
     <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="165" formatCode="0.0%"/>
     </dxf>
     <dxf>
@@ -1088,24 +1106,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="general"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
     </dxf>
     <dxf>
       <alignment horizontal="center"/>
@@ -15643,11 +15643,11 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>61</xdr:col>
-      <xdr:colOff>1218038</xdr:colOff>
+      <xdr:colOff>1268685</xdr:colOff>
       <xdr:row>36</xdr:row>
-      <xdr:rowOff>135466</xdr:rowOff>
+      <xdr:rowOff>136919</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="12625956" cy="2941446"/>
+    <xdr:ext cx="12584984" cy="1626471"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="46" name="CaixaDeTexto 45">
@@ -15661,8 +15661,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="67492988" y="7041091"/>
-          <a:ext cx="12625956" cy="2941446"/>
+          <a:off x="67417826" y="6973091"/>
+          <a:ext cx="12584984" cy="1626471"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -15744,22 +15744,7 @@
             <a:t>compradora</a:t>
           </a:r>
           <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
-            <a:t>.</a:t>
-          </a:r>
-          <a:br>
-            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
-          </a:br>
-          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
-        </a:p>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
-            <a:t>Entre as posições, os atacantes se destacam. Suas saídas renderam </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="1">
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="tx1"/>
               </a:solidFill>
@@ -15768,10 +15753,10 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>£126.3 milhões </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1400">
+            <a:t>, principalmente quando alinhados ao déficit de </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="tx1"/>
               </a:solidFill>
@@ -15780,22 +15765,10 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>aos cofres do clube,</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1400" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t> valor superior ao dobro da soma entre os meio-campistas e </a:t>
+            <a:t>-£373.4 milhões</a:t>
           </a:r>
           <a:br>
-            <a:rPr lang="pt-BR" sz="1400" baseline="0">
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="tx1"/>
               </a:solidFill>
@@ -15806,30 +15779,6 @@
             </a:rPr>
           </a:br>
           <a:r>
-            <a:rPr lang="pt-BR" sz="1400" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>defensores. Um peso ainda maior vai para Harry Kane </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1100" b="0" i="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>— </a:t>
-          </a:r>
-          <a:r>
             <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="tx1"/>
@@ -15839,32 +15788,15 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>sozinho, o inglês gerou </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="1">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>£95 milhões</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>, quantia que se sobrepõe à</a:t>
-          </a:r>
+            <a:t>registrado durante o período.</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+          </a:br>
+          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
               <a:solidFill>
@@ -15875,241 +15807,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t> adição dos valores de todos os jogadores</a:t>
-          </a:r>
-          <a:br>
-            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-          </a:br>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>restantes e que representa </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="1" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>52,8</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>% do retorno financeiro obtido ao longo de seis temporadas</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>. O</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t> impacto da categoria torna-se ainda mais visível quando Steve Bergwijn,</a:t>
-          </a:r>
-          <a:br>
-            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-          </a:br>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>seu companheiro, entra na equação: a saída do holandês garantiu </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="1">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>£31.3 milhões</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t> para a equipe, superando</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t> individualmente o preço de ambos os atletas responsáveis pela</a:t>
-          </a:r>
-          <a:br>
-            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-          </a:br>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>administração do meio-campo, sendo eles Christian Eriksen e Pierre-Emile Højbjerg.</a:t>
-          </a:r>
-          <a:br>
-            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-          </a:br>
-          <a:br>
-            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-          </a:br>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Em resumo, os </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="1" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>atacantes</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t> geraram maior retorno financeiro ao Tottenham Hotspur. Baseando-se na base de dados atual, não é possível identificar a razão por trás da</a:t>
-          </a:r>
-          <a:br>
-            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-          </a:br>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>valorização dos mesmos.</a:t>
+            <a:t>O investimento do Tottenham Hotspur em atletas</a:t>
           </a:r>
           <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
         </a:p>
@@ -18502,6 +18200,150 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6" rowHeaderCaption="Temporadas" colHeaderCaption="">
+  <location ref="A14:D22" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="10">
+    <pivotField axis="axisRow" showAll="0">
+      <items count="7">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="7">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="1"/>
+  </colFields>
+  <colItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Somas de Entradas e Saídas" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
+  </dataFields>
+  <formats count="6">
+    <format dxfId="5">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="4">
+      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="3">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="2">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="1" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="1">
+      <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="0">
+      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="2">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4F5027D2-D537-4505-8DBC-54A417F72129}" name="Tabela dinâmica8" cacheId="0" dataPosition="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10" rowHeaderCaption="Posições e Jogadores" colHeaderCaption="Tipo de Movimentação">
   <location ref="BA14:BC26" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
   <pivotFields count="10">
@@ -18631,7 +18473,7 @@
     <dataField name="Porcentagem (%) do Total" fld="6" showDataAs="percentOfTotal" baseField="0" baseItem="0" numFmtId="10"/>
   </dataFields>
   <formats count="18">
-    <format dxfId="17">
+    <format dxfId="23">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -18640,7 +18482,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="16">
+    <format dxfId="22">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -18653,7 +18495,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="15">
+    <format dxfId="21">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -18662,7 +18504,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="14">
+    <format dxfId="20">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -18675,7 +18517,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="13">
+    <format dxfId="19">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -18684,7 +18526,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="12">
+    <format dxfId="18">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -18697,26 +18539,26 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="11">
+    <format dxfId="17">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="10">
+    <format dxfId="16">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="9">
+    <format dxfId="15">
       <pivotArea field="-2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="1"/>
     </format>
-    <format dxfId="8">
+    <format dxfId="14">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="7">
+    <format dxfId="13">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="6">
+    <format dxfId="12">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -18729,7 +18571,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="5">
+    <format dxfId="11">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -18742,7 +18584,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="4">
+    <format dxfId="10">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -18755,14 +18597,14 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="3">
+    <format dxfId="9">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="2">
+    <format dxfId="8">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -18773,10 +18615,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="1">
+    <format dxfId="7">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="0">
+    <format dxfId="6">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
@@ -19155,7 +18997,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FB686887-B509-4E7E-B605-6A13972A6E0B}" name="Tabela dinâmica5" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Origem das Contratações" colHeaderCaption="Contagem de Jogadores">
   <location ref="AN14:AO47" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
@@ -19331,22 +19173,22 @@
     <dataField name="Clubes" fld="3" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="46">
-    <format dxfId="63">
+    <format dxfId="69">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="62">
+    <format dxfId="68">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="61">
+    <format dxfId="67">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="60">
+    <format dxfId="66">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="59">
+    <format dxfId="65">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="58">
+    <format dxfId="64">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="15">
@@ -19369,10 +19211,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="57">
+    <format dxfId="63">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="56">
+    <format dxfId="62">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19384,7 +19226,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="55">
+    <format dxfId="61">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19396,7 +19238,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="54">
+    <format dxfId="60">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19408,7 +19250,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="53">
+    <format dxfId="59">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19420,7 +19262,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="52">
+    <format dxfId="58">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19432,7 +19274,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="51">
+    <format dxfId="57">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="2">
@@ -19445,7 +19287,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="50">
+    <format dxfId="56">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19457,7 +19299,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="49">
+    <format dxfId="55">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19469,7 +19311,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="48">
+    <format dxfId="54">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19481,7 +19323,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="47">
+    <format dxfId="53">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19493,7 +19335,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="46">
+    <format dxfId="52">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19505,7 +19347,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="45">
+    <format dxfId="51">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19517,7 +19359,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="44">
+    <format dxfId="50">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19529,7 +19371,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="43">
+    <format dxfId="49">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19541,7 +19383,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="42">
+    <format dxfId="48">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19553,29 +19395,29 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="41">
+    <format dxfId="47">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="40">
+    <format dxfId="46">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="39">
+    <format dxfId="45">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="38">
+    <format dxfId="44">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="37">
+    <format dxfId="43">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="36">
+    <format dxfId="42">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="35">
+    <format dxfId="41">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="15">
@@ -19598,10 +19440,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="34">
+    <format dxfId="40">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="33">
+    <format dxfId="39">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19613,7 +19455,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="32">
+    <format dxfId="38">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19625,7 +19467,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="31">
+    <format dxfId="37">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19637,7 +19479,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="30">
+    <format dxfId="36">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19649,7 +19491,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="29">
+    <format dxfId="35">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19661,7 +19503,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="28">
+    <format dxfId="34">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="2">
@@ -19674,7 +19516,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="27">
+    <format dxfId="33">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19686,7 +19528,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="26">
+    <format dxfId="32">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19698,7 +19540,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="25">
+    <format dxfId="31">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19710,7 +19552,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="24">
+    <format dxfId="30">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19722,7 +19564,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="23">
+    <format dxfId="29">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19734,7 +19576,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="22">
+    <format dxfId="28">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19746,7 +19588,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="21">
+    <format dxfId="27">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19758,7 +19600,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="20">
+    <format dxfId="26">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19770,7 +19612,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="19">
+    <format dxfId="25">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19782,7 +19624,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="18">
+    <format dxfId="24">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
@@ -19802,7 +19644,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{996EC5F2-74EB-477F-A9D9-AF44A2544855}" name="Tabela dinâmica3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Faixa Etária" colHeaderCaption="Tipo de Movimentação">
   <location ref="Y14:Z20" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -19879,43 +19721,43 @@
     <dataField name="Contagem de Jogadores" fld="8" subtotal="count" baseField="8" baseItem="0"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="72">
+    <format dxfId="78">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="71">
+    <format dxfId="77">
       <pivotArea field="8" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="70">
+    <format dxfId="76">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="69">
+    <format dxfId="75">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="68">
+    <format dxfId="74">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="67">
+    <format dxfId="73">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="66">
+    <format dxfId="72">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="65">
+    <format dxfId="71">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="64">
+    <format dxfId="70">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -19942,7 +19784,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{904CEA3A-CD0A-459C-A420-1FB249800D4C}" name="Tabela dinâmica4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Nacionalidades" colHeaderCaption="Contagem de Jogadores">
   <location ref="AK14:AL29" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
@@ -20075,37 +19917,37 @@
     <dataField name="Contagem de Nacionalidades" fld="3" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="7">
-    <format dxfId="79">
+    <format dxfId="85">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="78">
+    <format dxfId="84">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="77">
+    <format dxfId="83">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="76">
+    <format dxfId="82">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="75">
+    <format dxfId="81">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="74">
+    <format dxfId="80">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="73">
+    <format dxfId="79">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -20132,7 +19974,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
   <location ref="O14:P19" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -20201,39 +20043,39 @@
     <dataField name="Soma do Valor das Transferências" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="88">
+    <format dxfId="94">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="87">
+    <format dxfId="93">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="86">
+    <format dxfId="92">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="85">
+    <format dxfId="91">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="84">
+    <format dxfId="90">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="83">
+    <format dxfId="89">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="82">
+    <format dxfId="88">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="81">
+    <format dxfId="87">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="80">
+    <format dxfId="86">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -20243,150 +20085,6 @@
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
             <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6" rowHeaderCaption="Temporadas" colHeaderCaption="">
-  <location ref="A14:D22" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="10">
-    <pivotField axis="axisRow" showAll="0">
-      <items count="7">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisCol" showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="7">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="1"/>
-  </colFields>
-  <colItems count="3">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Somas de Entradas e Saídas" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
-  </dataFields>
-  <formats count="6">
-    <format dxfId="94">
-      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
-        <references count="1">
-          <reference field="0" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="93">
-      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
-    </format>
-    <format dxfId="92">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="0" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="91">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="1" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="90">
-      <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="89">
-      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="2">
-    <chartFormat chart="0" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="1" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="1"/>
           </reference>
         </references>
       </pivotArea>

</xml_diff>

<commit_message>
49. Andamento da 6ª análise
Andamento da sexta análise.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8076D85-2031-4329-97B0-2DDCB4189AF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B61FF04C-C1E0-43A2-BA11-E16C9F996273}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15643,11 +15643,11 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>61</xdr:col>
-      <xdr:colOff>1268685</xdr:colOff>
+      <xdr:colOff>1086756</xdr:colOff>
       <xdr:row>36</xdr:row>
-      <xdr:rowOff>136919</xdr:rowOff>
+      <xdr:rowOff>119204</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="12584984" cy="1626471"/>
+    <xdr:ext cx="12907508" cy="2064796"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="46" name="CaixaDeTexto 45">
@@ -15661,8 +15661,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="67417826" y="6973091"/>
-          <a:ext cx="12584984" cy="1626471"/>
+          <a:off x="67460455" y="7165760"/>
+          <a:ext cx="12907508" cy="2064796"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -15807,9 +15807,234 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>O investimento do Tottenham Hotspur em atletas</a:t>
-          </a:r>
-          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
+            <a:t>O investimento do Tottenham Hotspur foi distribuído entre meio-campistas, atacantes e defensores </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>—</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1100" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>representando, respectivamente, </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>38,7%</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>; </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>36,2%</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> e </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>25,1% </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>do total.</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Os dados indicam que o clube possivelmente tenha desbravado o mercado de transferências visando jogadores com perfis </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>ofensivos</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> e que </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>controlem</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> o setor do meio-campo,</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>visto que, juntas, suas posições compõem aproximadamente </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>75</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>% das entradas.</a:t>
+          </a:r>
         </a:p>
       </xdr:txBody>
     </xdr:sp>
@@ -21127,7 +21352,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{121A8764-E71B-430A-8F79-2AFBC43701E9}">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <tabColor theme="6" tint="0.39997558519241921"/>
   </sheetPr>
   <dimension ref="A1:J24"/>
@@ -21275,7 +21500,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>9</v>
       </c>
@@ -21374,7 +21599,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>34</v>
       </c>
@@ -21506,7 +21731,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>55</v>
       </c>
@@ -21638,7 +21863,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>75</v>
       </c>
@@ -21770,7 +21995,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>93</v>
       </c>
@@ -21902,7 +22127,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>109</v>
       </c>
@@ -21936,7 +22161,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:J24" xr:uid="{121A8764-E71B-430A-8F79-2AFBC43701E9}"/>
+  <autoFilter ref="A2:J24" xr:uid="{121A8764-E71B-430A-8F79-2AFBC43701E9}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="Entrada"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:J25">
     <sortCondition ref="A3:A25"/>
   </sortState>

</xml_diff>

<commit_message>
50. Andamento da 6ª análise
Andamento da sexta análise.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B61FF04C-C1E0-43A2-BA11-E16C9F996273}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF923A03-95E0-4FFE-A249-A9551D355AAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15643,11 +15643,11 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>61</xdr:col>
-      <xdr:colOff>1086756</xdr:colOff>
+      <xdr:colOff>1125634</xdr:colOff>
       <xdr:row>36</xdr:row>
-      <xdr:rowOff>119204</xdr:rowOff>
+      <xdr:rowOff>130640</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="12907508" cy="2064796"/>
+    <xdr:ext cx="12907508" cy="2722284"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="46" name="CaixaDeTexto 45">
@@ -15661,8 +15661,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="67460455" y="7165760"/>
-          <a:ext cx="12907508" cy="2064796"/>
+          <a:off x="67274775" y="6966812"/>
+          <a:ext cx="12907508" cy="2722284"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -15796,7 +15796,23 @@
           <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0"/>
         </a:p>
         <a:p>
-          <a:pPr algn="ctr"/>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="ctr" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
           <a:r>
             <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
               <a:solidFill>
@@ -16035,6 +16051,138 @@
             </a:rPr>
             <a:t>% das entradas.</a:t>
           </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Em relação ao perfil etário das contratações, identificou-se que </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>69%</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> dos atletas eram jovens que possuíam entre 21 e 25 anos, enquanto </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>19% </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>concentravam-se em jogadores</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>experientes dos 26 aos 30 anos. Ativos muito jovens ou veteranos também marcaram presença, registrando </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>6% </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>cada. Notou-se que</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1400">
+            <a:effectLst/>
+          </a:endParaRPr>
         </a:p>
       </xdr:txBody>
     </xdr:sp>

</xml_diff>

<commit_message>
51. Andamento da 6ª análise
Andamento da sexta análise.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF923A03-95E0-4FFE-A249-A9551D355AAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{226EDEDF-29B0-4EC3-8429-9F93444E3C9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -847,6 +847,33 @@
   </cellStyles>
   <dxfs count="95">
     <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center"/>
     </dxf>
     <dxf>
@@ -1079,33 +1106,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general"/>
     </dxf>
     <dxf>
       <alignment horizontal="center"/>
@@ -15643,11 +15643,11 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>61</xdr:col>
-      <xdr:colOff>1125634</xdr:colOff>
-      <xdr:row>36</xdr:row>
-      <xdr:rowOff>130640</xdr:rowOff>
+      <xdr:colOff>954514</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>86530</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="12907508" cy="2722284"/>
+    <xdr:ext cx="13269595" cy="3598934"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="46" name="CaixaDeTexto 45">
@@ -15661,8 +15661,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="67274775" y="6966812"/>
-          <a:ext cx="12907508" cy="2722284"/>
+          <a:off x="67118416" y="6649487"/>
+          <a:ext cx="13269595" cy="3598934"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -16154,7 +16154,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>experientes dos 26 aos 30 anos. Ativos muito jovens ou veteranos também marcaram presença, registrando </a:t>
+            <a:t>experientes, dos 26 aos 30 anos. Ativos muito jovens ou veteranos também marcaram presença, registrando </a:t>
           </a:r>
           <a:r>
             <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
@@ -16178,7 +16178,255 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>cada. Notou-se que</a:t>
+            <a:t>cada. Embora os dados tenham apresentado um distanciamento</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>similar entre as duas categorias "extremas" citadas anteriormente e o restante do conjunto, uma delas tornou-se fundamental para compreender o comportamento do Tottenham</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Hotspur: a faixa etária batizada de </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>muito jovem</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> (16 até 20 anos)</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>e que conta com apenas um jogador, sendo ele Archie Gray. Somando-a à categoria </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>jovem</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>, é possível concluir que</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>75%</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> das contratações giraram em torno de ativos entre </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>16 e 25 anos</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>, portanto, jovens. O fato apresentado indica que o clube possivelmente adentrou o mercado de</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>transferências buscando um perfil </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>jovial</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>, que possui potencial para se desenvolver, sem desconsiderar jogadores consolidados e mais experientes, compondo um elenco </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>mesclado</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>.</a:t>
           </a:r>
           <a:endParaRPr lang="pt-BR" sz="1400">
             <a:effectLst/>
@@ -18573,6 +18821,134 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
+  <location ref="O14:P19" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="10">
+    <pivotField showAll="0"/>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="3">
+        <item h="1" x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0" sortType="descending">
+      <items count="4">
+        <item x="1"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="2">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+            <reference field="1" count="1" selected="0">
+              <x v="1"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="3"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="1"/>
+  </colFields>
+  <colItems count="1">
+    <i>
+      <x v="1"/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Soma do Valor das Transferências" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
+  </dataFields>
+  <formats count="9">
+    <format dxfId="8">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="7">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="6">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="5">
+      <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
+    </format>
+    <format dxfId="4">
+      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="3">
+      <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="2">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="3" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="1">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="1" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="0">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="1">
+    <chartFormat chart="1" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6" rowHeaderCaption="Temporadas" colHeaderCaption="">
   <location ref="A14:D22" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -18647,34 +19023,34 @@
     <dataField name="Somas de Entradas e Saídas" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="5">
+    <format dxfId="14">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="4">
+    <format dxfId="13">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="3">
+    <format dxfId="12">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="2">
+    <format dxfId="11">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="1">
+    <format dxfId="10">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="0">
+    <format dxfId="9">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -18716,7 +19092,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4F5027D2-D537-4505-8DBC-54A417F72129}" name="Tabela dinâmica8" cacheId="0" dataPosition="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10" rowHeaderCaption="Posições e Jogadores" colHeaderCaption="Tipo de Movimentação">
   <location ref="BA14:BC26" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
   <pivotFields count="10">
@@ -18846,7 +19222,7 @@
     <dataField name="Porcentagem (%) do Total" fld="6" showDataAs="percentOfTotal" baseField="0" baseItem="0" numFmtId="10"/>
   </dataFields>
   <formats count="18">
-    <format dxfId="23">
+    <format dxfId="32">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -18855,7 +19231,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="22">
+    <format dxfId="31">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -18868,7 +19244,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="21">
+    <format dxfId="30">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -18877,7 +19253,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="20">
+    <format dxfId="29">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -18890,7 +19266,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="19">
+    <format dxfId="28">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -18899,7 +19275,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="18">
+    <format dxfId="27">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -18912,26 +19288,26 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="17">
+    <format dxfId="26">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="16">
+    <format dxfId="25">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="15">
+    <format dxfId="24">
       <pivotArea field="-2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="1"/>
     </format>
-    <format dxfId="14">
+    <format dxfId="23">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="13">
+    <format dxfId="22">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="12">
+    <format dxfId="21">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -18944,7 +19320,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="11">
+    <format dxfId="20">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -18957,7 +19333,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="10">
+    <format dxfId="19">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -18970,14 +19346,14 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="9">
+    <format dxfId="18">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="8">
+    <format dxfId="17">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -18988,10 +19364,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="7">
+    <format dxfId="16">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="6">
+    <format dxfId="15">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
@@ -19370,7 +19746,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FB686887-B509-4E7E-B605-6A13972A6E0B}" name="Tabela dinâmica5" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Origem das Contratações" colHeaderCaption="Contagem de Jogadores">
   <location ref="AN14:AO47" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
@@ -19546,22 +19922,22 @@
     <dataField name="Clubes" fld="3" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="46">
-    <format dxfId="69">
+    <format dxfId="78">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="68">
+    <format dxfId="77">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="67">
+    <format dxfId="76">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="66">
+    <format dxfId="75">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="65">
+    <format dxfId="74">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="64">
+    <format dxfId="73">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="15">
@@ -19584,10 +19960,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="63">
+    <format dxfId="72">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="62">
+    <format dxfId="71">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19599,7 +19975,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="61">
+    <format dxfId="70">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19611,7 +19987,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="60">
+    <format dxfId="69">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19623,7 +19999,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="59">
+    <format dxfId="68">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19635,7 +20011,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="58">
+    <format dxfId="67">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19647,7 +20023,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="57">
+    <format dxfId="66">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="2">
@@ -19660,7 +20036,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="56">
+    <format dxfId="65">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19672,7 +20048,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="55">
+    <format dxfId="64">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19684,7 +20060,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="54">
+    <format dxfId="63">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19696,7 +20072,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="53">
+    <format dxfId="62">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19708,7 +20084,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="52">
+    <format dxfId="61">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19720,7 +20096,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="51">
+    <format dxfId="60">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19732,7 +20108,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="50">
+    <format dxfId="59">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19744,7 +20120,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="49">
+    <format dxfId="58">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19756,7 +20132,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="48">
+    <format dxfId="57">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19768,29 +20144,29 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="47">
+    <format dxfId="56">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="46">
+    <format dxfId="55">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="45">
+    <format dxfId="54">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="44">
+    <format dxfId="53">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="43">
+    <format dxfId="52">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="42">
+    <format dxfId="51">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="41">
+    <format dxfId="50">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="15">
@@ -19813,10 +20189,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="40">
+    <format dxfId="49">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="39">
+    <format dxfId="48">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19828,7 +20204,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="38">
+    <format dxfId="47">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19840,7 +20216,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="37">
+    <format dxfId="46">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19852,7 +20228,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="36">
+    <format dxfId="45">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19864,7 +20240,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="35">
+    <format dxfId="44">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19876,7 +20252,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="34">
+    <format dxfId="43">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="2">
@@ -19889,7 +20265,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="33">
+    <format dxfId="42">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19901,7 +20277,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="32">
+    <format dxfId="41">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19913,7 +20289,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="31">
+    <format dxfId="40">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19925,7 +20301,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="30">
+    <format dxfId="39">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19937,7 +20313,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="29">
+    <format dxfId="38">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19949,7 +20325,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="28">
+    <format dxfId="37">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19961,7 +20337,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="27">
+    <format dxfId="36">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19973,7 +20349,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="26">
+    <format dxfId="35">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19985,7 +20361,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="25">
+    <format dxfId="34">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -19997,7 +20373,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="24">
+    <format dxfId="33">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
@@ -20017,7 +20393,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{996EC5F2-74EB-477F-A9D9-AF44A2544855}" name="Tabela dinâmica3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Faixa Etária" colHeaderCaption="Tipo de Movimentação">
   <location ref="Y14:Z20" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -20094,43 +20470,43 @@
     <dataField name="Contagem de Jogadores" fld="8" subtotal="count" baseField="8" baseItem="0"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="78">
+    <format dxfId="87">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="77">
+    <format dxfId="86">
       <pivotArea field="8" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="76">
+    <format dxfId="85">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="75">
+    <format dxfId="84">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="74">
+    <format dxfId="83">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="73">
+    <format dxfId="82">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="72">
+    <format dxfId="81">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="71">
+    <format dxfId="80">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="70">
+    <format dxfId="79">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -20157,7 +20533,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{904CEA3A-CD0A-459C-A420-1FB249800D4C}" name="Tabela dinâmica4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Nacionalidades" colHeaderCaption="Contagem de Jogadores">
   <location ref="AK14:AL29" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
@@ -20290,166 +20666,38 @@
     <dataField name="Contagem de Nacionalidades" fld="3" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="7">
-    <format dxfId="85">
+    <format dxfId="94">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="84">
+    <format dxfId="93">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="83">
+    <format dxfId="92">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="82">
+    <format dxfId="91">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="81">
+    <format dxfId="90">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="80">
+    <format dxfId="89">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="79">
+    <format dxfId="88">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="1">
-    <chartFormat chart="1" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
-  <location ref="O14:P19" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="10">
-    <pivotField showAll="0"/>
-    <pivotField axis="axisCol" showAll="0">
-      <items count="3">
-        <item h="1" x="1"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0" sortType="descending">
-      <items count="4">
-        <item x="1"/>
-        <item x="2"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-      <autoSortScope>
-        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
-          <references count="2">
-            <reference field="4294967294" count="1" selected="0">
-              <x v="0"/>
-            </reference>
-            <reference field="1" count="1" selected="0">
-              <x v="1"/>
-            </reference>
-          </references>
-        </pivotArea>
-      </autoSortScope>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="3"/>
-  </rowFields>
-  <rowItems count="4">
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="1"/>
-  </colFields>
-  <colItems count="1">
-    <i>
-      <x v="1"/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Soma do Valor das Transferências" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
-  </dataFields>
-  <formats count="9">
-    <format dxfId="94">
-      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="93">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="92">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="91">
-      <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
-    </format>
-    <format dxfId="90">
-      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="89">
-      <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
-    </format>
-    <format dxfId="88">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="3" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="87">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="1" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="86">
-      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
   <chartFormats count="1">
@@ -21500,7 +21748,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{121A8764-E71B-430A-8F79-2AFBC43701E9}">
-  <sheetPr filterMode="1">
+  <sheetPr>
     <tabColor theme="6" tint="0.39997558519241921"/>
   </sheetPr>
   <dimension ref="A1:J24"/>
@@ -21648,7 +21896,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>9</v>
       </c>
@@ -21747,7 +21995,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>34</v>
       </c>
@@ -21879,7 +22127,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="12" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>55</v>
       </c>
@@ -22011,7 +22259,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>75</v>
       </c>
@@ -22143,7 +22391,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>93</v>
       </c>
@@ -22275,7 +22523,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="24" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>109</v>
       </c>
@@ -22309,13 +22557,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:J24" xr:uid="{121A8764-E71B-430A-8F79-2AFBC43701E9}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="Entrada"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A2:J24" xr:uid="{121A8764-E71B-430A-8F79-2AFBC43701E9}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:J25">
     <sortCondition ref="A3:A25"/>
   </sortState>

</xml_diff>

<commit_message>
52. Andamento da 6ª análise
Andamento da sexta análise.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{226EDEDF-29B0-4EC3-8429-9F93444E3C9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6474224B-34DD-4DE1-99A5-B3F58C035EB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15643,11 +15643,11 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>61</xdr:col>
-      <xdr:colOff>954514</xdr:colOff>
-      <xdr:row>35</xdr:row>
-      <xdr:rowOff>86530</xdr:rowOff>
+      <xdr:colOff>943520</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>118713</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="13269595" cy="3598934"/>
+    <xdr:ext cx="13284278" cy="4475584"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="46" name="CaixaDeTexto 45">
@@ -15661,8 +15661,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="67118416" y="6649487"/>
-          <a:ext cx="13269595" cy="3598934"/>
+          <a:off x="67222537" y="7107280"/>
+          <a:ext cx="13284278" cy="4475584"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -16427,6 +16427,158 @@
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
             <a:t>.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="ctr" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="ctr" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400">
+              <a:effectLst/>
+            </a:rPr>
+            <a:t>No que diz respeito às</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" baseline="0">
+              <a:effectLst/>
+            </a:rPr>
+            <a:t> nacionalidades dos atletas, não foi possível identificar um padrão quanto suas presenças nas contratações do clube. O principal fator resultante foi a</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1400" b="1" baseline="0">
+            <a:effectLst/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="ctr" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" baseline="0">
+              <a:effectLst/>
+            </a:rPr>
+            <a:t>diversidade</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:effectLst/>
+            </a:rPr>
+            <a:t> de nações encontradas, contabilizando </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" baseline="0">
+              <a:effectLst/>
+            </a:rPr>
+            <a:t>16</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:effectLst/>
+            </a:rPr>
+            <a:t> entre </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" baseline="0">
+              <a:effectLst/>
+            </a:rPr>
+            <a:t>13</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:effectLst/>
+            </a:rPr>
+            <a:t> jogadores. Em decorrência, ingleses e neerlandeses que contam com </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" baseline="0">
+              <a:effectLst/>
+            </a:rPr>
+            <a:t>3</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:effectLst/>
+            </a:rPr>
+            <a:t> e </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" baseline="0">
+              <a:effectLst/>
+            </a:rPr>
+            <a:t>2</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:effectLst/>
+            </a:rPr>
+            <a:t> atletas na lista, respectivamente,</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:effectLst/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:effectLst/>
+            </a:rPr>
+            <a:t>dificilmente podem ser considerados como modelos. </a:t>
           </a:r>
           <a:endParaRPr lang="pt-BR" sz="1400">
             <a:effectLst/>

</xml_diff>

<commit_message>
53. Andamento da 6ª análise
Andamento da sexta análise.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6474224B-34DD-4DE1-99A5-B3F58C035EB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F147AA7A-722D-44F0-B102-8F123C3DBC94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -847,6 +847,27 @@
   </cellStyles>
   <dxfs count="95">
     <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="general"/>
     </dxf>
     <dxf>
@@ -1082,27 +1103,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
     </dxf>
     <dxf>
       <alignment horizontal="center"/>
@@ -15643,11 +15643,11 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>61</xdr:col>
-      <xdr:colOff>943520</xdr:colOff>
+      <xdr:colOff>895894</xdr:colOff>
       <xdr:row>36</xdr:row>
-      <xdr:rowOff>118713</xdr:rowOff>
+      <xdr:rowOff>133864</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="13284278" cy="4475584"/>
+    <xdr:ext cx="13284278" cy="6009722"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="46" name="CaixaDeTexto 45">
@@ -15661,8 +15661,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="67222537" y="7107280"/>
-          <a:ext cx="13284278" cy="4475584"/>
+          <a:off x="67058925" y="7051395"/>
+          <a:ext cx="13284278" cy="6009722"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -16485,7 +16485,7 @@
             <a:rPr lang="pt-BR" sz="1400" baseline="0">
               <a:effectLst/>
             </a:rPr>
-            <a:t> nacionalidades dos atletas, não foi possível identificar um padrão quanto suas presenças nas contratações do clube. O principal fator resultante foi a</a:t>
+            <a:t> nacionalidades dos atletas, não foi possível identificar um padrão quanto suas presenças nas contratações do clube. O principal fator para tal foi a</a:t>
           </a:r>
           <a:endParaRPr lang="pt-BR" sz="1400" b="1" baseline="0">
             <a:effectLst/>
@@ -16543,7 +16543,7 @@
             <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
               <a:effectLst/>
             </a:rPr>
-            <a:t> jogadores. Em decorrência, ingleses e neerlandeses que contam com </a:t>
+            <a:t> jogadores. Em decorrência, ingleses e neerlandeses, líderes da lista com </a:t>
           </a:r>
           <a:r>
             <a:rPr lang="pt-BR" sz="1400" b="1" baseline="0">
@@ -16567,7 +16567,7 @@
             <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
               <a:effectLst/>
             </a:rPr>
-            <a:t> atletas na lista, respectivamente,</a:t>
+            <a:t> atletas respectivamente,</a:t>
           </a:r>
           <a:br>
             <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
@@ -16578,8 +16578,277 @@
             <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
               <a:effectLst/>
             </a:rPr>
-            <a:t>dificilmente podem ser considerados como modelos. </a:t>
-          </a:r>
+            <a:t>dificilmente podem ser considerados como modelos. No entanto, como forma de enriquecer a análise, é importante levar em consideração quais foram os clubes de origem dos</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:effectLst/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:effectLst/>
+            </a:rPr>
+            <a:t>jogadores envolvidos nas negociações, incluindo os representantes de ambas as nações. Notou-se que o Tottenham Hotspur, possivelmente alinhando-se com uma estratégia do</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:effectLst/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" baseline="0">
+              <a:effectLst/>
+            </a:rPr>
+            <a:t>seu departamento de </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="1" baseline="0">
+              <a:effectLst/>
+            </a:rPr>
+            <a:t>scouting</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:effectLst/>
+            </a:rPr>
+            <a:t>, mapeou ativos presentes em diversos mercados europeus</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1100" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>sem estarem necessariamente ligados à nacionalidade daquele país </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1100" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>— </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>como é o caso de</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Cristian Romero, defensor </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>argentino</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> adquirido enquanto atuava pela Atalanta, um clube </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>italiano</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>. Também foi possível identificar que a equipe não se distanciou do mercado</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>doméstico, visto que </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>todos</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> os atletas ingleses foram contratados enquanto jogavam por compatriotas dos Spurs, como Leeds United, Bournemouth e Leicester City. Todos os</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>indicadores apresentados reforçam a ideia de um elenco caracterizado pela </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>pluralidade</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>.</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
           <a:endParaRPr lang="pt-BR" sz="1400">
             <a:effectLst/>
           </a:endParaRPr>
@@ -18973,6 +19242,196 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{904CEA3A-CD0A-459C-A420-1FB249800D4C}" name="Tabela dinâmica4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Nacionalidades" colHeaderCaption="Contagem de Jogadores">
+  <location ref="AK14:AL29" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="9">
+    <pivotField axis="axisCol" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item h="1" x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" dataField="1" showAll="0" sortType="ascending">
+      <items count="15">
+        <item x="6"/>
+        <item x="4"/>
+        <item x="9"/>
+        <item x="11"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="12"/>
+        <item x="5"/>
+        <item x="10"/>
+        <item x="13"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="2">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+            <reference field="0" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="21">
+        <item x="12"/>
+        <item x="9"/>
+        <item x="7"/>
+        <item x="15"/>
+        <item x="5"/>
+        <item x="17"/>
+        <item x="11"/>
+        <item x="10"/>
+        <item x="2"/>
+        <item x="8"/>
+        <item x="18"/>
+        <item x="13"/>
+        <item x="0"/>
+        <item x="16"/>
+        <item x="19"/>
+        <item x="1"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item x="14"/>
+        <item x="6"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="3"/>
+  </rowFields>
+  <rowItems count="14">
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="0"/>
+  </colFields>
+  <colItems count="1">
+    <i>
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Contagem de Nacionalidades" fld="3" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="7">
+    <format dxfId="6">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="3" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="5">
+      <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="4">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="3" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="3">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+    <format dxfId="2">
+      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="1">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="0">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="1">
+    <chartFormat chart="1" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
   <location ref="O14:P19" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -19041,39 +19500,39 @@
     <dataField name="Soma do Valor das Transferências" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="8">
+    <format dxfId="15">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="7">
+    <format dxfId="14">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="6">
+    <format dxfId="13">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="5">
+    <format dxfId="12">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="4">
+    <format dxfId="11">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="3">
+    <format dxfId="10">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="2">
+    <format dxfId="9">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="1">
+    <format dxfId="8">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="0">
+    <format dxfId="7">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -19100,7 +19559,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6" rowHeaderCaption="Temporadas" colHeaderCaption="">
   <location ref="A14:D22" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -19175,34 +19634,34 @@
     <dataField name="Somas de Entradas e Saídas" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="14">
+    <format dxfId="21">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="13">
+    <format dxfId="20">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="12">
+    <format dxfId="19">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="11">
+    <format dxfId="18">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="10">
+    <format dxfId="17">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="9">
+    <format dxfId="16">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -19244,7 +19703,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4F5027D2-D537-4505-8DBC-54A417F72129}" name="Tabela dinâmica8" cacheId="0" dataPosition="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10" rowHeaderCaption="Posições e Jogadores" colHeaderCaption="Tipo de Movimentação">
   <location ref="BA14:BC26" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
   <pivotFields count="10">
@@ -19374,7 +19833,7 @@
     <dataField name="Porcentagem (%) do Total" fld="6" showDataAs="percentOfTotal" baseField="0" baseItem="0" numFmtId="10"/>
   </dataFields>
   <formats count="18">
-    <format dxfId="32">
+    <format dxfId="39">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -19383,7 +19842,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="31">
+    <format dxfId="38">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -19396,7 +19855,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="30">
+    <format dxfId="37">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -19405,7 +19864,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="29">
+    <format dxfId="36">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -19418,7 +19877,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="28">
+    <format dxfId="35">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -19427,7 +19886,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="27">
+    <format dxfId="34">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -19440,26 +19899,26 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="26">
+    <format dxfId="33">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="25">
+    <format dxfId="32">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="24">
+    <format dxfId="31">
       <pivotArea field="-2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="1"/>
     </format>
-    <format dxfId="23">
+    <format dxfId="30">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="22">
+    <format dxfId="29">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="21">
+    <format dxfId="28">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -19472,7 +19931,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="20">
+    <format dxfId="27">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -19485,7 +19944,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="19">
+    <format dxfId="26">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -19498,14 +19957,14 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="18">
+    <format dxfId="25">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="17">
+    <format dxfId="24">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -19516,10 +19975,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="16">
+    <format dxfId="23">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="15">
+    <format dxfId="22">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
@@ -19898,7 +20357,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FB686887-B509-4E7E-B605-6A13972A6E0B}" name="Tabela dinâmica5" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Origem das Contratações" colHeaderCaption="Contagem de Jogadores">
   <location ref="AN14:AO47" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
@@ -20074,22 +20533,22 @@
     <dataField name="Clubes" fld="3" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="46">
-    <format dxfId="78">
+    <format dxfId="85">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="77">
+    <format dxfId="84">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="76">
+    <format dxfId="83">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="75">
+    <format dxfId="82">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="74">
+    <format dxfId="81">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="73">
+    <format dxfId="80">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="15">
@@ -20112,10 +20571,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="72">
+    <format dxfId="79">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="71">
+    <format dxfId="78">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20127,7 +20586,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="70">
+    <format dxfId="77">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20139,7 +20598,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="69">
+    <format dxfId="76">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20151,7 +20610,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="68">
+    <format dxfId="75">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20163,7 +20622,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="67">
+    <format dxfId="74">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20175,7 +20634,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="66">
+    <format dxfId="73">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="2">
@@ -20188,7 +20647,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="65">
+    <format dxfId="72">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20200,7 +20659,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="64">
+    <format dxfId="71">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20212,7 +20671,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="63">
+    <format dxfId="70">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20224,7 +20683,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="62">
+    <format dxfId="69">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20236,7 +20695,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="61">
+    <format dxfId="68">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20248,7 +20707,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="60">
+    <format dxfId="67">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20260,7 +20719,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="59">
+    <format dxfId="66">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20272,7 +20731,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="58">
+    <format dxfId="65">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20284,7 +20743,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="57">
+    <format dxfId="64">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20296,29 +20755,29 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="56">
+    <format dxfId="63">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="55">
+    <format dxfId="62">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="54">
+    <format dxfId="61">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="53">
+    <format dxfId="60">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="52">
+    <format dxfId="59">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="51">
+    <format dxfId="58">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="50">
+    <format dxfId="57">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="15">
@@ -20341,10 +20800,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="49">
+    <format dxfId="56">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="48">
+    <format dxfId="55">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20356,7 +20815,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="47">
+    <format dxfId="54">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20368,7 +20827,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="46">
+    <format dxfId="53">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20380,7 +20839,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="45">
+    <format dxfId="52">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20392,7 +20851,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="44">
+    <format dxfId="51">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20404,7 +20863,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="43">
+    <format dxfId="50">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="2">
@@ -20417,7 +20876,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="42">
+    <format dxfId="49">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20429,7 +20888,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="41">
+    <format dxfId="48">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20441,7 +20900,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="40">
+    <format dxfId="47">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20453,7 +20912,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="39">
+    <format dxfId="46">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20465,7 +20924,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="38">
+    <format dxfId="45">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20477,7 +20936,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="37">
+    <format dxfId="44">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20489,7 +20948,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="36">
+    <format dxfId="43">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20501,7 +20960,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="35">
+    <format dxfId="42">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20513,7 +20972,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="34">
+    <format dxfId="41">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20525,7 +20984,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="33">
+    <format dxfId="40">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
@@ -20545,7 +21004,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{996EC5F2-74EB-477F-A9D9-AF44A2544855}" name="Tabela dinâmica3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Faixa Etária" colHeaderCaption="Tipo de Movimentação">
   <location ref="Y14:Z20" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -20622,216 +21081,20 @@
     <dataField name="Contagem de Jogadores" fld="8" subtotal="count" baseField="8" baseItem="0"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="87">
+    <format dxfId="94">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="86">
+    <format dxfId="93">
       <pivotArea field="8" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
-    </format>
-    <format dxfId="85">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="8" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="84">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
-    </format>
-    <format dxfId="83">
-      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="82">
-      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="81">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="1" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="80">
-      <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
-    </format>
-    <format dxfId="79">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="1">
-    <chartFormat chart="2" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{904CEA3A-CD0A-459C-A420-1FB249800D4C}" name="Tabela dinâmica4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Nacionalidades" colHeaderCaption="Contagem de Jogadores">
-  <location ref="AK14:AL29" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="9">
-    <pivotField axis="axisCol" showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item h="1" x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" dataField="1" showAll="0" sortType="ascending">
-      <items count="15">
-        <item x="6"/>
-        <item x="4"/>
-        <item x="9"/>
-        <item x="11"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="12"/>
-        <item x="5"/>
-        <item x="10"/>
-        <item x="13"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item t="default"/>
-      </items>
-      <autoSortScope>
-        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
-          <references count="2">
-            <reference field="4294967294" count="1" selected="0">
-              <x v="0"/>
-            </reference>
-            <reference field="0" count="1" selected="0">
-              <x v="0"/>
-            </reference>
-          </references>
-        </pivotArea>
-      </autoSortScope>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="21">
-        <item x="12"/>
-        <item x="9"/>
-        <item x="7"/>
-        <item x="15"/>
-        <item x="5"/>
-        <item x="17"/>
-        <item x="11"/>
-        <item x="10"/>
-        <item x="2"/>
-        <item x="8"/>
-        <item x="18"/>
-        <item x="13"/>
-        <item x="0"/>
-        <item x="16"/>
-        <item x="19"/>
-        <item x="1"/>
-        <item x="4"/>
-        <item x="3"/>
-        <item x="14"/>
-        <item x="6"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="3"/>
-  </rowFields>
-  <rowItems count="14">
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="13"/>
-    </i>
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="11"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="12"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="0"/>
-  </colFields>
-  <colItems count="1">
-    <i>
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Contagem de Nacionalidades" fld="3" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="7">
-    <format dxfId="94">
-      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
-        <references count="1">
-          <reference field="3" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="93">
-      <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
     <format dxfId="92">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
-          <reference field="3" count="0"/>
+          <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
@@ -20842,18 +21105,24 @@
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
     <format dxfId="89">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="88">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
-          <reference field="0" count="0"/>
+          <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="88">
+    <format dxfId="87">
+      <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
+    </format>
+    <format dxfId="86">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
   <chartFormats count="1">
-    <chartFormat chart="1" format="0" series="1">
+    <chartFormat chart="2" format="0" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -21900,7 +22169,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{121A8764-E71B-430A-8F79-2AFBC43701E9}">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <tabColor theme="6" tint="0.39997558519241921"/>
   </sheetPr>
   <dimension ref="A1:J24"/>
@@ -22048,7 +22317,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>9</v>
       </c>
@@ -22147,7 +22416,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>34</v>
       </c>
@@ -22279,7 +22548,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>55</v>
       </c>
@@ -22411,7 +22680,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>75</v>
       </c>
@@ -22543,7 +22812,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>93</v>
       </c>
@@ -22675,7 +22944,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>109</v>
       </c>
@@ -22709,7 +22978,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:J24" xr:uid="{121A8764-E71B-430A-8F79-2AFBC43701E9}"/>
+  <autoFilter ref="A2:J24" xr:uid="{121A8764-E71B-430A-8F79-2AFBC43701E9}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="Entrada"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:J25">
     <sortCondition ref="A3:A25"/>
   </sortState>

</xml_diff>

<commit_message>
54. Andamento da 6ª análise
Andamento do quinto parágrafo da sexta análise.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F147AA7A-722D-44F0-B102-8F123C3DBC94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AE303BD-6838-4226-B492-E992AC9BC217}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15645,9 +15645,9 @@
       <xdr:col>61</xdr:col>
       <xdr:colOff>895894</xdr:colOff>
       <xdr:row>36</xdr:row>
-      <xdr:rowOff>133864</xdr:rowOff>
+      <xdr:rowOff>24283</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="13284278" cy="6009722"/>
+    <xdr:ext cx="13284278" cy="6228885"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="46" name="CaixaDeTexto 45">
@@ -15661,8 +15661,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="67058925" y="7051395"/>
-          <a:ext cx="13284278" cy="6009722"/>
+          <a:off x="67058925" y="6941814"/>
+          <a:ext cx="13284278" cy="6228885"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -16849,6 +16849,113 @@
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
           </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Embora o valor gasto em contratações seja visto como destaque, a quantia </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>recebida</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> através das saídas de jogadores também impactou o clube. Foram registradas despedidas de</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>apenas </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>5</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> ativos que, juntas, reuniram </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>£179.8 milhões </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>aos cofres londrinos.</a:t>
+          </a:r>
           <a:endParaRPr lang="pt-BR" sz="1400">
             <a:effectLst/>
           </a:endParaRPr>
@@ -22251,7 +22358,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>9</v>
       </c>
@@ -22284,7 +22391,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
@@ -22317,7 +22424,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>9</v>
       </c>
@@ -22350,7 +22457,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>34</v>
       </c>
@@ -22383,7 +22490,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>34</v>
       </c>
@@ -22416,7 +22523,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>34</v>
       </c>
@@ -22449,7 +22556,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>34</v>
       </c>
@@ -22482,7 +22589,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>55</v>
       </c>
@@ -22515,7 +22622,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>55</v>
       </c>
@@ -22548,7 +22655,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="12" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>55</v>
       </c>
@@ -22581,7 +22688,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>55</v>
       </c>
@@ -22614,7 +22721,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>75</v>
       </c>
@@ -22647,7 +22754,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>75</v>
       </c>
@@ -22680,7 +22787,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>75</v>
       </c>
@@ -22713,7 +22820,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>75</v>
       </c>
@@ -22746,7 +22853,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>93</v>
       </c>
@@ -22779,7 +22886,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>93</v>
       </c>
@@ -22812,7 +22919,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>93</v>
       </c>
@@ -22845,7 +22952,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>93</v>
       </c>
@@ -22878,7 +22985,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>109</v>
       </c>
@@ -22911,7 +23018,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>109</v>
       </c>
@@ -22944,7 +23051,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="24" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>109</v>
       </c>
@@ -22981,7 +23088,7 @@
   <autoFilter ref="A2:J24" xr:uid="{121A8764-E71B-430A-8F79-2AFBC43701E9}">
     <filterColumn colId="1">
       <filters>
-        <filter val="Entrada"/>
+        <filter val="Saída"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
55. Andamento da 6ª análise
Andamento da sexta análise.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AE303BD-6838-4226-B492-E992AC9BC217}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{492FEDC9-F6A0-4F7F-8E4F-6A5BD7ECE0D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -868,6 +868,33 @@
       <alignment horizontal="center"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="general"/>
     </dxf>
     <dxf>
@@ -1103,33 +1130,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -15643,11 +15643,11 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>61</xdr:col>
-      <xdr:colOff>895894</xdr:colOff>
+      <xdr:colOff>935388</xdr:colOff>
       <xdr:row>36</xdr:row>
-      <xdr:rowOff>24283</xdr:rowOff>
+      <xdr:rowOff>128797</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="13284278" cy="6228885"/>
+    <xdr:ext cx="13514854" cy="7543860"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="46" name="CaixaDeTexto 45">
@@ -15661,8 +15661,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="67058925" y="6941814"/>
-          <a:ext cx="13284278" cy="6228885"/>
+          <a:off x="67098419" y="7046328"/>
+          <a:ext cx="13514854" cy="7543860"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -16918,6 +16918,77 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
+            <a:t>6</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> ativos que, juntas, reuniram </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>£179.8 milhões </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>aos cofres londrinos. Uma das movimentações mencionadas foi relacionada ao defensor belga Jan Vertoghen, que deixou</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>o clube livremente e sem custos na temporada 2020/21 — portanto, é possível concluir que </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
             <a:t>5</a:t>
           </a:r>
           <a:r>
@@ -16930,7 +17001,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t> ativos que, juntas, reuniram </a:t>
+            <a:t> das transferências realmente renderam à equipe. Cerca de </a:t>
           </a:r>
           <a:r>
             <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
@@ -16942,7 +17013,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>£179.8 milhões </a:t>
+            <a:t>70,2%</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
@@ -16954,7 +17025,254 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>aos cofres londrinos.</a:t>
+            <a:t> das vendas</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>pertenciam à atacantes, </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>22,5%</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> à meio-campistas e, por fim, </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>7,2%</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> aos defensores. Como citado anteriormente, </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>52,8%</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> do montante envolvia a saída de apenas um atleta: o atacante</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>inglês Harry Kane. Sozinha, sua venda gerou </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>£95 milhões</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>, quantia superior à soma de todas as outras. Seu companheiro de ataque, Steve Bergwijn, também arrecadou um valor</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>significativo ao Tottenham Hotspur: cerca de </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>£31 milhões</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>, se sobrepondo individualmente aos valores dos meio-campistas e defensores. Em resumo, as vendas acabaram</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>concentrando-se</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> nos atacantes e, embora não haja indícios suficientes para determinar quais foram as razões por trás delas, continuam sendo peças importantes para a compreensão</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>do comportamento financeiro do clube.</a:t>
           </a:r>
           <a:endParaRPr lang="pt-BR" sz="1400">
             <a:effectLst/>
@@ -19349,6 +19667,146 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{996EC5F2-74EB-477F-A9D9-AF44A2544855}" name="Tabela dinâmica3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Faixa Etária" colHeaderCaption="Tipo de Movimentação">
+  <location ref="Y14:Z20" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="10">
+    <pivotField showAll="0"/>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="3">
+        <item h="1" x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField axis="axisRow" dataField="1" showAll="0" sortType="ascending">
+      <items count="9">
+        <item m="1" x="5"/>
+        <item m="1" x="4"/>
+        <item m="1" x="7"/>
+        <item m="1" x="6"/>
+        <item x="3"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="2">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+            <reference field="1" count="1" selected="0">
+              <x v="1"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="8"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="1"/>
+  </colFields>
+  <colItems count="1">
+    <i>
+      <x v="1"/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Contagem de Jogadores" fld="8" subtotal="count" baseField="8" baseItem="0"/>
+  </dataFields>
+  <formats count="9">
+    <format dxfId="8">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="8" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="7">
+      <pivotArea field="8" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="6">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="8" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="5">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+    <format dxfId="4">
+      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="3">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="2">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="1" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="1">
+      <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
+    </format>
+    <format dxfId="0">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="1">
+    <chartFormat chart="2" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{904CEA3A-CD0A-459C-A420-1FB249800D4C}" name="Tabela dinâmica4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Nacionalidades" colHeaderCaption="Contagem de Jogadores">
   <location ref="AK14:AL29" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
@@ -19481,37 +19939,37 @@
     <dataField name="Contagem de Nacionalidades" fld="3" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="7">
-    <format dxfId="6">
+    <format dxfId="15">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="5">
+    <format dxfId="14">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="4">
+    <format dxfId="13">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="3">
+    <format dxfId="12">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="2">
+    <format dxfId="11">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="1">
+    <format dxfId="10">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="0">
+    <format dxfId="9">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -19538,7 +19996,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
   <location ref="O14:P19" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -19607,39 +20065,39 @@
     <dataField name="Soma do Valor das Transferências" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="15">
+    <format dxfId="24">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="14">
+    <format dxfId="23">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="13">
+    <format dxfId="22">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="12">
+    <format dxfId="21">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="11">
+    <format dxfId="20">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="10">
+    <format dxfId="19">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="9">
+    <format dxfId="18">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="8">
+    <format dxfId="17">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="7">
+    <format dxfId="16">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -19666,7 +20124,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6" rowHeaderCaption="Temporadas" colHeaderCaption="">
   <location ref="A14:D22" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -19741,34 +20199,34 @@
     <dataField name="Somas de Entradas e Saídas" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="21">
+    <format dxfId="30">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="20">
+    <format dxfId="29">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="19">
+    <format dxfId="28">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="18">
+    <format dxfId="27">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="17">
+    <format dxfId="26">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="16">
+    <format dxfId="25">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -19810,7 +20268,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4F5027D2-D537-4505-8DBC-54A417F72129}" name="Tabela dinâmica8" cacheId="0" dataPosition="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10" rowHeaderCaption="Posições e Jogadores" colHeaderCaption="Tipo de Movimentação">
   <location ref="BA14:BC26" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
   <pivotFields count="10">
@@ -19940,7 +20398,7 @@
     <dataField name="Porcentagem (%) do Total" fld="6" showDataAs="percentOfTotal" baseField="0" baseItem="0" numFmtId="10"/>
   </dataFields>
   <formats count="18">
-    <format dxfId="39">
+    <format dxfId="48">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -19949,7 +20407,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="38">
+    <format dxfId="47">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -19962,7 +20420,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="37">
+    <format dxfId="46">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -19971,7 +20429,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="36">
+    <format dxfId="45">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -19984,7 +20442,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="35">
+    <format dxfId="44">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -19993,7 +20451,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="34">
+    <format dxfId="43">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -20006,26 +20464,26 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="33">
+    <format dxfId="42">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="32">
+    <format dxfId="41">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="31">
+    <format dxfId="40">
       <pivotArea field="-2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="1"/>
     </format>
-    <format dxfId="30">
+    <format dxfId="39">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="29">
+    <format dxfId="38">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="28">
+    <format dxfId="37">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -20038,7 +20496,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="27">
+    <format dxfId="36">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -20051,7 +20509,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="26">
+    <format dxfId="35">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -20064,14 +20522,14 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="25">
+    <format dxfId="34">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="24">
+    <format dxfId="33">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -20082,10 +20540,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="23">
+    <format dxfId="32">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="22">
+    <format dxfId="31">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
@@ -20464,7 +20922,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FB686887-B509-4E7E-B605-6A13972A6E0B}" name="Tabela dinâmica5" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Origem das Contratações" colHeaderCaption="Contagem de Jogadores">
   <location ref="AN14:AO47" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
@@ -20640,22 +21098,22 @@
     <dataField name="Clubes" fld="3" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="46">
-    <format dxfId="85">
+    <format dxfId="94">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="84">
+    <format dxfId="93">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="83">
+    <format dxfId="92">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="82">
+    <format dxfId="91">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="81">
+    <format dxfId="90">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="80">
+    <format dxfId="89">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="15">
@@ -20678,10 +21136,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="79">
+    <format dxfId="88">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="78">
+    <format dxfId="87">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20693,7 +21151,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="77">
+    <format dxfId="86">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20705,7 +21163,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="76">
+    <format dxfId="85">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20717,7 +21175,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="75">
+    <format dxfId="84">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20729,7 +21187,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="74">
+    <format dxfId="83">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20741,7 +21199,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="73">
+    <format dxfId="82">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="2">
@@ -20754,7 +21212,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="72">
+    <format dxfId="81">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20766,7 +21224,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="71">
+    <format dxfId="80">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20778,7 +21236,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="70">
+    <format dxfId="79">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20790,7 +21248,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="69">
+    <format dxfId="78">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20802,7 +21260,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="68">
+    <format dxfId="77">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20814,7 +21272,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="67">
+    <format dxfId="76">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20826,7 +21284,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="66">
+    <format dxfId="75">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20838,7 +21296,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="65">
+    <format dxfId="74">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20850,7 +21308,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="64">
+    <format dxfId="73">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20862,29 +21320,29 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="63">
+    <format dxfId="72">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="62">
+    <format dxfId="71">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="61">
+    <format dxfId="70">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="60">
+    <format dxfId="69">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="59">
+    <format dxfId="68">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="58">
+    <format dxfId="67">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="57">
+    <format dxfId="66">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="15">
@@ -20907,10 +21365,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="56">
+    <format dxfId="65">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="55">
+    <format dxfId="64">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20922,7 +21380,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="54">
+    <format dxfId="63">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20934,7 +21392,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="53">
+    <format dxfId="62">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20946,7 +21404,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="52">
+    <format dxfId="61">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20958,7 +21416,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="51">
+    <format dxfId="60">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20970,7 +21428,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="50">
+    <format dxfId="59">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="2">
@@ -20983,7 +21441,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="49">
+    <format dxfId="58">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20995,7 +21453,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="48">
+    <format dxfId="57">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21007,7 +21465,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="47">
+    <format dxfId="56">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21019,7 +21477,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="46">
+    <format dxfId="55">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21031,7 +21489,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="45">
+    <format dxfId="54">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21043,7 +21501,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="44">
+    <format dxfId="53">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21055,7 +21513,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="43">
+    <format dxfId="52">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21067,7 +21525,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="42">
+    <format dxfId="51">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21079,7 +21537,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="41">
+    <format dxfId="50">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21091,7 +21549,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="40">
+    <format dxfId="49">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
@@ -21099,146 +21557,6 @@
       </pivotArea>
     </format>
   </formats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{996EC5F2-74EB-477F-A9D9-AF44A2544855}" name="Tabela dinâmica3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Faixa Etária" colHeaderCaption="Tipo de Movimentação">
-  <location ref="Y14:Z20" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="10">
-    <pivotField showAll="0"/>
-    <pivotField axis="axisCol" showAll="0">
-      <items count="3">
-        <item h="1" x="1"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField axis="axisRow" dataField="1" showAll="0" sortType="ascending">
-      <items count="9">
-        <item m="1" x="5"/>
-        <item m="1" x="4"/>
-        <item m="1" x="7"/>
-        <item m="1" x="6"/>
-        <item x="3"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-      <autoSortScope>
-        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
-          <references count="2">
-            <reference field="4294967294" count="1" selected="0">
-              <x v="0"/>
-            </reference>
-            <reference field="1" count="1" selected="0">
-              <x v="1"/>
-            </reference>
-          </references>
-        </pivotArea>
-      </autoSortScope>
-    </pivotField>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="8"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="1"/>
-  </colFields>
-  <colItems count="1">
-    <i>
-      <x v="1"/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Contagem de Jogadores" fld="8" subtotal="count" baseField="8" baseItem="0"/>
-  </dataFields>
-  <formats count="9">
-    <format dxfId="94">
-      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
-        <references count="1">
-          <reference field="8" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="93">
-      <pivotArea field="8" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
-    </format>
-    <format dxfId="92">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="8" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="91">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
-    </format>
-    <format dxfId="90">
-      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="89">
-      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="88">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="1" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="87">
-      <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
-    </format>
-    <format dxfId="86">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="1">
-    <chartFormat chart="2" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">

</xml_diff>

<commit_message>
56. Conclusão da 6ª análise
Conclusão da sexta análise.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{492FEDC9-F6A0-4F7F-8E4F-6A5BD7ECE0D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D15BDF6F-27AE-4031-8608-CC882EF7A127}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -895,6 +895,144 @@
       <alignment horizontal="center"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="general"/>
     </dxf>
     <dxf>
@@ -992,144 +1130,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="center" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" indent="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -15643,11 +15643,11 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>61</xdr:col>
-      <xdr:colOff>935388</xdr:colOff>
+      <xdr:colOff>727205</xdr:colOff>
       <xdr:row>36</xdr:row>
-      <xdr:rowOff>128797</xdr:rowOff>
+      <xdr:rowOff>87718</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="13514854" cy="7543860"/>
+    <xdr:ext cx="13856999" cy="8201348"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="46" name="CaixaDeTexto 45">
@@ -15661,8 +15661,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="67098419" y="7046328"/>
-          <a:ext cx="13514854" cy="7543860"/>
+          <a:off x="66907400" y="6829439"/>
+          <a:ext cx="13856999" cy="8201348"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -16390,7 +16390,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>jovial</a:t>
+            <a:t>jovem</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
@@ -17273,6 +17273,196 @@
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
             <a:t>do comportamento financeiro do clube.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="ctr" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:endParaRPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="ctr" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Resumidamente, pode-se dizer que as movimentações financeiras do Tottenham Hotspur entre as temporadas 2019/20 e 2024/25 foram caracterizadas pela </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>incisividade</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> em contratações,</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>diversidade</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> nas posições investidas, busca por </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>jovens</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>, </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>pluralidade</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> na questão de nacionalidades e </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>concentração</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> das vendas em atacantes.</a:t>
           </a:r>
           <a:endParaRPr lang="pt-BR" sz="1400">
             <a:effectLst/>
@@ -19667,6 +19857,653 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FB686887-B509-4E7E-B605-6A13972A6E0B}" name="Tabela dinâmica5" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Origem das Contratações" colHeaderCaption="Contagem de Jogadores">
+  <location ref="AN14:AO47" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="9">
+    <pivotField axis="axisCol" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item h="1" x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" dataField="1" showAll="0">
+      <items count="15">
+        <item x="6"/>
+        <item x="4"/>
+        <item x="9"/>
+        <item x="11"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="12"/>
+        <item x="5"/>
+        <item x="10"/>
+        <item x="13"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="21">
+        <item x="12"/>
+        <item x="9"/>
+        <item x="7"/>
+        <item x="15"/>
+        <item x="5"/>
+        <item x="17"/>
+        <item x="11"/>
+        <item x="10"/>
+        <item x="2"/>
+        <item x="8"/>
+        <item x="18"/>
+        <item x="13"/>
+        <item x="0"/>
+        <item x="16"/>
+        <item x="19"/>
+        <item x="1"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item x="14"/>
+        <item x="6"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="2">
+    <field x="4"/>
+    <field x="3"/>
+  </rowFields>
+  <rowItems count="32">
+    <i>
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i r="1">
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i r="1">
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i r="1">
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i r="1">
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i r="1">
+      <x v="12"/>
+    </i>
+    <i r="1">
+      <x v="13"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i r="1">
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i r="1">
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i r="1">
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i r="1">
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="15"/>
+    </i>
+    <i r="1">
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="16"/>
+    </i>
+    <i r="1">
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="17"/>
+    </i>
+    <i r="1">
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="18"/>
+    </i>
+    <i r="1">
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="19"/>
+    </i>
+    <i r="1">
+      <x v="9"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="0"/>
+  </colFields>
+  <colItems count="1">
+    <i>
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Clubes" fld="3" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="46">
+    <format dxfId="45">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="44">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="43">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="42">
+      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
+    </format>
+    <format dxfId="41">
+      <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="40">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="4" count="15">
+            <x v="2"/>
+            <x v="5"/>
+            <x v="6"/>
+            <x v="7"/>
+            <x v="8"/>
+            <x v="9"/>
+            <x v="10"/>
+            <x v="11"/>
+            <x v="12"/>
+            <x v="13"/>
+            <x v="15"/>
+            <x v="16"/>
+            <x v="17"/>
+            <x v="18"/>
+            <x v="19"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="39">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="38">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="0"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="37">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="8"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="5"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="36">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="10"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="6"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="35">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="2"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="7"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="34">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="3"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="8"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="33">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="2">
+            <x v="12"/>
+            <x v="13"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="9"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="32">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="8"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="10"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="31">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="8"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="11"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="30">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="6"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="12"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="29">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="11"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="13"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="28">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="7"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="15"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="27">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="5"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="16"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="26">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="4"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="17"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="25">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="7"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="18"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="24">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="9"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="19"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="23">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="22">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="21">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="20">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="19">
+      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
+    </format>
+    <format dxfId="18">
+      <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="17">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="4" count="15">
+            <x v="2"/>
+            <x v="5"/>
+            <x v="6"/>
+            <x v="7"/>
+            <x v="8"/>
+            <x v="9"/>
+            <x v="10"/>
+            <x v="11"/>
+            <x v="12"/>
+            <x v="13"/>
+            <x v="15"/>
+            <x v="16"/>
+            <x v="17"/>
+            <x v="18"/>
+            <x v="19"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="16">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="15">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="0"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="14">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="8"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="5"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="13">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="10"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="6"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="12">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="2"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="7"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="11">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="3"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="8"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="10">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="2">
+            <x v="12"/>
+            <x v="13"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="9"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="9">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="8"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="10"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="8">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="8"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="11"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="7">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="6"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="12"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="6">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="11"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="13"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="5">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="7"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="15"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="4">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="5"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="16"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="3">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="4"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="17"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="2">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="7"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="18"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="1">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="3" count="1">
+            <x v="9"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="19"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="0">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{996EC5F2-74EB-477F-A9D9-AF44A2544855}" name="Tabela dinâmica3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Faixa Etária" colHeaderCaption="Tipo de Movimentação">
   <location ref="Y14:Z20" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -19743,43 +20580,43 @@
     <dataField name="Contagem de Jogadores" fld="8" subtotal="count" baseField="8" baseItem="0"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="8">
+    <format dxfId="54">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="7">
+    <format dxfId="53">
       <pivotArea field="8" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="6">
+    <format dxfId="52">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="5">
+    <format dxfId="51">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="4">
+    <format dxfId="50">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="3">
+    <format dxfId="49">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="2">
+    <format dxfId="48">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="1">
+    <format dxfId="47">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="0">
+    <format dxfId="46">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -19806,7 +20643,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{904CEA3A-CD0A-459C-A420-1FB249800D4C}" name="Tabela dinâmica4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Nacionalidades" colHeaderCaption="Contagem de Jogadores">
   <location ref="AK14:AL29" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
@@ -19939,37 +20776,37 @@
     <dataField name="Contagem de Nacionalidades" fld="3" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="7">
-    <format dxfId="15">
+    <format dxfId="61">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="14">
+    <format dxfId="60">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="13">
+    <format dxfId="59">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="12">
+    <format dxfId="58">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="11">
+    <format dxfId="57">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="10">
+    <format dxfId="56">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="9">
+    <format dxfId="55">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -19996,7 +20833,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
   <location ref="O14:P19" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -20065,39 +20902,39 @@
     <dataField name="Soma do Valor das Transferências" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="24">
+    <format dxfId="70">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="23">
+    <format dxfId="69">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="22">
+    <format dxfId="68">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="21">
+    <format dxfId="67">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="20">
+    <format dxfId="66">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="19">
+    <format dxfId="65">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="18">
+    <format dxfId="64">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="17">
+    <format dxfId="63">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="16">
+    <format dxfId="62">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -20124,7 +20961,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6" rowHeaderCaption="Temporadas" colHeaderCaption="">
   <location ref="A14:D22" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -20199,34 +21036,34 @@
     <dataField name="Somas de Entradas e Saídas" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="30">
+    <format dxfId="76">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="29">
+    <format dxfId="75">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="28">
+    <format dxfId="74">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="27">
+    <format dxfId="73">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="26">
+    <format dxfId="72">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="25">
+    <format dxfId="71">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -20268,7 +21105,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4F5027D2-D537-4505-8DBC-54A417F72129}" name="Tabela dinâmica8" cacheId="0" dataPosition="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10" rowHeaderCaption="Posições e Jogadores" colHeaderCaption="Tipo de Movimentação">
   <location ref="BA14:BC26" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
   <pivotFields count="10">
@@ -20398,7 +21235,7 @@
     <dataField name="Porcentagem (%) do Total" fld="6" showDataAs="percentOfTotal" baseField="0" baseItem="0" numFmtId="10"/>
   </dataFields>
   <formats count="18">
-    <format dxfId="48">
+    <format dxfId="94">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -20407,7 +21244,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="47">
+    <format dxfId="93">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -20420,7 +21257,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="46">
+    <format dxfId="92">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -20429,7 +21266,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="45">
+    <format dxfId="91">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -20442,7 +21279,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="44">
+    <format dxfId="90">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -20451,7 +21288,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="43">
+    <format dxfId="89">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -20464,26 +21301,26 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="42">
+    <format dxfId="88">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="41">
+    <format dxfId="87">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="40">
+    <format dxfId="86">
       <pivotArea field="-2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="1"/>
     </format>
-    <format dxfId="39">
+    <format dxfId="85">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="38">
+    <format dxfId="84">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="37">
+    <format dxfId="83">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -20496,7 +21333,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="36">
+    <format dxfId="82">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -20509,7 +21346,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="35">
+    <format dxfId="81">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -20522,14 +21359,14 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="34">
+    <format dxfId="80">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="33">
+    <format dxfId="79">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -20540,10 +21377,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="32">
+    <format dxfId="78">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="31">
+    <format dxfId="77">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
@@ -20922,653 +21759,6 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FB686887-B509-4E7E-B605-6A13972A6E0B}" name="Tabela dinâmica5" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Origem das Contratações" colHeaderCaption="Contagem de Jogadores">
-  <location ref="AN14:AO47" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="9">
-    <pivotField axis="axisCol" showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item h="1" x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" dataField="1" showAll="0">
-      <items count="15">
-        <item x="6"/>
-        <item x="4"/>
-        <item x="9"/>
-        <item x="11"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="12"/>
-        <item x="5"/>
-        <item x="10"/>
-        <item x="13"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="21">
-        <item x="12"/>
-        <item x="9"/>
-        <item x="7"/>
-        <item x="15"/>
-        <item x="5"/>
-        <item x="17"/>
-        <item x="11"/>
-        <item x="10"/>
-        <item x="2"/>
-        <item x="8"/>
-        <item x="18"/>
-        <item x="13"/>
-        <item x="0"/>
-        <item x="16"/>
-        <item x="19"/>
-        <item x="1"/>
-        <item x="4"/>
-        <item x="3"/>
-        <item x="14"/>
-        <item x="6"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="2">
-    <field x="4"/>
-    <field x="3"/>
-  </rowFields>
-  <rowItems count="32">
-    <i>
-      <x v="2"/>
-    </i>
-    <i r="1">
-      <x/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i r="1">
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i r="1">
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i r="1">
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i r="1">
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i r="1">
-      <x v="12"/>
-    </i>
-    <i r="1">
-      <x v="13"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i r="1">
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="11"/>
-    </i>
-    <i r="1">
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="12"/>
-    </i>
-    <i r="1">
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="13"/>
-    </i>
-    <i r="1">
-      <x v="11"/>
-    </i>
-    <i>
-      <x v="15"/>
-    </i>
-    <i r="1">
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="16"/>
-    </i>
-    <i r="1">
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="17"/>
-    </i>
-    <i r="1">
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="18"/>
-    </i>
-    <i r="1">
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="19"/>
-    </i>
-    <i r="1">
-      <x v="9"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="0"/>
-  </colFields>
-  <colItems count="1">
-    <i>
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Clubes" fld="3" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="46">
-    <format dxfId="94">
-      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="93">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="92">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="91">
-      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
-    </format>
-    <format dxfId="90">
-      <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
-    </format>
-    <format dxfId="89">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="4" count="15">
-            <x v="2"/>
-            <x v="5"/>
-            <x v="6"/>
-            <x v="7"/>
-            <x v="8"/>
-            <x v="9"/>
-            <x v="10"/>
-            <x v="11"/>
-            <x v="12"/>
-            <x v="13"/>
-            <x v="15"/>
-            <x v="16"/>
-            <x v="17"/>
-            <x v="18"/>
-            <x v="19"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="88">
-      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="87">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="0"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="86">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="8"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="5"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="85">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="10"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="6"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="84">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="2"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="7"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="83">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="3"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="8"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="82">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="2">
-            <x v="12"/>
-            <x v="13"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="9"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="81">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="8"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="10"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="80">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="8"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="11"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="79">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="6"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="12"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="78">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="11"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="13"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="77">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="7"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="15"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="76">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="5"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="16"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="75">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="4"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="17"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="74">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="7"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="18"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="73">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="9"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="19"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="72">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="0" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="71">
-      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="70">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="69">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="68">
-      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
-    </format>
-    <format dxfId="67">
-      <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
-    </format>
-    <format dxfId="66">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="4" count="15">
-            <x v="2"/>
-            <x v="5"/>
-            <x v="6"/>
-            <x v="7"/>
-            <x v="8"/>
-            <x v="9"/>
-            <x v="10"/>
-            <x v="11"/>
-            <x v="12"/>
-            <x v="13"/>
-            <x v="15"/>
-            <x v="16"/>
-            <x v="17"/>
-            <x v="18"/>
-            <x v="19"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="65">
-      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="64">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="0"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="63">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="8"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="5"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="62">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="10"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="6"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="61">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="2"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="7"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="60">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="3"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="8"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="59">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="2">
-            <x v="12"/>
-            <x v="13"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="9"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="58">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="8"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="10"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="57">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="8"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="11"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="56">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="6"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="12"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="55">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="11"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="13"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="54">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="7"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="15"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="53">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="5"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="16"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="52">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="4"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="17"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="51">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="7"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="18"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="50">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="3" count="1">
-            <x v="9"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="19"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="49">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="0" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-  </formats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>

</xml_diff>

<commit_message>
57. Comentários sobre a Análise
Comentários sobre a sexta análise na aba Anotações.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D15BDF6F-27AE-4031-8608-CC882EF7A127}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2336FE0A-C6B5-4139-9893-38E32793DF67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Apresentação" sheetId="3" r:id="rId1"/>
@@ -18283,7 +18283,7 @@
       <xdr:row>41</xdr:row>
       <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="12148329" cy="7403693"/>
+    <xdr:ext cx="12148329" cy="7795083"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="6" name="CaixaDeTexto 5">
@@ -18298,7 +18298,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="190500" y="7867650"/>
-          <a:ext cx="12148329" cy="7403693"/>
+          <a:ext cx="12148329" cy="7795083"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -19028,7 +19028,43 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>•</a:t>
+            <a:t>• </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="1">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>6ª análise: </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>A sexta análise</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> consistiu, basicamente, em identificar quais foram as principais características que estiveram presentes durante o período analisado, sem a presença de qualquer tabela dinâmica ou gráfico. Este processo ocorreu por meio do resumo de todas as análises anteriores e como elas se conectavam umas com as outras. No final, foi possível concluir aspectos importantes sobre o comportamento do Tottenham Hotspur.</a:t>
           </a:r>
           <a:endParaRPr lang="pt-BR" sz="1200"/>
         </a:p>

</xml_diff>

<commit_message>
58. Ajuste do Comentário
Ajuste do comentário.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2336FE0A-C6B5-4139-9893-38E32793DF67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AE094A3-2398-4DF6-B1AE-789D5EEA3546}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19119,11 +19119,11 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>276225</xdr:colOff>
+      <xdr:colOff>177840</xdr:colOff>
       <xdr:row>82</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
+      <xdr:rowOff>123825</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="1089722" cy="327141"/>
+    <xdr:ext cx="2086598" cy="327141"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="7" name="CaixaDeTexto 6">
@@ -19137,8 +19137,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="276225" y="15697200"/>
-          <a:ext cx="1089722" cy="327141"/>
+          <a:off x="177840" y="15744825"/>
+          <a:ext cx="2086598" cy="327141"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -19168,8 +19168,72 @@
           <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="pt-BR" sz="1500" b="1"/>
-            <a:t>2. Análises:</a:t>
-          </a:r>
+            <a:t>3. Auxílio para Gráficos:</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>190500</xdr:colOff>
+      <xdr:row>84</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="12148329" cy="280205"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="9" name="CaixaDeTexto 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{65745CC7-F6D1-4837-864A-3EBFD68BB3F5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="190500" y="16097250"/>
+          <a:ext cx="12148329" cy="280205"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200"/>
+            <a:t>Essa</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1200" baseline="0"/>
+            <a:t> seção foi criada com o objetivo de auxiliar a criação dos gráficos presentes na aba anterior através da inserção de tabelas.</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1200"/>
         </a:p>
       </xdr:txBody>
     </xdr:sp>

</xml_diff>

<commit_message>
67. Ajuste na aba Apresentação
Leve ajuste na aba Apresentação.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F35F9247-9EE9-4CE2-8AC1-3003C89A2DCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{681008FF-7272-44B6-8A66-C8C4BF480717}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Apresentação" sheetId="3" r:id="rId1"/>
@@ -847,6 +847,24 @@
   </cellStyles>
   <dxfs count="95">
     <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="165" formatCode="0.0%"/>
     </dxf>
     <dxf>
@@ -1088,24 +1106,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="general"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
     </dxf>
     <dxf>
       <alignment horizontal="center"/>
@@ -11811,7 +11811,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Dashboard: </a:t>
+            <a:t>Anotações: </a:t>
           </a:r>
           <a:r>
             <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0">
@@ -11823,7 +11823,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>aba contendo o dashboard que será construído através da utilização de métricas importantes obtidas durante o processo das análises.</a:t>
+            <a:t>aba onde estarão disponíveis alguns de meus pensamentos e justificativas relacionadas a determinadas decisões que tomei durante a construção do projeto.</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -11873,52 +11873,16 @@
             <a:defRPr/>
           </a:pPr>
           <a:r>
-            <a:rPr lang="pt-BR" sz="1200" b="0">
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>•</a:t>
-          </a:r>
-          <a:r>
             <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0">
               <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t> </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1200" b="1" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Anotações: </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="pt-BR" sz="1200" b="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>aba onde estarão disponíveis alguns de meus pensamentos e justificativas relacionadas a determinadas decisões que tomei durante a construção do projeto.</a:t>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>O dashboard das análises estará disponível em um arquivo .pbix do Power BI e em uma pasta diferente.</a:t>
           </a:r>
           <a:endParaRPr lang="pt-BR" sz="1200">
             <a:solidFill>
@@ -19957,6 +19921,150 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6" rowHeaderCaption="Temporadas" colHeaderCaption="">
+  <location ref="A14:D22" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="10">
+    <pivotField axis="axisRow" showAll="0">
+      <items count="7">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="7">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="1"/>
+  </colFields>
+  <colItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Somas de Entradas e Saídas" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
+  </dataFields>
+  <formats count="6">
+    <format dxfId="5">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="4">
+      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="3">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="2">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="1" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="1">
+      <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="0">
+      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="2">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4F5027D2-D537-4505-8DBC-54A417F72129}" name="Tabela dinâmica8" cacheId="0" dataPosition="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10" rowHeaderCaption="Posições e Jogadores" colHeaderCaption="Tipo de Movimentação">
   <location ref="BA14:BC26" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
   <pivotFields count="10">
@@ -20086,7 +20194,7 @@
     <dataField name="Porcentagem (%) do Total" fld="6" showDataAs="percentOfTotal" baseField="0" baseItem="0" numFmtId="10"/>
   </dataFields>
   <formats count="18">
-    <format dxfId="17">
+    <format dxfId="23">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -20095,7 +20203,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="16">
+    <format dxfId="22">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -20108,7 +20216,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="15">
+    <format dxfId="21">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -20117,7 +20225,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="14">
+    <format dxfId="20">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -20130,7 +20238,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="13">
+    <format dxfId="19">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -20139,7 +20247,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="12">
+    <format dxfId="18">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -20152,26 +20260,26 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="11">
+    <format dxfId="17">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="10">
+    <format dxfId="16">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="9">
+    <format dxfId="15">
       <pivotArea field="-2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="1"/>
     </format>
-    <format dxfId="8">
+    <format dxfId="14">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="7">
+    <format dxfId="13">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="6">
+    <format dxfId="12">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -20184,7 +20292,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="5">
+    <format dxfId="11">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -20197,7 +20305,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="4">
+    <format dxfId="10">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -20210,14 +20318,14 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="3">
+    <format dxfId="9">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="2">
+    <format dxfId="8">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -20228,10 +20336,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="1">
+    <format dxfId="7">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="0">
+    <format dxfId="6">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
@@ -20610,7 +20718,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FB686887-B509-4E7E-B605-6A13972A6E0B}" name="Tabela dinâmica5" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Origem das Contratações" colHeaderCaption="Contagem de Jogadores">
   <location ref="AN14:AO47" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
@@ -20786,22 +20894,22 @@
     <dataField name="Clubes" fld="3" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="46">
-    <format dxfId="63">
+    <format dxfId="69">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="62">
+    <format dxfId="68">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="61">
+    <format dxfId="67">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="60">
+    <format dxfId="66">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="59">
+    <format dxfId="65">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="58">
+    <format dxfId="64">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="15">
@@ -20824,10 +20932,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="57">
+    <format dxfId="63">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="56">
+    <format dxfId="62">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20839,7 +20947,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="55">
+    <format dxfId="61">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20851,7 +20959,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="54">
+    <format dxfId="60">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20863,7 +20971,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="53">
+    <format dxfId="59">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20875,7 +20983,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="52">
+    <format dxfId="58">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20887,7 +20995,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="51">
+    <format dxfId="57">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="2">
@@ -20900,7 +21008,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="50">
+    <format dxfId="56">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20912,7 +21020,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="49">
+    <format dxfId="55">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20924,7 +21032,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="48">
+    <format dxfId="54">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20936,7 +21044,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="47">
+    <format dxfId="53">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20948,7 +21056,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="46">
+    <format dxfId="52">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20960,7 +21068,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="45">
+    <format dxfId="51">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20972,7 +21080,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="44">
+    <format dxfId="50">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20984,7 +21092,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="43">
+    <format dxfId="49">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20996,7 +21104,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="42">
+    <format dxfId="48">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21008,29 +21116,29 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="41">
+    <format dxfId="47">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="40">
+    <format dxfId="46">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="39">
+    <format dxfId="45">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="38">
+    <format dxfId="44">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="37">
+    <format dxfId="43">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="36">
+    <format dxfId="42">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="35">
+    <format dxfId="41">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="15">
@@ -21053,10 +21161,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="34">
+    <format dxfId="40">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="33">
+    <format dxfId="39">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21068,7 +21176,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="32">
+    <format dxfId="38">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21080,7 +21188,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="31">
+    <format dxfId="37">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21092,7 +21200,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="30">
+    <format dxfId="36">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21104,7 +21212,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="29">
+    <format dxfId="35">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21116,7 +21224,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="28">
+    <format dxfId="34">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="2">
@@ -21129,7 +21237,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="27">
+    <format dxfId="33">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21141,7 +21249,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="26">
+    <format dxfId="32">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21153,7 +21261,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="25">
+    <format dxfId="31">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21165,7 +21273,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="24">
+    <format dxfId="30">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21177,7 +21285,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="23">
+    <format dxfId="29">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21189,7 +21297,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="22">
+    <format dxfId="28">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21201,7 +21309,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="21">
+    <format dxfId="27">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21213,7 +21321,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="20">
+    <format dxfId="26">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21225,7 +21333,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="19">
+    <format dxfId="25">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21237,7 +21345,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="18">
+    <format dxfId="24">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
@@ -21257,7 +21365,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{996EC5F2-74EB-477F-A9D9-AF44A2544855}" name="Tabela dinâmica3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Faixa Etária" colHeaderCaption="Tipo de Movimentação">
   <location ref="Y14:Z20" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -21334,43 +21442,43 @@
     <dataField name="Contagem de Jogadores" fld="8" subtotal="count" baseField="8" baseItem="0"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="72">
+    <format dxfId="78">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="71">
+    <format dxfId="77">
       <pivotArea field="8" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="70">
+    <format dxfId="76">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="69">
+    <format dxfId="75">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="68">
+    <format dxfId="74">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="67">
+    <format dxfId="73">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="66">
+    <format dxfId="72">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="65">
+    <format dxfId="71">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="64">
+    <format dxfId="70">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -21397,7 +21505,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{904CEA3A-CD0A-459C-A420-1FB249800D4C}" name="Tabela dinâmica4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Nacionalidades" colHeaderCaption="Contagem de Jogadores">
   <location ref="AK14:AL29" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
@@ -21530,37 +21638,37 @@
     <dataField name="Contagem de Nacionalidades" fld="3" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="7">
-    <format dxfId="79">
+    <format dxfId="85">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="78">
+    <format dxfId="84">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="77">
+    <format dxfId="83">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="76">
+    <format dxfId="82">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="75">
+    <format dxfId="81">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="74">
+    <format dxfId="80">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="73">
+    <format dxfId="79">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -21587,7 +21695,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
   <location ref="O14:P19" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -21656,39 +21764,39 @@
     <dataField name="Soma do Valor das Transferências" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="88">
+    <format dxfId="94">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="87">
+    <format dxfId="93">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="86">
+    <format dxfId="92">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="85">
+    <format dxfId="91">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="84">
+    <format dxfId="90">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="83">
+    <format dxfId="89">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="82">
+    <format dxfId="88">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="81">
+    <format dxfId="87">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="80">
+    <format dxfId="86">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -21698,150 +21806,6 @@
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
             <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6" rowHeaderCaption="Temporadas" colHeaderCaption="">
-  <location ref="A14:D22" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="10">
-    <pivotField axis="axisRow" showAll="0">
-      <items count="7">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisCol" showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="7">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="1"/>
-  </colFields>
-  <colItems count="3">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Somas de Entradas e Saídas" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
-  </dataFields>
-  <formats count="6">
-    <format dxfId="94">
-      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
-        <references count="1">
-          <reference field="0" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="93">
-      <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
-    </format>
-    <format dxfId="92">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="0" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="91">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="1" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="90">
-      <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="89">
-      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="2">
-    <chartFormat chart="0" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="1" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="1"/>
           </reference>
         </references>
       </pivotArea>

</xml_diff>

<commit_message>
73. Estruturação das Pastas
Estruturação (possivelmente final) das pastas do projeto.
</commit_message>
<xml_diff>
--- a/notebooks/tottenham_transferencias.xlsx
+++ b/notebooks/tottenham_transferencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaike\OneDrive\Documentos\GitHub\projeto-tottenham\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{681008FF-7272-44B6-8A66-C8C4BF480717}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C56FFC4-1F7C-4017-9715-1981A18B29DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -847,6 +847,33 @@
   </cellStyles>
   <dxfs count="95">
     <dxf>
+      <alignment horizontal="general"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center"/>
     </dxf>
     <dxf>
@@ -1079,33 +1106,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general"/>
     </dxf>
     <dxf>
       <alignment horizontal="center"/>
@@ -11435,7 +11435,7 @@
           </a:r>
           <a:r>
             <a:rPr lang="pt-BR" sz="1200" baseline="0"/>
-            <a:t> com o total de 6 abas, cada uma representando uma etapa diferente. São elas:</a:t>
+            <a:t> com o total de 5 abas, cada uma representando uma etapa diferente. São elas:</a:t>
           </a:r>
           <a:endParaRPr lang="pt-BR" sz="1200" b="0" baseline="0"/>
         </a:p>
@@ -11882,7 +11882,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>O dashboard das análises estará disponível em um arquivo .pbix do Power BI e em uma pasta diferente.</a:t>
+            <a:t>O dashboard das análises está disponível em um arquivo .pbix do Power BI e em uma pasta diferente.</a:t>
           </a:r>
           <a:endParaRPr lang="pt-BR" sz="1200">
             <a:solidFill>
@@ -19921,6 +19921,134 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
+  <location ref="O14:P19" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="10">
+    <pivotField showAll="0"/>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="3">
+        <item h="1" x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0" sortType="descending">
+      <items count="4">
+        <item x="1"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="2">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+            <reference field="1" count="1" selected="0">
+              <x v="1"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="3"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="1"/>
+  </colFields>
+  <colItems count="1">
+    <i>
+      <x v="1"/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Soma do Valor das Transferências" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
+  </dataFields>
+  <formats count="9">
+    <format dxfId="8">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="7">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="6">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="5">
+      <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
+    </format>
+    <format dxfId="4">
+      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="3">
+      <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="2">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="3" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="1">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="1" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="0">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="1">
+    <chartFormat chart="1" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C0F863BA-AE4A-4439-B2F0-5F549C05D0FD}" name="Tabela dinâmica1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6" rowHeaderCaption="Temporadas" colHeaderCaption="">
   <location ref="A14:D22" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -19995,34 +20123,34 @@
     <dataField name="Somas de Entradas e Saídas" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="5">
+    <format dxfId="14">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="4">
+    <format dxfId="13">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="3">
+    <format dxfId="12">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="2">
+    <format dxfId="11">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="1">
+    <format dxfId="10">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="0">
+    <format dxfId="9">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -20064,7 +20192,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4F5027D2-D537-4505-8DBC-54A417F72129}" name="Tabela dinâmica8" cacheId="0" dataPosition="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10" rowHeaderCaption="Posições e Jogadores" colHeaderCaption="Tipo de Movimentação">
   <location ref="BA14:BC26" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
   <pivotFields count="10">
@@ -20194,7 +20322,7 @@
     <dataField name="Porcentagem (%) do Total" fld="6" showDataAs="percentOfTotal" baseField="0" baseItem="0" numFmtId="10"/>
   </dataFields>
   <formats count="18">
-    <format dxfId="23">
+    <format dxfId="32">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -20203,7 +20331,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="22">
+    <format dxfId="31">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -20216,7 +20344,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="21">
+    <format dxfId="30">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -20225,7 +20353,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="20">
+    <format dxfId="29">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -20238,7 +20366,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="19">
+    <format dxfId="28">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -20247,7 +20375,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="18">
+    <format dxfId="27">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -20260,26 +20388,26 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="17">
+    <format dxfId="26">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="16">
+    <format dxfId="25">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="15">
+    <format dxfId="24">
       <pivotArea field="-2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="1"/>
     </format>
-    <format dxfId="14">
+    <format dxfId="23">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="13">
+    <format dxfId="22">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="12">
+    <format dxfId="21">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -20292,7 +20420,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="11">
+    <format dxfId="20">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -20305,7 +20433,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="10">
+    <format dxfId="19">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="2">
@@ -20318,14 +20446,14 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="9">
+    <format dxfId="18">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="8">
+    <format dxfId="17">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -20336,10 +20464,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="7">
+    <format dxfId="16">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="6">
+    <format dxfId="15">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
@@ -20718,7 +20846,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FB686887-B509-4E7E-B605-6A13972A6E0B}" name="Tabela dinâmica5" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Origem das Contratações" colHeaderCaption="Contagem de Jogadores">
   <location ref="AN14:AO47" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
@@ -20894,22 +21022,22 @@
     <dataField name="Clubes" fld="3" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="46">
-    <format dxfId="69">
+    <format dxfId="78">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="68">
+    <format dxfId="77">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="67">
+    <format dxfId="76">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="66">
+    <format dxfId="75">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="65">
+    <format dxfId="74">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="64">
+    <format dxfId="73">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="15">
@@ -20932,10 +21060,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="63">
+    <format dxfId="72">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="62">
+    <format dxfId="71">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20947,7 +21075,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="61">
+    <format dxfId="70">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20959,7 +21087,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="60">
+    <format dxfId="69">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20971,7 +21099,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="59">
+    <format dxfId="68">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20983,7 +21111,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="58">
+    <format dxfId="67">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -20995,7 +21123,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="57">
+    <format dxfId="66">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="2">
@@ -21008,7 +21136,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="56">
+    <format dxfId="65">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21020,7 +21148,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="55">
+    <format dxfId="64">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21032,7 +21160,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="54">
+    <format dxfId="63">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21044,7 +21172,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="53">
+    <format dxfId="62">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21056,7 +21184,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="52">
+    <format dxfId="61">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21068,7 +21196,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="51">
+    <format dxfId="60">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21080,7 +21208,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="50">
+    <format dxfId="59">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21092,7 +21220,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="49">
+    <format dxfId="58">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21104,7 +21232,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="48">
+    <format dxfId="57">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21116,29 +21244,29 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="47">
+    <format dxfId="56">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="46">
+    <format dxfId="55">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="45">
+    <format dxfId="54">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="44">
+    <format dxfId="53">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="43">
+    <format dxfId="52">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="42">
+    <format dxfId="51">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="41">
+    <format dxfId="50">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="15">
@@ -21161,10 +21289,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="40">
+    <format dxfId="49">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="39">
+    <format dxfId="48">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21176,7 +21304,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="38">
+    <format dxfId="47">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21188,7 +21316,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="37">
+    <format dxfId="46">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21200,7 +21328,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="36">
+    <format dxfId="45">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21212,7 +21340,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="35">
+    <format dxfId="44">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21224,7 +21352,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="34">
+    <format dxfId="43">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="2">
@@ -21237,7 +21365,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="33">
+    <format dxfId="42">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21249,7 +21377,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="32">
+    <format dxfId="41">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21261,7 +21389,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="31">
+    <format dxfId="40">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21273,7 +21401,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="30">
+    <format dxfId="39">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21285,7 +21413,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="29">
+    <format dxfId="38">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21297,7 +21425,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="28">
+    <format dxfId="37">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21309,7 +21437,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="27">
+    <format dxfId="36">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21321,7 +21449,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="26">
+    <format dxfId="35">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21333,7 +21461,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="25">
+    <format dxfId="34">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1">
@@ -21345,7 +21473,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="24">
+    <format dxfId="33">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
@@ -21365,7 +21493,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{996EC5F2-74EB-477F-A9D9-AF44A2544855}" name="Tabela dinâmica3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Faixa Etária" colHeaderCaption="Tipo de Movimentação">
   <location ref="Y14:Z20" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
@@ -21442,43 +21570,43 @@
     <dataField name="Contagem de Jogadores" fld="8" subtotal="count" baseField="8" baseItem="0"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="78">
+    <format dxfId="87">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="77">
+    <format dxfId="86">
       <pivotArea field="8" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="76">
+    <format dxfId="85">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="8" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="75">
+    <format dxfId="84">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="74">
+    <format dxfId="83">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="73">
+    <format dxfId="82">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="72">
+    <format dxfId="81">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="71">
+    <format dxfId="80">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="70">
+    <format dxfId="79">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -21505,7 +21633,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{904CEA3A-CD0A-459C-A420-1FB249800D4C}" name="Tabela dinâmica4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Nacionalidades" colHeaderCaption="Contagem de Jogadores">
   <location ref="AK14:AL29" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="9">
@@ -21638,166 +21766,38 @@
     <dataField name="Contagem de Nacionalidades" fld="3" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="7">
-    <format dxfId="85">
+    <format dxfId="94">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="84">
+    <format dxfId="93">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="83">
+    <format dxfId="92">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="82">
+    <format dxfId="91">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="81">
+    <format dxfId="90">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="80">
+    <format dxfId="89">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="79">
+    <format dxfId="88">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="1">
-    <chartFormat chart="1" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70C1B1E3-0FD2-4659-8C22-185FC5338B5D}" name="Tabela dinâmica2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="Posições" colHeaderCaption="Tipo de Movimentação">
-  <location ref="O14:P19" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="10">
-    <pivotField showAll="0"/>
-    <pivotField axis="axisCol" showAll="0">
-      <items count="3">
-        <item h="1" x="1"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0" sortType="descending">
-      <items count="4">
-        <item x="1"/>
-        <item x="2"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-      <autoSortScope>
-        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
-          <references count="2">
-            <reference field="4294967294" count="1" selected="0">
-              <x v="0"/>
-            </reference>
-            <reference field="1" count="1" selected="0">
-              <x v="1"/>
-            </reference>
-          </references>
-        </pivotArea>
-      </autoSortScope>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="3"/>
-  </rowFields>
-  <rowItems count="4">
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="1"/>
-  </colFields>
-  <colItems count="1">
-    <i>
-      <x v="1"/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Soma do Valor das Transferências" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
-  </dataFields>
-  <formats count="9">
-    <format dxfId="94">
-      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="93">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="92">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="91">
-      <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
-    </format>
-    <format dxfId="90">
-      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="89">
-      <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
-    </format>
-    <format dxfId="88">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="3" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="87">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="1" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="86">
-      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
   <chartFormats count="1">

</xml_diff>